<commit_message>
Build: (de90e76) Add fights and enemies
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:D7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -409,72 +409,88 @@
       <c r="C1" t="str">
         <v>Element 2</v>
       </c>
+      <c r="D1" t="str">
+        <v>Damage</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Aqua</v>
+        <v>💧</v>
       </c>
       <c r="B2" t="str">
         <v/>
       </c>
+      <c r="D2" t="str">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Fire</v>
+        <v>🔥</v>
       </c>
       <c r="B3" t="str">
         <v/>
       </c>
+      <c r="D3" t="str">
+        <v>10</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Ground</v>
+        <v>🍃</v>
       </c>
       <c r="B4" t="str">
         <v/>
       </c>
+      <c r="D4" t="str">
+        <v>10</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Steam</v>
+        <v>💨</v>
       </c>
       <c r="B5" t="str">
-        <v>Aqua</v>
+        <v>💧</v>
       </c>
       <c r="C5" t="str">
-        <v>Fire</v>
+        <v>🔥</v>
+      </c>
+      <c r="D5" t="str">
+        <v>150</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Lava</v>
+        <v>💥</v>
       </c>
       <c r="B6" t="str">
-        <v>Ground</v>
+        <v>🍃</v>
       </c>
       <c r="C6" t="str">
-        <v>Fire</v>
+        <v>🔥</v>
+      </c>
+      <c r="D6" t="str">
+        <v>500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Rock</v>
+        <v>🌍</v>
       </c>
       <c r="B7" t="str">
-        <v>Water</v>
+        <v>💧</v>
       </c>
       <c r="C7" t="str">
-        <v>Ground</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Lightning</v>
+        <v>🍃</v>
+      </c>
+      <c r="D7" t="str">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (30e2c00) Add levels and experience
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -488,9 +488,14 @@
         <v>200</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>⚡</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (bf869e7) Add description and levels to elements
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:F8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,6 +412,12 @@
       <c r="D1" t="str">
         <v>Damage</v>
       </c>
+      <c r="E1" t="str">
+        <v>Level</v>
+      </c>
+      <c r="F1" t="str">
+        <v>description</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -420,8 +426,17 @@
       <c r="B2" t="str">
         <v/>
       </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
       <c r="D2" t="str">
         <v>10</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Flowing water, adaptable and steady.</v>
       </c>
     </row>
     <row r="3">
@@ -431,8 +446,17 @@
       <c r="B3" t="str">
         <v/>
       </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
       <c r="D3" t="str">
         <v>10</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Raw flame that burns fast and hot.</v>
       </c>
     </row>
     <row r="4">
@@ -442,8 +466,17 @@
       <c r="B4" t="str">
         <v/>
       </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
       <c r="D4" t="str">
         <v>10</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Living growth guided by nature.</v>
       </c>
     </row>
     <row r="5">
@@ -459,6 +492,12 @@
       <c r="D5" t="str">
         <v>150</v>
       </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Scalding vapor that blurs the field.</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -473,6 +512,12 @@
       <c r="D6" t="str">
         <v>500</v>
       </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Volatile blast from nature and fire.</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -487,15 +532,36 @@
       <c r="D7" t="str">
         <v>200</v>
       </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Rooted earth, resilient and heavy.</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
         <v>⚡</v>
       </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Charged spark that strikes instantly.</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (b6f391e) Add rewards
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,7 +432,7 @@
       <c r="D2" t="str">
         <v>10</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="str">
         <v>1</v>
       </c>
       <c r="F2" t="str">
@@ -452,7 +452,7 @@
       <c r="D3" t="str">
         <v>10</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="str">
         <v>1</v>
       </c>
       <c r="F3" t="str">
@@ -472,7 +472,7 @@
       <c r="D4" t="str">
         <v>10</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="str">
         <v>1</v>
       </c>
       <c r="F4" t="str">
@@ -481,87 +481,203 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>💨</v>
-      </c>
-      <c r="B5" t="str">
-        <v>💧</v>
-      </c>
-      <c r="C5" t="str">
-        <v>🔥</v>
+        <v>⚡</v>
       </c>
       <c r="D5" t="str">
-        <v>150</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
+        <v>10</v>
+      </c>
+      <c r="E5" t="str">
+        <v>1</v>
       </c>
       <c r="F5" t="str">
-        <v>Scalding vapor that blurs the field.</v>
+        <v>Charged spark that strikes instantly.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>💥</v>
+        <v>🌊</v>
       </c>
       <c r="B6" t="str">
-        <v>🍃</v>
+        <v>💧</v>
       </c>
       <c r="C6" t="str">
-        <v>🔥</v>
+        <v>💧</v>
       </c>
       <c r="D6" t="str">
-        <v>500</v>
-      </c>
-      <c r="E6">
-        <v>2</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Volatile blast from nature and fire.</v>
+        <v>150</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>🌍</v>
+        <v>💨</v>
       </c>
       <c r="B7" t="str">
         <v>💧</v>
       </c>
       <c r="C7" t="str">
-        <v>🍃</v>
+        <v>🔥</v>
       </c>
       <c r="D7" t="str">
-        <v>200</v>
-      </c>
-      <c r="E7">
+        <v>150</v>
+      </c>
+      <c r="E7" t="str">
         <v>2</v>
       </c>
       <c r="F7" t="str">
-        <v>Rooted earth, resilient and heavy.</v>
+        <v>Scalding vapor that blurs the field.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>🌍</v>
+      </c>
+      <c r="B8" t="str">
+        <v>💧</v>
+      </c>
+      <c r="C8" t="str">
+        <v>🍃</v>
+      </c>
+      <c r="D8" t="str">
+        <v>200</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Rooted earth, resilient and heavy.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>🚢</v>
+      </c>
+      <c r="B9" t="str">
+        <v>💧</v>
+      </c>
+      <c r="C9" t="str">
         <v>⚡</v>
       </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Charged spark that strikes instantly.</v>
+      <c r="D9" t="str">
+        <v>200</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>🌲</v>
+      </c>
+      <c r="B10" t="str">
+        <v>🍃</v>
+      </c>
+      <c r="C10" t="str">
+        <v>🍃</v>
+      </c>
+      <c r="D10" t="str">
+        <v>250</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>💥</v>
+      </c>
+      <c r="B11" t="str">
+        <v>🍃</v>
+      </c>
+      <c r="C11" t="str">
+        <v>🔥</v>
+      </c>
+      <c r="D11" t="str">
+        <v>500</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Volatile blast from nature and fire.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>🚑</v>
+      </c>
+      <c r="B12" t="str">
+        <v>🍃</v>
+      </c>
+      <c r="C12" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="D12" t="str">
+        <v>200</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>🌞</v>
+      </c>
+      <c r="B13" t="str">
+        <v>🔥</v>
+      </c>
+      <c r="C13" t="str">
+        <v>🔥</v>
+      </c>
+      <c r="D13" t="str">
+        <v>550</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2</v>
+      </c>
+      <c r="F13" t="str">
+        <v>:)</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B14" t="str">
+        <v>🔥</v>
+      </c>
+      <c r="C14" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="D14" t="str">
+        <v>300</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>🛸</v>
+      </c>
+      <c r="B15" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C15" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="D15" t="str">
+        <v>350</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (9013a45) Added types & weakness, updated battle with some QOL changes
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:H15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,6 +418,9 @@
       <c r="F1" t="str">
         <v>description</v>
       </c>
+      <c r="G1" t="str">
+        <v>Type1</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -438,6 +441,9 @@
       <c r="F2" t="str">
         <v>Flowing water, adaptable and steady.</v>
       </c>
+      <c r="G2" t="str">
+        <v>Water</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -458,6 +464,9 @@
       <c r="F3" t="str">
         <v>Raw flame that burns fast and hot.</v>
       </c>
+      <c r="G3" t="str">
+        <v>Fire</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -478,6 +487,9 @@
       <c r="F4" t="str">
         <v>Living growth guided by nature.</v>
       </c>
+      <c r="G4" t="str">
+        <v>Earth</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -492,6 +504,9 @@
       <c r="F5" t="str">
         <v>Charged spark that strikes instantly.</v>
       </c>
+      <c r="G5" t="str">
+        <v>Lightning</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -509,6 +524,9 @@
       <c r="E6" t="str">
         <v>2</v>
       </c>
+      <c r="G6" t="str">
+        <v>Water</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -529,6 +547,9 @@
       <c r="F7" t="str">
         <v>Scalding vapor that blurs the field.</v>
       </c>
+      <c r="G7" t="str">
+        <v>Air</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -549,6 +570,9 @@
       <c r="F8" t="str">
         <v>Rooted earth, resilient and heavy.</v>
       </c>
+      <c r="G8" t="str">
+        <v>Earth</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -566,6 +590,12 @@
       <c r="E9" t="str">
         <v>2</v>
       </c>
+      <c r="G9" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Water</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -583,6 +613,9 @@
       <c r="E10" t="str">
         <v>2</v>
       </c>
+      <c r="G10" t="str">
+        <v>Earth</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -603,6 +636,12 @@
       <c r="F11" t="str">
         <v>Volatile blast from nature and fire.</v>
       </c>
+      <c r="G11" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Light</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -620,6 +659,9 @@
       <c r="E12" t="str">
         <v>2</v>
       </c>
+      <c r="G12" t="str">
+        <v>Steel</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -640,6 +682,9 @@
       <c r="F13" t="str">
         <v>:)</v>
       </c>
+      <c r="G13" t="str">
+        <v>Fire</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -657,6 +702,12 @@
       <c r="E14" t="str">
         <v>2</v>
       </c>
+      <c r="G14" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Fire</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -674,10 +725,16 @@
       <c r="E15" t="str">
         <v>2</v>
       </c>
+      <c r="G15" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Lightning</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (cb82753) Scaled down enemy. Updated element info
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -439,7 +439,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="str">
-        <v>Flowing water, adaptable and steady.</v>
+        <v>A gift from the sky goddess</v>
       </c>
       <c r="G2" t="str">
         <v>Water</v>
@@ -456,13 +456,13 @@
         <v/>
       </c>
       <c r="D3" t="str">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E3" t="str">
         <v>1</v>
       </c>
       <c r="F3" t="str">
-        <v>Raw flame that burns fast and hot.</v>
+        <v>A bright flame burning hot</v>
       </c>
       <c r="G3" t="str">
         <v>Fire</v>
@@ -479,13 +479,13 @@
         <v/>
       </c>
       <c r="D4" t="str">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E4" t="str">
         <v>1</v>
       </c>
       <c r="F4" t="str">
-        <v>Living growth guided by nature.</v>
+        <v>It's a leaf</v>
       </c>
       <c r="G4" t="str">
         <v>Earth</v>
@@ -502,7 +502,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="str">
-        <v>Charged spark that strikes instantly.</v>
+        <v>Charged spark that strikes instantly</v>
       </c>
       <c r="G5" t="str">
         <v>Lightning</v>
@@ -519,10 +519,13 @@
         <v>💧</v>
       </c>
       <c r="D6" t="str">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="E6" t="str">
         <v>2</v>
+      </c>
+      <c r="F6" t="str">
+        <v>The tide is high today my friend</v>
       </c>
       <c r="G6" t="str">
         <v>Water</v>
@@ -539,13 +542,13 @@
         <v>🔥</v>
       </c>
       <c r="D7" t="str">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="E7" t="str">
         <v>2</v>
       </c>
       <c r="F7" t="str">
-        <v>Scalding vapor that blurs the field.</v>
+        <v>Scalding vapor that burns deeper than flame</v>
       </c>
       <c r="G7" t="str">
         <v>Air</v>
@@ -553,7 +556,7 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>🌍</v>
+        <v>🌴</v>
       </c>
       <c r="B8" t="str">
         <v>💧</v>
@@ -562,13 +565,13 @@
         <v>🍃</v>
       </c>
       <c r="D8" t="str">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="E8" t="str">
         <v>2</v>
       </c>
       <c r="F8" t="str">
-        <v>Rooted earth, resilient and heavy.</v>
+        <v>A prickly palm tree</v>
       </c>
       <c r="G8" t="str">
         <v>Earth</v>
@@ -585,10 +588,13 @@
         <v>⚡</v>
       </c>
       <c r="D9" t="str">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="E9" t="str">
         <v>2</v>
+      </c>
+      <c r="F9" t="str">
+        <v>A bit bigger than a tugboat</v>
       </c>
       <c r="G9" t="str">
         <v>Steel</v>
@@ -613,6 +619,9 @@
       <c r="E10" t="str">
         <v>2</v>
       </c>
+      <c r="F10" t="str">
+        <v>Its pines are sharper than you may think</v>
+      </c>
       <c r="G10" t="str">
         <v>Earth</v>
       </c>
@@ -634,7 +643,7 @@
         <v>2</v>
       </c>
       <c r="F11" t="str">
-        <v>Volatile blast from nature and fire.</v>
+        <v>BOOM</v>
       </c>
       <c r="G11" t="str">
         <v>Fire</v>
@@ -659,6 +668,9 @@
       <c r="E12" t="str">
         <v>2</v>
       </c>
+      <c r="F12" t="str">
+        <v>Hurts AND heals! (ok, healing isnt implemented yet but it WILL heal eventually)</v>
+      </c>
       <c r="G12" t="str">
         <v>Steel</v>
       </c>
@@ -680,7 +692,7 @@
         <v>2</v>
       </c>
       <c r="F13" t="str">
-        <v>:)</v>
+        <v>A miniature sun in the palm of your hand</v>
       </c>
       <c r="G13" t="str">
         <v>Fire</v>
@@ -697,10 +709,13 @@
         <v>⚡</v>
       </c>
       <c r="D14" t="str">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="E14" t="str">
         <v>2</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Away we go!</v>
       </c>
       <c r="G14" t="str">
         <v>Steel</v>
@@ -720,10 +735,13 @@
         <v>⚡</v>
       </c>
       <c r="D15" t="str">
-        <v>350</v>
+        <v>600</v>
       </c>
       <c r="E15" t="str">
         <v>2</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Sure why not</v>
       </c>
       <c r="G15" t="str">
         <v>Steel</v>

</xml_diff>

<commit_message>
Build: (1deedf3) Add special effects
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:W15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,6 +421,54 @@
       <c r="G1" t="str">
         <v>Type1</v>
       </c>
+      <c r="H1" t="str">
+        <v>Type2</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Effect 1 Kind</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Effect 1 Amount</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Effect 1 Hits</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Effect 1 Duration</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Effect 1 Target</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Effect 2 Kind</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Effect 2 Amount</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Effect 2 Hits</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Effect 2 Duration</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Effect 2 Target</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Effect 3 Kind</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Effect 3 Amount</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Effect 3 Hits</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Effect 3 Duration</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Effect 3 Target</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -444,6 +492,15 @@
       <c r="G2" t="str">
         <v>Water</v>
       </c>
+      <c r="I2" t="str">
+        <v>heal</v>
+      </c>
+      <c r="J2" t="str">
+        <v>5</v>
+      </c>
+      <c r="M2" t="str">
+        <v>self</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -467,6 +524,15 @@
       <c r="G3" t="str">
         <v>Fire</v>
       </c>
+      <c r="I3" t="str">
+        <v>burn</v>
+      </c>
+      <c r="J3" t="str">
+        <v>1</v>
+      </c>
+      <c r="L3" t="str">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -490,6 +556,12 @@
       <c r="G4" t="str">
         <v>Earth</v>
       </c>
+      <c r="I4" t="str">
+        <v>shield</v>
+      </c>
+      <c r="J4" t="str">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -507,6 +579,12 @@
       <c r="G5" t="str">
         <v>Lightning</v>
       </c>
+      <c r="I5" t="str">
+        <v>multihit</v>
+      </c>
+      <c r="K5" t="str">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -752,7 +830,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (0cb4488) Add soak, freeze. Elements play off eachother better. QOL changes
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -501,6 +501,15 @@
       <c r="M2" t="str">
         <v>self</v>
       </c>
+      <c r="N2" t="str">
+        <v>soak</v>
+      </c>
+      <c r="O2" t="str">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>3</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">

</xml_diff>

<commit_message>
Build: (d56e301) Updating icons to be new fresh clean maybe bad
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -472,7 +472,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>💧</v>
+        <v>Water</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -481,7 +481,7 @@
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E2" t="str">
         <v>1</v>
@@ -492,12 +492,21 @@
       <c r="G2" t="str">
         <v>Water</v>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
       <c r="I2" t="str">
         <v>heal</v>
       </c>
       <c r="J2" t="str">
         <v>5</v>
       </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
       <c r="M2" t="str">
         <v>self</v>
       </c>
@@ -507,13 +516,34 @@
       <c r="O2" t="str">
         <v>1</v>
       </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
       <c r="Q2" t="str">
         <v>3</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>🔥</v>
+        <v>Fire</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -522,7 +552,7 @@
         <v/>
       </c>
       <c r="D3" t="str">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E3" t="str">
         <v>1</v>
@@ -533,19 +563,58 @@
       <c r="G3" t="str">
         <v>Fire</v>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
       <c r="I3" t="str">
         <v>burn</v>
       </c>
       <c r="J3" t="str">
         <v>1</v>
       </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
       <c r="L3" t="str">
         <v>3</v>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>🍃</v>
+        <v>Earth</v>
       </c>
       <c r="B4" t="str">
         <v/>
@@ -554,7 +623,7 @@
         <v/>
       </c>
       <c r="D4" t="str">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E4" t="str">
         <v>1</v>
@@ -565,19 +634,67 @@
       <c r="G4" t="str">
         <v>Earth</v>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
       <c r="I4" t="str">
         <v>shield</v>
       </c>
       <c r="J4" t="str">
         <v>5</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>⚡</v>
+        <v>Lightning</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
       </c>
       <c r="D5" t="str">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" t="str">
         <v>1</v>
@@ -588,11 +705,53 @@
       <c r="G5" t="str">
         <v>Lightning</v>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
       <c r="I5" t="str">
         <v>multihit</v>
       </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
       <c r="K5" t="str">
         <v>2</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -606,7 +765,7 @@
         <v>💧</v>
       </c>
       <c r="D6" t="str">
-        <v>200</v>
+        <v>38</v>
       </c>
       <c r="E6" t="str">
         <v>2</v>
@@ -616,6 +775,54 @@
       </c>
       <c r="G6" t="str">
         <v>Water</v>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -629,7 +836,7 @@
         <v>🔥</v>
       </c>
       <c r="D7" t="str">
-        <v>300</v>
+        <v>52</v>
       </c>
       <c r="E7" t="str">
         <v>2</v>
@@ -639,6 +846,54 @@
       </c>
       <c r="G7" t="str">
         <v>Air</v>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -652,7 +907,7 @@
         <v>🍃</v>
       </c>
       <c r="D8" t="str">
-        <v>350</v>
+        <v>48</v>
       </c>
       <c r="E8" t="str">
         <v>2</v>
@@ -662,6 +917,54 @@
       </c>
       <c r="G8" t="str">
         <v>Earth</v>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -675,7 +978,7 @@
         <v>⚡</v>
       </c>
       <c r="D9" t="str">
-        <v>400</v>
+        <v>62</v>
       </c>
       <c r="E9" t="str">
         <v>2</v>
@@ -688,6 +991,51 @@
       </c>
       <c r="H9" t="str">
         <v>Water</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -701,7 +1049,7 @@
         <v>🍃</v>
       </c>
       <c r="D10" t="str">
-        <v>250</v>
+        <v>44</v>
       </c>
       <c r="E10" t="str">
         <v>2</v>
@@ -711,6 +1059,54 @@
       </c>
       <c r="G10" t="str">
         <v>Earth</v>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+      <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -724,7 +1120,7 @@
         <v>🔥</v>
       </c>
       <c r="D11" t="str">
-        <v>500</v>
+        <v>86</v>
       </c>
       <c r="E11" t="str">
         <v>2</v>
@@ -737,6 +1133,51 @@
       </c>
       <c r="H11" t="str">
         <v>Light</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -750,7 +1191,7 @@
         <v>⚡</v>
       </c>
       <c r="D12" t="str">
-        <v>200</v>
+        <v>58</v>
       </c>
       <c r="E12" t="str">
         <v>2</v>
@@ -760,6 +1201,54 @@
       </c>
       <c r="G12" t="str">
         <v>Steel</v>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -773,7 +1262,7 @@
         <v>🔥</v>
       </c>
       <c r="D13" t="str">
-        <v>550</v>
+        <v>94</v>
       </c>
       <c r="E13" t="str">
         <v>2</v>
@@ -783,6 +1272,54 @@
       </c>
       <c r="G13" t="str">
         <v>Fire</v>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -796,7 +1333,7 @@
         <v>⚡</v>
       </c>
       <c r="D14" t="str">
-        <v>450</v>
+        <v>78</v>
       </c>
       <c r="E14" t="str">
         <v>2</v>
@@ -809,6 +1346,51 @@
       </c>
       <c r="H14" t="str">
         <v>Fire</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
+        <v/>
+      </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
+        <v/>
+      </c>
+      <c r="R14" t="str">
+        <v/>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
+      <c r="U14" t="str">
+        <v/>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -822,7 +1404,7 @@
         <v>⚡</v>
       </c>
       <c r="D15" t="str">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="E15" t="str">
         <v>2</v>
@@ -835,6 +1417,51 @@
       </c>
       <c r="H15" t="str">
         <v>Lightning</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Build: (85b8755) Add PLASMA!
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:W16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -756,96 +756,51 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Worble</v>
+        <v>Plasma</v>
       </c>
       <c r="B6" t="str">
-        <v>💧</v>
+        <v>Fire</v>
       </c>
       <c r="C6" t="str">
-        <v>💧</v>
+        <v>Lightning</v>
       </c>
       <c r="D6" t="str">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="str">
-        <v>The tide is high today my friend</v>
+        <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="G6" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="H6" t="str">
-        <v/>
-      </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6" t="str">
-        <v/>
-      </c>
-      <c r="L6" t="str">
-        <v/>
-      </c>
-      <c r="M6" t="str">
-        <v/>
-      </c>
-      <c r="N6" t="str">
-        <v/>
-      </c>
-      <c r="O6" t="str">
-        <v/>
-      </c>
-      <c r="P6" t="str">
-        <v/>
-      </c>
-      <c r="Q6" t="str">
-        <v/>
-      </c>
-      <c r="R6" t="str">
-        <v/>
-      </c>
-      <c r="S6" t="str">
-        <v/>
-      </c>
-      <c r="T6" t="str">
-        <v/>
-      </c>
-      <c r="U6" t="str">
-        <v/>
-      </c>
-      <c r="V6" t="str">
-        <v/>
-      </c>
-      <c r="W6" t="str">
-        <v/>
+        <v>Lightning</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>💨</v>
+        <v>Worble</v>
       </c>
       <c r="B7" t="str">
         <v>💧</v>
       </c>
       <c r="C7" t="str">
-        <v>🔥</v>
+        <v>💧</v>
       </c>
       <c r="D7" t="str">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="E7" t="str">
         <v>2</v>
       </c>
       <c r="F7" t="str">
-        <v>Scalding vapor that burns deeper than flame</v>
+        <v>The tide is high today my friend</v>
       </c>
       <c r="G7" t="str">
-        <v>Air</v>
+        <v>Water</v>
       </c>
       <c r="H7" t="str">
         <v/>
@@ -898,25 +853,25 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>🌴</v>
+        <v>💨</v>
       </c>
       <c r="B8" t="str">
         <v>💧</v>
       </c>
       <c r="C8" t="str">
-        <v>🍃</v>
+        <v>🔥</v>
       </c>
       <c r="D8" t="str">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E8" t="str">
         <v>2</v>
       </c>
       <c r="F8" t="str">
-        <v>A prickly palm tree</v>
+        <v>Scalding vapor that burns deeper than flame</v>
       </c>
       <c r="G8" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="H8" t="str">
         <v/>
@@ -969,28 +924,28 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>🚢</v>
+        <v>🌴</v>
       </c>
       <c r="B9" t="str">
         <v>💧</v>
       </c>
       <c r="C9" t="str">
-        <v>⚡</v>
+        <v>🍃</v>
       </c>
       <c r="D9" t="str">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="E9" t="str">
         <v>2</v>
       </c>
       <c r="F9" t="str">
-        <v>A bit bigger than a tugboat</v>
+        <v>A prickly palm tree</v>
       </c>
       <c r="G9" t="str">
-        <v>Steel</v>
+        <v>Earth</v>
       </c>
       <c r="H9" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -1040,28 +995,28 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>🌲</v>
+        <v>🚢</v>
       </c>
       <c r="B10" t="str">
-        <v>🍃</v>
+        <v>💧</v>
       </c>
       <c r="C10" t="str">
-        <v>🍃</v>
+        <v>⚡</v>
       </c>
       <c r="D10" t="str">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="E10" t="str">
         <v>2</v>
       </c>
       <c r="F10" t="str">
-        <v>Its pines are sharper than you may think</v>
+        <v>A bit bigger than a tugboat</v>
       </c>
       <c r="G10" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="I10" t="str">
         <v/>
@@ -1111,28 +1066,28 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>💥</v>
+        <v>🌲</v>
       </c>
       <c r="B11" t="str">
         <v>🍃</v>
       </c>
       <c r="C11" t="str">
-        <v>🔥</v>
+        <v>🍃</v>
       </c>
       <c r="D11" t="str">
-        <v>86</v>
+        <v>44</v>
       </c>
       <c r="E11" t="str">
         <v>2</v>
       </c>
       <c r="F11" t="str">
-        <v>BOOM</v>
+        <v>Its pines are sharper than you may think</v>
       </c>
       <c r="G11" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="H11" t="str">
-        <v>Light</v>
+        <v/>
       </c>
       <c r="I11" t="str">
         <v/>
@@ -1182,28 +1137,28 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>🚑</v>
+        <v>💥</v>
       </c>
       <c r="B12" t="str">
         <v>🍃</v>
       </c>
       <c r="C12" t="str">
-        <v>⚡</v>
+        <v>🔥</v>
       </c>
       <c r="D12" t="str">
-        <v>58</v>
+        <v>86</v>
       </c>
       <c r="E12" t="str">
         <v>2</v>
       </c>
       <c r="F12" t="str">
-        <v>Hurts AND heals! (ok, healing isnt implemented yet but it WILL heal eventually)</v>
+        <v>BOOM</v>
       </c>
       <c r="G12" t="str">
-        <v>Steel</v>
+        <v>Fire</v>
       </c>
       <c r="H12" t="str">
-        <v/>
+        <v>Light</v>
       </c>
       <c r="I12" t="str">
         <v/>
@@ -1253,25 +1208,25 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>🌞</v>
+        <v>🚑</v>
       </c>
       <c r="B13" t="str">
-        <v>🔥</v>
+        <v>🍃</v>
       </c>
       <c r="C13" t="str">
-        <v>🔥</v>
+        <v>⚡</v>
       </c>
       <c r="D13" t="str">
-        <v>94</v>
+        <v>58</v>
       </c>
       <c r="E13" t="str">
         <v>2</v>
       </c>
       <c r="F13" t="str">
-        <v>A miniature sun in the palm of your hand</v>
+        <v>Hurts AND heals! (ok, healing isnt implemented yet but it WILL heal eventually)</v>
       </c>
       <c r="G13" t="str">
-        <v>Fire</v>
+        <v>Steel</v>
       </c>
       <c r="H13" t="str">
         <v/>
@@ -1324,28 +1279,28 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>🚀</v>
+        <v>🌞</v>
       </c>
       <c r="B14" t="str">
         <v>🔥</v>
       </c>
       <c r="C14" t="str">
-        <v>⚡</v>
+        <v>🔥</v>
       </c>
       <c r="D14" t="str">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="E14" t="str">
         <v>2</v>
       </c>
       <c r="F14" t="str">
-        <v>Away we go!</v>
+        <v>A miniature sun in the palm of your hand</v>
       </c>
       <c r="G14" t="str">
-        <v>Steel</v>
+        <v>Fire</v>
       </c>
       <c r="H14" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
       <c r="I14" t="str">
         <v/>
@@ -1395,78 +1350,149 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>🛸</v>
+        <v>🚀</v>
       </c>
       <c r="B15" t="str">
-        <v>⚡</v>
+        <v>🔥</v>
       </c>
       <c r="C15" t="str">
         <v>⚡</v>
       </c>
       <c r="D15" t="str">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="E15" t="str">
         <v>2</v>
       </c>
       <c r="F15" t="str">
-        <v>Sure why not</v>
+        <v>Away we go!</v>
       </c>
       <c r="G15" t="str">
         <v>Steel</v>
       </c>
       <c r="H15" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>🛸</v>
+      </c>
+      <c r="B16" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C16" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="D16" t="str">
+        <v>100</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Sure why not</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="H16" t="str">
         <v>Lightning</v>
       </c>
-      <c r="I15" t="str">
-        <v/>
-      </c>
-      <c r="J15" t="str">
-        <v/>
-      </c>
-      <c r="K15" t="str">
-        <v/>
-      </c>
-      <c r="L15" t="str">
-        <v/>
-      </c>
-      <c r="M15" t="str">
-        <v/>
-      </c>
-      <c r="N15" t="str">
-        <v/>
-      </c>
-      <c r="O15" t="str">
-        <v/>
-      </c>
-      <c r="P15" t="str">
-        <v/>
-      </c>
-      <c r="Q15" t="str">
-        <v/>
-      </c>
-      <c r="R15" t="str">
-        <v/>
-      </c>
-      <c r="S15" t="str">
-        <v/>
-      </c>
-      <c r="T15" t="str">
-        <v/>
-      </c>
-      <c r="U15" t="str">
-        <v/>
-      </c>
-      <c r="V15" t="str">
-        <v/>
-      </c>
-      <c r="W15" t="str">
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
+      <c r="W16" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (49bc1d3) Add Dark Matter & Sand
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W16"/>
+  <dimension ref="A1:X19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,57 +416,60 @@
         <v>Level</v>
       </c>
       <c r="F1" t="str">
+        <v>Energy</v>
+      </c>
+      <c r="G1" t="str">
         <v>description</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Type1</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Type2</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Effect 1 Kind</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Effect 1 Amount</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Effect 1 Hits</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Effect 1 Duration</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Effect 1 Target</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Effect 2 Kind</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Effect 2 Amount</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Effect 2 Hits</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Effect 2 Duration</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Effect 2 Target</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>Effect 3 Kind</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>Effect 3 Amount</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>Effect 3 Hits</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>Effect 3 Duration</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>Effect 3 Target</v>
       </c>
     </row>
@@ -475,10 +478,10 @@
         <v>Water</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Ice</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Fire</v>
       </c>
       <c r="D2" t="str">
         <v>8</v>
@@ -487,44 +490,44 @@
         <v>1</v>
       </c>
       <c r="F2" t="str">
+        <v>1</v>
+      </c>
+      <c r="G2" t="str">
         <v>A gift from the sky goddess</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Water</v>
       </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
         <v>heal</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>5</v>
       </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
       <c r="L2" t="str">
         <v/>
       </c>
       <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
         <v>self</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>soak</v>
       </c>
-      <c r="O2" t="str">
-        <v>1</v>
-      </c>
       <c r="P2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
         <v>3</v>
       </c>
-      <c r="R2" t="str">
-        <v/>
-      </c>
       <c r="S2" t="str">
         <v/>
       </c>
@@ -538,6 +541,9 @@
         <v/>
       </c>
       <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
         <v/>
       </c>
     </row>
@@ -558,29 +564,29 @@
         <v>1</v>
       </c>
       <c r="F3" t="str">
+        <v>1</v>
+      </c>
+      <c r="G3" t="str">
         <v>A bright flame burning hot</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Fire</v>
       </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
         <v>burn</v>
       </c>
-      <c r="J3" t="str">
-        <v>1</v>
-      </c>
       <c r="K3" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
         <v>3</v>
       </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
       <c r="N3" t="str">
         <v/>
       </c>
@@ -609,6 +615,9 @@
         <v/>
       </c>
       <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
         <v/>
       </c>
     </row>
@@ -629,23 +638,23 @@
         <v>1</v>
       </c>
       <c r="F4" t="str">
+        <v>1</v>
+      </c>
+      <c r="G4" t="str">
         <v>It's a leaf</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Earth</v>
       </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
         <v>shield</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>5</v>
       </c>
-      <c r="K4" t="str">
-        <v/>
-      </c>
       <c r="L4" t="str">
         <v/>
       </c>
@@ -680,6 +689,9 @@
         <v/>
       </c>
       <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
         <v/>
       </c>
     </row>
@@ -700,25 +712,25 @@
         <v>1</v>
       </c>
       <c r="F5" t="str">
+        <v>1</v>
+      </c>
+      <c r="G5" t="str">
         <v>Charged spark that strikes instantly</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>Lightning</v>
       </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
         <v>multihit</v>
       </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
       <c r="K5" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="L5" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="M5" t="str">
         <v/>
@@ -751,6 +763,9 @@
         <v/>
       </c>
       <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
         <v/>
       </c>
     </row>
@@ -771,249 +786,120 @@
         <v>1</v>
       </c>
       <c r="F6" t="str">
+        <v>1</v>
+      </c>
+      <c r="G6" t="str">
         <v>A deep sense of calm overwhelms you</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>Fire</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>Lightning</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Worble</v>
+        <v>Sand</v>
       </c>
       <c r="B7" t="str">
-        <v>💧</v>
+        <v>Earth</v>
       </c>
       <c r="C7" t="str">
-        <v>💧</v>
+        <v>Earth</v>
       </c>
       <c r="D7" t="str">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="E7" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="str">
-        <v>The tide is high today my friend</v>
+        <v>1</v>
       </c>
       <c r="G7" t="str">
-        <v>Water</v>
+        <v>Shifting grains dance between your fingertips</v>
       </c>
       <c r="H7" t="str">
-        <v/>
-      </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
-      <c r="J7" t="str">
-        <v/>
-      </c>
-      <c r="K7" t="str">
-        <v/>
-      </c>
-      <c r="L7" t="str">
-        <v/>
-      </c>
-      <c r="M7" t="str">
-        <v/>
-      </c>
-      <c r="N7" t="str">
-        <v/>
-      </c>
-      <c r="O7" t="str">
-        <v/>
-      </c>
-      <c r="P7" t="str">
-        <v/>
-      </c>
-      <c r="Q7" t="str">
-        <v/>
-      </c>
-      <c r="R7" t="str">
-        <v/>
-      </c>
-      <c r="S7" t="str">
-        <v/>
-      </c>
-      <c r="T7" t="str">
-        <v/>
-      </c>
-      <c r="U7" t="str">
-        <v/>
-      </c>
-      <c r="V7" t="str">
-        <v/>
-      </c>
-      <c r="W7" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>💨</v>
+        <v>Leaf</v>
       </c>
       <c r="B8" t="str">
-        <v>💧</v>
+        <v>Earth</v>
       </c>
       <c r="C8" t="str">
-        <v>🔥</v>
+        <v>Water</v>
       </c>
       <c r="D8" t="str">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="E8" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="str">
-        <v>Scalding vapor that burns deeper than flame</v>
+        <v>1</v>
       </c>
       <c r="G8" t="str">
-        <v>Air</v>
+        <v>Drops of dew glistle atop</v>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
       <c r="I8" t="str">
-        <v/>
-      </c>
-      <c r="J8" t="str">
-        <v/>
-      </c>
-      <c r="K8" t="str">
-        <v/>
-      </c>
-      <c r="L8" t="str">
-        <v/>
-      </c>
-      <c r="M8" t="str">
-        <v/>
-      </c>
-      <c r="N8" t="str">
-        <v/>
-      </c>
-      <c r="O8" t="str">
-        <v/>
-      </c>
-      <c r="P8" t="str">
-        <v/>
-      </c>
-      <c r="Q8" t="str">
-        <v/>
-      </c>
-      <c r="R8" t="str">
-        <v/>
-      </c>
-      <c r="S8" t="str">
-        <v/>
-      </c>
-      <c r="T8" t="str">
-        <v/>
-      </c>
-      <c r="U8" t="str">
-        <v/>
-      </c>
-      <c r="V8" t="str">
-        <v/>
-      </c>
-      <c r="W8" t="str">
-        <v/>
+        <v>Water</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>🌴</v>
+        <v>Dark Matter</v>
       </c>
       <c r="B9" t="str">
-        <v>💧</v>
+        <v>Unstable Element</v>
       </c>
       <c r="C9" t="str">
-        <v>🍃</v>
+        <v>Unstable Element</v>
       </c>
       <c r="D9" t="str">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="E9" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" t="str">
-        <v>A prickly palm tree</v>
+        <v>2</v>
       </c>
       <c r="G9" t="str">
-        <v>Earth</v>
+        <v>A quiet humming radiates from inside</v>
       </c>
       <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <v/>
-      </c>
-      <c r="K9" t="str">
-        <v/>
-      </c>
-      <c r="L9" t="str">
-        <v/>
-      </c>
-      <c r="M9" t="str">
-        <v/>
-      </c>
-      <c r="N9" t="str">
-        <v/>
-      </c>
-      <c r="O9" t="str">
-        <v/>
-      </c>
-      <c r="P9" t="str">
-        <v/>
-      </c>
-      <c r="Q9" t="str">
-        <v/>
-      </c>
-      <c r="R9" t="str">
-        <v/>
-      </c>
-      <c r="S9" t="str">
-        <v/>
-      </c>
-      <c r="T9" t="str">
-        <v/>
-      </c>
-      <c r="U9" t="str">
-        <v/>
-      </c>
-      <c r="V9" t="str">
-        <v/>
-      </c>
-      <c r="W9" t="str">
-        <v/>
+        <v>Void</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>🚢</v>
+        <v>Worble</v>
       </c>
       <c r="B10" t="str">
         <v>💧</v>
       </c>
       <c r="C10" t="str">
-        <v>⚡</v>
+        <v>💧</v>
       </c>
       <c r="D10" t="str">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="E10" t="str">
         <v>2</v>
       </c>
       <c r="F10" t="str">
-        <v>A bit bigger than a tugboat</v>
+        <v>2</v>
       </c>
       <c r="G10" t="str">
-        <v>Steel</v>
+        <v>The tide is high today my friend</v>
       </c>
       <c r="H10" t="str">
         <v>Water</v>
@@ -1063,31 +949,34 @@
       <c r="W10" t="str">
         <v/>
       </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>🌲</v>
+        <v>💨</v>
       </c>
       <c r="B11" t="str">
-        <v>🍃</v>
+        <v>💧</v>
       </c>
       <c r="C11" t="str">
-        <v>🍃</v>
+        <v>🔥</v>
       </c>
       <c r="D11" t="str">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="E11" t="str">
         <v>2</v>
       </c>
       <c r="F11" t="str">
-        <v>Its pines are sharper than you may think</v>
+        <v>2</v>
       </c>
       <c r="G11" t="str">
-        <v>Earth</v>
+        <v>Scalding vapor that burns deeper than flame</v>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>Air</v>
       </c>
       <c r="I11" t="str">
         <v/>
@@ -1132,33 +1021,36 @@
         <v/>
       </c>
       <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>💥</v>
+        <v>🌴</v>
       </c>
       <c r="B12" t="str">
+        <v>💧</v>
+      </c>
+      <c r="C12" t="str">
         <v>🍃</v>
       </c>
-      <c r="C12" t="str">
-        <v>🔥</v>
-      </c>
       <c r="D12" t="str">
-        <v>86</v>
+        <v>48</v>
       </c>
       <c r="E12" t="str">
         <v>2</v>
       </c>
       <c r="F12" t="str">
-        <v>BOOM</v>
+        <v>2</v>
       </c>
       <c r="G12" t="str">
-        <v>Fire</v>
+        <v>A prickly palm tree</v>
       </c>
       <c r="H12" t="str">
-        <v>Light</v>
+        <v>Earth</v>
       </c>
       <c r="I12" t="str">
         <v/>
@@ -1203,36 +1095,39 @@
         <v/>
       </c>
       <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>🚑</v>
+        <v>🚢</v>
       </c>
       <c r="B13" t="str">
-        <v>🍃</v>
+        <v>💧</v>
       </c>
       <c r="C13" t="str">
         <v>⚡</v>
       </c>
       <c r="D13" t="str">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E13" t="str">
         <v>2</v>
       </c>
       <c r="F13" t="str">
-        <v>Hurts AND heals! (ok, healing isnt implemented yet but it WILL heal eventually)</v>
+        <v>2</v>
       </c>
       <c r="G13" t="str">
+        <v>A bit bigger than a tugboat</v>
+      </c>
+      <c r="H13" t="str">
         <v>Steel</v>
       </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
       <c r="I13" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -1274,33 +1169,36 @@
         <v/>
       </c>
       <c r="W13" t="str">
+        <v/>
+      </c>
+      <c r="X13" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>🌞</v>
+        <v>🌲</v>
       </c>
       <c r="B14" t="str">
-        <v>🔥</v>
+        <v>🍃</v>
       </c>
       <c r="C14" t="str">
-        <v>🔥</v>
+        <v>🍃</v>
       </c>
       <c r="D14" t="str">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="E14" t="str">
         <v>2</v>
       </c>
       <c r="F14" t="str">
-        <v>A miniature sun in the palm of your hand</v>
+        <v>2</v>
       </c>
       <c r="G14" t="str">
-        <v>Fire</v>
+        <v>Its pines are sharper than you may think</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
       <c r="I14" t="str">
         <v/>
@@ -1345,36 +1243,39 @@
         <v/>
       </c>
       <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>🚀</v>
+        <v>💥</v>
       </c>
       <c r="B15" t="str">
+        <v>🍃</v>
+      </c>
+      <c r="C15" t="str">
         <v>🔥</v>
       </c>
-      <c r="C15" t="str">
-        <v>⚡</v>
-      </c>
       <c r="D15" t="str">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="E15" t="str">
         <v>2</v>
       </c>
       <c r="F15" t="str">
-        <v>Away we go!</v>
+        <v>2</v>
       </c>
       <c r="G15" t="str">
-        <v>Steel</v>
+        <v>BOOM</v>
       </c>
       <c r="H15" t="str">
         <v>Fire</v>
       </c>
       <c r="I15" t="str">
-        <v/>
+        <v>Light</v>
       </c>
       <c r="J15" t="str">
         <v/>
@@ -1416,83 +1317,311 @@
         <v/>
       </c>
       <c r="W15" t="str">
+        <v/>
+      </c>
+      <c r="X15" t="str">
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>🛸</v>
+        <v>🚑</v>
       </c>
       <c r="B16" t="str">
-        <v>⚡</v>
+        <v>🍃</v>
       </c>
       <c r="C16" t="str">
         <v>⚡</v>
       </c>
       <c r="D16" t="str">
+        <v>58</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2</v>
+      </c>
+      <c r="G16" t="str">
+        <v>Hurts AND heals! (ok, healing isnt implemented yet but it WILL heal eventually)</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
+        <v/>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
+      <c r="R16" t="str">
+        <v/>
+      </c>
+      <c r="S16" t="str">
+        <v/>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v/>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
+      <c r="W16" t="str">
+        <v/>
+      </c>
+      <c r="X16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>🌞</v>
+      </c>
+      <c r="B17" t="str">
+        <v>🔥</v>
+      </c>
+      <c r="C17" t="str">
+        <v>🔥</v>
+      </c>
+      <c r="D17" t="str">
+        <v>94</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2</v>
+      </c>
+      <c r="F17" t="str">
+        <v>2</v>
+      </c>
+      <c r="G17" t="str">
+        <v>A miniature sun in the palm of your hand</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+      <c r="V17" t="str">
+        <v/>
+      </c>
+      <c r="W17" t="str">
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>🚀</v>
+      </c>
+      <c r="B18" t="str">
+        <v>🔥</v>
+      </c>
+      <c r="C18" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="D18" t="str">
+        <v>78</v>
+      </c>
+      <c r="E18" t="str">
+        <v>2</v>
+      </c>
+      <c r="F18" t="str">
+        <v>2</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Away we go!</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+      <c r="V18" t="str">
+        <v/>
+      </c>
+      <c r="W18" t="str">
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>🛸</v>
+      </c>
+      <c r="B19" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="C19" t="str">
+        <v>⚡</v>
+      </c>
+      <c r="D19" t="str">
         <v>100</v>
       </c>
-      <c r="E16" t="str">
-        <v>2</v>
-      </c>
-      <c r="F16" t="str">
+      <c r="E19" t="str">
+        <v>2</v>
+      </c>
+      <c r="F19" t="str">
+        <v>2</v>
+      </c>
+      <c r="G19" t="str">
         <v>Sure why not</v>
       </c>
-      <c r="G16" t="str">
+      <c r="H19" t="str">
         <v>Steel</v>
       </c>
-      <c r="H16" t="str">
+      <c r="I19" t="str">
         <v>Lightning</v>
       </c>
-      <c r="I16" t="str">
-        <v/>
-      </c>
-      <c r="J16" t="str">
-        <v/>
-      </c>
-      <c r="K16" t="str">
-        <v/>
-      </c>
-      <c r="L16" t="str">
-        <v/>
-      </c>
-      <c r="M16" t="str">
-        <v/>
-      </c>
-      <c r="N16" t="str">
-        <v/>
-      </c>
-      <c r="O16" t="str">
-        <v/>
-      </c>
-      <c r="P16" t="str">
-        <v/>
-      </c>
-      <c r="Q16" t="str">
-        <v/>
-      </c>
-      <c r="R16" t="str">
-        <v/>
-      </c>
-      <c r="S16" t="str">
-        <v/>
-      </c>
-      <c r="T16" t="str">
-        <v/>
-      </c>
-      <c r="U16" t="str">
-        <v/>
-      </c>
-      <c r="V16" t="str">
-        <v/>
-      </c>
-      <c r="W16" t="str">
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+      <c r="V19" t="str">
+        <v/>
+      </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (b8daa9f) (WIP) Adding elements
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X19"/>
+  <dimension ref="A1:X55"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -884,10 +884,10 @@
         <v>Worble</v>
       </c>
       <c r="B10" t="str">
-        <v>💧</v>
+        <v>Water</v>
       </c>
       <c r="C10" t="str">
-        <v>💧</v>
+        <v>Water</v>
       </c>
       <c r="D10" t="str">
         <v>38</v>
@@ -955,28 +955,22 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>💨</v>
+        <v>Blaze</v>
       </c>
       <c r="B11" t="str">
-        <v>💧</v>
+        <v>Leaf</v>
       </c>
       <c r="C11" t="str">
-        <v>🔥</v>
+        <v>Fire</v>
       </c>
       <c r="D11" t="str">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E11" t="str">
         <v>2</v>
       </c>
       <c r="F11" t="str">
         <v>2</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Scalding vapor that burns deeper than flame</v>
-      </c>
-      <c r="H11" t="str">
-        <v>Air</v>
       </c>
       <c r="I11" t="str">
         <v/>
@@ -1029,28 +1023,22 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>🌴</v>
+        <v>Regen</v>
       </c>
       <c r="B12" t="str">
-        <v>💧</v>
+        <v>Leaf</v>
       </c>
       <c r="C12" t="str">
-        <v>🍃</v>
+        <v>Water</v>
       </c>
       <c r="D12" t="str">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E12" t="str">
         <v>2</v>
       </c>
       <c r="F12" t="str">
         <v>2</v>
-      </c>
-      <c r="G12" t="str">
-        <v>A prickly palm tree</v>
-      </c>
-      <c r="H12" t="str">
-        <v>Earth</v>
       </c>
       <c r="I12" t="str">
         <v/>
@@ -1103,16 +1091,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>🚢</v>
+        <v>Leaf Shield</v>
       </c>
       <c r="B13" t="str">
-        <v>💧</v>
+        <v>Leaf</v>
       </c>
       <c r="C13" t="str">
-        <v>⚡</v>
+        <v>Earth</v>
       </c>
       <c r="D13" t="str">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="E13" t="str">
         <v>2</v>
@@ -1121,22 +1109,16 @@
         <v>2</v>
       </c>
       <c r="G13" t="str">
-        <v>A bit bigger than a tugboat</v>
+        <v>Leaves swirl around you</v>
       </c>
       <c r="H13" t="str">
-        <v>Steel</v>
-      </c>
-      <c r="I13" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="K13" t="str">
-        <v/>
-      </c>
-      <c r="L13" t="str">
-        <v/>
+        <v>15</v>
       </c>
       <c r="M13" t="str">
         <v/>
@@ -1177,16 +1159,16 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>🌲</v>
+        <v>Tornado</v>
       </c>
       <c r="B14" t="str">
-        <v>🍃</v>
+        <v>Leaf</v>
       </c>
       <c r="C14" t="str">
-        <v>🍃</v>
+        <v>Air</v>
       </c>
       <c r="D14" t="str">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="E14" t="str">
         <v>2</v>
@@ -1195,22 +1177,22 @@
         <v>2</v>
       </c>
       <c r="G14" t="str">
-        <v>Its pines are sharper than you may think</v>
+        <v>Wind whips and slashes about</v>
       </c>
       <c r="H14" t="str">
         <v>Earth</v>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>Air</v>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>multihit</v>
       </c>
       <c r="K14" t="str">
         <v/>
       </c>
       <c r="L14" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="M14" t="str">
         <v/>
@@ -1251,16 +1233,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>💥</v>
+        <v>Blizzard</v>
       </c>
       <c r="B15" t="str">
-        <v>🍃</v>
+        <v>Leaf</v>
       </c>
       <c r="C15" t="str">
-        <v>🔥</v>
-      </c>
-      <c r="D15" t="str">
-        <v>86</v>
+        <v>Ice</v>
       </c>
       <c r="E15" t="str">
         <v>2</v>
@@ -1269,13 +1248,13 @@
         <v>2</v>
       </c>
       <c r="G15" t="str">
-        <v>BOOM</v>
+        <v>Snow flurries and blocks your vision</v>
       </c>
       <c r="H15" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="I15" t="str">
-        <v>Light</v>
+        <v>Ice</v>
       </c>
       <c r="J15" t="str">
         <v/>
@@ -1325,28 +1304,19 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>🚑</v>
+        <v>Leaf Blade</v>
       </c>
       <c r="B16" t="str">
-        <v>🍃</v>
+        <v>Leaf</v>
       </c>
       <c r="C16" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="D16" t="str">
-        <v>58</v>
+        <v>Steel</v>
       </c>
       <c r="E16" t="str">
         <v>2</v>
       </c>
       <c r="F16" t="str">
         <v>2</v>
-      </c>
-      <c r="G16" t="str">
-        <v>Hurts AND heals! (ok, healing isnt implemented yet but it WILL heal eventually)</v>
-      </c>
-      <c r="H16" t="str">
-        <v>Steel</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -1399,16 +1369,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>🌞</v>
+        <v>1000 Needles</v>
       </c>
       <c r="B17" t="str">
-        <v>🔥</v>
+        <v>Leaf</v>
       </c>
       <c r="C17" t="str">
-        <v>🔥</v>
+        <v>Sand</v>
       </c>
       <c r="D17" t="str">
-        <v>94</v>
+        <v>20</v>
       </c>
       <c r="E17" t="str">
         <v>2</v>
@@ -1416,23 +1386,17 @@
       <c r="F17" t="str">
         <v>2</v>
       </c>
-      <c r="G17" t="str">
-        <v>A miniature sun in the palm of your hand</v>
-      </c>
       <c r="H17" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="I17" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
       <c r="J17" t="str">
-        <v/>
+        <v>multihit</v>
       </c>
       <c r="K17" t="str">
         <v/>
       </c>
       <c r="L17" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="M17" t="str">
         <v/>
@@ -1473,31 +1437,19 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>🚀</v>
+        <v>Fire</v>
       </c>
       <c r="B18" t="str">
-        <v>🔥</v>
+        <v>Leaf</v>
       </c>
       <c r="C18" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="D18" t="str">
-        <v>78</v>
+        <v>Lightning</v>
       </c>
       <c r="E18" t="str">
         <v>2</v>
       </c>
       <c r="F18" t="str">
         <v>2</v>
-      </c>
-      <c r="G18" t="str">
-        <v>Away we go!</v>
-      </c>
-      <c r="H18" t="str">
-        <v>Steel</v>
-      </c>
-      <c r="I18" t="str">
-        <v>Fire</v>
       </c>
       <c r="J18" t="str">
         <v/>
@@ -1547,16 +1499,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>🛸</v>
+        <v>Photosynthesis</v>
       </c>
       <c r="B19" t="str">
-        <v>⚡</v>
+        <v>Leaf</v>
       </c>
       <c r="C19" t="str">
-        <v>⚡</v>
-      </c>
-      <c r="D19" t="str">
-        <v>100</v>
+        <v>Leaf</v>
       </c>
       <c r="E19" t="str">
         <v>2</v>
@@ -1564,64 +1513,622 @@
       <c r="F19" t="str">
         <v>2</v>
       </c>
-      <c r="G19" t="str">
-        <v>Sure why not</v>
-      </c>
-      <c r="H19" t="str">
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Steel Sand</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="C20" t="str">
         <v>Steel</v>
       </c>
-      <c r="I19" t="str">
+      <c r="E20" t="str">
+        <v>2</v>
+      </c>
+      <c r="F20" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Glass</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2</v>
+      </c>
+      <c r="F21" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Mud Shot</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Water</v>
+      </c>
+      <c r="E22" t="str">
+        <v>2</v>
+      </c>
+      <c r="F22" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Glass</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="C23" t="str">
         <v>Lightning</v>
       </c>
-      <c r="J19" t="str">
-        <v/>
-      </c>
-      <c r="K19" t="str">
-        <v/>
-      </c>
-      <c r="L19" t="str">
-        <v/>
-      </c>
-      <c r="M19" t="str">
-        <v/>
-      </c>
-      <c r="N19" t="str">
-        <v/>
-      </c>
-      <c r="O19" t="str">
-        <v/>
-      </c>
-      <c r="P19" t="str">
-        <v/>
-      </c>
-      <c r="Q19" t="str">
-        <v/>
-      </c>
-      <c r="R19" t="str">
-        <v/>
-      </c>
-      <c r="S19" t="str">
-        <v/>
-      </c>
-      <c r="T19" t="str">
-        <v/>
-      </c>
-      <c r="U19" t="str">
-        <v/>
-      </c>
-      <c r="V19" t="str">
-        <v/>
-      </c>
-      <c r="W19" t="str">
-        <v/>
-      </c>
-      <c r="X19" t="str">
-        <v/>
+      <c r="E23" t="str">
+        <v>2</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Sand Shield</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2</v>
+      </c>
+      <c r="F24" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Sandstorm</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Air</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2</v>
+      </c>
+      <c r="F25" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Iceblast</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2</v>
+      </c>
+      <c r="F26" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2</v>
+      </c>
+      <c r="F27" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Blaze Blade</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2</v>
+      </c>
+      <c r="F28" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Aqua Blade</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Water</v>
+      </c>
+      <c r="E29" t="str">
+        <v>2</v>
+      </c>
+      <c r="F29" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Voltage</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2</v>
+      </c>
+      <c r="F30" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Cleave</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="E31" t="str">
+        <v>2</v>
+      </c>
+      <c r="F31" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Quick Strike</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Air</v>
+      </c>
+      <c r="E32" t="str">
+        <v>2</v>
+      </c>
+      <c r="F32" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Ice Blade</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="E33" t="str">
+        <v>2</v>
+      </c>
+      <c r="F33" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Refined Steel</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="E34" t="str">
+        <v>2</v>
+      </c>
+      <c r="F34" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Plasma</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="E35" t="str">
+        <v>2</v>
+      </c>
+      <c r="F35" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Water Bolt</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Water</v>
+      </c>
+      <c r="E36" t="str">
+        <v>2</v>
+      </c>
+      <c r="F36" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Plasma</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="E37" t="str">
+        <v>2</v>
+      </c>
+      <c r="F37" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Plasma</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Air</v>
+      </c>
+      <c r="E38" t="str">
+        <v>2</v>
+      </c>
+      <c r="F38" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Ice Bolt</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="E39" t="str">
+        <v>2</v>
+      </c>
+      <c r="F39" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Thunder</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="E40" t="str">
+        <v>2</v>
+      </c>
+      <c r="F40" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Air</v>
+      </c>
+      <c r="E41" t="str">
+        <v>2</v>
+      </c>
+      <c r="F41" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Mud Shot</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="E42" t="str">
+        <v>2</v>
+      </c>
+      <c r="F42" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Worble</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Water</v>
+      </c>
+      <c r="E43" t="str">
+        <v>2</v>
+      </c>
+      <c r="F43" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Air</v>
+      </c>
+      <c r="E44" t="str">
+        <v>2</v>
+      </c>
+      <c r="F44" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Air</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="E45" t="str">
+        <v>2</v>
+      </c>
+      <c r="F45" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Tornado</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Air</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Air</v>
+      </c>
+      <c r="E46" t="str">
+        <v>2</v>
+      </c>
+      <c r="F46" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Air</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="E47" t="str">
+        <v>2</v>
+      </c>
+      <c r="F47" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Hailstorm</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Air</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="E48" t="str">
+        <v>2</v>
+      </c>
+      <c r="F48" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Air</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="E49" t="str">
+        <v>2</v>
+      </c>
+      <c r="F49" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Water</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="E50" t="str">
+        <v>2</v>
+      </c>
+      <c r="F50" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="E51" t="str">
+        <v>2</v>
+      </c>
+      <c r="F51" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Pyreball</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="E52" t="str">
+        <v>2</v>
+      </c>
+      <c r="F52" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Ice Shield</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="E53" t="str">
+        <v>2</v>
+      </c>
+      <c r="F53" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Tundra</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="E54" t="str">
+        <v>2</v>
+      </c>
+      <c r="F54" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Earthquake</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="E55" t="str">
+        <v>2</v>
+      </c>
+      <c r="F55" t="str">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X55"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (a9ff39d) Add images for all spells and elements
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X55"/>
+  <dimension ref="A1:Z51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -552,10 +552,10 @@
         <v>Fire</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Air</v>
       </c>
       <c r="D3" t="str">
         <v>10</v>
@@ -623,16 +623,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>Leaf</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>Lightning</v>
       </c>
       <c r="D4" t="str">
-        <v>10</v>
+        <v/>
       </c>
       <c r="E4" t="str">
         <v>1</v>
@@ -641,19 +641,19 @@
         <v>1</v>
       </c>
       <c r="G4" t="str">
-        <v>It's a leaf</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="I4" t="str">
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="K4" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="L4" t="str">
         <v/>
@@ -692,21 +692,27 @@
         <v/>
       </c>
       <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>Sand</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>Sand</v>
       </c>
       <c r="D5" t="str">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E5" t="str">
         <v>1</v>
@@ -715,22 +721,22 @@
         <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v>Charged spark that strikes instantly</v>
+        <v>It's a leaf</v>
       </c>
       <c r="H5" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="I5" t="str">
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>multihit</v>
+        <v>shield</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="L5" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="M5" t="str">
         <v/>
@@ -771,71 +777,107 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Plasma</v>
+        <v>Lightning</v>
       </c>
       <c r="B6" t="str">
+        <v>Air</v>
+      </c>
+      <c r="C6" t="str">
         <v>Fire</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
+        <v>11</v>
+      </c>
+      <c r="E6" t="str">
+        <v>1</v>
+      </c>
+      <c r="F6" t="str">
+        <v>1</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Charged spark that strikes instantly</v>
+      </c>
+      <c r="H6" t="str">
         <v>Lightning</v>
       </c>
-      <c r="D6" t="str">
-        <v>1</v>
-      </c>
-      <c r="E6" t="str">
-        <v>1</v>
-      </c>
-      <c r="F6" t="str">
-        <v>1</v>
-      </c>
-      <c r="G6" t="str">
-        <v>A deep sense of calm overwhelms you</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Fire</v>
-      </c>
       <c r="I6" t="str">
-        <v>Lightning</v>
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v>multihit</v>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v>2</v>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v/>
+      </c>
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Sand</v>
+        <v>Plasma</v>
       </c>
       <c r="B7" t="str">
-        <v>Earth</v>
+        <v>Lightning</v>
       </c>
       <c r="C7" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="D7" t="str">
-        <v>10</v>
+        <v>Air</v>
       </c>
       <c r="E7" t="str">
         <v>1</v>
       </c>
       <c r="F7" t="str">
         <v>1</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Shifting grains dance between your fingertips</v>
-      </c>
-      <c r="H7" t="str">
-        <v>Earth</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Leaf</v>
+        <v>Plasma</v>
       </c>
       <c r="B8" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C8" t="str">
         <v>Earth</v>
       </c>
-      <c r="C8" t="str">
-        <v>Water</v>
-      </c>
       <c r="D8" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="E8" t="str">
         <v>1</v>
@@ -844,201 +886,162 @@
         <v>1</v>
       </c>
       <c r="G8" t="str">
-        <v>Drops of dew glistle atop</v>
+        <v/>
       </c>
       <c r="H8" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="I8" t="str">
-        <v>Water</v>
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v/>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+      <c r="X8" t="str">
+        <v/>
+      </c>
+      <c r="Y8" t="str">
+        <v/>
+      </c>
+      <c r="Z8" t="str">
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Dark Matter</v>
+        <v>Plasma</v>
       </c>
       <c r="B9" t="str">
-        <v>Unstable Element</v>
+        <v>Lightning</v>
       </c>
       <c r="C9" t="str">
-        <v>Unstable Element</v>
-      </c>
-      <c r="D9" t="str">
-        <v>18</v>
+        <v>Fire</v>
       </c>
       <c r="E9" t="str">
         <v>1</v>
       </c>
       <c r="F9" t="str">
-        <v>2</v>
-      </c>
-      <c r="G9" t="str">
-        <v>A quiet humming radiates from inside</v>
-      </c>
-      <c r="H9" t="str">
-        <v>Void</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Worble</v>
+        <v>Plasma</v>
       </c>
       <c r="B10" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="C10" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="D10" t="str">
-        <v>38</v>
+        <v>1</v>
       </c>
       <c r="E10" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10" t="str">
-        <v>The tide is high today my friend</v>
+        <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H10" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="I10" t="str">
-        <v/>
-      </c>
-      <c r="J10" t="str">
-        <v/>
-      </c>
-      <c r="K10" t="str">
-        <v/>
-      </c>
-      <c r="L10" t="str">
-        <v/>
-      </c>
-      <c r="M10" t="str">
-        <v/>
-      </c>
-      <c r="N10" t="str">
-        <v/>
-      </c>
-      <c r="O10" t="str">
-        <v/>
-      </c>
-      <c r="P10" t="str">
-        <v/>
-      </c>
-      <c r="Q10" t="str">
-        <v/>
-      </c>
-      <c r="R10" t="str">
-        <v/>
-      </c>
-      <c r="S10" t="str">
-        <v/>
-      </c>
-      <c r="T10" t="str">
-        <v/>
-      </c>
-      <c r="U10" t="str">
-        <v/>
-      </c>
-      <c r="V10" t="str">
-        <v/>
-      </c>
-      <c r="W10" t="str">
-        <v/>
-      </c>
-      <c r="X10" t="str">
-        <v/>
+        <v>Lightning</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Blaze</v>
+        <v>Sand</v>
       </c>
       <c r="B11" t="str">
-        <v>Leaf</v>
+        <v>Earth</v>
       </c>
       <c r="C11" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D11" t="str">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="E11" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" t="str">
-        <v>2</v>
-      </c>
-      <c r="I11" t="str">
-        <v/>
-      </c>
-      <c r="J11" t="str">
-        <v/>
-      </c>
-      <c r="K11" t="str">
-        <v/>
-      </c>
-      <c r="L11" t="str">
-        <v/>
-      </c>
-      <c r="M11" t="str">
-        <v/>
-      </c>
-      <c r="N11" t="str">
-        <v/>
-      </c>
-      <c r="O11" t="str">
-        <v/>
-      </c>
-      <c r="P11" t="str">
-        <v/>
-      </c>
-      <c r="Q11" t="str">
-        <v/>
-      </c>
-      <c r="R11" t="str">
-        <v/>
-      </c>
-      <c r="S11" t="str">
-        <v/>
-      </c>
-      <c r="T11" t="str">
-        <v/>
-      </c>
-      <c r="U11" t="str">
-        <v/>
-      </c>
-      <c r="V11" t="str">
-        <v/>
-      </c>
-      <c r="W11" t="str">
-        <v/>
-      </c>
-      <c r="X11" t="str">
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Shifting grains dance between your fingertips</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Regen</v>
+        <v>Sand</v>
       </c>
       <c r="B12" t="str">
-        <v>Leaf</v>
+        <v>Air</v>
       </c>
       <c r="C12" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="D12" t="str">
-        <v>40</v>
+        <v/>
       </c>
       <c r="E12" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="str">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
       </c>
       <c r="I12" t="str">
         <v/>
@@ -1086,39 +1089,51 @@
         <v/>
       </c>
       <c r="X12" t="str">
+        <v/>
+      </c>
+      <c r="Y12" t="str">
+        <v/>
+      </c>
+      <c r="Z12" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Leaf Shield</v>
+        <v>Steel</v>
       </c>
       <c r="B13" t="str">
-        <v>Leaf</v>
+        <v>Fire</v>
       </c>
       <c r="C13" t="str">
         <v>Earth</v>
       </c>
       <c r="D13" t="str">
-        <v>32</v>
+        <v/>
       </c>
       <c r="E13" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" t="str">
-        <v>Leaves swirl around you</v>
+        <v/>
       </c>
       <c r="H13" t="str">
-        <v>Earth</v>
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v/>
       </c>
       <c r="J13" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="K13" t="str">
-        <v>15</v>
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
       </c>
       <c r="M13" t="str">
         <v/>
@@ -1154,45 +1169,51 @@
         <v/>
       </c>
       <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
+        <v/>
+      </c>
+      <c r="Z13" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Tornado</v>
+        <v>Air</v>
       </c>
       <c r="B14" t="str">
-        <v>Leaf</v>
+        <v>Water</v>
       </c>
       <c r="C14" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="D14" t="str">
-        <v>25</v>
+        <v/>
       </c>
       <c r="E14" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G14" t="str">
-        <v>Wind whips and slashes about</v>
+        <v/>
       </c>
       <c r="H14" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="I14" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="J14" t="str">
-        <v>multihit</v>
+        <v/>
       </c>
       <c r="K14" t="str">
         <v/>
       </c>
       <c r="L14" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="M14" t="str">
         <v/>
@@ -1228,95 +1249,68 @@
         <v/>
       </c>
       <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14" t="str">
+        <v/>
+      </c>
+      <c r="Z14" t="str">
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Blizzard</v>
+        <v>Leaf</v>
       </c>
       <c r="B15" t="str">
-        <v>Leaf</v>
+        <v>Earth</v>
       </c>
       <c r="C15" t="str">
-        <v>Ice</v>
+        <v>Water</v>
+      </c>
+      <c r="D15" t="str">
+        <v>8</v>
       </c>
       <c r="E15" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G15" t="str">
-        <v>Snow flurries and blocks your vision</v>
+        <v>Drops of dew glistle atop</v>
       </c>
       <c r="H15" t="str">
         <v>Earth</v>
       </c>
       <c r="I15" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="J15" t="str">
-        <v/>
-      </c>
-      <c r="K15" t="str">
-        <v/>
-      </c>
-      <c r="L15" t="str">
-        <v/>
-      </c>
-      <c r="M15" t="str">
-        <v/>
-      </c>
-      <c r="N15" t="str">
-        <v/>
-      </c>
-      <c r="O15" t="str">
-        <v/>
-      </c>
-      <c r="P15" t="str">
-        <v/>
-      </c>
-      <c r="Q15" t="str">
-        <v/>
-      </c>
-      <c r="R15" t="str">
-        <v/>
-      </c>
-      <c r="S15" t="str">
-        <v/>
-      </c>
-      <c r="T15" t="str">
-        <v/>
-      </c>
-      <c r="U15" t="str">
-        <v/>
-      </c>
-      <c r="V15" t="str">
-        <v/>
-      </c>
-      <c r="W15" t="str">
-        <v/>
-      </c>
-      <c r="X15" t="str">
-        <v/>
+        <v>Water</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Leaf Blade</v>
+        <v>Ice</v>
       </c>
       <c r="B16" t="str">
-        <v>Leaf</v>
+        <v>Water</v>
       </c>
       <c r="C16" t="str">
-        <v>Steel</v>
+        <v>Air</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
       </c>
       <c r="E16" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="str">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -1364,301 +1358,640 @@
         <v/>
       </c>
       <c r="X16" t="str">
+        <v/>
+      </c>
+      <c r="Y16" t="str">
+        <v/>
+      </c>
+      <c r="Z16" t="str">
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>1000 Needles</v>
+        <v>Glass</v>
       </c>
       <c r="B17" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C17" t="str">
-        <v>Sand</v>
-      </c>
-      <c r="D17" t="str">
-        <v>20</v>
+        <v>Fire</v>
       </c>
       <c r="E17" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" t="str">
-        <v>2</v>
-      </c>
-      <c r="H17" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="J17" t="str">
-        <v>multihit</v>
-      </c>
-      <c r="K17" t="str">
-        <v/>
-      </c>
-      <c r="L17" t="str">
-        <v>10</v>
-      </c>
-      <c r="M17" t="str">
-        <v/>
-      </c>
-      <c r="N17" t="str">
-        <v/>
-      </c>
-      <c r="O17" t="str">
-        <v/>
-      </c>
-      <c r="P17" t="str">
-        <v/>
-      </c>
-      <c r="Q17" t="str">
-        <v/>
-      </c>
-      <c r="R17" t="str">
-        <v/>
-      </c>
-      <c r="S17" t="str">
-        <v/>
-      </c>
-      <c r="T17" t="str">
-        <v/>
-      </c>
-      <c r="U17" t="str">
-        <v/>
-      </c>
-      <c r="V17" t="str">
-        <v/>
-      </c>
-      <c r="W17" t="str">
-        <v/>
-      </c>
-      <c r="X17" t="str">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Fire</v>
+        <v>Glass</v>
       </c>
       <c r="B18" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C18" t="str">
         <v>Lightning</v>
       </c>
       <c r="E18" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" t="str">
-        <v>2</v>
-      </c>
-      <c r="J18" t="str">
-        <v/>
-      </c>
-      <c r="K18" t="str">
-        <v/>
-      </c>
-      <c r="L18" t="str">
-        <v/>
-      </c>
-      <c r="M18" t="str">
-        <v/>
-      </c>
-      <c r="N18" t="str">
-        <v/>
-      </c>
-      <c r="O18" t="str">
-        <v/>
-      </c>
-      <c r="P18" t="str">
-        <v/>
-      </c>
-      <c r="Q18" t="str">
-        <v/>
-      </c>
-      <c r="R18" t="str">
-        <v/>
-      </c>
-      <c r="S18" t="str">
-        <v/>
-      </c>
-      <c r="T18" t="str">
-        <v/>
-      </c>
-      <c r="U18" t="str">
-        <v/>
-      </c>
-      <c r="V18" t="str">
-        <v/>
-      </c>
-      <c r="W18" t="str">
-        <v/>
-      </c>
-      <c r="X18" t="str">
-        <v/>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Photosynthesis</v>
+        <v>Dark Matter</v>
       </c>
       <c r="B19" t="str">
-        <v>Leaf</v>
+        <v>Unstable Element</v>
       </c>
       <c r="C19" t="str">
-        <v>Leaf</v>
+        <v>Unstable Element</v>
+      </c>
+      <c r="D19" t="str">
+        <v>18</v>
       </c>
       <c r="E19" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="str">
         <v>2</v>
+      </c>
+      <c r="G19" t="str">
+        <v>A quiet humming radiates from inside</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Void</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Steel Sand</v>
+        <v>Worble</v>
       </c>
       <c r="B20" t="str">
-        <v>Sand</v>
+        <v>Water</v>
       </c>
       <c r="C20" t="str">
-        <v>Steel</v>
+        <v>Water</v>
+      </c>
+      <c r="D20" t="str">
+        <v>38</v>
       </c>
       <c r="E20" t="str">
         <v>2</v>
       </c>
       <c r="F20" t="str">
         <v>2</v>
+      </c>
+      <c r="G20" t="str">
+        <v>The tide is high today my friend</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Water</v>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+      <c r="V20" t="str">
+        <v/>
+      </c>
+      <c r="W20" t="str">
+        <v/>
+      </c>
+      <c r="X20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Glass</v>
+        <v>Blaze</v>
       </c>
       <c r="B21" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="C21" t="str">
         <v>Fire</v>
       </c>
+      <c r="D21" t="str">
+        <v>53</v>
+      </c>
       <c r="E21" t="str">
         <v>2</v>
       </c>
       <c r="F21" t="str">
         <v>2</v>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
+      <c r="U21" t="str">
+        <v/>
+      </c>
+      <c r="V21" t="str">
+        <v/>
+      </c>
+      <c r="W21" t="str">
+        <v/>
+      </c>
+      <c r="X21" t="str">
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Mud Shot</v>
+        <v>Regen</v>
       </c>
       <c r="B22" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="C22" t="str">
         <v>Water</v>
       </c>
+      <c r="D22" t="str">
+        <v>40</v>
+      </c>
       <c r="E22" t="str">
         <v>2</v>
       </c>
       <c r="F22" t="str">
         <v>2</v>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+      <c r="T22" t="str">
+        <v/>
+      </c>
+      <c r="U22" t="str">
+        <v/>
+      </c>
+      <c r="V22" t="str">
+        <v/>
+      </c>
+      <c r="W22" t="str">
+        <v/>
+      </c>
+      <c r="X22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Glass</v>
+        <v>Thorns</v>
       </c>
       <c r="B23" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="C23" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
+      </c>
+      <c r="D23" t="str">
+        <v>32</v>
       </c>
       <c r="E23" t="str">
         <v>2</v>
       </c>
       <c r="F23" t="str">
         <v>2</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Leaves swirl around you</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J23" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K23" t="str">
+        <v>15</v>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Sand Shield</v>
+        <v>Tornado</v>
       </c>
       <c r="B24" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="C24" t="str">
+        <v>Air</v>
+      </c>
+      <c r="D24" t="str">
+        <v>25</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2</v>
+      </c>
+      <c r="F24" t="str">
+        <v>2</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Wind whips and slashes about</v>
+      </c>
+      <c r="H24" t="str">
         <v>Earth</v>
       </c>
-      <c r="E24" t="str">
-        <v>2</v>
-      </c>
-      <c r="F24" t="str">
-        <v>2</v>
+      <c r="I24" t="str">
+        <v>Air</v>
+      </c>
+      <c r="J24" t="str">
+        <v>multihit</v>
+      </c>
+      <c r="K24" t="str">
+        <v/>
+      </c>
+      <c r="L24" t="str">
+        <v>5</v>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
+        <v/>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
+        <v/>
+      </c>
+      <c r="X24" t="str">
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Sandstorm</v>
+        <v>Blizzard</v>
       </c>
       <c r="B25" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="C25" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="E25" t="str">
         <v>2</v>
       </c>
       <c r="F25" t="str">
         <v>2</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Snow flurries and blocks your vision</v>
+      </c>
+      <c r="H25" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
+        <v/>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
+        <v/>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+      <c r="T25" t="str">
+        <v/>
+      </c>
+      <c r="U25" t="str">
+        <v/>
+      </c>
+      <c r="V25" t="str">
+        <v/>
+      </c>
+      <c r="W25" t="str">
+        <v/>
+      </c>
+      <c r="X25" t="str">
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Iceblast</v>
+        <v>Leaf Blade</v>
       </c>
       <c r="B26" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="C26" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="E26" t="str">
         <v>2</v>
       </c>
       <c r="F26" t="str">
         <v>2</v>
+      </c>
+      <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
+        <v/>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v/>
+      </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+      <c r="T26" t="str">
+        <v/>
+      </c>
+      <c r="U26" t="str">
+        <v/>
+      </c>
+      <c r="V26" t="str">
+        <v/>
+      </c>
+      <c r="W26" t="str">
+        <v/>
+      </c>
+      <c r="X26" t="str">
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Earth</v>
+        <v>Needle Storm</v>
       </c>
       <c r="B27" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="C27" t="str">
         <v>Sand</v>
       </c>
+      <c r="D27" t="str">
+        <v>20</v>
+      </c>
       <c r="E27" t="str">
         <v>2</v>
       </c>
       <c r="F27" t="str">
         <v>2</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J27" t="str">
+        <v>multihit</v>
+      </c>
+      <c r="K27" t="str">
+        <v/>
+      </c>
+      <c r="L27" t="str">
+        <v>10</v>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+      <c r="U27" t="str">
+        <v/>
+      </c>
+      <c r="V27" t="str">
+        <v/>
+      </c>
+      <c r="W27" t="str">
+        <v/>
+      </c>
+      <c r="X27" t="str">
+        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Blaze Blade</v>
+        <v>Photosynthesis</v>
       </c>
       <c r="B28" t="str">
-        <v>Steel</v>
+        <v>Leaf</v>
       </c>
       <c r="C28" t="str">
-        <v>Fire</v>
+        <v>Leaf</v>
       </c>
       <c r="E28" t="str">
         <v>2</v>
@@ -1669,13 +2002,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Aqua Blade</v>
+        <v>Desert Blade</v>
       </c>
       <c r="B29" t="str">
+        <v>Sand</v>
+      </c>
+      <c r="C29" t="str">
         <v>Steel</v>
-      </c>
-      <c r="C29" t="str">
-        <v>Water</v>
       </c>
       <c r="E29" t="str">
         <v>2</v>
@@ -1686,13 +2019,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Voltage</v>
+        <v>Mud Shot</v>
       </c>
       <c r="B30" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="C30" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="E30" t="str">
         <v>2</v>
@@ -1703,10 +2036,10 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Cleave</v>
+        <v>Sand Shield</v>
       </c>
       <c r="B31" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="C31" t="str">
         <v>Earth</v>
@@ -1720,10 +2053,10 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Quick Strike</v>
+        <v>Sandstorm</v>
       </c>
       <c r="B32" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="C32" t="str">
         <v>Air</v>
@@ -1737,10 +2070,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Ice Blade</v>
+        <v>Iceblast</v>
       </c>
       <c r="B33" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="C33" t="str">
         <v>Ice</v>
@@ -1754,13 +2087,13 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Refined Steel</v>
+        <v>Blaze Blade</v>
       </c>
       <c r="B34" t="str">
         <v>Steel</v>
       </c>
       <c r="C34" t="str">
-        <v>Steel</v>
+        <v>Fire</v>
       </c>
       <c r="E34" t="str">
         <v>2</v>
@@ -1771,13 +2104,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Plasma</v>
+        <v>Aqua Blade</v>
       </c>
       <c r="B35" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
       </c>
       <c r="C35" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="E35" t="str">
         <v>2</v>
@@ -1788,13 +2121,13 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Water Bolt</v>
+        <v>Thunder Blade</v>
       </c>
       <c r="B36" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="C36" t="str">
         <v>Lightning</v>
-      </c>
-      <c r="C36" t="str">
-        <v>Water</v>
       </c>
       <c r="E36" t="str">
         <v>2</v>
@@ -1805,10 +2138,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Plasma</v>
+        <v>Earth Blade</v>
       </c>
       <c r="B37" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
       </c>
       <c r="C37" t="str">
         <v>Earth</v>
@@ -1822,10 +2155,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Plasma</v>
+        <v>Air Blade</v>
       </c>
       <c r="B38" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
       </c>
       <c r="C38" t="str">
         <v>Air</v>
@@ -1839,10 +2172,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Ice Bolt</v>
+        <v>Ice Blade</v>
       </c>
       <c r="B39" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
       </c>
       <c r="C39" t="str">
         <v>Ice</v>
@@ -1856,13 +2189,13 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Thunder</v>
+        <v>Refined Steel</v>
       </c>
       <c r="B40" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
       </c>
       <c r="C40" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
       </c>
       <c r="E40" t="str">
         <v>2</v>
@@ -1873,13 +2206,13 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Fire</v>
+        <v>Water Bolt</v>
       </c>
       <c r="B41" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C41" t="str">
         <v>Water</v>
-      </c>
-      <c r="C41" t="str">
-        <v>Air</v>
       </c>
       <c r="E41" t="str">
         <v>2</v>
@@ -1890,13 +2223,13 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Mud Shot</v>
+        <v>Ice Bolt</v>
       </c>
       <c r="B42" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="C42" t="str">
-        <v>Sand</v>
+        <v>Ice</v>
       </c>
       <c r="E42" t="str">
         <v>2</v>
@@ -1907,13 +2240,13 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Worble</v>
+        <v>Thunder</v>
       </c>
       <c r="B43" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="C43" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="E43" t="str">
         <v>2</v>
@@ -1924,13 +2257,13 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Ice</v>
+        <v>Mud Shot</v>
       </c>
       <c r="B44" t="str">
         <v>Water</v>
       </c>
       <c r="C44" t="str">
-        <v>Air</v>
+        <v>Sand</v>
       </c>
       <c r="E44" t="str">
         <v>2</v>
@@ -1941,13 +2274,13 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Air</v>
+        <v>Worble</v>
       </c>
       <c r="B45" t="str">
         <v>Water</v>
       </c>
       <c r="C45" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="E45" t="str">
         <v>2</v>
@@ -1975,13 +2308,13 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Lightning</v>
+        <v>Hailstorm</v>
       </c>
       <c r="B47" t="str">
         <v>Air</v>
       </c>
       <c r="C47" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="E47" t="str">
         <v>2</v>
@@ -1992,13 +2325,13 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Hailstorm</v>
+        <v>Pyreball</v>
       </c>
       <c r="B48" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="C48" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="E48" t="str">
         <v>2</v>
@@ -2009,10 +2342,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Sand</v>
+        <v>Ice Shield</v>
       </c>
       <c r="B49" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="C49" t="str">
         <v>Earth</v>
@@ -2026,10 +2359,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Water</v>
+        <v>Glacier</v>
       </c>
       <c r="B50" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="C50" t="str">
         <v>Ice</v>
@@ -2043,10 +2376,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Steel</v>
+        <v>Earthquake</v>
       </c>
       <c r="B51" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="C51" t="str">
         <v>Earth</v>
@@ -2058,77 +2391,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <v>Pyreball</v>
-      </c>
-      <c r="B52" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="C52" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="E52" t="str">
-        <v>2</v>
-      </c>
-      <c r="F52" t="str">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>Ice Shield</v>
-      </c>
-      <c r="B53" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="C53" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="E53" t="str">
-        <v>2</v>
-      </c>
-      <c r="F53" t="str">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>Tundra</v>
-      </c>
-      <c r="B54" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="C54" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="E54" t="str">
-        <v>2</v>
-      </c>
-      <c r="F54" t="str">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>Earthquake</v>
-      </c>
-      <c r="B55" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="C55" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="E55" t="str">
-        <v>2</v>
-      </c>
-      <c r="F55" t="str">
-        <v>2</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X55"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (f677367) Update potion
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z51"/>
+  <dimension ref="A1:AB53"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -472,19 +472,31 @@
       <c r="X1" t="str">
         <v>Effect 3 Target</v>
       </c>
+      <c r="Y1" t="str">
+        <v>__EMPTY</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>__EMPTY_1</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Type 1</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>Type 2</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="B2" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
       <c r="C2" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E2" t="str">
         <v>1</v>
@@ -493,19 +505,19 @@
         <v>1</v>
       </c>
       <c r="G2" t="str">
-        <v>A gift from the sky goddess</v>
+        <v>A bright flame burning hot</v>
       </c>
       <c r="H2" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="I2" t="str">
         <v/>
       </c>
       <c r="J2" t="str">
-        <v>heal</v>
+        <v/>
       </c>
       <c r="K2" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="L2" t="str">
         <v/>
@@ -514,19 +526,19 @@
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O2" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P2" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="Q2" t="str">
         <v/>
       </c>
       <c r="R2" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -544,21 +556,33 @@
         <v/>
       </c>
       <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="AB2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="B3" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="C3" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E3" t="str">
         <v>1</v>
@@ -567,25 +591,25 @@
         <v>1</v>
       </c>
       <c r="G3" t="str">
-        <v>A bright flame burning hot</v>
+        <v>A gift from the sky goddess</v>
       </c>
       <c r="H3" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="I3" t="str">
         <v/>
       </c>
       <c r="J3" t="str">
-        <v>burn</v>
+        <v/>
       </c>
       <c r="K3" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="L3" t="str">
         <v/>
       </c>
       <c r="M3" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="N3" t="str">
         <v/>
@@ -618,21 +642,33 @@
         <v/>
       </c>
       <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AB3" t="str">
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="B4" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
       <c r="C4" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
       <c r="D4" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="E4" t="str">
         <v>1</v>
@@ -641,10 +677,10 @@
         <v>1</v>
       </c>
       <c r="G4" t="str">
-        <v/>
+        <v>It's a rock</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -698,21 +734,27 @@
         <v/>
       </c>
       <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB4" t="str">
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="B5" t="str">
-        <v>Sand</v>
+        <v>Ice</v>
       </c>
       <c r="C5" t="str">
-        <v>Sand</v>
+        <v>Fire</v>
       </c>
       <c r="D5" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E5" t="str">
         <v>1</v>
@@ -721,16 +763,16 @@
         <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v>It's a leaf</v>
+        <v>A gift from the sky goddess</v>
       </c>
       <c r="H5" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="I5" t="str">
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>shield</v>
+        <v>heal</v>
       </c>
       <c r="K5" t="str">
         <v>5</v>
@@ -742,19 +784,19 @@
         <v/>
       </c>
       <c r="N5" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O5" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="P5" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q5" t="str">
         <v/>
       </c>
       <c r="R5" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="S5" t="str">
         <v/>
@@ -772,21 +814,33 @@
         <v/>
       </c>
       <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5" t="str">
+        <v/>
+      </c>
+      <c r="AB5" t="str">
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Lightning</v>
+        <v>Fire</v>
       </c>
       <c r="B6" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C6" t="str">
         <v>Air</v>
       </c>
-      <c r="C6" t="str">
-        <v>Fire</v>
-      </c>
       <c r="D6" t="str">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E6" t="str">
         <v>1</v>
@@ -795,25 +849,25 @@
         <v>1</v>
       </c>
       <c r="G6" t="str">
-        <v>Charged spark that strikes instantly</v>
+        <v>A bright flame burning hot</v>
       </c>
       <c r="H6" t="str">
-        <v>Lightning</v>
+        <v>Fire</v>
       </c>
       <c r="I6" t="str">
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>multihit</v>
+        <v>burn</v>
       </c>
       <c r="K6" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="L6" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="N6" t="str">
         <v/>
@@ -846,18 +900,33 @@
         <v/>
       </c>
       <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
+        <v/>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+      <c r="AA6" t="str">
+        <v/>
+      </c>
+      <c r="AB6" t="str">
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Plasma</v>
+        <v>Fire</v>
       </c>
       <c r="B7" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="C7" t="str">
         <v>Lightning</v>
       </c>
-      <c r="C7" t="str">
-        <v>Air</v>
+      <c r="D7" t="str">
+        <v>10</v>
       </c>
       <c r="E7" t="str">
         <v>1</v>
@@ -865,19 +934,85 @@
       <c r="F7" t="str">
         <v>1</v>
       </c>
+      <c r="G7" t="str">
+        <v>A bright flame burning hot</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v/>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+      <c r="X7" t="str">
+        <v/>
+      </c>
+      <c r="Y7" t="str">
+        <v/>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
+      </c>
+      <c r="AA7" t="str">
+        <v/>
+      </c>
+      <c r="AB7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Plasma</v>
+        <v>Earth</v>
       </c>
       <c r="B8" t="str">
-        <v>Lightning</v>
+        <v>Sand</v>
       </c>
       <c r="C8" t="str">
-        <v>Earth</v>
+        <v>Sand</v>
       </c>
       <c r="D8" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="E8" t="str">
         <v>1</v>
@@ -886,19 +1021,19 @@
         <v>1</v>
       </c>
       <c r="G8" t="str">
-        <v/>
+        <v>It's a rock</v>
       </c>
       <c r="H8" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
       <c r="I8" t="str">
         <v/>
       </c>
       <c r="J8" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="K8" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="L8" t="str">
         <v/>
@@ -943,24 +1078,99 @@
         <v/>
       </c>
       <c r="Z8" t="str">
+        <v/>
+      </c>
+      <c r="AA8" t="str">
+        <v/>
+      </c>
+      <c r="AB8" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Plasma</v>
+        <v>Lightning</v>
       </c>
       <c r="B9" t="str">
-        <v>Lightning</v>
+        <v>Air</v>
       </c>
       <c r="C9" t="str">
         <v>Fire</v>
       </c>
+      <c r="D9" t="str">
+        <v>7</v>
+      </c>
       <c r="E9" t="str">
         <v>1</v>
       </c>
       <c r="F9" t="str">
         <v>1</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Charged spark that strikes instantly</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v>multihit</v>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v>2</v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v/>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
+      </c>
+      <c r="AA9" t="str">
+        <v/>
+      </c>
+      <c r="AB9" t="str">
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -968,10 +1178,10 @@
         <v>Plasma</v>
       </c>
       <c r="B10" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="C10" t="str">
-        <v>Lightning</v>
+        <v>Air</v>
       </c>
       <c r="D10" t="str">
         <v>1</v>
@@ -986,24 +1196,81 @@
         <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H10" t="str">
-        <v>Fire</v>
+        <v>Plasma</v>
       </c>
       <c r="I10" t="str">
-        <v>Lightning</v>
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v/>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+      <c r="AA10" t="str">
+        <v/>
+      </c>
+      <c r="AB10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Sand</v>
+        <v>Plasma</v>
       </c>
       <c r="B11" t="str">
-        <v>Earth</v>
+        <v>Lightning</v>
       </c>
       <c r="C11" t="str">
         <v>Earth</v>
       </c>
       <c r="D11" t="str">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E11" t="str">
         <v>1</v>
@@ -1012,24 +1279,84 @@
         <v>1</v>
       </c>
       <c r="G11" t="str">
-        <v>Shifting grains dance between your fingertips</v>
+        <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H11" t="str">
-        <v>Earth</v>
+        <v>Plasma</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v/>
+      </c>
+      <c r="Z11" t="str">
+        <v/>
+      </c>
+      <c r="AA11" t="str">
+        <v/>
+      </c>
+      <c r="AB11" t="str">
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Sand</v>
+        <v>Plasma</v>
       </c>
       <c r="B12" t="str">
-        <v>Air</v>
+        <v>Lightning</v>
       </c>
       <c r="C12" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="D12" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E12" t="str">
         <v>1</v>
@@ -1038,10 +1365,10 @@
         <v>1</v>
       </c>
       <c r="G12" t="str">
-        <v/>
+        <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H12" t="str">
-        <v/>
+        <v>Plasma</v>
       </c>
       <c r="I12" t="str">
         <v/>
@@ -1095,21 +1422,27 @@
         <v/>
       </c>
       <c r="Z12" t="str">
+        <v/>
+      </c>
+      <c r="AA12" t="str">
+        <v/>
+      </c>
+      <c r="AB12" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Steel</v>
+        <v>Plasma</v>
       </c>
       <c r="B13" t="str">
         <v>Fire</v>
       </c>
       <c r="C13" t="str">
-        <v>Earth</v>
+        <v>Lightning</v>
       </c>
       <c r="D13" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="E13" t="str">
         <v>1</v>
@@ -1118,13 +1451,13 @@
         <v>1</v>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>Fire</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>Lightning</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -1175,21 +1508,27 @@
         <v/>
       </c>
       <c r="Z13" t="str">
+        <v/>
+      </c>
+      <c r="AA13" t="str">
+        <v/>
+      </c>
+      <c r="AB13" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Air</v>
+        <v>Sand</v>
       </c>
       <c r="B14" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="C14" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D14" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="E14" t="str">
         <v>1</v>
@@ -1198,10 +1537,10 @@
         <v>1</v>
       </c>
       <c r="G14" t="str">
-        <v/>
+        <v>Shifting grains dance between your fingertips</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
       <c r="I14" t="str">
         <v/>
@@ -1255,21 +1594,27 @@
         <v/>
       </c>
       <c r="Z14" t="str">
+        <v/>
+      </c>
+      <c r="AA14" t="str">
+        <v/>
+      </c>
+      <c r="AB14" t="str">
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="B15" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="C15" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="D15" t="str">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E15" t="str">
         <v>1</v>
@@ -1278,27 +1623,84 @@
         <v>1</v>
       </c>
       <c r="G15" t="str">
-        <v>Drops of dew glistle atop</v>
+        <v>Shifting grains dance between your fingertips</v>
       </c>
       <c r="H15" t="str">
         <v>Earth</v>
       </c>
       <c r="I15" t="str">
-        <v>Water</v>
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
+        <v/>
+      </c>
+      <c r="M15" t="str">
+        <v/>
+      </c>
+      <c r="N15" t="str">
+        <v/>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
+        <v/>
+      </c>
+      <c r="R15" t="str">
+        <v/>
+      </c>
+      <c r="S15" t="str">
+        <v/>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v/>
+      </c>
+      <c r="V15" t="str">
+        <v/>
+      </c>
+      <c r="W15" t="str">
+        <v/>
+      </c>
+      <c r="X15" t="str">
+        <v/>
+      </c>
+      <c r="Y15" t="str">
+        <v/>
+      </c>
+      <c r="Z15" t="str">
+        <v/>
+      </c>
+      <c r="AA15" t="str">
+        <v/>
+      </c>
+      <c r="AB15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="B16" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="C16" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
       <c r="D16" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="E16" t="str">
         <v>1</v>
@@ -1307,10 +1709,10 @@
         <v>1</v>
       </c>
       <c r="G16" t="str">
-        <v/>
+        <v>Forged from fire and stone, hammered hard</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>Steel</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -1364,35 +1766,113 @@
         <v/>
       </c>
       <c r="Z16" t="str">
+        <v/>
+      </c>
+      <c r="AA16" t="str">
+        <v/>
+      </c>
+      <c r="AB16" t="str">
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Glass</v>
+        <v>Air</v>
       </c>
       <c r="B17" t="str">
-        <v>Sand</v>
+        <v>Water</v>
       </c>
       <c r="C17" t="str">
         <v>Fire</v>
       </c>
+      <c r="D17" t="str">
+        <v>10</v>
+      </c>
       <c r="E17" t="str">
         <v>1</v>
       </c>
       <c r="F17" t="str">
         <v>1</v>
       </c>
+      <c r="G17" t="str">
+        <v>A cool rush of wind drifts past your face</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Air</v>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v/>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
+        <v/>
+      </c>
+      <c r="R17" t="str">
+        <v/>
+      </c>
+      <c r="S17" t="str">
+        <v/>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v/>
+      </c>
+      <c r="V17" t="str">
+        <v/>
+      </c>
+      <c r="W17" t="str">
+        <v/>
+      </c>
+      <c r="X17" t="str">
+        <v/>
+      </c>
+      <c r="Y17" t="str">
+        <v/>
+      </c>
+      <c r="Z17" t="str">
+        <v/>
+      </c>
+      <c r="AA17" t="str">
+        <v/>
+      </c>
+      <c r="AB17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Glass</v>
+        <v>Leaf</v>
       </c>
       <c r="B18" t="str">
-        <v>Sand</v>
+        <v>Earth</v>
       </c>
       <c r="C18" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
+      </c>
+      <c r="D18" t="str">
+        <v>8</v>
       </c>
       <c r="E18" t="str">
         <v>1</v>
@@ -1400,57 +1880,183 @@
       <c r="F18" t="str">
         <v>1</v>
       </c>
+      <c r="G18" t="str">
+        <v>Drops of dew glistle atop</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Water</v>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v/>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+      <c r="V18" t="str">
+        <v/>
+      </c>
+      <c r="W18" t="str">
+        <v/>
+      </c>
+      <c r="X18" t="str">
+        <v/>
+      </c>
+      <c r="Y18" t="str">
+        <v/>
+      </c>
+      <c r="Z18" t="str">
+        <v/>
+      </c>
+      <c r="AA18" t="str">
+        <v/>
+      </c>
+      <c r="AB18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Dark Matter</v>
+        <v>Ice</v>
       </c>
       <c r="B19" t="str">
-        <v>Unstable Element</v>
+        <v>Water</v>
       </c>
       <c r="C19" t="str">
-        <v>Unstable Element</v>
+        <v>Air</v>
       </c>
       <c r="D19" t="str">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E19" t="str">
         <v>1</v>
       </c>
       <c r="F19" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" t="str">
-        <v>A quiet humming radiates from inside</v>
+        <v>A biting chill that settles in your bones</v>
       </c>
       <c r="H19" t="str">
-        <v>Void</v>
+        <v>Ice</v>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+      <c r="V19" t="str">
+        <v/>
+      </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <v/>
+      </c>
+      <c r="Y19" t="str">
+        <v/>
+      </c>
+      <c r="Z19" t="str">
+        <v/>
+      </c>
+      <c r="AA19" t="str">
+        <v/>
+      </c>
+      <c r="AB19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Worble</v>
+        <v>Glass</v>
       </c>
       <c r="B20" t="str">
-        <v>Water</v>
+        <v>Sand</v>
       </c>
       <c r="C20" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="D20" t="str">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="E20" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G20" t="str">
-        <v>The tide is high today my friend</v>
+        <v>Smooth and brittle, it catches the light</v>
       </c>
       <c r="H20" t="str">
-        <v>Water</v>
+        <v>Glass</v>
       </c>
       <c r="I20" t="str">
         <v/>
@@ -1498,27 +2104,45 @@
         <v/>
       </c>
       <c r="X20" t="str">
+        <v/>
+      </c>
+      <c r="Y20" t="str">
+        <v/>
+      </c>
+      <c r="Z20" t="str">
+        <v/>
+      </c>
+      <c r="AA20" t="str">
+        <v/>
+      </c>
+      <c r="AB20" t="str">
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Blaze</v>
+        <v>Glass</v>
       </c>
       <c r="B21" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C21" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="D21" t="str">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="E21" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="str">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Smooth and brittle, it catches the light</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Glass</v>
       </c>
       <c r="I21" t="str">
         <v/>
@@ -1566,28 +2190,46 @@
         <v/>
       </c>
       <c r="X21" t="str">
+        <v/>
+      </c>
+      <c r="Y21" t="str">
+        <v/>
+      </c>
+      <c r="Z21" t="str">
+        <v/>
+      </c>
+      <c r="AA21" t="str">
+        <v/>
+      </c>
+      <c r="AB21" t="str">
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Regen</v>
+        <v>Dark Matter</v>
       </c>
       <c r="B22" t="str">
-        <v>Leaf</v>
+        <v>Unstable Element</v>
       </c>
       <c r="C22" t="str">
-        <v>Water</v>
+        <v>Unstable Element</v>
       </c>
       <c r="D22" t="str">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="E22" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="str">
         <v>2</v>
       </c>
+      <c r="G22" t="str">
+        <v>A quiet humming radiates from inside</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Void</v>
+      </c>
       <c r="I22" t="str">
         <v/>
       </c>
@@ -1634,45 +2276,63 @@
         <v/>
       </c>
       <c r="X22" t="str">
+        <v/>
+      </c>
+      <c r="Y22" t="str">
+        <v/>
+      </c>
+      <c r="Z22" t="str">
+        <v/>
+      </c>
+      <c r="AA22" t="str">
+        <v/>
+      </c>
+      <c r="AB22" t="str">
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Thorns</v>
+        <v>Worble</v>
       </c>
       <c r="B23" t="str">
-        <v>Leaf</v>
+        <v>Water</v>
       </c>
       <c r="C23" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="D23" t="str">
-        <v>32</v>
+        <v>126</v>
       </c>
       <c r="E23" t="str">
         <v>2</v>
       </c>
       <c r="F23" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G23" t="str">
-        <v>Leaves swirl around you</v>
+        <v>The tide is high today my friend</v>
       </c>
       <c r="H23" t="str">
-        <v>Earth</v>
+        <v>Water</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Water</v>
       </c>
       <c r="J23" t="str">
-        <v>shield</v>
+        <v>soak</v>
       </c>
       <c r="K23" t="str">
-        <v>15</v>
+        <v>4</v>
+      </c>
+      <c r="L23" t="str">
+        <v/>
       </c>
       <c r="M23" t="str">
         <v/>
       </c>
       <c r="N23" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="O23" t="str">
         <v/>
@@ -1703,56 +2363,68 @@
       </c>
       <c r="X23" t="str">
         <v/>
+      </c>
+      <c r="Y23" t="str">
+        <v/>
+      </c>
+      <c r="Z23" t="str">
+        <v/>
+      </c>
+      <c r="AA23" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AB23" t="str">
+        <v>Water</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Tornado</v>
+        <v>Blaze</v>
       </c>
       <c r="B24" t="str">
         <v>Leaf</v>
       </c>
       <c r="C24" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="D24" t="str">
-        <v>25</v>
+        <v>109</v>
       </c>
       <c r="E24" t="str">
         <v>2</v>
       </c>
       <c r="F24" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G24" t="str">
-        <v>Wind whips and slashes about</v>
+        <v>Forest floor erupts in scorching flame</v>
       </c>
       <c r="H24" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="I24" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
       <c r="J24" t="str">
-        <v>multihit</v>
+        <v>burn</v>
       </c>
       <c r="K24" t="str">
-        <v/>
+        <v>6</v>
       </c>
       <c r="L24" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="M24" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="N24" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="O24" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="P24" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="Q24" t="str">
         <v/>
@@ -1761,7 +2433,7 @@
         <v/>
       </c>
       <c r="S24" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="T24" t="str">
         <v/>
@@ -1777,38 +2449,53 @@
       </c>
       <c r="X24" t="str">
         <v/>
+      </c>
+      <c r="Y24" t="str">
+        <v/>
+      </c>
+      <c r="Z24" t="str">
+        <v/>
+      </c>
+      <c r="AA24" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="AB24" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Blizzard</v>
+        <v>Regen</v>
       </c>
       <c r="B25" t="str">
         <v>Leaf</v>
       </c>
       <c r="C25" t="str">
-        <v>Ice</v>
+        <v>Water</v>
+      </c>
+      <c r="D25" t="str">
+        <v>109</v>
       </c>
       <c r="E25" t="str">
         <v>2</v>
       </c>
       <c r="F25" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G25" t="str">
-        <v>Snow flurries and blocks your vision</v>
+        <v>Living vines wrap wounds in cool water</v>
       </c>
       <c r="H25" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="I25" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="J25" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="K25" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="L25" t="str">
         <v/>
@@ -1817,13 +2504,13 @@
         <v/>
       </c>
       <c r="N25" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O25" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="P25" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="Q25" t="str">
         <v/>
@@ -1832,7 +2519,7 @@
         <v/>
       </c>
       <c r="S25" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="T25" t="str">
         <v/>
@@ -1848,32 +2535,53 @@
       </c>
       <c r="X25" t="str">
         <v/>
+      </c>
+      <c r="Y25" t="str">
+        <v/>
+      </c>
+      <c r="Z25" t="str">
+        <v/>
+      </c>
+      <c r="AA25" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AB25" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Leaf Blade</v>
+        <v>Thorns</v>
       </c>
       <c r="B26" t="str">
         <v>Leaf</v>
       </c>
       <c r="C26" t="str">
-        <v>Steel</v>
+        <v>Earth</v>
+      </c>
+      <c r="D26" t="str">
+        <v>109</v>
       </c>
       <c r="E26" t="str">
         <v>2</v>
       </c>
       <c r="F26" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Spiked vines protect you</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Earth</v>
       </c>
       <c r="I26" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="J26" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="K26" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="L26" t="str">
         <v/>
@@ -1882,13 +2590,13 @@
         <v/>
       </c>
       <c r="N26" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O26" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="P26" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="Q26" t="str">
         <v/>
@@ -1897,7 +2605,7 @@
         <v/>
       </c>
       <c r="S26" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="T26" t="str">
         <v/>
@@ -1913,44 +2621,62 @@
       </c>
       <c r="X26" t="str">
         <v/>
+      </c>
+      <c r="Y26" t="str">
+        <v/>
+      </c>
+      <c r="Z26" t="str">
+        <v/>
+      </c>
+      <c r="AA26" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB26" t="str">
+        <v>Water</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Needle Storm</v>
+        <v>Tornado</v>
       </c>
       <c r="B27" t="str">
         <v>Leaf</v>
       </c>
       <c r="C27" t="str">
-        <v>Sand</v>
+        <v>Air</v>
       </c>
       <c r="D27" t="str">
-        <v>20</v>
+        <v>109</v>
       </c>
       <c r="E27" t="str">
         <v>2</v>
       </c>
       <c r="F27" t="str">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Wind whips and slashes about</v>
       </c>
       <c r="H27" t="str">
+        <v>Air</v>
+      </c>
+      <c r="I27" t="str">
         <v>Earth</v>
       </c>
       <c r="J27" t="str">
-        <v>multihit</v>
+        <v>shield</v>
       </c>
       <c r="K27" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="L27" t="str">
-        <v>10</v>
+        <v/>
       </c>
       <c r="M27" t="str">
         <v/>
       </c>
       <c r="N27" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O27" t="str">
         <v/>
@@ -1981,419 +2707,2259 @@
       </c>
       <c r="X27" t="str">
         <v/>
+      </c>
+      <c r="Y27" t="str">
+        <v/>
+      </c>
+      <c r="Z27" t="str">
+        <v/>
+      </c>
+      <c r="AA27" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AB27" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Photosynthesis</v>
+        <v>Blizzard</v>
       </c>
       <c r="B28" t="str">
         <v>Leaf</v>
       </c>
       <c r="C28" t="str">
-        <v>Leaf</v>
+        <v>Ice</v>
+      </c>
+      <c r="D28" t="str">
+        <v>109</v>
       </c>
       <c r="E28" t="str">
         <v>2</v>
       </c>
       <c r="F28" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Snow flurries block your vision</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J28" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K28" t="str">
+        <v>8</v>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v>self</v>
+      </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
+      <c r="T28" t="str">
+        <v/>
+      </c>
+      <c r="U28" t="str">
+        <v/>
+      </c>
+      <c r="V28" t="str">
+        <v/>
+      </c>
+      <c r="W28" t="str">
+        <v/>
+      </c>
+      <c r="X28" t="str">
+        <v/>
+      </c>
+      <c r="Y28" t="str">
+        <v/>
+      </c>
+      <c r="Z28" t="str">
+        <v/>
+      </c>
+      <c r="AA28" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="AB28" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Desert Blade</v>
+        <v>Leaf Blade</v>
       </c>
       <c r="B29" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="C29" t="str">
         <v>Steel</v>
       </c>
+      <c r="D29" t="str">
+        <v>159</v>
+      </c>
       <c r="E29" t="str">
         <v>2</v>
       </c>
       <c r="F29" t="str">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="G29" t="str">
+        <v>A razor edge honed from living wood</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Water</v>
+      </c>
+      <c r="J29" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K29" t="str">
+        <v>8</v>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v>self</v>
+      </c>
+      <c r="O29" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P29" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="T29" t="str">
+        <v/>
+      </c>
+      <c r="U29" t="str">
+        <v/>
+      </c>
+      <c r="V29" t="str">
+        <v/>
+      </c>
+      <c r="W29" t="str">
+        <v/>
+      </c>
+      <c r="X29" t="str">
+        <v/>
+      </c>
+      <c r="Y29" t="str">
+        <v/>
+      </c>
+      <c r="Z29" t="str">
+        <v/>
+      </c>
+      <c r="AA29" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB29" t="str">
+        <v>Water</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Mud Shot</v>
+        <v>Needle Storm</v>
       </c>
       <c r="B30" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="C30" t="str">
         <v>Sand</v>
       </c>
-      <c r="C30" t="str">
+      <c r="D30" t="str">
+        <v>159</v>
+      </c>
+      <c r="E30" t="str">
+        <v>2</v>
+      </c>
+      <c r="F30" t="str">
+        <v>7</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Tiny needles prick from every angle</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I30" t="str">
         <v>Water</v>
       </c>
-      <c r="E30" t="str">
-        <v>2</v>
-      </c>
-      <c r="F30" t="str">
-        <v>2</v>
+      <c r="J30" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K30" t="str">
+        <v>8</v>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v>self</v>
+      </c>
+      <c r="O30" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P30" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
+      <c r="R30" t="str">
+        <v/>
+      </c>
+      <c r="S30" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="T30" t="str">
+        <v/>
+      </c>
+      <c r="U30" t="str">
+        <v/>
+      </c>
+      <c r="V30" t="str">
+        <v/>
+      </c>
+      <c r="W30" t="str">
+        <v/>
+      </c>
+      <c r="X30" t="str">
+        <v/>
+      </c>
+      <c r="Y30" t="str">
+        <v/>
+      </c>
+      <c r="Z30" t="str">
+        <v/>
+      </c>
+      <c r="AA30" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB30" t="str">
+        <v>Water</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Sand Shield</v>
+        <v>Photosynthesis</v>
       </c>
       <c r="B31" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="C31" t="str">
-        <v>Earth</v>
+        <v>Leaf</v>
+      </c>
+      <c r="D31" t="str">
+        <v>210</v>
       </c>
       <c r="E31" t="str">
         <v>2</v>
       </c>
       <c r="F31" t="str">
-        <v>2</v>
+        <v>9</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Nature feeds itself to grow ever stronger</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Water</v>
+      </c>
+      <c r="J31" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K31" t="str">
+        <v>8</v>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
+      <c r="N31" t="str">
+        <v>self</v>
+      </c>
+      <c r="O31" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P31" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
+      <c r="R31" t="str">
+        <v/>
+      </c>
+      <c r="S31" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="T31" t="str">
+        <v/>
+      </c>
+      <c r="U31" t="str">
+        <v/>
+      </c>
+      <c r="V31" t="str">
+        <v/>
+      </c>
+      <c r="W31" t="str">
+        <v/>
+      </c>
+      <c r="X31" t="str">
+        <v/>
+      </c>
+      <c r="Y31" t="str">
+        <v/>
+      </c>
+      <c r="Z31" t="str">
+        <v/>
+      </c>
+      <c r="AA31" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB31" t="str">
+        <v>Water</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Sandstorm</v>
+        <v>Desert Blade</v>
       </c>
       <c r="B32" t="str">
         <v>Sand</v>
       </c>
       <c r="C32" t="str">
-        <v>Air</v>
+        <v>Steel</v>
+      </c>
+      <c r="D32" t="str">
+        <v>159</v>
       </c>
       <c r="E32" t="str">
         <v>2</v>
       </c>
       <c r="F32" t="str">
-        <v>2</v>
+        <v>7</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Sand-forged steel scorched by the desert sun</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="J32" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K32" t="str">
+        <v>6</v>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v>2</v>
+      </c>
+      <c r="N32" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O32" t="str">
+        <v>shield</v>
+      </c>
+      <c r="P32" t="str">
+        <v>8</v>
+      </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
+      <c r="R32" t="str">
+        <v/>
+      </c>
+      <c r="S32" t="str">
+        <v>self</v>
+      </c>
+      <c r="T32" t="str">
+        <v/>
+      </c>
+      <c r="U32" t="str">
+        <v/>
+      </c>
+      <c r="V32" t="str">
+        <v/>
+      </c>
+      <c r="W32" t="str">
+        <v/>
+      </c>
+      <c r="X32" t="str">
+        <v/>
+      </c>
+      <c r="Y32" t="str">
+        <v/>
+      </c>
+      <c r="Z32" t="str">
+        <v/>
+      </c>
+      <c r="AA32" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB32" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Iceblast</v>
+        <v>Mud Shot</v>
       </c>
       <c r="B33" t="str">
         <v>Sand</v>
       </c>
       <c r="C33" t="str">
-        <v>Ice</v>
+        <v>Water</v>
+      </c>
+      <c r="D33" t="str">
+        <v>109</v>
       </c>
       <c r="E33" t="str">
         <v>2</v>
       </c>
       <c r="F33" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Thick sludge launched with surprising force</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Water</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J33" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K33" t="str">
+        <v>8</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v>self</v>
+      </c>
+      <c r="O33" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P33" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
+      <c r="S33" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
+        <v/>
+      </c>
+      <c r="V33" t="str">
+        <v/>
+      </c>
+      <c r="W33" t="str">
+        <v/>
+      </c>
+      <c r="X33" t="str">
+        <v/>
+      </c>
+      <c r="Y33" t="str">
+        <v/>
+      </c>
+      <c r="Z33" t="str">
+        <v/>
+      </c>
+      <c r="AA33" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AB33" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Blaze Blade</v>
+        <v>Sand Shield</v>
       </c>
       <c r="B34" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="C34" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
+      </c>
+      <c r="D34" t="str">
+        <v>109</v>
       </c>
       <c r="E34" t="str">
         <v>2</v>
       </c>
       <c r="F34" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Grains pack tight into an earthen wall</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K34" t="str">
+        <v>8</v>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v>self</v>
+      </c>
+      <c r="O34" t="str">
+        <v/>
+      </c>
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
+      <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
+        <v/>
+      </c>
+      <c r="U34" t="str">
+        <v/>
+      </c>
+      <c r="V34" t="str">
+        <v/>
+      </c>
+      <c r="W34" t="str">
+        <v/>
+      </c>
+      <c r="X34" t="str">
+        <v/>
+      </c>
+      <c r="Y34" t="str">
+        <v/>
+      </c>
+      <c r="Z34" t="str">
+        <v/>
+      </c>
+      <c r="AA34" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB34" t="str">
+        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Aqua Blade</v>
+        <v>Sandstorm</v>
       </c>
       <c r="B35" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="C35" t="str">
-        <v>Water</v>
+        <v>Air</v>
+      </c>
+      <c r="D35" t="str">
+        <v>109</v>
       </c>
       <c r="E35" t="str">
         <v>2</v>
       </c>
       <c r="F35" t="str">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Blinding grit swirls on howling winds</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Air</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J35" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K35" t="str">
+        <v>8</v>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v>self</v>
+      </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
+      <c r="S35" t="str">
+        <v/>
+      </c>
+      <c r="T35" t="str">
+        <v/>
+      </c>
+      <c r="U35" t="str">
+        <v/>
+      </c>
+      <c r="V35" t="str">
+        <v/>
+      </c>
+      <c r="W35" t="str">
+        <v/>
+      </c>
+      <c r="X35" t="str">
+        <v/>
+      </c>
+      <c r="Y35" t="str">
+        <v/>
+      </c>
+      <c r="Z35" t="str">
+        <v/>
+      </c>
+      <c r="AA35" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AB35" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Thunder Blade</v>
+        <v>Iceblast</v>
       </c>
       <c r="B36" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="C36" t="str">
-        <v>Lightning</v>
+        <v>Ice</v>
+      </c>
+      <c r="D36" t="str">
+        <v>109</v>
       </c>
       <c r="E36" t="str">
         <v>2</v>
       </c>
       <c r="F36" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Cold grit bites with a frosty sting</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J36" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K36" t="str">
+        <v>8</v>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v>self</v>
+      </c>
+      <c r="O36" t="str">
+        <v/>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
+      <c r="R36" t="str">
+        <v/>
+      </c>
+      <c r="S36" t="str">
+        <v/>
+      </c>
+      <c r="T36" t="str">
+        <v/>
+      </c>
+      <c r="U36" t="str">
+        <v/>
+      </c>
+      <c r="V36" t="str">
+        <v/>
+      </c>
+      <c r="W36" t="str">
+        <v/>
+      </c>
+      <c r="X36" t="str">
+        <v/>
+      </c>
+      <c r="Y36" t="str">
+        <v/>
+      </c>
+      <c r="Z36" t="str">
+        <v/>
+      </c>
+      <c r="AA36" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="AB36" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Earth Blade</v>
+        <v>Blaze Blade</v>
       </c>
       <c r="B37" t="str">
         <v>Steel</v>
       </c>
       <c r="C37" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
+      </c>
+      <c r="D37" t="str">
+        <v>109</v>
       </c>
       <c r="E37" t="str">
         <v>2</v>
       </c>
       <c r="F37" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G37" t="str">
+        <v>A steel blade bathed in white-hot flame</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J37" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K37" t="str">
+        <v>6</v>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <v>2</v>
+      </c>
+      <c r="N37" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O37" t="str">
+        <v>shield</v>
+      </c>
+      <c r="P37" t="str">
+        <v>8</v>
+      </c>
+      <c r="Q37" t="str">
+        <v/>
+      </c>
+      <c r="R37" t="str">
+        <v/>
+      </c>
+      <c r="S37" t="str">
+        <v>self</v>
+      </c>
+      <c r="T37" t="str">
+        <v/>
+      </c>
+      <c r="U37" t="str">
+        <v/>
+      </c>
+      <c r="V37" t="str">
+        <v/>
+      </c>
+      <c r="W37" t="str">
+        <v/>
+      </c>
+      <c r="X37" t="str">
+        <v/>
+      </c>
+      <c r="Y37" t="str">
+        <v/>
+      </c>
+      <c r="Z37" t="str">
+        <v/>
+      </c>
+      <c r="AA37" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="AB37" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Air Blade</v>
+        <v>Aqua Blade</v>
       </c>
       <c r="B38" t="str">
         <v>Steel</v>
       </c>
       <c r="C38" t="str">
-        <v>Air</v>
+        <v>Water</v>
+      </c>
+      <c r="D38" t="str">
+        <v>109</v>
       </c>
       <c r="E38" t="str">
         <v>2</v>
       </c>
       <c r="F38" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Steam rises where cold steel meets the wave</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Water</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="J38" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K38" t="str">
+        <v>6</v>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <v>2</v>
+      </c>
+      <c r="N38" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O38" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P38" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
+      <c r="R38" t="str">
+        <v/>
+      </c>
+      <c r="S38" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="T38" t="str">
+        <v/>
+      </c>
+      <c r="U38" t="str">
+        <v/>
+      </c>
+      <c r="V38" t="str">
+        <v/>
+      </c>
+      <c r="W38" t="str">
+        <v/>
+      </c>
+      <c r="X38" t="str">
+        <v/>
+      </c>
+      <c r="Y38" t="str">
+        <v/>
+      </c>
+      <c r="Z38" t="str">
+        <v/>
+      </c>
+      <c r="AA38" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AB38" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Ice Blade</v>
+        <v>Thunder Blade</v>
       </c>
       <c r="B39" t="str">
         <v>Steel</v>
       </c>
       <c r="C39" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
+      </c>
+      <c r="D39" t="str">
+        <v>109</v>
       </c>
       <c r="E39" t="str">
         <v>2</v>
       </c>
       <c r="F39" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Lightning arcs along the edge with every swing</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="J39" t="str">
+        <v>multi_hit</v>
+      </c>
+      <c r="K39" t="str">
+        <v/>
+      </c>
+      <c r="L39" t="str">
+        <v>2</v>
+      </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+      <c r="N39" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O39" t="str">
+        <v>burn</v>
+      </c>
+      <c r="P39" t="str">
+        <v>6</v>
+      </c>
+      <c r="Q39" t="str">
+        <v/>
+      </c>
+      <c r="R39" t="str">
+        <v>2</v>
+      </c>
+      <c r="S39" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="T39" t="str">
+        <v/>
+      </c>
+      <c r="U39" t="str">
+        <v/>
+      </c>
+      <c r="V39" t="str">
+        <v/>
+      </c>
+      <c r="W39" t="str">
+        <v/>
+      </c>
+      <c r="X39" t="str">
+        <v/>
+      </c>
+      <c r="Y39" t="str">
+        <v/>
+      </c>
+      <c r="Z39" t="str">
+        <v/>
+      </c>
+      <c r="AA39" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="AB39" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Refined Steel</v>
+        <v>Earth Blade</v>
       </c>
       <c r="B40" t="str">
         <v>Steel</v>
       </c>
       <c r="C40" t="str">
-        <v>Steel</v>
+        <v>Earth</v>
+      </c>
+      <c r="D40" t="str">
+        <v>109</v>
       </c>
       <c r="E40" t="str">
         <v>2</v>
       </c>
       <c r="F40" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Heavy as bedrock, it burns on impact</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="J40" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K40" t="str">
+        <v>6</v>
+      </c>
+      <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
+        <v>2</v>
+      </c>
+      <c r="N40" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O40" t="str">
+        <v>shield</v>
+      </c>
+      <c r="P40" t="str">
+        <v>8</v>
+      </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
+      <c r="R40" t="str">
+        <v/>
+      </c>
+      <c r="S40" t="str">
+        <v>self</v>
+      </c>
+      <c r="T40" t="str">
+        <v/>
+      </c>
+      <c r="U40" t="str">
+        <v/>
+      </c>
+      <c r="V40" t="str">
+        <v/>
+      </c>
+      <c r="W40" t="str">
+        <v/>
+      </c>
+      <c r="X40" t="str">
+        <v/>
+      </c>
+      <c r="Y40" t="str">
+        <v/>
+      </c>
+      <c r="Z40" t="str">
+        <v/>
+      </c>
+      <c r="AA40" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB40" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Water Bolt</v>
+        <v>Air Blade</v>
       </c>
       <c r="B41" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
       </c>
       <c r="C41" t="str">
-        <v>Water</v>
+        <v>Air</v>
+      </c>
+      <c r="D41" t="str">
+        <v>109</v>
       </c>
       <c r="E41" t="str">
         <v>2</v>
       </c>
       <c r="F41" t="str">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Cuts the air so fast it ignites</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Air</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="J41" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K41" t="str">
+        <v>6</v>
+      </c>
+      <c r="L41" t="str">
+        <v/>
+      </c>
+      <c r="M41" t="str">
+        <v>2</v>
+      </c>
+      <c r="N41" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O41" t="str">
+        <v/>
+      </c>
+      <c r="P41" t="str">
+        <v/>
+      </c>
+      <c r="Q41" t="str">
+        <v/>
+      </c>
+      <c r="R41" t="str">
+        <v/>
+      </c>
+      <c r="S41" t="str">
+        <v/>
+      </c>
+      <c r="T41" t="str">
+        <v/>
+      </c>
+      <c r="U41" t="str">
+        <v/>
+      </c>
+      <c r="V41" t="str">
+        <v/>
+      </c>
+      <c r="W41" t="str">
+        <v/>
+      </c>
+      <c r="X41" t="str">
+        <v/>
+      </c>
+      <c r="Y41" t="str">
+        <v/>
+      </c>
+      <c r="Z41" t="str">
+        <v/>
+      </c>
+      <c r="AA41" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AB41" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Ice Bolt</v>
+        <v>Ice Blade</v>
       </c>
       <c r="B42" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
       </c>
       <c r="C42" t="str">
         <v>Ice</v>
       </c>
+      <c r="D42" t="str">
+        <v>109</v>
+      </c>
       <c r="E42" t="str">
         <v>2</v>
       </c>
       <c r="F42" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Cold steel that somehow scorches on contact</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="J42" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K42" t="str">
+        <v>6</v>
+      </c>
+      <c r="L42" t="str">
+        <v/>
+      </c>
+      <c r="M42" t="str">
+        <v>2</v>
+      </c>
+      <c r="N42" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O42" t="str">
+        <v/>
+      </c>
+      <c r="P42" t="str">
+        <v/>
+      </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
+      <c r="R42" t="str">
+        <v/>
+      </c>
+      <c r="S42" t="str">
+        <v/>
+      </c>
+      <c r="T42" t="str">
+        <v/>
+      </c>
+      <c r="U42" t="str">
+        <v/>
+      </c>
+      <c r="V42" t="str">
+        <v/>
+      </c>
+      <c r="W42" t="str">
+        <v/>
+      </c>
+      <c r="X42" t="str">
+        <v/>
+      </c>
+      <c r="Y42" t="str">
+        <v/>
+      </c>
+      <c r="Z42" t="str">
+        <v/>
+      </c>
+      <c r="AA42" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="AB42" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Thunder</v>
+        <v>Refined Steel</v>
       </c>
       <c r="B43" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
       </c>
       <c r="C43" t="str">
-        <v>Lightning</v>
+        <v>Steel</v>
+      </c>
+      <c r="D43" t="str">
+        <v>210</v>
       </c>
       <c r="E43" t="str">
         <v>2</v>
       </c>
       <c r="F43" t="str">
-        <v>2</v>
+        <v>9</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Folded a thousand times until perfect</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J43" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K43" t="str">
+        <v>6</v>
+      </c>
+      <c r="L43" t="str">
+        <v/>
+      </c>
+      <c r="M43" t="str">
+        <v>2</v>
+      </c>
+      <c r="N43" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O43" t="str">
+        <v>shield</v>
+      </c>
+      <c r="P43" t="str">
+        <v>8</v>
+      </c>
+      <c r="Q43" t="str">
+        <v/>
+      </c>
+      <c r="R43" t="str">
+        <v/>
+      </c>
+      <c r="S43" t="str">
+        <v>self</v>
+      </c>
+      <c r="T43" t="str">
+        <v/>
+      </c>
+      <c r="U43" t="str">
+        <v/>
+      </c>
+      <c r="V43" t="str">
+        <v/>
+      </c>
+      <c r="W43" t="str">
+        <v/>
+      </c>
+      <c r="X43" t="str">
+        <v/>
+      </c>
+      <c r="Y43" t="str">
+        <v/>
+      </c>
+      <c r="Z43" t="str">
+        <v/>
+      </c>
+      <c r="AA43" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="AB43" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Mud Shot</v>
+        <v>Water Bolt</v>
       </c>
       <c r="B44" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="C44" t="str">
         <v>Water</v>
       </c>
-      <c r="C44" t="str">
-        <v>Sand</v>
+      <c r="D44" t="str">
+        <v>58</v>
       </c>
       <c r="E44" t="str">
         <v>2</v>
       </c>
       <c r="F44" t="str">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Crackling bolts that drench what they strike</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="I44" t="str">
+        <v>Water</v>
+      </c>
+      <c r="J44" t="str">
+        <v>multi_hit</v>
+      </c>
+      <c r="K44" t="str">
+        <v/>
+      </c>
+      <c r="L44" t="str">
+        <v>2</v>
+      </c>
+      <c r="M44" t="str">
+        <v/>
+      </c>
+      <c r="N44" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O44" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P44" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q44" t="str">
+        <v/>
+      </c>
+      <c r="R44" t="str">
+        <v/>
+      </c>
+      <c r="S44" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="T44" t="str">
+        <v/>
+      </c>
+      <c r="U44" t="str">
+        <v/>
+      </c>
+      <c r="V44" t="str">
+        <v/>
+      </c>
+      <c r="W44" t="str">
+        <v/>
+      </c>
+      <c r="X44" t="str">
+        <v/>
+      </c>
+      <c r="Y44" t="str">
+        <v/>
+      </c>
+      <c r="Z44" t="str">
+        <v/>
+      </c>
+      <c r="AA44" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="AB44" t="str">
+        <v>Water</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Worble</v>
+        <v>Ice Bolt</v>
       </c>
       <c r="B45" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="C45" t="str">
-        <v>Water</v>
+        <v>Ice</v>
+      </c>
+      <c r="D45" t="str">
+        <v>58</v>
       </c>
       <c r="E45" t="str">
         <v>2</v>
       </c>
       <c r="F45" t="str">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="G45" t="str">
+        <v>A frozen shard launched like a thunderbolt</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="I45" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="J45" t="str">
+        <v>multi_hit</v>
+      </c>
+      <c r="K45" t="str">
+        <v/>
+      </c>
+      <c r="L45" t="str">
+        <v>2</v>
+      </c>
+      <c r="M45" t="str">
+        <v/>
+      </c>
+      <c r="N45" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O45" t="str">
+        <v/>
+      </c>
+      <c r="P45" t="str">
+        <v/>
+      </c>
+      <c r="Q45" t="str">
+        <v/>
+      </c>
+      <c r="R45" t="str">
+        <v/>
+      </c>
+      <c r="S45" t="str">
+        <v/>
+      </c>
+      <c r="T45" t="str">
+        <v/>
+      </c>
+      <c r="U45" t="str">
+        <v/>
+      </c>
+      <c r="V45" t="str">
+        <v/>
+      </c>
+      <c r="W45" t="str">
+        <v/>
+      </c>
+      <c r="X45" t="str">
+        <v/>
+      </c>
+      <c r="Y45" t="str">
+        <v/>
+      </c>
+      <c r="Z45" t="str">
+        <v/>
+      </c>
+      <c r="AA45" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="AB45" t="str">
+        <v>Ice</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Tornado</v>
+        <v>Thunder</v>
       </c>
       <c r="B46" t="str">
-        <v>Air</v>
+        <v>Lightning</v>
       </c>
       <c r="C46" t="str">
-        <v>Air</v>
+        <v>Lightning</v>
+      </c>
+      <c r="D46" t="str">
+        <v>126</v>
       </c>
       <c r="E46" t="str">
         <v>2</v>
       </c>
       <c r="F46" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Strikes once, twice, three times in a flash</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="I46" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="J46" t="str">
+        <v>multi_hit</v>
+      </c>
+      <c r="K46" t="str">
+        <v/>
+      </c>
+      <c r="L46" t="str">
+        <v>3</v>
+      </c>
+      <c r="M46" t="str">
+        <v/>
+      </c>
+      <c r="N46" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O46" t="str">
+        <v/>
+      </c>
+      <c r="P46" t="str">
+        <v/>
+      </c>
+      <c r="Q46" t="str">
+        <v/>
+      </c>
+      <c r="R46" t="str">
+        <v/>
+      </c>
+      <c r="S46" t="str">
+        <v/>
+      </c>
+      <c r="T46" t="str">
+        <v/>
+      </c>
+      <c r="U46" t="str">
+        <v/>
+      </c>
+      <c r="V46" t="str">
+        <v/>
+      </c>
+      <c r="W46" t="str">
+        <v/>
+      </c>
+      <c r="X46" t="str">
+        <v/>
+      </c>
+      <c r="Y46" t="str">
+        <v/>
+      </c>
+      <c r="Z46" t="str">
+        <v/>
+      </c>
+      <c r="AA46" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="AB46" t="str">
+        <v>Lightning</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Hailstorm</v>
+        <v>Mud Shot</v>
       </c>
       <c r="B47" t="str">
-        <v>Air</v>
+        <v>Water</v>
       </c>
       <c r="C47" t="str">
-        <v>Ice</v>
+        <v>Sand</v>
+      </c>
+      <c r="D47" t="str">
+        <v>109</v>
       </c>
       <c r="E47" t="str">
         <v>2</v>
       </c>
       <c r="F47" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G47" t="str">
+        <v>Thick sludge launched with surprising force</v>
+      </c>
+      <c r="H47" t="str">
+        <v>Water</v>
+      </c>
+      <c r="I47" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J47" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K47" t="str">
+        <v>8</v>
+      </c>
+      <c r="L47" t="str">
+        <v/>
+      </c>
+      <c r="M47" t="str">
+        <v/>
+      </c>
+      <c r="N47" t="str">
+        <v>self</v>
+      </c>
+      <c r="O47" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P47" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q47" t="str">
+        <v/>
+      </c>
+      <c r="R47" t="str">
+        <v/>
+      </c>
+      <c r="S47" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="T47" t="str">
+        <v/>
+      </c>
+      <c r="U47" t="str">
+        <v/>
+      </c>
+      <c r="V47" t="str">
+        <v/>
+      </c>
+      <c r="W47" t="str">
+        <v/>
+      </c>
+      <c r="X47" t="str">
+        <v/>
+      </c>
+      <c r="Y47" t="str">
+        <v/>
+      </c>
+      <c r="Z47" t="str">
+        <v/>
+      </c>
+      <c r="AA47" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AB47" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Pyreball</v>
+        <v>Tornado</v>
       </c>
       <c r="B48" t="str">
-        <v>Fire</v>
+        <v>Air</v>
       </c>
       <c r="C48" t="str">
-        <v>Fire</v>
+        <v>Air</v>
+      </c>
+      <c r="D48" t="str">
+        <v>126</v>
       </c>
       <c r="E48" t="str">
         <v>2</v>
       </c>
       <c r="F48" t="str">
         <v>2</v>
+      </c>
+      <c r="G48" t="str">
+        <v>A perfect spiral of destruction and fury</v>
+      </c>
+      <c r="H48" t="str">
+        <v>Air</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Air</v>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+      <c r="K48" t="str">
+        <v/>
+      </c>
+      <c r="L48" t="str">
+        <v/>
+      </c>
+      <c r="M48" t="str">
+        <v/>
+      </c>
+      <c r="N48" t="str">
+        <v/>
+      </c>
+      <c r="O48" t="str">
+        <v/>
+      </c>
+      <c r="P48" t="str">
+        <v/>
+      </c>
+      <c r="Q48" t="str">
+        <v/>
+      </c>
+      <c r="R48" t="str">
+        <v/>
+      </c>
+      <c r="S48" t="str">
+        <v/>
+      </c>
+      <c r="T48" t="str">
+        <v/>
+      </c>
+      <c r="U48" t="str">
+        <v/>
+      </c>
+      <c r="V48" t="str">
+        <v/>
+      </c>
+      <c r="W48" t="str">
+        <v/>
+      </c>
+      <c r="X48" t="str">
+        <v/>
+      </c>
+      <c r="Y48" t="str">
+        <v/>
+      </c>
+      <c r="Z48" t="str">
+        <v/>
+      </c>
+      <c r="AA48" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AB48" t="str">
+        <v>Air</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Ice Shield</v>
+        <v>Hailstorm</v>
       </c>
       <c r="B49" t="str">
+        <v>Air</v>
+      </c>
+      <c r="C49" t="str">
         <v>Ice</v>
       </c>
-      <c r="C49" t="str">
-        <v>Earth</v>
+      <c r="D49" t="str">
+        <v>58</v>
       </c>
       <c r="E49" t="str">
         <v>2</v>
       </c>
       <c r="F49" t="str">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G49" t="str">
+        <v>Ice pellets rain down in a furious torrent</v>
+      </c>
+      <c r="H49" t="str">
+        <v>Air</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+      <c r="K49" t="str">
+        <v/>
+      </c>
+      <c r="L49" t="str">
+        <v/>
+      </c>
+      <c r="M49" t="str">
+        <v/>
+      </c>
+      <c r="N49" t="str">
+        <v/>
+      </c>
+      <c r="O49" t="str">
+        <v/>
+      </c>
+      <c r="P49" t="str">
+        <v/>
+      </c>
+      <c r="Q49" t="str">
+        <v/>
+      </c>
+      <c r="R49" t="str">
+        <v/>
+      </c>
+      <c r="S49" t="str">
+        <v/>
+      </c>
+      <c r="T49" t="str">
+        <v/>
+      </c>
+      <c r="U49" t="str">
+        <v/>
+      </c>
+      <c r="V49" t="str">
+        <v/>
+      </c>
+      <c r="W49" t="str">
+        <v/>
+      </c>
+      <c r="X49" t="str">
+        <v/>
+      </c>
+      <c r="Y49" t="str">
+        <v/>
+      </c>
+      <c r="Z49" t="str">
+        <v/>
+      </c>
+      <c r="AA49" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AB49" t="str">
+        <v>Ice</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Glacier</v>
+        <v>Pyreball</v>
       </c>
       <c r="B50" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="C50" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
+      </c>
+      <c r="D50" t="str">
+        <v>126</v>
       </c>
       <c r="E50" t="str">
         <v>2</v>
       </c>
       <c r="F50" t="str">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="G50" t="str">
+        <v>A massive fireball of pure concentrated flame</v>
+      </c>
+      <c r="H50" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="J50" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K50" t="str">
+        <v>10</v>
+      </c>
+      <c r="L50" t="str">
+        <v/>
+      </c>
+      <c r="M50" t="str">
+        <v>3</v>
+      </c>
+      <c r="N50" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O50" t="str">
+        <v/>
+      </c>
+      <c r="P50" t="str">
+        <v/>
+      </c>
+      <c r="Q50" t="str">
+        <v/>
+      </c>
+      <c r="R50" t="str">
+        <v/>
+      </c>
+      <c r="S50" t="str">
+        <v/>
+      </c>
+      <c r="T50" t="str">
+        <v/>
+      </c>
+      <c r="U50" t="str">
+        <v/>
+      </c>
+      <c r="V50" t="str">
+        <v/>
+      </c>
+      <c r="W50" t="str">
+        <v/>
+      </c>
+      <c r="X50" t="str">
+        <v/>
+      </c>
+      <c r="Y50" t="str">
+        <v/>
+      </c>
+      <c r="Z50" t="str">
+        <v/>
+      </c>
+      <c r="AA50" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="AB50" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
+        <v>Ice Shield</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="D51" t="str">
+        <v>58</v>
+      </c>
+      <c r="E51" t="str">
+        <v>2</v>
+      </c>
+      <c r="F51" t="str">
+        <v>3</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Frozen barrier as solid and cold as bedrock</v>
+      </c>
+      <c r="H51" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="I51" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J51" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K51" t="str">
+        <v>8</v>
+      </c>
+      <c r="L51" t="str">
+        <v/>
+      </c>
+      <c r="M51" t="str">
+        <v/>
+      </c>
+      <c r="N51" t="str">
+        <v>self</v>
+      </c>
+      <c r="O51" t="str">
+        <v/>
+      </c>
+      <c r="P51" t="str">
+        <v/>
+      </c>
+      <c r="Q51" t="str">
+        <v/>
+      </c>
+      <c r="R51" t="str">
+        <v/>
+      </c>
+      <c r="S51" t="str">
+        <v/>
+      </c>
+      <c r="T51" t="str">
+        <v/>
+      </c>
+      <c r="U51" t="str">
+        <v/>
+      </c>
+      <c r="V51" t="str">
+        <v/>
+      </c>
+      <c r="W51" t="str">
+        <v/>
+      </c>
+      <c r="X51" t="str">
+        <v/>
+      </c>
+      <c r="Y51" t="str">
+        <v/>
+      </c>
+      <c r="Z51" t="str">
+        <v/>
+      </c>
+      <c r="AA51" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="AB51" t="str">
+        <v>Earth</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Glacier</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="D52" t="str">
+        <v>126</v>
+      </c>
+      <c r="E52" t="str">
+        <v>2</v>
+      </c>
+      <c r="F52" t="str">
+        <v>5</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Ancient ice creaks and grinds slowly forward</v>
+      </c>
+      <c r="H52" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="I52" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
+        <v/>
+      </c>
+      <c r="L52" t="str">
+        <v/>
+      </c>
+      <c r="M52" t="str">
+        <v/>
+      </c>
+      <c r="N52" t="str">
+        <v/>
+      </c>
+      <c r="O52" t="str">
+        <v/>
+      </c>
+      <c r="P52" t="str">
+        <v/>
+      </c>
+      <c r="Q52" t="str">
+        <v/>
+      </c>
+      <c r="R52" t="str">
+        <v/>
+      </c>
+      <c r="S52" t="str">
+        <v/>
+      </c>
+      <c r="T52" t="str">
+        <v/>
+      </c>
+      <c r="U52" t="str">
+        <v/>
+      </c>
+      <c r="V52" t="str">
+        <v/>
+      </c>
+      <c r="W52" t="str">
+        <v/>
+      </c>
+      <c r="X52" t="str">
+        <v/>
+      </c>
+      <c r="Y52" t="str">
+        <v/>
+      </c>
+      <c r="Z52" t="str">
+        <v/>
+      </c>
+      <c r="AA52" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="AB52" t="str">
+        <v>Ice</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
         <v>Earthquake</v>
       </c>
-      <c r="B51" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="C51" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="E51" t="str">
-        <v>2</v>
-      </c>
-      <c r="F51" t="str">
-        <v>2</v>
+      <c r="B53" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="D53" t="str">
+        <v>126</v>
+      </c>
+      <c r="E53" t="str">
+        <v>2</v>
+      </c>
+      <c r="F53" t="str">
+        <v>5</v>
+      </c>
+      <c r="G53" t="str">
+        <v>The ground splits open beneath your foe</v>
+      </c>
+      <c r="H53" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I53" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J53" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K53" t="str">
+        <v>16</v>
+      </c>
+      <c r="L53" t="str">
+        <v/>
+      </c>
+      <c r="M53" t="str">
+        <v/>
+      </c>
+      <c r="N53" t="str">
+        <v>self</v>
+      </c>
+      <c r="O53" t="str">
+        <v/>
+      </c>
+      <c r="P53" t="str">
+        <v/>
+      </c>
+      <c r="Q53" t="str">
+        <v/>
+      </c>
+      <c r="R53" t="str">
+        <v/>
+      </c>
+      <c r="S53" t="str">
+        <v/>
+      </c>
+      <c r="T53" t="str">
+        <v/>
+      </c>
+      <c r="U53" t="str">
+        <v/>
+      </c>
+      <c r="V53" t="str">
+        <v/>
+      </c>
+      <c r="W53" t="str">
+        <v/>
+      </c>
+      <c r="X53" t="str">
+        <v/>
+      </c>
+      <c r="Y53" t="str">
+        <v/>
+      </c>
+      <c r="Z53" t="str">
+        <v/>
+      </c>
+      <c r="AA53" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB53" t="str">
+        <v>Earth</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB53"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (02791cd) Balancing Elements a bit more, Updating UI
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB53"/>
+  <dimension ref="A1:AB52"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -487,7 +487,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -496,7 +496,7 @@
         <v/>
       </c>
       <c r="D2" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E2" t="str">
         <v>1</v>
@@ -505,10 +505,10 @@
         <v>1</v>
       </c>
       <c r="G2" t="str">
-        <v>A bright flame burning hot</v>
+        <v>A gift from the sky goddess</v>
       </c>
       <c r="H2" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -565,7 +565,7 @@
         <v/>
       </c>
       <c r="AA2" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="AB2" t="str">
         <v/>
@@ -573,7 +573,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -582,7 +582,7 @@
         <v/>
       </c>
       <c r="D3" t="str">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E3" t="str">
         <v>1</v>
@@ -591,10 +591,10 @@
         <v>1</v>
       </c>
       <c r="G3" t="str">
-        <v>A gift from the sky goddess</v>
+        <v>It's a rock</v>
       </c>
       <c r="H3" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="I3" t="str">
         <v/>
@@ -651,7 +651,7 @@
         <v/>
       </c>
       <c r="AA3" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="AB3" t="str">
         <v/>
@@ -659,16 +659,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>Ice</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>Fire</v>
       </c>
       <c r="D4" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E4" t="str">
         <v>1</v>
@@ -677,19 +677,19 @@
         <v>1</v>
       </c>
       <c r="G4" t="str">
-        <v>It's a rock</v>
+        <v>A gift from the sky goddess</v>
       </c>
       <c r="H4" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="I4" t="str">
         <v/>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>heal</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="L4" t="str">
         <v/>
@@ -698,19 +698,19 @@
         <v/>
       </c>
       <c r="N4" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O4" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="P4" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q4" t="str">
         <v/>
       </c>
       <c r="R4" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="S4" t="str">
         <v/>
@@ -737,7 +737,7 @@
         <v/>
       </c>
       <c r="AA4" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AB4" t="str">
         <v/>
@@ -745,16 +745,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="B5" t="str">
         <v>Water</v>
       </c>
-      <c r="B5" t="str">
-        <v>Ice</v>
-      </c>
       <c r="C5" t="str">
-        <v>Fire</v>
+        <v>Air</v>
       </c>
       <c r="D5" t="str">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E5" t="str">
         <v>1</v>
@@ -763,40 +763,40 @@
         <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v>A gift from the sky goddess</v>
+        <v>A bright flame burning hot</v>
       </c>
       <c r="H5" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="I5" t="str">
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>heal</v>
+        <v>burn</v>
       </c>
       <c r="K5" t="str">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L5" t="str">
         <v/>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="N5" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O5" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P5" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="Q5" t="str">
         <v/>
       </c>
       <c r="R5" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="S5" t="str">
         <v/>
@@ -834,10 +834,10 @@
         <v>Fire</v>
       </c>
       <c r="B6" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="C6" t="str">
-        <v>Air</v>
+        <v>Lightning</v>
       </c>
       <c r="D6" t="str">
         <v>10</v>
@@ -858,16 +858,16 @@
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>burn</v>
+        <v/>
       </c>
       <c r="K6" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="L6" t="str">
         <v/>
       </c>
       <c r="M6" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="N6" t="str">
         <v/>
@@ -917,13 +917,13 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="B7" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C7" t="str">
-        <v>Lightning</v>
+        <v>Sand</v>
       </c>
       <c r="D7" t="str">
         <v>10</v>
@@ -935,19 +935,19 @@
         <v>1</v>
       </c>
       <c r="G7" t="str">
-        <v>A bright flame burning hot</v>
+        <v>It's a rock</v>
       </c>
       <c r="H7" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="I7" t="str">
         <v/>
       </c>
       <c r="J7" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="L7" t="str">
         <v/>
@@ -1003,16 +1003,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Earth</v>
+        <v>Lightning</v>
       </c>
       <c r="B8" t="str">
-        <v>Sand</v>
+        <v>Air</v>
       </c>
       <c r="C8" t="str">
-        <v>Sand</v>
+        <v>Fire</v>
       </c>
       <c r="D8" t="str">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E8" t="str">
         <v>1</v>
@@ -1021,22 +1021,22 @@
         <v>1</v>
       </c>
       <c r="G8" t="str">
-        <v>It's a rock</v>
+        <v>Charged spark that strikes instantly</v>
       </c>
       <c r="H8" t="str">
-        <v>Earth</v>
+        <v>Lightning</v>
       </c>
       <c r="I8" t="str">
         <v/>
       </c>
       <c r="J8" t="str">
-        <v>shield</v>
+        <v>multihit</v>
       </c>
       <c r="K8" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="L8" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="M8" t="str">
         <v/>
@@ -1089,16 +1089,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Plasma</v>
+      </c>
+      <c r="B9" t="str">
         <v>Lightning</v>
       </c>
-      <c r="B9" t="str">
+      <c r="C9" t="str">
         <v>Air</v>
       </c>
-      <c r="C9" t="str">
-        <v>Fire</v>
-      </c>
       <c r="D9" t="str">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E9" t="str">
         <v>1</v>
@@ -1107,22 +1107,22 @@
         <v>1</v>
       </c>
       <c r="G9" t="str">
-        <v>Charged spark that strikes instantly</v>
+        <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H9" t="str">
-        <v>Lightning</v>
+        <v>Plasma</v>
       </c>
       <c r="I9" t="str">
         <v/>
       </c>
       <c r="J9" t="str">
-        <v>multihit</v>
+        <v/>
       </c>
       <c r="K9" t="str">
         <v/>
       </c>
       <c r="L9" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="M9" t="str">
         <v/>
@@ -1181,7 +1181,7 @@
         <v>Lightning</v>
       </c>
       <c r="C10" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
       <c r="D10" t="str">
         <v>1</v>
@@ -1267,7 +1267,7 @@
         <v>Lightning</v>
       </c>
       <c r="C11" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="D11" t="str">
         <v>1</v>
@@ -1350,10 +1350,10 @@
         <v>Plasma</v>
       </c>
       <c r="B12" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="C12" t="str">
         <v>Lightning</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Fire</v>
       </c>
       <c r="D12" t="str">
         <v>1</v>
@@ -1368,10 +1368,10 @@
         <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H12" t="str">
-        <v>Plasma</v>
+        <v>Fire</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>Lightning</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -1433,16 +1433,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Plasma</v>
+        <v>Sand</v>
       </c>
       <c r="B13" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="C13" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="D13" t="str">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E13" t="str">
         <v>1</v>
@@ -1451,13 +1451,13 @@
         <v>1</v>
       </c>
       <c r="G13" t="str">
-        <v>A deep sense of calm overwhelms you</v>
+        <v>Shifting grains dance between your fingertips</v>
       </c>
       <c r="H13" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="I13" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -1522,7 +1522,7 @@
         <v>Sand</v>
       </c>
       <c r="B14" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="C14" t="str">
         <v>Earth</v>
@@ -1605,10 +1605,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="B15" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="C15" t="str">
         <v>Earth</v>
@@ -1623,10 +1623,10 @@
         <v>1</v>
       </c>
       <c r="G15" t="str">
-        <v>Shifting grains dance between your fingertips</v>
+        <v>Forged from fire and stone, hammered hard</v>
       </c>
       <c r="H15" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="I15" t="str">
         <v/>
@@ -1691,13 +1691,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Steel</v>
+        <v>Air</v>
       </c>
       <c r="B16" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C16" t="str">
         <v>Fire</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Earth</v>
       </c>
       <c r="D16" t="str">
         <v>10</v>
@@ -1709,10 +1709,10 @@
         <v>1</v>
       </c>
       <c r="G16" t="str">
-        <v>Forged from fire and stone, hammered hard</v>
+        <v>A cool rush of wind drifts past your face</v>
       </c>
       <c r="H16" t="str">
-        <v>Steel</v>
+        <v>Air</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -1777,16 +1777,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Air</v>
+        <v>Leaf</v>
       </c>
       <c r="B17" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="C17" t="str">
         <v>Water</v>
       </c>
-      <c r="C17" t="str">
-        <v>Fire</v>
-      </c>
       <c r="D17" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E17" t="str">
         <v>1</v>
@@ -1795,13 +1795,13 @@
         <v>1</v>
       </c>
       <c r="G17" t="str">
-        <v>A cool rush of wind drifts past your face</v>
+        <v>Drops of dew glistle atop</v>
       </c>
       <c r="H17" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -1863,16 +1863,16 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Leaf</v>
+        <v>Ice</v>
       </c>
       <c r="B18" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="C18" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="D18" t="str">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E18" t="str">
         <v>1</v>
@@ -1881,13 +1881,13 @@
         <v>1</v>
       </c>
       <c r="G18" t="str">
-        <v>Drops of dew glistle atop</v>
+        <v>A biting chill that settles in your bones</v>
       </c>
       <c r="H18" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
       <c r="I18" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="J18" t="str">
         <v/>
@@ -1949,16 +1949,16 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Ice</v>
+        <v>Glass</v>
       </c>
       <c r="B19" t="str">
-        <v>Water</v>
+        <v>Sand</v>
       </c>
       <c r="C19" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="D19" t="str">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E19" t="str">
         <v>1</v>
@@ -1967,10 +1967,10 @@
         <v>1</v>
       </c>
       <c r="G19" t="str">
-        <v>A biting chill that settles in your bones</v>
+        <v>Smooth and brittle, it catches the light</v>
       </c>
       <c r="H19" t="str">
-        <v>Ice</v>
+        <v>Glass</v>
       </c>
       <c r="I19" t="str">
         <v/>
@@ -2041,7 +2041,7 @@
         <v>Sand</v>
       </c>
       <c r="C20" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="D20" t="str">
         <v>12</v>
@@ -2121,28 +2121,28 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Glass</v>
+        <v>Dark Matter</v>
       </c>
       <c r="B21" t="str">
-        <v>Sand</v>
+        <v>Unstable Element</v>
       </c>
       <c r="C21" t="str">
-        <v>Lightning</v>
+        <v>Unstable Element</v>
       </c>
       <c r="D21" t="str">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E21" t="str">
         <v>1</v>
       </c>
       <c r="F21" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" t="str">
-        <v>Smooth and brittle, it catches the light</v>
+        <v>A quiet humming radiates from inside</v>
       </c>
       <c r="H21" t="str">
-        <v>Glass</v>
+        <v>Void</v>
       </c>
       <c r="I21" t="str">
         <v/>
@@ -2207,37 +2207,37 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Dark Matter</v>
+        <v>Worble</v>
       </c>
       <c r="B22" t="str">
-        <v>Unstable Element</v>
+        <v>Water</v>
       </c>
       <c r="C22" t="str">
-        <v>Unstable Element</v>
+        <v>Water</v>
       </c>
       <c r="D22" t="str">
-        <v>18</v>
+        <v>126</v>
       </c>
       <c r="E22" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G22" t="str">
-        <v>A quiet humming radiates from inside</v>
+        <v>The tide is high today my friend</v>
       </c>
       <c r="H22" t="str">
-        <v>Void</v>
+        <v>Water</v>
       </c>
       <c r="I22" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="J22" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="K22" t="str">
-        <v/>
+        <v>4</v>
       </c>
       <c r="L22" t="str">
         <v/>
@@ -2246,7 +2246,7 @@
         <v/>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="O22" t="str">
         <v/>
@@ -2285,24 +2285,24 @@
         <v/>
       </c>
       <c r="AA22" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="AB22" t="str">
-        <v/>
+        <v>Water</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Worble</v>
+        <v>Blaze</v>
       </c>
       <c r="B23" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="C23" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="D23" t="str">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="E23" t="str">
         <v>2</v>
@@ -2311,34 +2311,34 @@
         <v>5</v>
       </c>
       <c r="G23" t="str">
-        <v>The tide is high today my friend</v>
+        <v>Forest floor erupts in scorching flame</v>
       </c>
       <c r="H23" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="I23" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="J23" t="str">
-        <v>soak</v>
+        <v>burn</v>
       </c>
       <c r="K23" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L23" t="str">
         <v/>
       </c>
       <c r="M23" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="N23" t="str">
         <v>enemy</v>
       </c>
       <c r="O23" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="P23" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="Q23" t="str">
         <v/>
@@ -2347,7 +2347,7 @@
         <v/>
       </c>
       <c r="S23" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="T23" t="str">
         <v/>
@@ -2371,21 +2371,21 @@
         <v/>
       </c>
       <c r="AA23" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="AB23" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Blaze</v>
+        <v>Regen</v>
       </c>
       <c r="B24" t="str">
         <v>Leaf</v>
       </c>
       <c r="C24" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="D24" t="str">
         <v>109</v>
@@ -2397,44 +2397,44 @@
         <v>5</v>
       </c>
       <c r="G24" t="str">
-        <v>Forest floor erupts in scorching flame</v>
+        <v>Living vines wrap wounds in cool water</v>
       </c>
       <c r="H24" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="I24" t="str">
         <v>Earth</v>
       </c>
       <c r="J24" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="K24" t="str">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L24" t="str">
         <v/>
       </c>
       <c r="M24" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N24" t="str">
+        <v>self</v>
+      </c>
+      <c r="O24" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P24" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
         <v>enemy</v>
       </c>
-      <c r="O24" t="str">
-        <v>shield</v>
-      </c>
-      <c r="P24" t="str">
-        <v>8</v>
-      </c>
-      <c r="Q24" t="str">
-        <v/>
-      </c>
-      <c r="R24" t="str">
-        <v/>
-      </c>
-      <c r="S24" t="str">
-        <v>self</v>
-      </c>
       <c r="T24" t="str">
         <v/>
       </c>
@@ -2457,7 +2457,7 @@
         <v/>
       </c>
       <c r="AA24" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="AB24" t="str">
         <v>Earth</v>
@@ -2465,13 +2465,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Regen</v>
+        <v>Thorns</v>
       </c>
       <c r="B25" t="str">
         <v>Leaf</v>
       </c>
       <c r="C25" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="D25" t="str">
         <v>109</v>
@@ -2483,13 +2483,13 @@
         <v>5</v>
       </c>
       <c r="G25" t="str">
-        <v>Living vines wrap wounds in cool water</v>
+        <v>Spiked vines protect you</v>
       </c>
       <c r="H25" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="I25" t="str">
         <v>Water</v>
-      </c>
-      <c r="I25" t="str">
-        <v>Earth</v>
       </c>
       <c r="J25" t="str">
         <v>shield</v>
@@ -2543,21 +2543,21 @@
         <v/>
       </c>
       <c r="AA25" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB25" t="str">
         <v>Water</v>
-      </c>
-      <c r="AB25" t="str">
-        <v>Earth</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Thorns</v>
+        <v>Tornado</v>
       </c>
       <c r="B26" t="str">
         <v>Leaf</v>
       </c>
       <c r="C26" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="D26" t="str">
         <v>109</v>
@@ -2566,16 +2566,16 @@
         <v>2</v>
       </c>
       <c r="F26" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G26" t="str">
-        <v>Spiked vines protect you</v>
+        <v>Wind whips and slashes about</v>
       </c>
       <c r="H26" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="I26" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="J26" t="str">
         <v>shield</v>
@@ -2593,10 +2593,10 @@
         <v>self</v>
       </c>
       <c r="O26" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P26" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q26" t="str">
         <v/>
@@ -2605,7 +2605,7 @@
         <v/>
       </c>
       <c r="S26" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T26" t="str">
         <v/>
@@ -2629,21 +2629,21 @@
         <v/>
       </c>
       <c r="AA26" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="AB26" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Tornado</v>
+        <v>Blizzard</v>
       </c>
       <c r="B27" t="str">
         <v>Leaf</v>
       </c>
       <c r="C27" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D27" t="str">
         <v>109</v>
@@ -2652,13 +2652,13 @@
         <v>2</v>
       </c>
       <c r="F27" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G27" t="str">
-        <v>Wind whips and slashes about</v>
+        <v>Snow flurries block your vision</v>
       </c>
       <c r="H27" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="I27" t="str">
         <v>Earth</v>
@@ -2715,7 +2715,7 @@
         <v/>
       </c>
       <c r="AA27" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="AB27" t="str">
         <v>Earth</v>
@@ -2723,31 +2723,31 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Blizzard</v>
+        <v>Leaf Blade</v>
       </c>
       <c r="B28" t="str">
         <v>Leaf</v>
       </c>
       <c r="C28" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="D28" t="str">
-        <v>109</v>
+        <v>159</v>
       </c>
       <c r="E28" t="str">
         <v>2</v>
       </c>
       <c r="F28" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G28" t="str">
-        <v>Snow flurries block your vision</v>
+        <v>A razor edge honed from living wood</v>
       </c>
       <c r="H28" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="I28" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="J28" t="str">
         <v>shield</v>
@@ -2765,10 +2765,10 @@
         <v>self</v>
       </c>
       <c r="O28" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="P28" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="Q28" t="str">
         <v/>
@@ -2777,7 +2777,7 @@
         <v/>
       </c>
       <c r="S28" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="T28" t="str">
         <v/>
@@ -2801,21 +2801,21 @@
         <v/>
       </c>
       <c r="AA28" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="AB28" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Leaf Blade</v>
+        <v>Needle Storm</v>
       </c>
       <c r="B29" t="str">
         <v>Leaf</v>
       </c>
       <c r="C29" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="D29" t="str">
         <v>159</v>
@@ -2827,7 +2827,7 @@
         <v>7</v>
       </c>
       <c r="G29" t="str">
-        <v>A razor edge honed from living wood</v>
+        <v>Tiny needles prick from every angle</v>
       </c>
       <c r="H29" t="str">
         <v>Earth</v>
@@ -2895,25 +2895,25 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Needle Storm</v>
+        <v>Photosynthesis</v>
       </c>
       <c r="B30" t="str">
         <v>Leaf</v>
       </c>
       <c r="C30" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="D30" t="str">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="E30" t="str">
         <v>2</v>
       </c>
       <c r="F30" t="str">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G30" t="str">
-        <v>Tiny needles prick from every angle</v>
+        <v>Nature feeds itself to grow ever stronger</v>
       </c>
       <c r="H30" t="str">
         <v>Earth</v>
@@ -2981,62 +2981,62 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Photosynthesis</v>
+        <v>Desert Blade</v>
       </c>
       <c r="B31" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C31" t="str">
-        <v>Leaf</v>
+        <v>Steel</v>
       </c>
       <c r="D31" t="str">
-        <v>210</v>
+        <v>159</v>
       </c>
       <c r="E31" t="str">
         <v>2</v>
       </c>
       <c r="F31" t="str">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G31" t="str">
-        <v>Nature feeds itself to grow ever stronger</v>
+        <v>Sand-forged steel scorched by the desert sun</v>
       </c>
       <c r="H31" t="str">
         <v>Earth</v>
       </c>
       <c r="I31" t="str">
-        <v>Water</v>
+        <v>Steel</v>
       </c>
       <c r="J31" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K31" t="str">
+        <v>6</v>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v>2</v>
+      </c>
+      <c r="N31" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O31" t="str">
         <v>shield</v>
       </c>
-      <c r="K31" t="str">
+      <c r="P31" t="str">
         <v>8</v>
       </c>
-      <c r="L31" t="str">
-        <v/>
-      </c>
-      <c r="M31" t="str">
-        <v/>
-      </c>
-      <c r="N31" t="str">
+      <c r="Q31" t="str">
+        <v/>
+      </c>
+      <c r="R31" t="str">
+        <v/>
+      </c>
+      <c r="S31" t="str">
         <v>self</v>
       </c>
-      <c r="O31" t="str">
-        <v>soak</v>
-      </c>
-      <c r="P31" t="str">
-        <v>2</v>
-      </c>
-      <c r="Q31" t="str">
-        <v/>
-      </c>
-      <c r="R31" t="str">
-        <v/>
-      </c>
-      <c r="S31" t="str">
-        <v>enemy</v>
-      </c>
       <c r="T31" t="str">
         <v/>
       </c>
@@ -3062,67 +3062,67 @@
         <v>Earth</v>
       </c>
       <c r="AB31" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Desert Blade</v>
+        <v>Mud Shot</v>
       </c>
       <c r="B32" t="str">
         <v>Sand</v>
       </c>
       <c r="C32" t="str">
-        <v>Steel</v>
+        <v>Water</v>
       </c>
       <c r="D32" t="str">
-        <v>159</v>
+        <v>109</v>
       </c>
       <c r="E32" t="str">
         <v>2</v>
       </c>
       <c r="F32" t="str">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G32" t="str">
-        <v>Sand-forged steel scorched by the desert sun</v>
+        <v>Thick sludge launched with surprising force</v>
       </c>
       <c r="H32" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="I32" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="J32" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="K32" t="str">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L32" t="str">
         <v/>
       </c>
       <c r="M32" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N32" t="str">
+        <v>self</v>
+      </c>
+      <c r="O32" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P32" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
+      <c r="R32" t="str">
+        <v/>
+      </c>
+      <c r="S32" t="str">
         <v>enemy</v>
       </c>
-      <c r="O32" t="str">
-        <v>shield</v>
-      </c>
-      <c r="P32" t="str">
-        <v>8</v>
-      </c>
-      <c r="Q32" t="str">
-        <v/>
-      </c>
-      <c r="R32" t="str">
-        <v/>
-      </c>
-      <c r="S32" t="str">
-        <v>self</v>
-      </c>
       <c r="T32" t="str">
         <v/>
       </c>
@@ -3145,21 +3145,21 @@
         <v/>
       </c>
       <c r="AA32" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="AB32" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Mud Shot</v>
+        <v>Sand Shield</v>
       </c>
       <c r="B33" t="str">
         <v>Sand</v>
       </c>
       <c r="C33" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="D33" t="str">
         <v>109</v>
@@ -3171,13 +3171,13 @@
         <v>5</v>
       </c>
       <c r="G33" t="str">
-        <v>Thick sludge launched with surprising force</v>
+        <v>Grains pack tight into an earthen wall</v>
       </c>
       <c r="H33" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="I33" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="J33" t="str">
         <v>shield</v>
@@ -3195,10 +3195,10 @@
         <v>self</v>
       </c>
       <c r="O33" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P33" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q33" t="str">
         <v/>
@@ -3207,7 +3207,7 @@
         <v/>
       </c>
       <c r="S33" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T33" t="str">
         <v/>
@@ -3231,21 +3231,21 @@
         <v/>
       </c>
       <c r="AA33" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="AB33" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Sand Shield</v>
+        <v>Sandstorm</v>
       </c>
       <c r="B34" t="str">
         <v>Sand</v>
       </c>
       <c r="C34" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="D34" t="str">
         <v>109</v>
@@ -3254,16 +3254,16 @@
         <v>2</v>
       </c>
       <c r="F34" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G34" t="str">
-        <v>Grains pack tight into an earthen wall</v>
+        <v>Blinding grit swirls on howling winds</v>
       </c>
       <c r="H34" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="I34" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
       <c r="J34" t="str">
         <v>shield</v>
@@ -3317,21 +3317,21 @@
         <v/>
       </c>
       <c r="AA34" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="AB34" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Sandstorm</v>
+        <v>Iceblast</v>
       </c>
       <c r="B35" t="str">
         <v>Sand</v>
       </c>
       <c r="C35" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D35" t="str">
         <v>109</v>
@@ -3340,13 +3340,13 @@
         <v>2</v>
       </c>
       <c r="F35" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G35" t="str">
-        <v>Blinding grit swirls on howling winds</v>
+        <v>Cold grit bites with a frosty sting</v>
       </c>
       <c r="H35" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="I35" t="str">
         <v>Earth</v>
@@ -3403,7 +3403,7 @@
         <v/>
       </c>
       <c r="AA35" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="AB35" t="str">
         <v>Earth</v>
@@ -3411,13 +3411,13 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Iceblast</v>
+        <v>Blaze Blade</v>
       </c>
       <c r="B36" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="C36" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="D36" t="str">
         <v>109</v>
@@ -3426,47 +3426,47 @@
         <v>2</v>
       </c>
       <c r="F36" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G36" t="str">
-        <v>Cold grit bites with a frosty sting</v>
+        <v>A steel blade bathed in white-hot flame</v>
       </c>
       <c r="H36" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="I36" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="J36" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K36" t="str">
+        <v>6</v>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v>2</v>
+      </c>
+      <c r="N36" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O36" t="str">
         <v>shield</v>
       </c>
-      <c r="K36" t="str">
+      <c r="P36" t="str">
         <v>8</v>
       </c>
-      <c r="L36" t="str">
-        <v/>
-      </c>
-      <c r="M36" t="str">
-        <v/>
-      </c>
-      <c r="N36" t="str">
+      <c r="Q36" t="str">
+        <v/>
+      </c>
+      <c r="R36" t="str">
+        <v/>
+      </c>
+      <c r="S36" t="str">
         <v>self</v>
       </c>
-      <c r="O36" t="str">
-        <v/>
-      </c>
-      <c r="P36" t="str">
-        <v/>
-      </c>
-      <c r="Q36" t="str">
-        <v/>
-      </c>
-      <c r="R36" t="str">
-        <v/>
-      </c>
-      <c r="S36" t="str">
-        <v/>
-      </c>
       <c r="T36" t="str">
         <v/>
       </c>
@@ -3489,7 +3489,7 @@
         <v/>
       </c>
       <c r="AA36" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="AB36" t="str">
         <v>Earth</v>
@@ -3497,13 +3497,13 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Blaze Blade</v>
+        <v>Aqua Blade</v>
       </c>
       <c r="B37" t="str">
         <v>Steel</v>
       </c>
       <c r="C37" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="D37" t="str">
         <v>109</v>
@@ -3512,16 +3512,16 @@
         <v>2</v>
       </c>
       <c r="F37" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G37" t="str">
-        <v>A steel blade bathed in white-hot flame</v>
+        <v>Steam rises where cold steel meets the wave</v>
       </c>
       <c r="H37" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="I37" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="J37" t="str">
         <v>burn</v>
@@ -3539,10 +3539,10 @@
         <v>enemy</v>
       </c>
       <c r="O37" t="str">
-        <v>shield</v>
+        <v>soak</v>
       </c>
       <c r="P37" t="str">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Q37" t="str">
         <v/>
@@ -3551,7 +3551,7 @@
         <v/>
       </c>
       <c r="S37" t="str">
-        <v>self</v>
+        <v>enemy</v>
       </c>
       <c r="T37" t="str">
         <v/>
@@ -3575,21 +3575,21 @@
         <v/>
       </c>
       <c r="AA37" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AB37" t="str">
         <v>Fire</v>
-      </c>
-      <c r="AB37" t="str">
-        <v>Earth</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Aqua Blade</v>
+        <v>Thunder Blade</v>
       </c>
       <c r="B38" t="str">
         <v>Steel</v>
       </c>
       <c r="C38" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="D38" t="str">
         <v>109</v>
@@ -3598,43 +3598,43 @@
         <v>2</v>
       </c>
       <c r="F38" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G38" t="str">
-        <v>Steam rises where cold steel meets the wave</v>
+        <v>Sparks dance across the blades edge</v>
       </c>
       <c r="H38" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="I38" t="str">
-        <v>Fire</v>
+        <v>Steel</v>
       </c>
       <c r="J38" t="str">
-        <v>burn</v>
+        <v>multi_hit</v>
       </c>
       <c r="K38" t="str">
-        <v>6</v>
+        <v/>
       </c>
       <c r="L38" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="M38" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N38" t="str">
         <v>enemy</v>
       </c>
       <c r="O38" t="str">
-        <v>soak</v>
+        <v>burn</v>
       </c>
       <c r="P38" t="str">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="Q38" t="str">
         <v/>
       </c>
       <c r="R38" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="S38" t="str">
         <v>enemy</v>
@@ -3661,7 +3661,7 @@
         <v/>
       </c>
       <c r="AA38" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="AB38" t="str">
         <v>Fire</v>
@@ -3669,13 +3669,13 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Thunder Blade</v>
+        <v>Earth Blade</v>
       </c>
       <c r="B39" t="str">
         <v>Steel</v>
       </c>
       <c r="C39" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="D39" t="str">
         <v>109</v>
@@ -3684,46 +3684,46 @@
         <v>2</v>
       </c>
       <c r="F39" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G39" t="str">
-        <v>Lightning arcs along the edge with every swing</v>
+        <v>Heavy as bedrock</v>
       </c>
       <c r="H39" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="I39" t="str">
-        <v>Fire</v>
+        <v>Steel</v>
       </c>
       <c r="J39" t="str">
-        <v>multi_hit</v>
+        <v>burn</v>
       </c>
       <c r="K39" t="str">
-        <v/>
+        <v>6</v>
       </c>
       <c r="L39" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="M39" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="N39" t="str">
         <v>enemy</v>
       </c>
       <c r="O39" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="P39" t="str">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q39" t="str">
         <v/>
       </c>
       <c r="R39" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="S39" t="str">
-        <v>enemy</v>
+        <v>self</v>
       </c>
       <c r="T39" t="str">
         <v/>
@@ -3747,7 +3747,7 @@
         <v/>
       </c>
       <c r="AA39" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="AB39" t="str">
         <v>Fire</v>
@@ -3755,13 +3755,13 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Earth Blade</v>
+        <v>Air Blade</v>
       </c>
       <c r="B40" t="str">
         <v>Steel</v>
       </c>
       <c r="C40" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="D40" t="str">
         <v>109</v>
@@ -3770,16 +3770,16 @@
         <v>2</v>
       </c>
       <c r="F40" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G40" t="str">
-        <v>Heavy as bedrock, it burns on impact</v>
+        <v>Cuts the air so fast it ignites</v>
       </c>
       <c r="H40" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="I40" t="str">
-        <v>Fire</v>
+        <v>Steel</v>
       </c>
       <c r="J40" t="str">
         <v>burn</v>
@@ -3797,10 +3797,10 @@
         <v>enemy</v>
       </c>
       <c r="O40" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="P40" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="Q40" t="str">
         <v/>
@@ -3809,7 +3809,7 @@
         <v/>
       </c>
       <c r="S40" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="T40" t="str">
         <v/>
@@ -3833,7 +3833,7 @@
         <v/>
       </c>
       <c r="AA40" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="AB40" t="str">
         <v>Fire</v>
@@ -3841,13 +3841,13 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Air Blade</v>
+        <v>Ice Blade</v>
       </c>
       <c r="B41" t="str">
         <v>Steel</v>
       </c>
       <c r="C41" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D41" t="str">
         <v>109</v>
@@ -3856,16 +3856,16 @@
         <v>2</v>
       </c>
       <c r="F41" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G41" t="str">
-        <v>Cuts the air so fast it ignites</v>
+        <v>Cold steel that somehow scorches on contact</v>
       </c>
       <c r="H41" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="I41" t="str">
-        <v>Fire</v>
+        <v>Steel</v>
       </c>
       <c r="J41" t="str">
         <v>burn</v>
@@ -3919,7 +3919,7 @@
         <v/>
       </c>
       <c r="AA41" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="AB41" t="str">
         <v>Fire</v>
@@ -3927,31 +3927,31 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Ice Blade</v>
+        <v>Refined Steel</v>
       </c>
       <c r="B42" t="str">
         <v>Steel</v>
       </c>
       <c r="C42" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="D42" t="str">
-        <v>109</v>
+        <v>210</v>
       </c>
       <c r="E42" t="str">
         <v>2</v>
       </c>
       <c r="F42" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G42" t="str">
-        <v>Cold steel that somehow scorches on contact</v>
+        <v>Folded a thousand times until perfect</v>
       </c>
       <c r="H42" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="I42" t="str">
-        <v>Fire</v>
+        <v>Steel</v>
       </c>
       <c r="J42" t="str">
         <v>burn</v>
@@ -3969,10 +3969,10 @@
         <v>enemy</v>
       </c>
       <c r="O42" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="P42" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="Q42" t="str">
         <v/>
@@ -3981,7 +3981,7 @@
         <v/>
       </c>
       <c r="S42" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="T42" t="str">
         <v/>
@@ -4005,60 +4005,60 @@
         <v/>
       </c>
       <c r="AA42" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="AB42" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Refined Steel</v>
+        <v>Water Bolt</v>
       </c>
       <c r="B43" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="C43" t="str">
-        <v>Steel</v>
+        <v>Water</v>
       </c>
       <c r="D43" t="str">
-        <v>210</v>
+        <v>58</v>
       </c>
       <c r="E43" t="str">
         <v>2</v>
       </c>
       <c r="F43" t="str">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G43" t="str">
-        <v>Folded a thousand times until perfect</v>
+        <v>Crackling bolts that drench what they strike</v>
       </c>
       <c r="H43" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="I43" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="J43" t="str">
-        <v>burn</v>
+        <v>multi_hit</v>
       </c>
       <c r="K43" t="str">
-        <v>6</v>
+        <v/>
       </c>
       <c r="L43" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="M43" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N43" t="str">
         <v>enemy</v>
       </c>
       <c r="O43" t="str">
-        <v>shield</v>
+        <v>soak</v>
       </c>
       <c r="P43" t="str">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="Q43" t="str">
         <v/>
@@ -4067,7 +4067,7 @@
         <v/>
       </c>
       <c r="S43" t="str">
-        <v>self</v>
+        <v>enemy</v>
       </c>
       <c r="T43" t="str">
         <v/>
@@ -4091,21 +4091,21 @@
         <v/>
       </c>
       <c r="AA43" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="AB43" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Water Bolt</v>
+        <v>Ice Bolt</v>
       </c>
       <c r="B44" t="str">
         <v>Lightning</v>
       </c>
       <c r="C44" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="D44" t="str">
         <v>58</v>
@@ -4117,13 +4117,13 @@
         <v>3</v>
       </c>
       <c r="G44" t="str">
-        <v>Crackling bolts that drench what they strike</v>
+        <v>A frozen shard launched like a thunderbolt</v>
       </c>
       <c r="H44" t="str">
         <v>Lightning</v>
       </c>
       <c r="I44" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="J44" t="str">
         <v>multi_hit</v>
@@ -4141,10 +4141,10 @@
         <v>enemy</v>
       </c>
       <c r="O44" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P44" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q44" t="str">
         <v/>
@@ -4153,7 +4153,7 @@
         <v/>
       </c>
       <c r="S44" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T44" t="str">
         <v/>
@@ -4180,36 +4180,36 @@
         <v>Lightning</v>
       </c>
       <c r="AB44" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Ice Bolt</v>
+        <v>Thunder</v>
       </c>
       <c r="B45" t="str">
         <v>Lightning</v>
       </c>
       <c r="C45" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
       <c r="D45" t="str">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="E45" t="str">
         <v>2</v>
       </c>
       <c r="F45" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G45" t="str">
-        <v>A frozen shard launched like a thunderbolt</v>
+        <v>Strikes once, twice, three times in a flash</v>
       </c>
       <c r="H45" t="str">
         <v>Lightning</v>
       </c>
       <c r="I45" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
       <c r="J45" t="str">
         <v>multi_hit</v>
@@ -4218,7 +4218,7 @@
         <v/>
       </c>
       <c r="L45" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M45" t="str">
         <v/>
@@ -4266,21 +4266,21 @@
         <v>Lightning</v>
       </c>
       <c r="AB45" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Thunder</v>
+        <v>Mud Shot</v>
       </c>
       <c r="B46" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="C46" t="str">
-        <v>Lightning</v>
+        <v>Sand</v>
       </c>
       <c r="D46" t="str">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="E46" t="str">
         <v>2</v>
@@ -4289,44 +4289,44 @@
         <v>5</v>
       </c>
       <c r="G46" t="str">
-        <v>Strikes once, twice, three times in a flash</v>
+        <v>Thick sludge launched with surprising force</v>
       </c>
       <c r="H46" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="I46" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="J46" t="str">
-        <v>multi_hit</v>
+        <v>shield</v>
       </c>
       <c r="K46" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="L46" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="M46" t="str">
         <v/>
       </c>
       <c r="N46" t="str">
+        <v>self</v>
+      </c>
+      <c r="O46" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P46" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q46" t="str">
+        <v/>
+      </c>
+      <c r="R46" t="str">
+        <v/>
+      </c>
+      <c r="S46" t="str">
         <v>enemy</v>
       </c>
-      <c r="O46" t="str">
-        <v/>
-      </c>
-      <c r="P46" t="str">
-        <v/>
-      </c>
-      <c r="Q46" t="str">
-        <v/>
-      </c>
-      <c r="R46" t="str">
-        <v/>
-      </c>
-      <c r="S46" t="str">
-        <v/>
-      </c>
       <c r="T46" t="str">
         <v/>
       </c>
@@ -4349,45 +4349,45 @@
         <v/>
       </c>
       <c r="AA46" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="AB46" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Mud Shot</v>
+        <v>Tornado</v>
       </c>
       <c r="B47" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="C47" t="str">
-        <v>Sand</v>
+        <v>Air</v>
       </c>
       <c r="D47" t="str">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="E47" t="str">
         <v>2</v>
       </c>
       <c r="F47" t="str">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G47" t="str">
-        <v>Thick sludge launched with surprising force</v>
+        <v>A perfect spiral of destruction and fury</v>
       </c>
       <c r="H47" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="I47" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="J47" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="K47" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="L47" t="str">
         <v/>
@@ -4396,13 +4396,13 @@
         <v/>
       </c>
       <c r="N47" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O47" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P47" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q47" t="str">
         <v/>
@@ -4411,7 +4411,7 @@
         <v/>
       </c>
       <c r="S47" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T47" t="str">
         <v/>
@@ -4435,39 +4435,39 @@
         <v/>
       </c>
       <c r="AA47" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="AB47" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Tornado</v>
+        <v>Hailstorm</v>
       </c>
       <c r="B48" t="str">
         <v>Air</v>
       </c>
       <c r="C48" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D48" t="str">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="E48" t="str">
         <v>2</v>
       </c>
       <c r="F48" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G48" t="str">
-        <v>A perfect spiral of destruction and fury</v>
+        <v>Ice pellets rain down in a furious torrent</v>
       </c>
       <c r="H48" t="str">
         <v>Air</v>
       </c>
       <c r="I48" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="J48" t="str">
         <v/>
@@ -4524,51 +4524,51 @@
         <v>Air</v>
       </c>
       <c r="AB48" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Hailstorm</v>
+        <v>Pyreball</v>
       </c>
       <c r="B49" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="C49" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="D49" t="str">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="E49" t="str">
         <v>2</v>
       </c>
       <c r="F49" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G49" t="str">
-        <v>Ice pellets rain down in a furious torrent</v>
+        <v>A massive fireball of pure concentrated flame</v>
       </c>
       <c r="H49" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="I49" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="J49" t="str">
-        <v/>
+        <v>burn</v>
       </c>
       <c r="K49" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="L49" t="str">
         <v/>
       </c>
       <c r="M49" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="N49" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="O49" t="str">
         <v/>
@@ -4607,54 +4607,54 @@
         <v/>
       </c>
       <c r="AA49" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="AB49" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Pyreball</v>
+        <v>Ice Shield</v>
       </c>
       <c r="B50" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="C50" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D50" t="str">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="E50" t="str">
         <v>2</v>
       </c>
       <c r="F50" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G50" t="str">
-        <v>A massive fireball of pure concentrated flame</v>
+        <v>Frozen barrier as solid and cold as bedrock</v>
       </c>
       <c r="H50" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="I50" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="J50" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="K50" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L50" t="str">
         <v/>
       </c>
       <c r="M50" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="N50" t="str">
-        <v>enemy</v>
+        <v>self</v>
       </c>
       <c r="O50" t="str">
         <v/>
@@ -4693,45 +4693,45 @@
         <v/>
       </c>
       <c r="AA50" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="AB50" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Ice Shield</v>
+        <v>Glacier</v>
       </c>
       <c r="B51" t="str">
         <v>Ice</v>
       </c>
       <c r="C51" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
       <c r="D51" t="str">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="E51" t="str">
         <v>2</v>
       </c>
       <c r="F51" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G51" t="str">
-        <v>Frozen barrier as solid and cold as bedrock</v>
+        <v>Ancient ice creaks and grinds slowly forward</v>
       </c>
       <c r="H51" t="str">
         <v>Ice</v>
       </c>
       <c r="I51" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
       <c r="J51" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="K51" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="L51" t="str">
         <v/>
@@ -4740,7 +4740,7 @@
         <v/>
       </c>
       <c r="N51" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O51" t="str">
         <v/>
@@ -4782,18 +4782,18 @@
         <v>Ice</v>
       </c>
       <c r="AB51" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Glacier</v>
+        <v>Earthquake</v>
       </c>
       <c r="B52" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="C52" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="D52" t="str">
         <v>126</v>
@@ -4805,19 +4805,19 @@
         <v>5</v>
       </c>
       <c r="G52" t="str">
-        <v>Ancient ice creaks and grinds slowly forward</v>
+        <v>The ground splits open beneath your foe</v>
       </c>
       <c r="H52" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="I52" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="J52" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="K52" t="str">
-        <v/>
+        <v>16</v>
       </c>
       <c r="L52" t="str">
         <v/>
@@ -4826,7 +4826,7 @@
         <v/>
       </c>
       <c r="N52" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O52" t="str">
         <v/>
@@ -4865,101 +4865,15 @@
         <v/>
       </c>
       <c r="AA52" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="AB52" t="str">
-        <v>Ice</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>Earthquake</v>
-      </c>
-      <c r="B53" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="C53" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="D53" t="str">
-        <v>126</v>
-      </c>
-      <c r="E53" t="str">
-        <v>2</v>
-      </c>
-      <c r="F53" t="str">
-        <v>5</v>
-      </c>
-      <c r="G53" t="str">
-        <v>The ground splits open beneath your foe</v>
-      </c>
-      <c r="H53" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="I53" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="J53" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K53" t="str">
-        <v>16</v>
-      </c>
-      <c r="L53" t="str">
-        <v/>
-      </c>
-      <c r="M53" t="str">
-        <v/>
-      </c>
-      <c r="N53" t="str">
-        <v>self</v>
-      </c>
-      <c r="O53" t="str">
-        <v/>
-      </c>
-      <c r="P53" t="str">
-        <v/>
-      </c>
-      <c r="Q53" t="str">
-        <v/>
-      </c>
-      <c r="R53" t="str">
-        <v/>
-      </c>
-      <c r="S53" t="str">
-        <v/>
-      </c>
-      <c r="T53" t="str">
-        <v/>
-      </c>
-      <c r="U53" t="str">
-        <v/>
-      </c>
-      <c r="V53" t="str">
-        <v/>
-      </c>
-      <c r="W53" t="str">
-        <v/>
-      </c>
-      <c r="X53" t="str">
-        <v/>
-      </c>
-      <c r="Y53" t="str">
-        <v/>
-      </c>
-      <c r="Z53" t="str">
-        <v/>
-      </c>
-      <c r="AA53" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="AB53" t="str">
         <v>Earth</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB53"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB52"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (f8e57bf) Add energize status effect
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB52"/>
+  <dimension ref="A1:AB49"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -490,16 +490,16 @@
         <v>Water</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>Ice</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Fire</v>
       </c>
       <c r="D2" t="str">
         <v>8</v>
       </c>
       <c r="E2" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="str">
         <v>1</v>
@@ -514,10 +514,10 @@
         <v/>
       </c>
       <c r="J2" t="str">
-        <v/>
+        <v>heal</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="L2" t="str">
         <v/>
@@ -526,19 +526,19 @@
         <v/>
       </c>
       <c r="N2" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O2" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="P2" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q2" t="str">
         <v/>
       </c>
       <c r="R2" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -565,7 +565,7 @@
         <v/>
       </c>
       <c r="AA2" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="AB2" t="str">
         <v/>
@@ -573,43 +573,43 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Air</v>
       </c>
       <c r="D3" t="str">
         <v>10</v>
       </c>
       <c r="E3" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="str">
         <v>1</v>
       </c>
       <c r="G3" t="str">
-        <v>It's a rock</v>
+        <v>A bright flame burning hot</v>
       </c>
       <c r="H3" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="I3" t="str">
         <v/>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>burn</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="L3" t="str">
         <v/>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="N3" t="str">
         <v/>
@@ -651,7 +651,7 @@
         <v/>
       </c>
       <c r="AA3" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AB3" t="str">
         <v/>
@@ -659,37 +659,37 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="B4" t="str">
-        <v>Ice</v>
+        <v>Leaf</v>
       </c>
       <c r="C4" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="D4" t="str">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="str">
         <v>1</v>
       </c>
       <c r="G4" t="str">
-        <v>A gift from the sky goddess</v>
+        <v>A bright flame burning hot</v>
       </c>
       <c r="H4" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="I4" t="str">
         <v/>
       </c>
       <c r="J4" t="str">
-        <v>heal</v>
+        <v/>
       </c>
       <c r="K4" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="L4" t="str">
         <v/>
@@ -698,19 +698,19 @@
         <v/>
       </c>
       <c r="N4" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O4" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P4" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="Q4" t="str">
         <v/>
       </c>
       <c r="R4" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="S4" t="str">
         <v/>
@@ -740,48 +740,48 @@
         <v/>
       </c>
       <c r="AB4" t="str">
-        <v/>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="B5" t="str">
-        <v>Water</v>
+        <v>Sand</v>
       </c>
       <c r="C5" t="str">
-        <v>Air</v>
+        <v>Sand</v>
       </c>
       <c r="D5" t="str">
         <v>10</v>
       </c>
       <c r="E5" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="str">
         <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v>A bright flame burning hot</v>
+        <v>It's a rock</v>
       </c>
       <c r="H5" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="I5" t="str">
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="K5" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L5" t="str">
         <v/>
       </c>
       <c r="M5" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="N5" t="str">
         <v/>
@@ -831,40 +831,40 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Air</v>
+      </c>
+      <c r="C6" t="str">
         <v>Fire</v>
       </c>
-      <c r="B6" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Lightning</v>
-      </c>
       <c r="D6" t="str">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E6" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="str">
         <v>1</v>
       </c>
       <c r="G6" t="str">
-        <v>A bright flame burning hot</v>
+        <v>Charged spark that strikes instantly</v>
       </c>
       <c r="H6" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="I6" t="str">
         <v/>
       </c>
       <c r="J6" t="str">
-        <v/>
+        <v>multihit</v>
       </c>
       <c r="K6" t="str">
         <v/>
       </c>
       <c r="L6" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="M6" t="str">
         <v/>
@@ -917,16 +917,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Earth</v>
+        <v>Plasma</v>
       </c>
       <c r="B7" t="str">
-        <v>Sand</v>
+        <v>Lightning</v>
       </c>
       <c r="C7" t="str">
-        <v>Sand</v>
+        <v>Air</v>
       </c>
       <c r="D7" t="str">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E7" t="str">
         <v>1</v>
@@ -935,19 +935,19 @@
         <v>1</v>
       </c>
       <c r="G7" t="str">
-        <v>It's a rock</v>
+        <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H7" t="str">
-        <v>Earth</v>
+        <v>Plasma</v>
       </c>
       <c r="I7" t="str">
         <v/>
       </c>
       <c r="J7" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="K7" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="L7" t="str">
         <v/>
@@ -1003,16 +1003,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>Plasma</v>
+      </c>
+      <c r="B8" t="str">
         <v>Lightning</v>
       </c>
-      <c r="B8" t="str">
-        <v>Air</v>
-      </c>
       <c r="C8" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D8" t="str">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E8" t="str">
         <v>1</v>
@@ -1021,22 +1021,22 @@
         <v>1</v>
       </c>
       <c r="G8" t="str">
-        <v>Charged spark that strikes instantly</v>
+        <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H8" t="str">
-        <v>Lightning</v>
+        <v>Plasma</v>
       </c>
       <c r="I8" t="str">
         <v/>
       </c>
       <c r="J8" t="str">
-        <v>multihit</v>
+        <v/>
       </c>
       <c r="K8" t="str">
         <v/>
       </c>
       <c r="L8" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="M8" t="str">
         <v/>
@@ -1095,7 +1095,7 @@
         <v>Lightning</v>
       </c>
       <c r="C9" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="D9" t="str">
         <v>1</v>
@@ -1178,10 +1178,10 @@
         <v>Plasma</v>
       </c>
       <c r="B10" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="C10" t="str">
         <v>Lightning</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Earth</v>
       </c>
       <c r="D10" t="str">
         <v>1</v>
@@ -1196,10 +1196,10 @@
         <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H10" t="str">
-        <v>Plasma</v>
+        <v>Fire</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>Lightning</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1261,16 +1261,16 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Plasma</v>
+        <v>Sand</v>
       </c>
       <c r="B11" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="C11" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D11" t="str">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E11" t="str">
         <v>1</v>
@@ -1279,10 +1279,10 @@
         <v>1</v>
       </c>
       <c r="G11" t="str">
-        <v>A deep sense of calm overwhelms you</v>
+        <v>Shifting grains dance between your fingertips</v>
       </c>
       <c r="H11" t="str">
-        <v>Plasma</v>
+        <v>Earth</v>
       </c>
       <c r="I11" t="str">
         <v/>
@@ -1347,16 +1347,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Plasma</v>
+        <v>Sand</v>
       </c>
       <c r="B12" t="str">
-        <v>Fire</v>
+        <v>Air</v>
       </c>
       <c r="C12" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="D12" t="str">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E12" t="str">
         <v>1</v>
@@ -1365,13 +1365,13 @@
         <v>1</v>
       </c>
       <c r="G12" t="str">
-        <v>A deep sense of calm overwhelms you</v>
+        <v>Shifting grains dance between your fingertips</v>
       </c>
       <c r="H12" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="I12" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -1433,10 +1433,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="B13" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="C13" t="str">
         <v>Earth</v>
@@ -1451,10 +1451,10 @@
         <v>1</v>
       </c>
       <c r="G13" t="str">
-        <v>Shifting grains dance between your fingertips</v>
+        <v>Forged from fire and stone, hammered hard</v>
       </c>
       <c r="H13" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="I13" t="str">
         <v/>
@@ -1519,28 +1519,28 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Sand</v>
+        <v>Air</v>
       </c>
       <c r="B14" t="str">
-        <v>Air</v>
+        <v>Water</v>
       </c>
       <c r="C14" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="D14" t="str">
         <v>10</v>
       </c>
       <c r="E14" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" t="str">
         <v>1</v>
       </c>
       <c r="G14" t="str">
-        <v>Shifting grains dance between your fingertips</v>
+        <v>A cool rush of wind drifts past your face</v>
       </c>
       <c r="H14" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="I14" t="str">
         <v/>
@@ -1605,46 +1605,46 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Steel</v>
+        <v>Leaf</v>
       </c>
       <c r="B15" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="C15" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="D15" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E15" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" t="str">
         <v>1</v>
       </c>
       <c r="G15" t="str">
-        <v>Forged from fire and stone, hammered hard</v>
+        <v>Drops of dew glistle atop</v>
       </c>
       <c r="H15" t="str">
-        <v>Steel</v>
+        <v>Earth</v>
       </c>
       <c r="I15" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>energize</v>
       </c>
       <c r="K15" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="L15" t="str">
         <v/>
       </c>
       <c r="M15" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="N15" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -1683,7 +1683,7 @@
         <v/>
       </c>
       <c r="AA15" t="str">
-        <v/>
+        <v>Leaf</v>
       </c>
       <c r="AB15" t="str">
         <v/>
@@ -1691,13 +1691,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="B16" t="str">
         <v>Water</v>
       </c>
       <c r="C16" t="str">
-        <v>Fire</v>
+        <v>Air</v>
       </c>
       <c r="D16" t="str">
         <v>10</v>
@@ -1709,10 +1709,10 @@
         <v>1</v>
       </c>
       <c r="G16" t="str">
-        <v>A cool rush of wind drifts past your face</v>
+        <v>A biting chill that settles in your bones</v>
       </c>
       <c r="H16" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -1777,16 +1777,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Leaf</v>
+        <v>Glass</v>
       </c>
       <c r="B17" t="str">
-        <v>Earth</v>
+        <v>Sand</v>
       </c>
       <c r="C17" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="D17" t="str">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E17" t="str">
         <v>1</v>
@@ -1795,13 +1795,13 @@
         <v>1</v>
       </c>
       <c r="G17" t="str">
-        <v>Drops of dew glistle atop</v>
+        <v>Smooth and brittle, it catches the light</v>
       </c>
       <c r="H17" t="str">
-        <v>Earth</v>
+        <v>Glass</v>
       </c>
       <c r="I17" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -1863,16 +1863,16 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Ice</v>
+        <v>Glass</v>
       </c>
       <c r="B18" t="str">
-        <v>Water</v>
+        <v>Sand</v>
       </c>
       <c r="C18" t="str">
-        <v>Air</v>
+        <v>Lightning</v>
       </c>
       <c r="D18" t="str">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E18" t="str">
         <v>1</v>
@@ -1881,10 +1881,10 @@
         <v>1</v>
       </c>
       <c r="G18" t="str">
-        <v>A biting chill that settles in your bones</v>
+        <v>Smooth and brittle, it catches the light</v>
       </c>
       <c r="H18" t="str">
-        <v>Ice</v>
+        <v>Glass</v>
       </c>
       <c r="I18" t="str">
         <v/>
@@ -1949,28 +1949,28 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Glass</v>
+        <v>Dark Matter</v>
       </c>
       <c r="B19" t="str">
-        <v>Sand</v>
+        <v>Unstable Element</v>
       </c>
       <c r="C19" t="str">
-        <v>Fire</v>
+        <v>Unstable Element</v>
       </c>
       <c r="D19" t="str">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E19" t="str">
         <v>1</v>
       </c>
       <c r="F19" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" t="str">
-        <v>Smooth and brittle, it catches the light</v>
+        <v>A quiet humming radiates from inside</v>
       </c>
       <c r="H19" t="str">
-        <v>Glass</v>
+        <v>Void</v>
       </c>
       <c r="I19" t="str">
         <v/>
@@ -2035,37 +2035,37 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Glass</v>
+        <v>Worble</v>
       </c>
       <c r="B20" t="str">
-        <v>Sand</v>
+        <v>Water</v>
       </c>
       <c r="C20" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="D20" t="str">
-        <v>12</v>
+        <v>126</v>
       </c>
       <c r="E20" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F20" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G20" t="str">
-        <v>Smooth and brittle, it catches the light</v>
+        <v>The tide is high today my friend</v>
       </c>
       <c r="H20" t="str">
-        <v>Glass</v>
+        <v>Water</v>
       </c>
       <c r="I20" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="K20" t="str">
-        <v/>
+        <v>4</v>
       </c>
       <c r="L20" t="str">
         <v/>
@@ -2074,7 +2074,7 @@
         <v/>
       </c>
       <c r="N20" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="O20" t="str">
         <v/>
@@ -2113,60 +2113,54 @@
         <v/>
       </c>
       <c r="AA20" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="AB20" t="str">
-        <v/>
+        <v>Water</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Dark Matter</v>
+        <v>Blaze</v>
       </c>
       <c r="B21" t="str">
-        <v>Unstable Element</v>
+        <v>Leaf</v>
       </c>
       <c r="C21" t="str">
-        <v>Unstable Element</v>
+        <v>Fire</v>
       </c>
       <c r="D21" t="str">
-        <v>18</v>
+        <v>109</v>
       </c>
       <c r="E21" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21" t="str">
+        <v>5</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Forest floor erupts in scorching flame</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="J21" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K21" t="str">
+        <v>6</v>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
         <v>2</v>
       </c>
-      <c r="G21" t="str">
-        <v>A quiet humming radiates from inside</v>
-      </c>
-      <c r="H21" t="str">
-        <v>Void</v>
-      </c>
-      <c r="I21" t="str">
-        <v/>
-      </c>
-      <c r="J21" t="str">
-        <v/>
-      </c>
-      <c r="K21" t="str">
-        <v/>
-      </c>
-      <c r="L21" t="str">
-        <v/>
-      </c>
-      <c r="M21" t="str">
-        <v/>
-      </c>
       <c r="N21" t="str">
-        <v/>
-      </c>
-      <c r="O21" t="str">
-        <v/>
-      </c>
-      <c r="P21" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="Q21" t="str">
         <v/>
@@ -2174,9 +2168,6 @@
       <c r="R21" t="str">
         <v/>
       </c>
-      <c r="S21" t="str">
-        <v/>
-      </c>
       <c r="T21" t="str">
         <v/>
       </c>
@@ -2199,24 +2190,24 @@
         <v/>
       </c>
       <c r="AA21" t="str">
-        <v/>
+        <v>Fire</v>
       </c>
       <c r="AB21" t="str">
-        <v/>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Worble</v>
+        <v>Regen</v>
       </c>
       <c r="B22" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="C22" t="str">
         <v>Water</v>
       </c>
       <c r="D22" t="str">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="E22" t="str">
         <v>2</v>
@@ -2225,19 +2216,19 @@
         <v>5</v>
       </c>
       <c r="G22" t="str">
-        <v>The tide is high today my friend</v>
+        <v>Living vines wrap wounds in cool water</v>
       </c>
       <c r="H22" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="I22" t="str">
         <v>Water</v>
       </c>
       <c r="J22" t="str">
-        <v>soak</v>
+        <v>shield</v>
       </c>
       <c r="K22" t="str">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L22" t="str">
         <v/>
@@ -2246,21 +2237,12 @@
         <v/>
       </c>
       <c r="N22" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="O22" t="str">
-        <v/>
-      </c>
-      <c r="P22" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="Q22" t="str">
         <v/>
       </c>
       <c r="R22" t="str">
-        <v/>
-      </c>
-      <c r="S22" t="str">
         <v/>
       </c>
       <c r="T22" t="str">
@@ -2288,18 +2270,18 @@
         <v>Water</v>
       </c>
       <c r="AB22" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Blaze</v>
+        <v>Thorns</v>
       </c>
       <c r="B23" t="str">
         <v>Leaf</v>
       </c>
       <c r="C23" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D23" t="str">
         <v>109</v>
@@ -2311,81 +2293,72 @@
         <v>5</v>
       </c>
       <c r="G23" t="str">
-        <v>Forest floor erupts in scorching flame</v>
+        <v>Spiked vines protect you</v>
       </c>
       <c r="H23" t="str">
-        <v>Fire</v>
+        <v>Leaf</v>
       </c>
       <c r="I23" t="str">
+        <v>Water</v>
+      </c>
+      <c r="J23" t="str">
+        <v>shield</v>
+      </c>
+      <c r="K23" t="str">
+        <v>8</v>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v>self</v>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
+      </c>
+      <c r="Y23" t="str">
+        <v/>
+      </c>
+      <c r="Z23" t="str">
+        <v/>
+      </c>
+      <c r="AA23" t="str">
         <v>Earth</v>
       </c>
-      <c r="J23" t="str">
-        <v>burn</v>
-      </c>
-      <c r="K23" t="str">
-        <v>6</v>
-      </c>
-      <c r="L23" t="str">
-        <v/>
-      </c>
-      <c r="M23" t="str">
-        <v>2</v>
-      </c>
-      <c r="N23" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="O23" t="str">
-        <v>shield</v>
-      </c>
-      <c r="P23" t="str">
-        <v>8</v>
-      </c>
-      <c r="Q23" t="str">
-        <v/>
-      </c>
-      <c r="R23" t="str">
-        <v/>
-      </c>
-      <c r="S23" t="str">
-        <v>self</v>
-      </c>
-      <c r="T23" t="str">
-        <v/>
-      </c>
-      <c r="U23" t="str">
-        <v/>
-      </c>
-      <c r="V23" t="str">
-        <v/>
-      </c>
-      <c r="W23" t="str">
-        <v/>
-      </c>
-      <c r="X23" t="str">
-        <v/>
-      </c>
-      <c r="Y23" t="str">
-        <v/>
-      </c>
-      <c r="Z23" t="str">
-        <v/>
-      </c>
-      <c r="AA23" t="str">
-        <v>Fire</v>
-      </c>
       <c r="AB23" t="str">
-        <v>Earth</v>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Regen</v>
+        <v>Tornado</v>
       </c>
       <c r="B24" t="str">
         <v>Leaf</v>
       </c>
       <c r="C24" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="D24" t="str">
         <v>109</v>
@@ -2394,16 +2367,16 @@
         <v>2</v>
       </c>
       <c r="F24" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G24" t="str">
-        <v>Living vines wrap wounds in cool water</v>
+        <v>Wind whips and slashes about</v>
       </c>
       <c r="H24" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="I24" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="J24" t="str">
         <v>shield</v>
@@ -2421,10 +2394,10 @@
         <v>self</v>
       </c>
       <c r="O24" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P24" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q24" t="str">
         <v/>
@@ -2433,7 +2406,7 @@
         <v/>
       </c>
       <c r="S24" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T24" t="str">
         <v/>
@@ -2457,21 +2430,21 @@
         <v/>
       </c>
       <c r="AA24" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="AB24" t="str">
-        <v>Earth</v>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Thorns</v>
+        <v>Blizzard</v>
       </c>
       <c r="B25" t="str">
         <v>Leaf</v>
       </c>
       <c r="C25" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
       <c r="D25" t="str">
         <v>109</v>
@@ -2483,13 +2456,13 @@
         <v>5</v>
       </c>
       <c r="G25" t="str">
-        <v>Spiked vines protect you</v>
+        <v>Snow flurries block your vision</v>
       </c>
       <c r="H25" t="str">
-        <v>Earth</v>
+        <v>Leaf</v>
       </c>
       <c r="I25" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="J25" t="str">
         <v>shield</v>
@@ -2507,10 +2480,10 @@
         <v>self</v>
       </c>
       <c r="O25" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P25" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q25" t="str">
         <v/>
@@ -2519,7 +2492,7 @@
         <v/>
       </c>
       <c r="S25" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T25" t="str">
         <v/>
@@ -2543,39 +2516,39 @@
         <v/>
       </c>
       <c r="AA25" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
       <c r="AB25" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Tornado</v>
+        <v>Leaf Blade</v>
       </c>
       <c r="B26" t="str">
         <v>Leaf</v>
       </c>
       <c r="C26" t="str">
-        <v>Air</v>
+        <v>Steel</v>
       </c>
       <c r="D26" t="str">
-        <v>109</v>
+        <v>159</v>
       </c>
       <c r="E26" t="str">
         <v>2</v>
       </c>
       <c r="F26" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G26" t="str">
-        <v>Wind whips and slashes about</v>
+        <v>A razor edge honed from living wood</v>
       </c>
       <c r="H26" t="str">
-        <v>Air</v>
+        <v>Leaf</v>
       </c>
       <c r="I26" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="J26" t="str">
         <v>shield</v>
@@ -2592,21 +2565,12 @@
       <c r="N26" t="str">
         <v>self</v>
       </c>
-      <c r="O26" t="str">
-        <v/>
-      </c>
-      <c r="P26" t="str">
-        <v/>
-      </c>
       <c r="Q26" t="str">
         <v/>
       </c>
       <c r="R26" t="str">
         <v/>
       </c>
-      <c r="S26" t="str">
-        <v/>
-      </c>
       <c r="T26" t="str">
         <v/>
       </c>
@@ -2629,36 +2593,36 @@
         <v/>
       </c>
       <c r="AA26" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
       <c r="AB26" t="str">
-        <v>Earth</v>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Blizzard</v>
+        <v>Needle Storm</v>
       </c>
       <c r="B27" t="str">
         <v>Leaf</v>
       </c>
       <c r="C27" t="str">
-        <v>Ice</v>
+        <v>Sand</v>
       </c>
       <c r="D27" t="str">
-        <v>109</v>
+        <v>159</v>
       </c>
       <c r="E27" t="str">
         <v>2</v>
       </c>
       <c r="F27" t="str">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G27" t="str">
-        <v>Snow flurries block your vision</v>
+        <v>Tiny needles prick from every angle</v>
       </c>
       <c r="H27" t="str">
-        <v>Ice</v>
+        <v>Leaf</v>
       </c>
       <c r="I27" t="str">
         <v>Earth</v>
@@ -2678,21 +2642,12 @@
       <c r="N27" t="str">
         <v>self</v>
       </c>
-      <c r="O27" t="str">
-        <v/>
-      </c>
-      <c r="P27" t="str">
-        <v/>
-      </c>
       <c r="Q27" t="str">
         <v/>
       </c>
       <c r="R27" t="str">
         <v/>
       </c>
-      <c r="S27" t="str">
-        <v/>
-      </c>
       <c r="T27" t="str">
         <v/>
       </c>
@@ -2715,45 +2670,45 @@
         <v/>
       </c>
       <c r="AA27" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="AB27" t="str">
-        <v>Earth</v>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Leaf Blade</v>
+        <v>Photosynthesis</v>
       </c>
       <c r="B28" t="str">
         <v>Leaf</v>
       </c>
       <c r="C28" t="str">
-        <v>Steel</v>
+        <v>Leaf</v>
       </c>
       <c r="D28" t="str">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="E28" t="str">
         <v>2</v>
       </c>
       <c r="F28" t="str">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G28" t="str">
-        <v>A razor edge honed from living wood</v>
+        <v>Nature feeds itself to grow ever stronger</v>
       </c>
       <c r="H28" t="str">
-        <v>Earth</v>
+        <v>Leaf</v>
       </c>
       <c r="I28" t="str">
-        <v>Steel</v>
+        <v>Water</v>
       </c>
       <c r="J28" t="str">
-        <v>shield</v>
+        <v>soak</v>
       </c>
       <c r="K28" t="str">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L28" t="str">
         <v/>
@@ -2762,22 +2717,13 @@
         <v/>
       </c>
       <c r="N28" t="str">
-        <v>self</v>
-      </c>
-      <c r="O28" t="str">
-        <v>soak</v>
-      </c>
-      <c r="P28" t="str">
-        <v>2</v>
+        <v>enemy</v>
       </c>
       <c r="Q28" t="str">
         <v/>
       </c>
       <c r="R28" t="str">
         <v/>
-      </c>
-      <c r="S28" t="str">
-        <v>enemy</v>
       </c>
       <c r="T28" t="str">
         <v/>
@@ -2804,18 +2750,18 @@
         <v>Earth</v>
       </c>
       <c r="AB28" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Needle Storm</v>
+        <v>Desert Blade</v>
       </c>
       <c r="B29" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C29" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="D29" t="str">
         <v>159</v>
@@ -2824,16 +2770,16 @@
         <v>2</v>
       </c>
       <c r="F29" t="str">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G29" t="str">
-        <v>Tiny needles prick from every angle</v>
+        <v>Sand-forged steel scorched by the desert sun</v>
       </c>
       <c r="H29" t="str">
         <v>Earth</v>
       </c>
       <c r="I29" t="str">
-        <v>Water</v>
+        <v>Steel</v>
       </c>
       <c r="J29" t="str">
         <v>shield</v>
@@ -2850,20 +2796,11 @@
       <c r="N29" t="str">
         <v>self</v>
       </c>
-      <c r="O29" t="str">
-        <v>soak</v>
-      </c>
-      <c r="P29" t="str">
-        <v>2</v>
-      </c>
       <c r="Q29" t="str">
         <v/>
       </c>
       <c r="R29" t="str">
         <v/>
-      </c>
-      <c r="S29" t="str">
-        <v>enemy</v>
       </c>
       <c r="T29" t="str">
         <v/>
@@ -2890,36 +2827,36 @@
         <v>Earth</v>
       </c>
       <c r="AB29" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Photosynthesis</v>
+        <v>Sand Shield</v>
       </c>
       <c r="B30" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C30" t="str">
-        <v>Leaf</v>
+        <v>Earth</v>
       </c>
       <c r="D30" t="str">
-        <v>210</v>
+        <v>109</v>
       </c>
       <c r="E30" t="str">
         <v>2</v>
       </c>
       <c r="F30" t="str">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G30" t="str">
-        <v>Nature feeds itself to grow ever stronger</v>
+        <v>Grains pack tight into an earthen wall</v>
       </c>
       <c r="H30" t="str">
         <v>Earth</v>
       </c>
       <c r="I30" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="J30" t="str">
         <v>shield</v>
@@ -2937,10 +2874,10 @@
         <v>self</v>
       </c>
       <c r="O30" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P30" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q30" t="str">
         <v/>
@@ -2949,7 +2886,7 @@
         <v/>
       </c>
       <c r="S30" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T30" t="str">
         <v/>
@@ -2976,57 +2913,57 @@
         <v>Earth</v>
       </c>
       <c r="AB30" t="str">
-        <v>Water</v>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Desert Blade</v>
+        <v>Sandstorm</v>
       </c>
       <c r="B31" t="str">
         <v>Sand</v>
       </c>
       <c r="C31" t="str">
-        <v>Steel</v>
+        <v>Air</v>
       </c>
       <c r="D31" t="str">
-        <v>159</v>
+        <v>109</v>
       </c>
       <c r="E31" t="str">
         <v>2</v>
       </c>
       <c r="F31" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G31" t="str">
-        <v>Sand-forged steel scorched by the desert sun</v>
+        <v>Blinding grit swirls on howling winds</v>
       </c>
       <c r="H31" t="str">
+        <v>Air</v>
+      </c>
+      <c r="I31" t="str">
         <v>Earth</v>
       </c>
-      <c r="I31" t="str">
-        <v>Steel</v>
-      </c>
       <c r="J31" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="K31" t="str">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L31" t="str">
         <v/>
       </c>
       <c r="M31" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N31" t="str">
-        <v>enemy</v>
+        <v>self</v>
       </c>
       <c r="O31" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="P31" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="Q31" t="str">
         <v/>
@@ -3035,7 +2972,7 @@
         <v/>
       </c>
       <c r="S31" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="T31" t="str">
         <v/>
@@ -3059,21 +2996,21 @@
         <v/>
       </c>
       <c r="AA31" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AB31" t="str">
         <v>Earth</v>
-      </c>
-      <c r="AB31" t="str">
-        <v>Fire</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Mud Shot</v>
+        <v>Iceblast</v>
       </c>
       <c r="B32" t="str">
         <v>Sand</v>
       </c>
       <c r="C32" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="D32" t="str">
         <v>109</v>
@@ -3085,10 +3022,10 @@
         <v>5</v>
       </c>
       <c r="G32" t="str">
-        <v>Thick sludge launched with surprising force</v>
+        <v>Cold grit bites with a frosty sting</v>
       </c>
       <c r="H32" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="I32" t="str">
         <v>Earth</v>
@@ -3109,10 +3046,10 @@
         <v>self</v>
       </c>
       <c r="O32" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P32" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q32" t="str">
         <v/>
@@ -3121,7 +3058,7 @@
         <v/>
       </c>
       <c r="S32" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T32" t="str">
         <v/>
@@ -3145,7 +3082,7 @@
         <v/>
       </c>
       <c r="AA32" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="AB32" t="str">
         <v>Earth</v>
@@ -3153,13 +3090,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Sand Shield</v>
+        <v>Blaze Blade</v>
       </c>
       <c r="B33" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="C33" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="D33" t="str">
         <v>109</v>
@@ -3168,84 +3105,75 @@
         <v>2</v>
       </c>
       <c r="F33" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G33" t="str">
-        <v>Grains pack tight into an earthen wall</v>
+        <v>A steel blade bathed in white-hot flame</v>
       </c>
       <c r="H33" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="J33" t="str">
+        <v>burn</v>
+      </c>
+      <c r="K33" t="str">
+        <v>6</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v>2</v>
+      </c>
+      <c r="N33" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
+        <v/>
+      </c>
+      <c r="V33" t="str">
+        <v/>
+      </c>
+      <c r="W33" t="str">
+        <v/>
+      </c>
+      <c r="X33" t="str">
+        <v/>
+      </c>
+      <c r="Y33" t="str">
+        <v/>
+      </c>
+      <c r="Z33" t="str">
+        <v/>
+      </c>
+      <c r="AA33" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="AB33" t="str">
         <v>Earth</v>
-      </c>
-      <c r="I33" t="str">
-        <v/>
-      </c>
-      <c r="J33" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K33" t="str">
-        <v>8</v>
-      </c>
-      <c r="L33" t="str">
-        <v/>
-      </c>
-      <c r="M33" t="str">
-        <v/>
-      </c>
-      <c r="N33" t="str">
-        <v>self</v>
-      </c>
-      <c r="O33" t="str">
-        <v/>
-      </c>
-      <c r="P33" t="str">
-        <v/>
-      </c>
-      <c r="Q33" t="str">
-        <v/>
-      </c>
-      <c r="R33" t="str">
-        <v/>
-      </c>
-      <c r="S33" t="str">
-        <v/>
-      </c>
-      <c r="T33" t="str">
-        <v/>
-      </c>
-      <c r="U33" t="str">
-        <v/>
-      </c>
-      <c r="V33" t="str">
-        <v/>
-      </c>
-      <c r="W33" t="str">
-        <v/>
-      </c>
-      <c r="X33" t="str">
-        <v/>
-      </c>
-      <c r="Y33" t="str">
-        <v/>
-      </c>
-      <c r="Z33" t="str">
-        <v/>
-      </c>
-      <c r="AA33" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="AB33" t="str">
-        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Sandstorm</v>
+        <v>Aqua Blade</v>
       </c>
       <c r="B34" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="C34" t="str">
-        <v>Air</v>
+        <v>Water</v>
       </c>
       <c r="D34" t="str">
         <v>109</v>
@@ -3254,22 +3182,22 @@
         <v>2</v>
       </c>
       <c r="F34" t="str">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G34" t="str">
-        <v>Blinding grit swirls on howling winds</v>
+        <v>Steam rises where cold steel meets the wave</v>
       </c>
       <c r="H34" t="str">
-        <v>Air</v>
+        <v>Water</v>
       </c>
       <c r="I34" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="J34" t="str">
-        <v>shield</v>
+        <v>soak</v>
       </c>
       <c r="K34" t="str">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L34" t="str">
         <v/>
@@ -3278,22 +3206,7 @@
         <v/>
       </c>
       <c r="N34" t="str">
-        <v>self</v>
-      </c>
-      <c r="O34" t="str">
-        <v/>
-      </c>
-      <c r="P34" t="str">
-        <v/>
-      </c>
-      <c r="Q34" t="str">
-        <v/>
-      </c>
-      <c r="R34" t="str">
-        <v/>
-      </c>
-      <c r="S34" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="T34" t="str">
         <v/>
@@ -3317,21 +3230,21 @@
         <v/>
       </c>
       <c r="AA34" t="str">
-        <v>Air</v>
+        <v>Water</v>
       </c>
       <c r="AB34" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Iceblast</v>
+        <v>Thunder Blade</v>
       </c>
       <c r="B35" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="C35" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
       <c r="D35" t="str">
         <v>109</v>
@@ -3340,47 +3253,35 @@
         <v>2</v>
       </c>
       <c r="F35" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G35" t="str">
-        <v>Cold grit bites with a frosty sting</v>
+        <v>Sparks dance across the blades edge</v>
       </c>
       <c r="H35" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
       <c r="I35" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="J35" t="str">
-        <v>shield</v>
+        <v>multi_hit</v>
       </c>
       <c r="K35" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="L35" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="M35" t="str">
         <v/>
       </c>
       <c r="N35" t="str">
-        <v>self</v>
-      </c>
-      <c r="O35" t="str">
-        <v/>
-      </c>
-      <c r="P35" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="Q35" t="str">
         <v/>
       </c>
-      <c r="R35" t="str">
-        <v/>
-      </c>
-      <c r="S35" t="str">
-        <v/>
-      </c>
       <c r="T35" t="str">
         <v/>
       </c>
@@ -3403,21 +3304,21 @@
         <v/>
       </c>
       <c r="AA35" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
       <c r="AB35" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Blaze Blade</v>
+        <v>Earth Blade</v>
       </c>
       <c r="B36" t="str">
         <v>Steel</v>
       </c>
       <c r="C36" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D36" t="str">
         <v>109</v>
@@ -3429,42 +3330,27 @@
         <v>0</v>
       </c>
       <c r="G36" t="str">
-        <v>A steel blade bathed in white-hot flame</v>
+        <v>Heavy as bedrock</v>
       </c>
       <c r="H36" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="I36" t="str">
         <v>Steel</v>
       </c>
       <c r="J36" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="K36" t="str">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L36" t="str">
         <v/>
       </c>
       <c r="M36" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N36" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="O36" t="str">
-        <v>shield</v>
-      </c>
-      <c r="P36" t="str">
-        <v>8</v>
-      </c>
-      <c r="Q36" t="str">
-        <v/>
-      </c>
-      <c r="R36" t="str">
-        <v/>
-      </c>
-      <c r="S36" t="str">
         <v>self</v>
       </c>
       <c r="T36" t="str">
@@ -3489,21 +3375,21 @@
         <v/>
       </c>
       <c r="AA36" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AB36" t="str">
         <v>Fire</v>
-      </c>
-      <c r="AB36" t="str">
-        <v>Earth</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Aqua Blade</v>
+        <v>Air Blade</v>
       </c>
       <c r="B37" t="str">
         <v>Steel</v>
       </c>
       <c r="C37" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="D37" t="str">
         <v>109</v>
@@ -3515,34 +3401,22 @@
         <v>0</v>
       </c>
       <c r="G37" t="str">
-        <v>Steam rises where cold steel meets the wave</v>
+        <v>Cuts the air so fast it ignites</v>
       </c>
       <c r="H37" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="I37" t="str">
         <v>Steel</v>
       </c>
-      <c r="J37" t="str">
-        <v>burn</v>
-      </c>
-      <c r="K37" t="str">
-        <v>6</v>
-      </c>
       <c r="L37" t="str">
         <v/>
       </c>
-      <c r="M37" t="str">
-        <v>2</v>
-      </c>
-      <c r="N37" t="str">
-        <v>enemy</v>
-      </c>
       <c r="O37" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P37" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q37" t="str">
         <v/>
@@ -3551,7 +3425,7 @@
         <v/>
       </c>
       <c r="S37" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T37" t="str">
         <v/>
@@ -3575,7 +3449,7 @@
         <v/>
       </c>
       <c r="AA37" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="AB37" t="str">
         <v>Fire</v>
@@ -3583,13 +3457,13 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Thunder Blade</v>
+        <v>Ice Blade</v>
       </c>
       <c r="B38" t="str">
         <v>Steel</v>
       </c>
       <c r="C38" t="str">
-        <v>Lightning</v>
+        <v>Ice</v>
       </c>
       <c r="D38" t="str">
         <v>109</v>
@@ -3601,43 +3475,31 @@
         <v>0</v>
       </c>
       <c r="G38" t="str">
-        <v>Sparks dance across the blades edge</v>
+        <v>Cold steel that somehow scorches on contact</v>
       </c>
       <c r="H38" t="str">
-        <v>Lightning</v>
+        <v>Ice</v>
       </c>
       <c r="I38" t="str">
         <v>Steel</v>
       </c>
-      <c r="J38" t="str">
-        <v>multi_hit</v>
-      </c>
-      <c r="K38" t="str">
-        <v/>
-      </c>
       <c r="L38" t="str">
-        <v>2</v>
-      </c>
-      <c r="M38" t="str">
-        <v/>
-      </c>
-      <c r="N38" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="O38" t="str">
-        <v>burn</v>
+        <v/>
       </c>
       <c r="P38" t="str">
-        <v>6</v>
+        <v/>
       </c>
       <c r="Q38" t="str">
         <v/>
       </c>
       <c r="R38" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="S38" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T38" t="str">
         <v/>
@@ -3661,7 +3523,7 @@
         <v/>
       </c>
       <c r="AA38" t="str">
-        <v>Lightning</v>
+        <v>Ice</v>
       </c>
       <c r="AB38" t="str">
         <v>Fire</v>
@@ -3669,16 +3531,16 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Earth Blade</v>
+        <v>Refined Steel</v>
       </c>
       <c r="B39" t="str">
         <v>Steel</v>
       </c>
       <c r="C39" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="D39" t="str">
-        <v>109</v>
+        <v>210</v>
       </c>
       <c r="E39" t="str">
         <v>2</v>
@@ -3687,44 +3549,23 @@
         <v>0</v>
       </c>
       <c r="G39" t="str">
-        <v>Heavy as bedrock</v>
+        <v>Folded a thousand times until perfect</v>
       </c>
       <c r="H39" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="I39" t="str">
         <v>Steel</v>
       </c>
-      <c r="J39" t="str">
-        <v>burn</v>
-      </c>
-      <c r="K39" t="str">
-        <v>6</v>
-      </c>
       <c r="L39" t="str">
         <v/>
       </c>
-      <c r="M39" t="str">
-        <v>2</v>
-      </c>
-      <c r="N39" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="O39" t="str">
-        <v>shield</v>
-      </c>
-      <c r="P39" t="str">
-        <v>8</v>
-      </c>
       <c r="Q39" t="str">
         <v/>
       </c>
       <c r="R39" t="str">
         <v/>
       </c>
-      <c r="S39" t="str">
-        <v>self</v>
-      </c>
       <c r="T39" t="str">
         <v/>
       </c>
@@ -3747,60 +3588,60 @@
         <v/>
       </c>
       <c r="AA39" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="AB39" t="str">
         <v>Earth</v>
-      </c>
-      <c r="AB39" t="str">
-        <v>Fire</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Air Blade</v>
+        <v>Water Bolt</v>
       </c>
       <c r="B40" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="C40" t="str">
-        <v>Air</v>
+        <v>Water</v>
       </c>
       <c r="D40" t="str">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E40" t="str">
         <v>2</v>
       </c>
       <c r="F40" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G40" t="str">
-        <v>Cuts the air so fast it ignites</v>
+        <v>Crackling bolts that drench what they strike</v>
       </c>
       <c r="H40" t="str">
-        <v>Air</v>
+        <v>Lightning</v>
       </c>
       <c r="I40" t="str">
-        <v>Steel</v>
+        <v>Water</v>
       </c>
       <c r="J40" t="str">
-        <v>burn</v>
+        <v>multi_hit</v>
       </c>
       <c r="K40" t="str">
-        <v>6</v>
+        <v/>
       </c>
       <c r="L40" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="M40" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N40" t="str">
         <v>enemy</v>
       </c>
       <c r="O40" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="P40" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="Q40" t="str">
         <v/>
@@ -3809,7 +3650,7 @@
         <v/>
       </c>
       <c r="S40" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="T40" t="str">
         <v/>
@@ -3833,51 +3674,51 @@
         <v/>
       </c>
       <c r="AA40" t="str">
-        <v>Air</v>
+        <v>Lightning</v>
       </c>
       <c r="AB40" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Ice Blade</v>
+        <v>Ice Bolt</v>
       </c>
       <c r="B41" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="C41" t="str">
         <v>Ice</v>
       </c>
       <c r="D41" t="str">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E41" t="str">
         <v>2</v>
       </c>
       <c r="F41" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G41" t="str">
-        <v>Cold steel that somehow scorches on contact</v>
+        <v>A frozen shard launched like a thunderbolt</v>
       </c>
       <c r="H41" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="I41" t="str">
         <v>Ice</v>
       </c>
-      <c r="I41" t="str">
-        <v>Steel</v>
-      </c>
       <c r="J41" t="str">
-        <v>burn</v>
+        <v>multi_hit</v>
       </c>
       <c r="K41" t="str">
-        <v>6</v>
+        <v/>
       </c>
       <c r="L41" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="M41" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N41" t="str">
         <v>enemy</v>
@@ -3919,60 +3760,60 @@
         <v/>
       </c>
       <c r="AA41" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="AB41" t="str">
         <v>Ice</v>
-      </c>
-      <c r="AB41" t="str">
-        <v>Fire</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Refined Steel</v>
+        <v>Thunder</v>
       </c>
       <c r="B42" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="C42" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="D42" t="str">
-        <v>210</v>
+        <v>126</v>
       </c>
       <c r="E42" t="str">
         <v>2</v>
       </c>
       <c r="F42" t="str">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G42" t="str">
-        <v>Folded a thousand times until perfect</v>
+        <v>Strikes once, twice, three times in a flash</v>
       </c>
       <c r="H42" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="I42" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="J42" t="str">
-        <v>burn</v>
+        <v>multi_hit</v>
       </c>
       <c r="K42" t="str">
-        <v>6</v>
+        <v/>
       </c>
       <c r="L42" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="M42" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N42" t="str">
         <v>enemy</v>
       </c>
       <c r="O42" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="P42" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="Q42" t="str">
         <v/>
@@ -3981,7 +3822,7 @@
         <v/>
       </c>
       <c r="S42" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="T42" t="str">
         <v/>
@@ -4005,54 +3846,54 @@
         <v/>
       </c>
       <c r="AA42" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="AB42" t="str">
-        <v>Earth</v>
+        <v>Lightning</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Water Bolt</v>
+        <v>Mud Shot</v>
       </c>
       <c r="B43" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="C43" t="str">
-        <v>Water</v>
+        <v>Sand</v>
       </c>
       <c r="D43" t="str">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E43" t="str">
         <v>2</v>
       </c>
       <c r="F43" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G43" t="str">
-        <v>Crackling bolts that drench what they strike</v>
+        <v>Thick sludge launched with surprising force</v>
       </c>
       <c r="H43" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="I43" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="J43" t="str">
-        <v>multi_hit</v>
+        <v>shield</v>
       </c>
       <c r="K43" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="L43" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="M43" t="str">
         <v/>
       </c>
       <c r="N43" t="str">
-        <v>enemy</v>
+        <v>self</v>
       </c>
       <c r="O43" t="str">
         <v>soak</v>
@@ -4091,54 +3932,54 @@
         <v/>
       </c>
       <c r="AA43" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="AB43" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Ice Bolt</v>
+        <v>Tornado</v>
       </c>
       <c r="B44" t="str">
-        <v>Lightning</v>
+        <v>Air</v>
       </c>
       <c r="C44" t="str">
-        <v>Ice</v>
+        <v>Air</v>
       </c>
       <c r="D44" t="str">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="E44" t="str">
         <v>2</v>
       </c>
       <c r="F44" t="str">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G44" t="str">
-        <v>A frozen shard launched like a thunderbolt</v>
+        <v>A perfect spiral of destruction and fury</v>
       </c>
       <c r="H44" t="str">
-        <v>Lightning</v>
+        <v>Air</v>
       </c>
       <c r="I44" t="str">
-        <v>Ice</v>
+        <v>Air</v>
       </c>
       <c r="J44" t="str">
-        <v>multi_hit</v>
+        <v/>
       </c>
       <c r="K44" t="str">
         <v/>
       </c>
       <c r="L44" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="M44" t="str">
         <v/>
       </c>
       <c r="N44" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="O44" t="str">
         <v/>
@@ -4177,54 +4018,54 @@
         <v/>
       </c>
       <c r="AA44" t="str">
-        <v>Lightning</v>
+        <v>Air</v>
       </c>
       <c r="AB44" t="str">
-        <v>Ice</v>
+        <v>Air</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Thunder</v>
+        <v>Hailstorm</v>
       </c>
       <c r="B45" t="str">
-        <v>Lightning</v>
+        <v>Air</v>
       </c>
       <c r="C45" t="str">
-        <v>Lightning</v>
+        <v>Ice</v>
       </c>
       <c r="D45" t="str">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="E45" t="str">
         <v>2</v>
       </c>
       <c r="F45" t="str">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G45" t="str">
-        <v>Strikes once, twice, three times in a flash</v>
+        <v>Ice pellets rain down in a furious torrent</v>
       </c>
       <c r="H45" t="str">
-        <v>Lightning</v>
+        <v>Air</v>
       </c>
       <c r="I45" t="str">
-        <v>Lightning</v>
+        <v>Ice</v>
       </c>
       <c r="J45" t="str">
-        <v>multi_hit</v>
+        <v/>
       </c>
       <c r="K45" t="str">
         <v/>
       </c>
       <c r="L45" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="M45" t="str">
         <v/>
       </c>
       <c r="N45" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -4263,24 +4104,24 @@
         <v/>
       </c>
       <c r="AA45" t="str">
-        <v>Lightning</v>
+        <v>Air</v>
       </c>
       <c r="AB45" t="str">
-        <v>Lightning</v>
+        <v>Ice</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Mud Shot</v>
+        <v>Pyreball</v>
       </c>
       <c r="B46" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="C46" t="str">
-        <v>Sand</v>
+        <v>Fire</v>
       </c>
       <c r="D46" t="str">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="E46" t="str">
         <v>2</v>
@@ -4289,34 +4130,34 @@
         <v>5</v>
       </c>
       <c r="G46" t="str">
-        <v>Thick sludge launched with surprising force</v>
+        <v>A massive fireball of pure concentrated flame</v>
       </c>
       <c r="H46" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="I46" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="J46" t="str">
-        <v>shield</v>
+        <v>burn</v>
       </c>
       <c r="K46" t="str">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L46" t="str">
         <v/>
       </c>
       <c r="M46" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="N46" t="str">
-        <v>self</v>
+        <v>enemy</v>
       </c>
       <c r="O46" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P46" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q46" t="str">
         <v/>
@@ -4325,7 +4166,7 @@
         <v/>
       </c>
       <c r="S46" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T46" t="str">
         <v/>
@@ -4349,45 +4190,45 @@
         <v/>
       </c>
       <c r="AA46" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="AB46" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Tornado</v>
+        <v>Ice Shield</v>
       </c>
       <c r="B47" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="C47" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
       <c r="D47" t="str">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="E47" t="str">
         <v>2</v>
       </c>
       <c r="F47" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G47" t="str">
-        <v>A perfect spiral of destruction and fury</v>
+        <v>Frozen barrier as solid and cold as bedrock</v>
       </c>
       <c r="H47" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="I47" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
       <c r="J47" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="K47" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="L47" t="str">
         <v/>
@@ -4396,7 +4237,7 @@
         <v/>
       </c>
       <c r="N47" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O47" t="str">
         <v/>
@@ -4435,36 +4276,36 @@
         <v/>
       </c>
       <c r="AA47" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="AB47" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Hailstorm</v>
+        <v>Glacier</v>
       </c>
       <c r="B48" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="C48" t="str">
         <v>Ice</v>
       </c>
       <c r="D48" t="str">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="E48" t="str">
         <v>2</v>
       </c>
       <c r="F48" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G48" t="str">
-        <v>Ice pellets rain down in a furious torrent</v>
+        <v>Ancient ice creaks and grinds slowly forward</v>
       </c>
       <c r="H48" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="I48" t="str">
         <v>Ice</v>
@@ -4521,7 +4362,7 @@
         <v/>
       </c>
       <c r="AA48" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="AB48" t="str">
         <v>Ice</v>
@@ -4529,13 +4370,13 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Pyreball</v>
+        <v>Earthquake</v>
       </c>
       <c r="B49" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="C49" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D49" t="str">
         <v>126</v>
@@ -4547,28 +4388,28 @@
         <v>5</v>
       </c>
       <c r="G49" t="str">
-        <v>A massive fireball of pure concentrated flame</v>
+        <v>The ground splits open beneath your foe</v>
       </c>
       <c r="H49" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="I49" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="J49" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="K49" t="str">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="L49" t="str">
         <v/>
       </c>
       <c r="M49" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="N49" t="str">
-        <v>enemy</v>
+        <v>self</v>
       </c>
       <c r="O49" t="str">
         <v/>
@@ -4607,273 +4448,15 @@
         <v/>
       </c>
       <c r="AA49" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="AB49" t="str">
-        <v>Fire</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <v>Ice Shield</v>
-      </c>
-      <c r="B50" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="C50" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="D50" t="str">
-        <v>58</v>
-      </c>
-      <c r="E50" t="str">
-        <v>2</v>
-      </c>
-      <c r="F50" t="str">
-        <v>3</v>
-      </c>
-      <c r="G50" t="str">
-        <v>Frozen barrier as solid and cold as bedrock</v>
-      </c>
-      <c r="H50" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="I50" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="J50" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K50" t="str">
-        <v>8</v>
-      </c>
-      <c r="L50" t="str">
-        <v/>
-      </c>
-      <c r="M50" t="str">
-        <v/>
-      </c>
-      <c r="N50" t="str">
-        <v>self</v>
-      </c>
-      <c r="O50" t="str">
-        <v/>
-      </c>
-      <c r="P50" t="str">
-        <v/>
-      </c>
-      <c r="Q50" t="str">
-        <v/>
-      </c>
-      <c r="R50" t="str">
-        <v/>
-      </c>
-      <c r="S50" t="str">
-        <v/>
-      </c>
-      <c r="T50" t="str">
-        <v/>
-      </c>
-      <c r="U50" t="str">
-        <v/>
-      </c>
-      <c r="V50" t="str">
-        <v/>
-      </c>
-      <c r="W50" t="str">
-        <v/>
-      </c>
-      <c r="X50" t="str">
-        <v/>
-      </c>
-      <c r="Y50" t="str">
-        <v/>
-      </c>
-      <c r="Z50" t="str">
-        <v/>
-      </c>
-      <c r="AA50" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="AB50" t="str">
-        <v>Earth</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>Glacier</v>
-      </c>
-      <c r="B51" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="C51" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="D51" t="str">
-        <v>126</v>
-      </c>
-      <c r="E51" t="str">
-        <v>2</v>
-      </c>
-      <c r="F51" t="str">
-        <v>5</v>
-      </c>
-      <c r="G51" t="str">
-        <v>Ancient ice creaks and grinds slowly forward</v>
-      </c>
-      <c r="H51" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="I51" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="J51" t="str">
-        <v/>
-      </c>
-      <c r="K51" t="str">
-        <v/>
-      </c>
-      <c r="L51" t="str">
-        <v/>
-      </c>
-      <c r="M51" t="str">
-        <v/>
-      </c>
-      <c r="N51" t="str">
-        <v/>
-      </c>
-      <c r="O51" t="str">
-        <v/>
-      </c>
-      <c r="P51" t="str">
-        <v/>
-      </c>
-      <c r="Q51" t="str">
-        <v/>
-      </c>
-      <c r="R51" t="str">
-        <v/>
-      </c>
-      <c r="S51" t="str">
-        <v/>
-      </c>
-      <c r="T51" t="str">
-        <v/>
-      </c>
-      <c r="U51" t="str">
-        <v/>
-      </c>
-      <c r="V51" t="str">
-        <v/>
-      </c>
-      <c r="W51" t="str">
-        <v/>
-      </c>
-      <c r="X51" t="str">
-        <v/>
-      </c>
-      <c r="Y51" t="str">
-        <v/>
-      </c>
-      <c r="Z51" t="str">
-        <v/>
-      </c>
-      <c r="AA51" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="AB51" t="str">
-        <v>Ice</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <v>Earthquake</v>
-      </c>
-      <c r="B52" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="C52" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="D52" t="str">
-        <v>126</v>
-      </c>
-      <c r="E52" t="str">
-        <v>2</v>
-      </c>
-      <c r="F52" t="str">
-        <v>5</v>
-      </c>
-      <c r="G52" t="str">
-        <v>The ground splits open beneath your foe</v>
-      </c>
-      <c r="H52" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="I52" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="J52" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K52" t="str">
-        <v>16</v>
-      </c>
-      <c r="L52" t="str">
-        <v/>
-      </c>
-      <c r="M52" t="str">
-        <v/>
-      </c>
-      <c r="N52" t="str">
-        <v>self</v>
-      </c>
-      <c r="O52" t="str">
-        <v/>
-      </c>
-      <c r="P52" t="str">
-        <v/>
-      </c>
-      <c r="Q52" t="str">
-        <v/>
-      </c>
-      <c r="R52" t="str">
-        <v/>
-      </c>
-      <c r="S52" t="str">
-        <v/>
-      </c>
-      <c r="T52" t="str">
-        <v/>
-      </c>
-      <c r="U52" t="str">
-        <v/>
-      </c>
-      <c r="V52" t="str">
-        <v/>
-      </c>
-      <c r="W52" t="str">
-        <v/>
-      </c>
-      <c r="X52" t="str">
-        <v/>
-      </c>
-      <c r="Y52" t="str">
-        <v/>
-      </c>
-      <c r="Z52" t="str">
-        <v/>
-      </c>
-      <c r="AA52" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="AB52" t="str">
         <v>Earth</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB52"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB49"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (8d6f564) Remove StartMenuModal, use reward modal as the generic version
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB49"/>
+  <dimension ref="A1:AB48"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -576,16 +576,16 @@
         <v>Fire</v>
       </c>
       <c r="B3" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="C3" t="str">
-        <v>Air</v>
+        <v>Lightning</v>
       </c>
       <c r="D3" t="str">
         <v>10</v>
       </c>
       <c r="E3" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="str">
         <v>1</v>
@@ -654,18 +654,18 @@
         <v/>
       </c>
       <c r="AB3" t="str">
-        <v/>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="B4" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C4" t="str">
-        <v>Lightning</v>
+        <v>Sand</v>
       </c>
       <c r="D4" t="str">
         <v>10</v>
@@ -677,19 +677,19 @@
         <v>1</v>
       </c>
       <c r="G4" t="str">
-        <v>A bright flame burning hot</v>
+        <v>It's a rock</v>
       </c>
       <c r="H4" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="I4" t="str">
         <v/>
       </c>
       <c r="J4" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>5</v>
       </c>
       <c r="L4" t="str">
         <v/>
@@ -740,21 +740,21 @@
         <v/>
       </c>
       <c r="AB4" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Earth</v>
+        <v>Lightning</v>
       </c>
       <c r="B5" t="str">
-        <v>Sand</v>
+        <v>Air</v>
       </c>
       <c r="C5" t="str">
-        <v>Sand</v>
+        <v>Fire</v>
       </c>
       <c r="D5" t="str">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E5" t="str">
         <v>0</v>
@@ -763,22 +763,22 @@
         <v>1</v>
       </c>
       <c r="G5" t="str">
-        <v>It's a rock</v>
+        <v>Charged spark that strikes instantly</v>
       </c>
       <c r="H5" t="str">
-        <v>Earth</v>
+        <v>Lightning</v>
       </c>
       <c r="I5" t="str">
         <v/>
       </c>
       <c r="J5" t="str">
-        <v>shield</v>
+        <v>multihit</v>
       </c>
       <c r="K5" t="str">
-        <v>5</v>
+        <v/>
       </c>
       <c r="L5" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="M5" t="str">
         <v/>
@@ -831,40 +831,40 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Plasma</v>
+      </c>
+      <c r="B6" t="str">
         <v>Lightning</v>
       </c>
-      <c r="B6" t="str">
+      <c r="C6" t="str">
         <v>Air</v>
       </c>
-      <c r="C6" t="str">
-        <v>Fire</v>
-      </c>
       <c r="D6" t="str">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="str">
         <v>1</v>
       </c>
       <c r="G6" t="str">
-        <v>Charged spark that strikes instantly</v>
+        <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H6" t="str">
-        <v>Lightning</v>
+        <v>Plasma</v>
       </c>
       <c r="I6" t="str">
         <v/>
       </c>
       <c r="J6" t="str">
-        <v>multihit</v>
+        <v/>
       </c>
       <c r="K6" t="str">
         <v/>
       </c>
       <c r="L6" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="M6" t="str">
         <v/>
@@ -923,7 +923,7 @@
         <v>Lightning</v>
       </c>
       <c r="C7" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
       <c r="D7" t="str">
         <v>1</v>
@@ -1009,7 +1009,7 @@
         <v>Lightning</v>
       </c>
       <c r="C8" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="D8" t="str">
         <v>1</v>
@@ -1092,10 +1092,10 @@
         <v>Plasma</v>
       </c>
       <c r="B9" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="C9" t="str">
         <v>Lightning</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Fire</v>
       </c>
       <c r="D9" t="str">
         <v>1</v>
@@ -1110,10 +1110,10 @@
         <v>A deep sense of calm overwhelms you</v>
       </c>
       <c r="H9" t="str">
-        <v>Plasma</v>
+        <v>Fire</v>
       </c>
       <c r="I9" t="str">
-        <v/>
+        <v>Lightning</v>
       </c>
       <c r="J9" t="str">
         <v/>
@@ -1175,16 +1175,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Plasma</v>
+        <v>Sand</v>
       </c>
       <c r="B10" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="C10" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="D10" t="str">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E10" t="str">
         <v>1</v>
@@ -1193,13 +1193,13 @@
         <v>1</v>
       </c>
       <c r="G10" t="str">
-        <v>A deep sense of calm overwhelms you</v>
+        <v>Shifting grains dance between your fingertips</v>
       </c>
       <c r="H10" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="I10" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1264,7 +1264,7 @@
         <v>Sand</v>
       </c>
       <c r="B11" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="C11" t="str">
         <v>Earth</v>
@@ -1347,10 +1347,10 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="B12" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="C12" t="str">
         <v>Earth</v>
@@ -1365,10 +1365,10 @@
         <v>1</v>
       </c>
       <c r="G12" t="str">
-        <v>Shifting grains dance between your fingertips</v>
+        <v>Forged from fire and stone, hammered hard</v>
       </c>
       <c r="H12" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="I12" t="str">
         <v/>
@@ -1433,28 +1433,28 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Steel</v>
+        <v>Air</v>
       </c>
       <c r="B13" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C13" t="str">
         <v>Fire</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Earth</v>
       </c>
       <c r="D13" t="str">
         <v>10</v>
       </c>
       <c r="E13" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="str">
         <v>1</v>
       </c>
       <c r="G13" t="str">
-        <v>Forged from fire and stone, hammered hard</v>
+        <v>A cool rush of wind drifts past your face</v>
       </c>
       <c r="H13" t="str">
-        <v>Steel</v>
+        <v>Air</v>
       </c>
       <c r="I13" t="str">
         <v/>
@@ -1519,46 +1519,46 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Air</v>
+        <v>Leaf</v>
       </c>
       <c r="B14" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="C14" t="str">
         <v>Water</v>
       </c>
-      <c r="C14" t="str">
-        <v>Fire</v>
-      </c>
       <c r="D14" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E14" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" t="str">
         <v>1</v>
       </c>
       <c r="G14" t="str">
-        <v>A cool rush of wind drifts past your face</v>
+        <v>Drops of dew glistle atop</v>
       </c>
       <c r="H14" t="str">
-        <v>Air</v>
+        <v>Earth</v>
       </c>
       <c r="I14" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="J14" t="str">
-        <v/>
+        <v>energize</v>
       </c>
       <c r="K14" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="L14" t="str">
         <v/>
       </c>
       <c r="M14" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="N14" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O14" t="str">
         <v/>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
       <c r="AA14" t="str">
-        <v/>
+        <v>Leaf</v>
       </c>
       <c r="AB14" t="str">
         <v/>
@@ -1605,46 +1605,46 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Leaf</v>
+        <v>Ice</v>
       </c>
       <c r="B15" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="C15" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="D15" t="str">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E15" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" t="str">
         <v>1</v>
       </c>
       <c r="G15" t="str">
-        <v>Drops of dew glistle atop</v>
+        <v>A biting chill that settles in your bones</v>
       </c>
       <c r="H15" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
       <c r="I15" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="J15" t="str">
-        <v>energize</v>
+        <v/>
       </c>
       <c r="K15" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="L15" t="str">
         <v/>
       </c>
       <c r="M15" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="N15" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -1683,7 +1683,7 @@
         <v/>
       </c>
       <c r="AA15" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
       <c r="AB15" t="str">
         <v/>
@@ -1691,16 +1691,16 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Ice</v>
+        <v>Glass</v>
       </c>
       <c r="B16" t="str">
-        <v>Water</v>
+        <v>Sand</v>
       </c>
       <c r="C16" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="D16" t="str">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E16" t="str">
         <v>1</v>
@@ -1709,10 +1709,10 @@
         <v>1</v>
       </c>
       <c r="G16" t="str">
-        <v>A biting chill that settles in your bones</v>
+        <v>Smooth and brittle, it catches the light</v>
       </c>
       <c r="H16" t="str">
-        <v>Ice</v>
+        <v>Glass</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -1783,7 +1783,7 @@
         <v>Sand</v>
       </c>
       <c r="C17" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="D17" t="str">
         <v>12</v>
@@ -1863,28 +1863,28 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Glass</v>
+        <v>Dark Matter</v>
       </c>
       <c r="B18" t="str">
-        <v>Sand</v>
+        <v>Unstable Element</v>
       </c>
       <c r="C18" t="str">
-        <v>Lightning</v>
+        <v>Unstable Element</v>
       </c>
       <c r="D18" t="str">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E18" t="str">
         <v>1</v>
       </c>
       <c r="F18" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18" t="str">
-        <v>Smooth and brittle, it catches the light</v>
+        <v>A quiet humming radiates from inside</v>
       </c>
       <c r="H18" t="str">
-        <v>Glass</v>
+        <v>Void</v>
       </c>
       <c r="I18" t="str">
         <v/>
@@ -1949,37 +1949,37 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Dark Matter</v>
+        <v>Worble</v>
       </c>
       <c r="B19" t="str">
-        <v>Unstable Element</v>
+        <v>Water</v>
       </c>
       <c r="C19" t="str">
-        <v>Unstable Element</v>
+        <v>Water</v>
       </c>
       <c r="D19" t="str">
-        <v>18</v>
+        <v>126</v>
       </c>
       <c r="E19" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F19" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G19" t="str">
-        <v>A quiet humming radiates from inside</v>
+        <v>The tide is high today my friend</v>
       </c>
       <c r="H19" t="str">
-        <v>Void</v>
+        <v>Water</v>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="J19" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="K19" t="str">
-        <v/>
+        <v>4</v>
       </c>
       <c r="L19" t="str">
         <v/>
@@ -1988,7 +1988,7 @@
         <v/>
       </c>
       <c r="N19" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="O19" t="str">
         <v/>
@@ -2027,24 +2027,24 @@
         <v/>
       </c>
       <c r="AA19" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="AB19" t="str">
-        <v/>
+        <v>Water</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Worble</v>
+        <v>Blaze</v>
       </c>
       <c r="B20" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="C20" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="D20" t="str">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="E20" t="str">
         <v>2</v>
@@ -2053,44 +2053,35 @@
         <v>5</v>
       </c>
       <c r="G20" t="str">
-        <v>The tide is high today my friend</v>
+        <v>Forest floor erupts in scorching flame</v>
       </c>
       <c r="H20" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="I20" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="J20" t="str">
-        <v>soak</v>
+        <v>burn</v>
       </c>
       <c r="K20" t="str">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L20" t="str">
         <v/>
       </c>
       <c r="M20" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="N20" t="str">
         <v>enemy</v>
       </c>
-      <c r="O20" t="str">
-        <v/>
-      </c>
-      <c r="P20" t="str">
-        <v/>
-      </c>
       <c r="Q20" t="str">
         <v/>
       </c>
       <c r="R20" t="str">
         <v/>
       </c>
-      <c r="S20" t="str">
-        <v/>
-      </c>
       <c r="T20" t="str">
         <v/>
       </c>
@@ -2113,21 +2104,21 @@
         <v/>
       </c>
       <c r="AA20" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="AB20" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Blaze</v>
+        <v>Regen</v>
       </c>
       <c r="B21" t="str">
         <v>Leaf</v>
       </c>
       <c r="C21" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="D21" t="str">
         <v>109</v>
@@ -2139,28 +2130,28 @@
         <v>5</v>
       </c>
       <c r="G21" t="str">
-        <v>Forest floor erupts in scorching flame</v>
+        <v>Living vines wrap wounds in cool water</v>
       </c>
       <c r="H21" t="str">
         <v>Leaf</v>
       </c>
       <c r="I21" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="J21" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="K21" t="str">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L21" t="str">
         <v/>
       </c>
       <c r="M21" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N21" t="str">
-        <v>enemy</v>
+        <v>self</v>
       </c>
       <c r="Q21" t="str">
         <v/>
@@ -2190,7 +2181,7 @@
         <v/>
       </c>
       <c r="AA21" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="AB21" t="str">
         <v>Leaf</v>
@@ -2198,13 +2189,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Regen</v>
+        <v>Thorns</v>
       </c>
       <c r="B22" t="str">
         <v>Leaf</v>
       </c>
       <c r="C22" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="D22" t="str">
         <v>109</v>
@@ -2216,7 +2207,7 @@
         <v>5</v>
       </c>
       <c r="G22" t="str">
-        <v>Living vines wrap wounds in cool water</v>
+        <v>Spiked vines protect you</v>
       </c>
       <c r="H22" t="str">
         <v>Leaf</v>
@@ -2267,7 +2258,7 @@
         <v/>
       </c>
       <c r="AA22" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="AB22" t="str">
         <v>Leaf</v>
@@ -2275,13 +2266,13 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Thorns</v>
+        <v>Tornado</v>
       </c>
       <c r="B23" t="str">
         <v>Leaf</v>
       </c>
       <c r="C23" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="D23" t="str">
         <v>109</v>
@@ -2290,16 +2281,16 @@
         <v>2</v>
       </c>
       <c r="F23" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G23" t="str">
-        <v>Spiked vines protect you</v>
+        <v>Wind whips and slashes about</v>
       </c>
       <c r="H23" t="str">
         <v>Leaf</v>
       </c>
       <c r="I23" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="J23" t="str">
         <v>shield</v>
@@ -2316,12 +2307,21 @@
       <c r="N23" t="str">
         <v>self</v>
       </c>
+      <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
       <c r="Q23" t="str">
         <v/>
       </c>
       <c r="R23" t="str">
         <v/>
       </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
       <c r="T23" t="str">
         <v/>
       </c>
@@ -2344,7 +2344,7 @@
         <v/>
       </c>
       <c r="AA23" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="AB23" t="str">
         <v>Leaf</v>
@@ -2352,13 +2352,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Tornado</v>
+        <v>Blizzard</v>
       </c>
       <c r="B24" t="str">
         <v>Leaf</v>
       </c>
       <c r="C24" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D24" t="str">
         <v>109</v>
@@ -2367,16 +2367,16 @@
         <v>2</v>
       </c>
       <c r="F24" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G24" t="str">
-        <v>Wind whips and slashes about</v>
+        <v>Snow flurries block your vision</v>
       </c>
       <c r="H24" t="str">
         <v>Leaf</v>
       </c>
       <c r="I24" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="J24" t="str">
         <v>shield</v>
@@ -2430,7 +2430,7 @@
         <v/>
       </c>
       <c r="AA24" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="AB24" t="str">
         <v>Leaf</v>
@@ -2438,31 +2438,31 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Blizzard</v>
+        <v>Leaf Blade</v>
       </c>
       <c r="B25" t="str">
         <v>Leaf</v>
       </c>
       <c r="C25" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="D25" t="str">
-        <v>109</v>
+        <v>159</v>
       </c>
       <c r="E25" t="str">
         <v>2</v>
       </c>
       <c r="F25" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G25" t="str">
-        <v>Snow flurries block your vision</v>
+        <v>A razor edge honed from living wood</v>
       </c>
       <c r="H25" t="str">
         <v>Leaf</v>
       </c>
       <c r="I25" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="J25" t="str">
         <v>shield</v>
@@ -2479,21 +2479,12 @@
       <c r="N25" t="str">
         <v>self</v>
       </c>
-      <c r="O25" t="str">
-        <v/>
-      </c>
-      <c r="P25" t="str">
-        <v/>
-      </c>
       <c r="Q25" t="str">
         <v/>
       </c>
       <c r="R25" t="str">
         <v/>
       </c>
-      <c r="S25" t="str">
-        <v/>
-      </c>
       <c r="T25" t="str">
         <v/>
       </c>
@@ -2516,7 +2507,7 @@
         <v/>
       </c>
       <c r="AA25" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="AB25" t="str">
         <v>Leaf</v>
@@ -2524,13 +2515,13 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Leaf Blade</v>
+        <v>Needle Storm</v>
       </c>
       <c r="B26" t="str">
         <v>Leaf</v>
       </c>
       <c r="C26" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="D26" t="str">
         <v>159</v>
@@ -2539,16 +2530,16 @@
         <v>2</v>
       </c>
       <c r="F26" t="str">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G26" t="str">
-        <v>A razor edge honed from living wood</v>
+        <v>Tiny needles prick from every angle</v>
       </c>
       <c r="H26" t="str">
         <v>Leaf</v>
       </c>
       <c r="I26" t="str">
-        <v>Steel</v>
+        <v>Earth</v>
       </c>
       <c r="J26" t="str">
         <v>shield</v>
@@ -2601,37 +2592,37 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Needle Storm</v>
+        <v>Photosynthesis</v>
       </c>
       <c r="B27" t="str">
         <v>Leaf</v>
       </c>
       <c r="C27" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="D27" t="str">
-        <v>159</v>
+        <v>210</v>
       </c>
       <c r="E27" t="str">
         <v>2</v>
       </c>
       <c r="F27" t="str">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G27" t="str">
-        <v>Tiny needles prick from every angle</v>
+        <v>Nature feeds itself to grow ever stronger</v>
       </c>
       <c r="H27" t="str">
         <v>Leaf</v>
       </c>
       <c r="I27" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="J27" t="str">
-        <v>shield</v>
+        <v>soak</v>
       </c>
       <c r="K27" t="str">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L27" t="str">
         <v/>
@@ -2640,7 +2631,7 @@
         <v/>
       </c>
       <c r="N27" t="str">
-        <v>self</v>
+        <v>enemy</v>
       </c>
       <c r="Q27" t="str">
         <v/>
@@ -2678,37 +2669,37 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Photosynthesis</v>
+        <v>Desert Blade</v>
       </c>
       <c r="B28" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C28" t="str">
-        <v>Leaf</v>
+        <v>Steel</v>
       </c>
       <c r="D28" t="str">
-        <v>210</v>
+        <v>159</v>
       </c>
       <c r="E28" t="str">
         <v>2</v>
       </c>
       <c r="F28" t="str">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G28" t="str">
-        <v>Nature feeds itself to grow ever stronger</v>
+        <v>Sand-forged steel scorched by the desert sun</v>
       </c>
       <c r="H28" t="str">
-        <v>Leaf</v>
+        <v>Earth</v>
       </c>
       <c r="I28" t="str">
-        <v>Water</v>
+        <v>Steel</v>
       </c>
       <c r="J28" t="str">
-        <v>soak</v>
+        <v>shield</v>
       </c>
       <c r="K28" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="L28" t="str">
         <v/>
@@ -2717,7 +2708,7 @@
         <v/>
       </c>
       <c r="N28" t="str">
-        <v>enemy</v>
+        <v>self</v>
       </c>
       <c r="Q28" t="str">
         <v/>
@@ -2750,36 +2741,36 @@
         <v>Earth</v>
       </c>
       <c r="AB28" t="str">
-        <v>Leaf</v>
+        <v>Fire</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Desert Blade</v>
+        <v>Sand Shield</v>
       </c>
       <c r="B29" t="str">
         <v>Sand</v>
       </c>
       <c r="C29" t="str">
-        <v>Steel</v>
+        <v>Earth</v>
       </c>
       <c r="D29" t="str">
-        <v>159</v>
+        <v>109</v>
       </c>
       <c r="E29" t="str">
         <v>2</v>
       </c>
       <c r="F29" t="str">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G29" t="str">
-        <v>Sand-forged steel scorched by the desert sun</v>
+        <v>Grains pack tight into an earthen wall</v>
       </c>
       <c r="H29" t="str">
         <v>Earth</v>
       </c>
       <c r="I29" t="str">
-        <v>Steel</v>
+        <v/>
       </c>
       <c r="J29" t="str">
         <v>shield</v>
@@ -2796,10 +2787,19 @@
       <c r="N29" t="str">
         <v>self</v>
       </c>
+      <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
       <c r="Q29" t="str">
         <v/>
       </c>
       <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
         <v/>
       </c>
       <c r="T29" t="str">
@@ -2827,18 +2827,18 @@
         <v>Earth</v>
       </c>
       <c r="AB29" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Sand Shield</v>
+        <v>Sandstorm</v>
       </c>
       <c r="B30" t="str">
         <v>Sand</v>
       </c>
       <c r="C30" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="D30" t="str">
         <v>109</v>
@@ -2847,16 +2847,16 @@
         <v>2</v>
       </c>
       <c r="F30" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G30" t="str">
-        <v>Grains pack tight into an earthen wall</v>
+        <v>Blinding grit swirls on howling winds</v>
       </c>
       <c r="H30" t="str">
+        <v>Air</v>
+      </c>
+      <c r="I30" t="str">
         <v>Earth</v>
-      </c>
-      <c r="I30" t="str">
-        <v/>
       </c>
       <c r="J30" t="str">
         <v>shield</v>
@@ -2910,21 +2910,21 @@
         <v/>
       </c>
       <c r="AA30" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AB30" t="str">
         <v>Earth</v>
-      </c>
-      <c r="AB30" t="str">
-        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Sandstorm</v>
+        <v>Iceblast</v>
       </c>
       <c r="B31" t="str">
         <v>Sand</v>
       </c>
       <c r="C31" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D31" t="str">
         <v>109</v>
@@ -2933,13 +2933,13 @@
         <v>2</v>
       </c>
       <c r="F31" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G31" t="str">
-        <v>Blinding grit swirls on howling winds</v>
+        <v>Cold grit bites with a frosty sting</v>
       </c>
       <c r="H31" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="I31" t="str">
         <v>Earth</v>
@@ -2996,7 +2996,7 @@
         <v/>
       </c>
       <c r="AA31" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="AB31" t="str">
         <v>Earth</v>
@@ -3004,13 +3004,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Iceblast</v>
+        <v>Blaze Blade</v>
       </c>
       <c r="B32" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="C32" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="D32" t="str">
         <v>109</v>
@@ -3019,37 +3019,31 @@
         <v>2</v>
       </c>
       <c r="F32" t="str">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G32" t="str">
-        <v>Cold grit bites with a frosty sting</v>
+        <v>A steel blade bathed in white-hot flame</v>
       </c>
       <c r="H32" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="I32" t="str">
-        <v>Earth</v>
+        <v>Steel</v>
       </c>
       <c r="J32" t="str">
-        <v>shield</v>
+        <v>burn</v>
       </c>
       <c r="K32" t="str">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L32" t="str">
         <v/>
       </c>
       <c r="M32" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="N32" t="str">
-        <v>self</v>
-      </c>
-      <c r="O32" t="str">
-        <v/>
-      </c>
-      <c r="P32" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="Q32" t="str">
         <v/>
@@ -3057,9 +3051,6 @@
       <c r="R32" t="str">
         <v/>
       </c>
-      <c r="S32" t="str">
-        <v/>
-      </c>
       <c r="T32" t="str">
         <v/>
       </c>
@@ -3082,7 +3073,7 @@
         <v/>
       </c>
       <c r="AA32" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="AB32" t="str">
         <v>Earth</v>
@@ -3090,13 +3081,13 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Blaze Blade</v>
+        <v>Aqua Blade</v>
       </c>
       <c r="B33" t="str">
         <v>Steel</v>
       </c>
       <c r="C33" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="D33" t="str">
         <v>109</v>
@@ -3108,35 +3099,29 @@
         <v>0</v>
       </c>
       <c r="G33" t="str">
-        <v>A steel blade bathed in white-hot flame</v>
+        <v>Steam rises where cold steel meets the wave</v>
       </c>
       <c r="H33" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="I33" t="str">
         <v>Steel</v>
       </c>
       <c r="J33" t="str">
-        <v>burn</v>
+        <v>soak</v>
       </c>
       <c r="K33" t="str">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="L33" t="str">
         <v/>
       </c>
       <c r="M33" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N33" t="str">
         <v>enemy</v>
       </c>
-      <c r="Q33" t="str">
-        <v/>
-      </c>
-      <c r="R33" t="str">
-        <v/>
-      </c>
       <c r="T33" t="str">
         <v/>
       </c>
@@ -3159,21 +3144,21 @@
         <v/>
       </c>
       <c r="AA33" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AB33" t="str">
         <v>Fire</v>
-      </c>
-      <c r="AB33" t="str">
-        <v>Earth</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Aqua Blade</v>
+        <v>Thunder Blade</v>
       </c>
       <c r="B34" t="str">
         <v>Steel</v>
       </c>
       <c r="C34" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="D34" t="str">
         <v>109</v>
@@ -3185,22 +3170,22 @@
         <v>0</v>
       </c>
       <c r="G34" t="str">
-        <v>Steam rises where cold steel meets the wave</v>
+        <v>Sparks dance across the blades edge</v>
       </c>
       <c r="H34" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="I34" t="str">
         <v>Steel</v>
       </c>
       <c r="J34" t="str">
-        <v>soak</v>
+        <v>multi_hit</v>
       </c>
       <c r="K34" t="str">
+        <v/>
+      </c>
+      <c r="L34" t="str">
         <v>2</v>
-      </c>
-      <c r="L34" t="str">
-        <v/>
       </c>
       <c r="M34" t="str">
         <v/>
@@ -3208,6 +3193,9 @@
       <c r="N34" t="str">
         <v>enemy</v>
       </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
       <c r="T34" t="str">
         <v/>
       </c>
@@ -3230,7 +3218,7 @@
         <v/>
       </c>
       <c r="AA34" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="AB34" t="str">
         <v>Fire</v>
@@ -3238,13 +3226,13 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Thunder Blade</v>
+        <v>Earth Blade</v>
       </c>
       <c r="B35" t="str">
         <v>Steel</v>
       </c>
       <c r="C35" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="D35" t="str">
         <v>109</v>
@@ -3256,31 +3244,28 @@
         <v>0</v>
       </c>
       <c r="G35" t="str">
-        <v>Sparks dance across the blades edge</v>
+        <v>Heavy as bedrock</v>
       </c>
       <c r="H35" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="I35" t="str">
         <v>Steel</v>
       </c>
       <c r="J35" t="str">
-        <v>multi_hit</v>
+        <v>shield</v>
       </c>
       <c r="K35" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="L35" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="M35" t="str">
         <v/>
       </c>
       <c r="N35" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="Q35" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="T35" t="str">
         <v/>
@@ -3304,7 +3289,7 @@
         <v/>
       </c>
       <c r="AA35" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="AB35" t="str">
         <v>Fire</v>
@@ -3312,13 +3297,13 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Earth Blade</v>
+        <v>Air Blade</v>
       </c>
       <c r="B36" t="str">
         <v>Steel</v>
       </c>
       <c r="C36" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="D36" t="str">
         <v>109</v>
@@ -3330,28 +3315,31 @@
         <v>0</v>
       </c>
       <c r="G36" t="str">
-        <v>Heavy as bedrock</v>
+        <v>Cuts the air so fast it ignites</v>
       </c>
       <c r="H36" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="I36" t="str">
         <v>Steel</v>
       </c>
-      <c r="J36" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K36" t="str">
-        <v>8</v>
-      </c>
       <c r="L36" t="str">
         <v/>
       </c>
-      <c r="M36" t="str">
-        <v/>
-      </c>
-      <c r="N36" t="str">
-        <v>self</v>
+      <c r="O36" t="str">
+        <v/>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
+      <c r="R36" t="str">
+        <v/>
+      </c>
+      <c r="S36" t="str">
+        <v/>
       </c>
       <c r="T36" t="str">
         <v/>
@@ -3375,7 +3363,7 @@
         <v/>
       </c>
       <c r="AA36" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="AB36" t="str">
         <v>Fire</v>
@@ -3383,13 +3371,13 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Air Blade</v>
+        <v>Ice Blade</v>
       </c>
       <c r="B37" t="str">
         <v>Steel</v>
       </c>
       <c r="C37" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D37" t="str">
         <v>109</v>
@@ -3401,10 +3389,10 @@
         <v>0</v>
       </c>
       <c r="G37" t="str">
-        <v>Cuts the air so fast it ignites</v>
+        <v>Cold steel that somehow scorches on contact</v>
       </c>
       <c r="H37" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="I37" t="str">
         <v>Steel</v>
@@ -3449,7 +3437,7 @@
         <v/>
       </c>
       <c r="AA37" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="AB37" t="str">
         <v>Fire</v>
@@ -3457,16 +3445,16 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Ice Blade</v>
+        <v>Refined Steel</v>
       </c>
       <c r="B38" t="str">
         <v>Steel</v>
       </c>
       <c r="C38" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="D38" t="str">
-        <v>109</v>
+        <v>210</v>
       </c>
       <c r="E38" t="str">
         <v>2</v>
@@ -3475,10 +3463,10 @@
         <v>0</v>
       </c>
       <c r="G38" t="str">
-        <v>Cold steel that somehow scorches on contact</v>
+        <v>Folded a thousand times until perfect</v>
       </c>
       <c r="H38" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="I38" t="str">
         <v>Steel</v>
@@ -3486,21 +3474,12 @@
       <c r="L38" t="str">
         <v/>
       </c>
-      <c r="O38" t="str">
-        <v/>
-      </c>
-      <c r="P38" t="str">
-        <v/>
-      </c>
       <c r="Q38" t="str">
         <v/>
       </c>
       <c r="R38" t="str">
         <v/>
       </c>
-      <c r="S38" t="str">
-        <v/>
-      </c>
       <c r="T38" t="str">
         <v/>
       </c>
@@ -3523,42 +3502,60 @@
         <v/>
       </c>
       <c r="AA38" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="AB38" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Refined Steel</v>
+        <v>Water Bolt</v>
       </c>
       <c r="B39" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="C39" t="str">
-        <v>Steel</v>
+        <v>Water</v>
       </c>
       <c r="D39" t="str">
-        <v>210</v>
+        <v>58</v>
       </c>
       <c r="E39" t="str">
         <v>2</v>
       </c>
       <c r="F39" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G39" t="str">
-        <v>Folded a thousand times until perfect</v>
+        <v>Crackling bolts that drench what they strike</v>
       </c>
       <c r="H39" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="I39" t="str">
-        <v>Steel</v>
+        <v>Water</v>
+      </c>
+      <c r="J39" t="str">
+        <v>multi_hit</v>
+      </c>
+      <c r="K39" t="str">
+        <v/>
       </c>
       <c r="L39" t="str">
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+      <c r="N39" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="O39" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P39" t="str">
+        <v>2</v>
       </c>
       <c r="Q39" t="str">
         <v/>
@@ -3566,6 +3563,9 @@
       <c r="R39" t="str">
         <v/>
       </c>
+      <c r="S39" t="str">
+        <v>enemy</v>
+      </c>
       <c r="T39" t="str">
         <v/>
       </c>
@@ -3588,21 +3588,21 @@
         <v/>
       </c>
       <c r="AA39" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="AB39" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Water Bolt</v>
+        <v>Ice Bolt</v>
       </c>
       <c r="B40" t="str">
         <v>Lightning</v>
       </c>
       <c r="C40" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="D40" t="str">
         <v>58</v>
@@ -3614,13 +3614,13 @@
         <v>3</v>
       </c>
       <c r="G40" t="str">
-        <v>Crackling bolts that drench what they strike</v>
+        <v>A frozen shard launched like a thunderbolt</v>
       </c>
       <c r="H40" t="str">
         <v>Lightning</v>
       </c>
       <c r="I40" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="J40" t="str">
         <v>multi_hit</v>
@@ -3638,10 +3638,10 @@
         <v>enemy</v>
       </c>
       <c r="O40" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P40" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q40" t="str">
         <v/>
@@ -3650,7 +3650,7 @@
         <v/>
       </c>
       <c r="S40" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T40" t="str">
         <v/>
@@ -3677,36 +3677,36 @@
         <v>Lightning</v>
       </c>
       <c r="AB40" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Ice Bolt</v>
+        <v>Thunder</v>
       </c>
       <c r="B41" t="str">
         <v>Lightning</v>
       </c>
       <c r="C41" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
       <c r="D41" t="str">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="E41" t="str">
         <v>2</v>
       </c>
       <c r="F41" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G41" t="str">
-        <v>A frozen shard launched like a thunderbolt</v>
+        <v>Strikes once, twice, three times in a flash</v>
       </c>
       <c r="H41" t="str">
         <v>Lightning</v>
       </c>
       <c r="I41" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
       <c r="J41" t="str">
         <v>multi_hit</v>
@@ -3715,7 +3715,7 @@
         <v/>
       </c>
       <c r="L41" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M41" t="str">
         <v/>
@@ -3763,21 +3763,21 @@
         <v>Lightning</v>
       </c>
       <c r="AB41" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Thunder</v>
+        <v>Mud Shot</v>
       </c>
       <c r="B42" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="C42" t="str">
-        <v>Lightning</v>
+        <v>Sand</v>
       </c>
       <c r="D42" t="str">
-        <v>126</v>
+        <v>60</v>
       </c>
       <c r="E42" t="str">
         <v>2</v>
@@ -3786,44 +3786,44 @@
         <v>5</v>
       </c>
       <c r="G42" t="str">
-        <v>Strikes once, twice, three times in a flash</v>
+        <v>Thick sludge launched with surprising force</v>
       </c>
       <c r="H42" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="I42" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="J42" t="str">
-        <v>multi_hit</v>
+        <v>shield</v>
       </c>
       <c r="K42" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="L42" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="M42" t="str">
         <v/>
       </c>
       <c r="N42" t="str">
+        <v>self</v>
+      </c>
+      <c r="O42" t="str">
+        <v>soak</v>
+      </c>
+      <c r="P42" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q42" t="str">
+        <v/>
+      </c>
+      <c r="R42" t="str">
+        <v/>
+      </c>
+      <c r="S42" t="str">
         <v>enemy</v>
       </c>
-      <c r="O42" t="str">
-        <v/>
-      </c>
-      <c r="P42" t="str">
-        <v/>
-      </c>
-      <c r="Q42" t="str">
-        <v/>
-      </c>
-      <c r="R42" t="str">
-        <v/>
-      </c>
-      <c r="S42" t="str">
-        <v/>
-      </c>
       <c r="T42" t="str">
         <v/>
       </c>
@@ -3846,45 +3846,45 @@
         <v/>
       </c>
       <c r="AA42" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="AB42" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Mud Shot</v>
+        <v>Tornado</v>
       </c>
       <c r="B43" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="C43" t="str">
-        <v>Sand</v>
+        <v>Air</v>
       </c>
       <c r="D43" t="str">
-        <v>60</v>
+        <v>126</v>
       </c>
       <c r="E43" t="str">
         <v>2</v>
       </c>
       <c r="F43" t="str">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G43" t="str">
-        <v>Thick sludge launched with surprising force</v>
+        <v>A perfect spiral of destruction and fury</v>
       </c>
       <c r="H43" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="I43" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="J43" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="K43" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="L43" t="str">
         <v/>
@@ -3893,13 +3893,13 @@
         <v/>
       </c>
       <c r="N43" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O43" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P43" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q43" t="str">
         <v/>
@@ -3908,7 +3908,7 @@
         <v/>
       </c>
       <c r="S43" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T43" t="str">
         <v/>
@@ -3932,39 +3932,39 @@
         <v/>
       </c>
       <c r="AA43" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="AB43" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Tornado</v>
+        <v>Hailstorm</v>
       </c>
       <c r="B44" t="str">
         <v>Air</v>
       </c>
       <c r="C44" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D44" t="str">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="E44" t="str">
         <v>2</v>
       </c>
       <c r="F44" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G44" t="str">
-        <v>A perfect spiral of destruction and fury</v>
+        <v>Ice pellets rain down in a furious torrent</v>
       </c>
       <c r="H44" t="str">
         <v>Air</v>
       </c>
       <c r="I44" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="J44" t="str">
         <v/>
@@ -4021,51 +4021,51 @@
         <v>Air</v>
       </c>
       <c r="AB44" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Hailstorm</v>
+        <v>Pyreball</v>
       </c>
       <c r="B45" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="C45" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="D45" t="str">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="E45" t="str">
         <v>2</v>
       </c>
       <c r="F45" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G45" t="str">
-        <v>Ice pellets rain down in a furious torrent</v>
+        <v>A massive fireball of pure concentrated flame</v>
       </c>
       <c r="H45" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="I45" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="J45" t="str">
-        <v/>
+        <v>burn</v>
       </c>
       <c r="K45" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="L45" t="str">
         <v/>
       </c>
       <c r="M45" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="N45" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -4104,54 +4104,54 @@
         <v/>
       </c>
       <c r="AA45" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="AB45" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Pyreball</v>
+        <v>Ice Shield</v>
       </c>
       <c r="B46" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="C46" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D46" t="str">
-        <v>126</v>
+        <v>58</v>
       </c>
       <c r="E46" t="str">
         <v>2</v>
       </c>
       <c r="F46" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G46" t="str">
-        <v>A massive fireball of pure concentrated flame</v>
+        <v>Frozen barrier as solid and cold as bedrock</v>
       </c>
       <c r="H46" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="I46" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="J46" t="str">
-        <v>burn</v>
+        <v>shield</v>
       </c>
       <c r="K46" t="str">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="L46" t="str">
         <v/>
       </c>
       <c r="M46" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="N46" t="str">
-        <v>enemy</v>
+        <v>self</v>
       </c>
       <c r="O46" t="str">
         <v/>
@@ -4190,45 +4190,45 @@
         <v/>
       </c>
       <c r="AA46" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="AB46" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Ice Shield</v>
+        <v>Glacier</v>
       </c>
       <c r="B47" t="str">
         <v>Ice</v>
       </c>
       <c r="C47" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
       <c r="D47" t="str">
-        <v>58</v>
+        <v>126</v>
       </c>
       <c r="E47" t="str">
         <v>2</v>
       </c>
       <c r="F47" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G47" t="str">
-        <v>Frozen barrier as solid and cold as bedrock</v>
+        <v>Ancient ice creaks and grinds slowly forward</v>
       </c>
       <c r="H47" t="str">
         <v>Ice</v>
       </c>
       <c r="I47" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
       <c r="J47" t="str">
-        <v>shield</v>
+        <v/>
       </c>
       <c r="K47" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="L47" t="str">
         <v/>
@@ -4237,7 +4237,7 @@
         <v/>
       </c>
       <c r="N47" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O47" t="str">
         <v/>
@@ -4279,18 +4279,18 @@
         <v>Ice</v>
       </c>
       <c r="AB47" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Glacier</v>
+        <v>Earthquake</v>
       </c>
       <c r="B48" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="C48" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="D48" t="str">
         <v>126</v>
@@ -4302,19 +4302,19 @@
         <v>5</v>
       </c>
       <c r="G48" t="str">
-        <v>Ancient ice creaks and grinds slowly forward</v>
+        <v>The ground splits open beneath your foe</v>
       </c>
       <c r="H48" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="I48" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="J48" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="K48" t="str">
-        <v/>
+        <v>16</v>
       </c>
       <c r="L48" t="str">
         <v/>
@@ -4323,7 +4323,7 @@
         <v/>
       </c>
       <c r="N48" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="O48" t="str">
         <v/>
@@ -4362,101 +4362,15 @@
         <v/>
       </c>
       <c r="AA48" t="str">
-        <v>Ice</v>
+        <v>Earth</v>
       </c>
       <c r="AB48" t="str">
-        <v>Ice</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>Earthquake</v>
-      </c>
-      <c r="B49" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="C49" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="D49" t="str">
-        <v>126</v>
-      </c>
-      <c r="E49" t="str">
-        <v>2</v>
-      </c>
-      <c r="F49" t="str">
-        <v>5</v>
-      </c>
-      <c r="G49" t="str">
-        <v>The ground splits open beneath your foe</v>
-      </c>
-      <c r="H49" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="I49" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="J49" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K49" t="str">
-        <v>16</v>
-      </c>
-      <c r="L49" t="str">
-        <v/>
-      </c>
-      <c r="M49" t="str">
-        <v/>
-      </c>
-      <c r="N49" t="str">
-        <v>self</v>
-      </c>
-      <c r="O49" t="str">
-        <v/>
-      </c>
-      <c r="P49" t="str">
-        <v/>
-      </c>
-      <c r="Q49" t="str">
-        <v/>
-      </c>
-      <c r="R49" t="str">
-        <v/>
-      </c>
-      <c r="S49" t="str">
-        <v/>
-      </c>
-      <c r="T49" t="str">
-        <v/>
-      </c>
-      <c r="U49" t="str">
-        <v/>
-      </c>
-      <c r="V49" t="str">
-        <v/>
-      </c>
-      <c r="W49" t="str">
-        <v/>
-      </c>
-      <c r="X49" t="str">
-        <v/>
-      </c>
-      <c r="Y49" t="str">
-        <v/>
-      </c>
-      <c r="Z49" t="str">
-        <v/>
-      </c>
-      <c r="AA49" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="AB49" t="str">
         <v>Earth</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AB48"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (1281a14) Change potions meter to remain across battles. QoL changes.
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -514,30 +514,15 @@
         <v/>
       </c>
       <c r="J2" t="str">
-        <v>heal</v>
+        <v>soak</v>
       </c>
       <c r="K2" t="str">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L2" t="str">
         <v/>
       </c>
       <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
-        <v>self</v>
-      </c>
-      <c r="O2" t="str">
-        <v>soak</v>
-      </c>
-      <c r="P2" t="str">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2" t="str">
         <v>3</v>
       </c>
       <c r="S2" t="str">

</xml_diff>

<commit_message>
Build: (5668b9f) elemental map upgrades
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -570,7 +570,7 @@
         <v>10</v>
       </c>
       <c r="E3" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="str">
         <v>1</v>
@@ -742,7 +742,7 @@
         <v>7</v>
       </c>
       <c r="E5" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" t="str">
         <v>1</v>
@@ -828,7 +828,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="str">
         <v>1</v>
@@ -914,7 +914,7 @@
         <v>1</v>
       </c>
       <c r="E7" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F7" t="str">
         <v>1</v>
@@ -1000,7 +1000,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F8" t="str">
         <v>1</v>
@@ -1086,7 +1086,7 @@
         <v>1</v>
       </c>
       <c r="E9" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" t="str">
         <v>1</v>
@@ -1430,7 +1430,7 @@
         <v>10</v>
       </c>
       <c r="E13" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" t="str">
         <v>1</v>
@@ -1688,7 +1688,7 @@
         <v>12</v>
       </c>
       <c r="E16" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16" t="str">
         <v>1</v>
@@ -1774,7 +1774,7 @@
         <v>12</v>
       </c>
       <c r="E17" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" t="str">
         <v>1</v>

</xml_diff>

<commit_message>
Build: (f69e628) Balance element levels + add additional icons
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AB48"/>
+  <dimension ref="A1:AC46"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,78 +410,81 @@
         <v>Element 2</v>
       </c>
       <c r="D1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="E1" t="str">
         <v>Damage</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Level</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Energy</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>description</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Type1</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Type2</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Effect 1 Kind</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Effect 1 Amount</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Effect 1 Hits</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Effect 1 Duration</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>Effect 1 Target</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Effect 2 Kind</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Effect 2 Amount</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="R1" t="str">
         <v>Effect 2 Hits</v>
       </c>
-      <c r="R1" t="str">
+      <c r="S1" t="str">
         <v>Effect 2 Duration</v>
       </c>
-      <c r="S1" t="str">
+      <c r="T1" t="str">
         <v>Effect 2 Target</v>
       </c>
-      <c r="T1" t="str">
+      <c r="U1" t="str">
         <v>Effect 3 Kind</v>
       </c>
-      <c r="U1" t="str">
+      <c r="V1" t="str">
         <v>Effect 3 Amount</v>
       </c>
-      <c r="V1" t="str">
+      <c r="W1" t="str">
         <v>Effect 3 Hits</v>
       </c>
-      <c r="W1" t="str">
+      <c r="X1" t="str">
         <v>Effect 3 Duration</v>
       </c>
-      <c r="X1" t="str">
+      <c r="Y1" t="str">
         <v>Effect 3 Target</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="Z1" t="str">
         <v>__EMPTY</v>
       </c>
-      <c r="Z1" t="str">
+      <c r="AA1" t="str">
         <v>__EMPTY_1</v>
       </c>
-      <c r="AA1" t="str">
+      <c r="AB1" t="str">
         <v>Type 1</v>
       </c>
-      <c r="AB1" t="str">
+      <c r="AC1" t="str">
         <v>Type 2</v>
       </c>
     </row>
@@ -496,38 +499,38 @@
         <v>Fire</v>
       </c>
       <c r="D2" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E2" t="str">
         <v>8</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>0</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>1</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>A gift from the sky goddess</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>Water</v>
       </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
       <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
         <v>soak</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>1</v>
       </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
       <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
         <v>3</v>
       </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
       <c r="T2" t="str">
         <v/>
       </c>
@@ -553,6 +556,9 @@
         <v/>
       </c>
       <c r="AB2" t="str">
+        <v/>
+      </c>
+      <c r="AC2" t="str">
         <v/>
       </c>
     </row>
@@ -567,38 +573,38 @@
         <v>Lightning</v>
       </c>
       <c r="D3" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E3" t="str">
         <v>10</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>0</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>1</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>A bright flame burning hot</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>Fire</v>
       </c>
-      <c r="I3" t="str">
-        <v/>
-      </c>
       <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
         <v>burn</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>1</v>
       </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
       <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
         <v>3</v>
       </c>
-      <c r="N3" t="str">
-        <v/>
-      </c>
       <c r="O3" t="str">
         <v/>
       </c>
@@ -639,6 +645,9 @@
         <v/>
       </c>
       <c r="AB3" t="str">
+        <v/>
+      </c>
+      <c r="AC3" t="str">
         <v>Leaf</v>
       </c>
     </row>
@@ -653,32 +662,32 @@
         <v>Sand</v>
       </c>
       <c r="D4" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E4" t="str">
         <v>10</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>0</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G4" t="str">
         <v>1</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>It's a rock</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>Earth</v>
       </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
       <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
         <v>shield</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>5</v>
       </c>
-      <c r="L4" t="str">
-        <v/>
-      </c>
       <c r="M4" t="str">
         <v/>
       </c>
@@ -725,6 +734,9 @@
         <v/>
       </c>
       <c r="AB4" t="str">
+        <v/>
+      </c>
+      <c r="AC4" t="str">
         <v/>
       </c>
     </row>
@@ -739,35 +751,35 @@
         <v>Fire</v>
       </c>
       <c r="D5" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E5" t="str">
         <v>7</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
+        <v>2</v>
+      </c>
+      <c r="G5" t="str">
         <v>1</v>
       </c>
-      <c r="F5" t="str">
-        <v>1</v>
-      </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>Charged spark that strikes instantly</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>Lightning</v>
       </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
       <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
         <v>multihit</v>
       </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
       <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
         <v>2</v>
       </c>
-      <c r="M5" t="str">
-        <v/>
-      </c>
       <c r="N5" t="str">
         <v/>
       </c>
@@ -811,6 +823,9 @@
         <v/>
       </c>
       <c r="AB5" t="str">
+        <v/>
+      </c>
+      <c r="AC5" t="str">
         <v/>
       </c>
     </row>
@@ -825,23 +840,23 @@
         <v>Air</v>
       </c>
       <c r="D6" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E6" t="str">
         <v>1</v>
       </c>
-      <c r="E6" t="str">
-        <v>2</v>
-      </c>
       <c r="F6" t="str">
+        <v>3</v>
+      </c>
+      <c r="G6" t="str">
         <v>1</v>
       </c>
-      <c r="G6" t="str">
-        <v>A deep sense of calm overwhelms you</v>
-      </c>
       <c r="H6" t="str">
+        <v>Enhances existing elements</v>
+      </c>
+      <c r="I6" t="str">
         <v>Plasma</v>
       </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
       <c r="J6" t="str">
         <v/>
       </c>
@@ -897,6 +912,9 @@
         <v/>
       </c>
       <c r="AB6" t="str">
+        <v/>
+      </c>
+      <c r="AC6" t="str">
         <v/>
       </c>
     </row>
@@ -911,23 +929,23 @@
         <v>Earth</v>
       </c>
       <c r="D7" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E7" t="str">
         <v>1</v>
       </c>
-      <c r="E7" t="str">
-        <v>2</v>
-      </c>
       <c r="F7" t="str">
+        <v>3</v>
+      </c>
+      <c r="G7" t="str">
         <v>1</v>
       </c>
-      <c r="G7" t="str">
-        <v>A deep sense of calm overwhelms you</v>
-      </c>
       <c r="H7" t="str">
+        <v>Enhances existing elements</v>
+      </c>
+      <c r="I7" t="str">
         <v>Plasma</v>
       </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
       <c r="J7" t="str">
         <v/>
       </c>
@@ -983,6 +1001,9 @@
         <v/>
       </c>
       <c r="AB7" t="str">
+        <v/>
+      </c>
+      <c r="AC7" t="str">
         <v/>
       </c>
     </row>
@@ -997,23 +1018,23 @@
         <v>Fire</v>
       </c>
       <c r="D8" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E8" t="str">
         <v>1</v>
       </c>
-      <c r="E8" t="str">
-        <v>2</v>
-      </c>
       <c r="F8" t="str">
+        <v>3</v>
+      </c>
+      <c r="G8" t="str">
         <v>1</v>
       </c>
-      <c r="G8" t="str">
-        <v>A deep sense of calm overwhelms you</v>
-      </c>
       <c r="H8" t="str">
+        <v>Enhances existing elements</v>
+      </c>
+      <c r="I8" t="str">
         <v>Plasma</v>
       </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
       <c r="J8" t="str">
         <v/>
       </c>
@@ -1069,45 +1090,48 @@
         <v/>
       </c>
       <c r="AB8" t="str">
+        <v/>
+      </c>
+      <c r="AC8" t="str">
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Plasma</v>
+        <v>Bulwark</v>
       </c>
       <c r="B9" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="C9" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="D9" t="str">
-        <v>1</v>
+        <v>Spell</v>
       </c>
       <c r="E9" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F9" t="str">
         <v>1</v>
       </c>
       <c r="G9" t="str">
-        <v>A deep sense of calm overwhelms you</v>
+        <v>1</v>
       </c>
       <c r="H9" t="str">
-        <v>Fire</v>
+        <v>An earthen barrier that stops incoming damage</v>
       </c>
       <c r="I9" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="J9" t="str">
         <v/>
       </c>
       <c r="K9" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="L9" t="str">
-        <v/>
+        <v>12</v>
       </c>
       <c r="M9" t="str">
         <v/>
@@ -1155,6 +1179,9 @@
         <v/>
       </c>
       <c r="AB9" t="str">
+        <v/>
+      </c>
+      <c r="AC9" t="str">
         <v/>
       </c>
     </row>
@@ -1163,29 +1190,29 @@
         <v>Sand</v>
       </c>
       <c r="B10" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="C10" t="str">
         <v>Earth</v>
       </c>
       <c r="D10" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E10" t="str">
         <v>10</v>
       </c>
-      <c r="E10" t="str">
+      <c r="F10" t="str">
+        <v>2</v>
+      </c>
+      <c r="G10" t="str">
         <v>1</v>
       </c>
-      <c r="F10" t="str">
-        <v>1</v>
-      </c>
-      <c r="G10" t="str">
+      <c r="H10" t="str">
         <v>Shifting grains dance between your fingertips</v>
       </c>
-      <c r="H10" t="str">
+      <c r="I10" t="str">
         <v>Earth</v>
       </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
       <c r="J10" t="str">
         <v/>
       </c>
@@ -1241,36 +1268,39 @@
         <v/>
       </c>
       <c r="AB10" t="str">
+        <v/>
+      </c>
+      <c r="AC10" t="str">
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="B11" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="C11" t="str">
         <v>Earth</v>
       </c>
       <c r="D11" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E11" t="str">
         <v>10</v>
-      </c>
-      <c r="E11" t="str">
-        <v>1</v>
       </c>
       <c r="F11" t="str">
         <v>1</v>
       </c>
       <c r="G11" t="str">
-        <v>Shifting grains dance between your fingertips</v>
+        <v>1</v>
       </c>
       <c r="H11" t="str">
-        <v>Earth</v>
+        <v>Forged from fire and stone, hammered hard</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>Steel</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1327,36 +1357,39 @@
         <v/>
       </c>
       <c r="AB11" t="str">
+        <v/>
+      </c>
+      <c r="AC11" t="str">
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Steel</v>
+        <v>Air</v>
       </c>
       <c r="B12" t="str">
+        <v>Water</v>
+      </c>
+      <c r="C12" t="str">
         <v>Fire</v>
       </c>
-      <c r="C12" t="str">
-        <v>Earth</v>
-      </c>
       <c r="D12" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E12" t="str">
         <v>10</v>
-      </c>
-      <c r="E12" t="str">
-        <v>1</v>
       </c>
       <c r="F12" t="str">
         <v>1</v>
       </c>
       <c r="G12" t="str">
-        <v>Forged from fire and stone, hammered hard</v>
+        <v>1</v>
       </c>
       <c r="H12" t="str">
-        <v>Steel</v>
+        <v>A cool rush of wind drifts past your face</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>Air</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -1413,54 +1446,54 @@
         <v/>
       </c>
       <c r="AB12" t="str">
+        <v/>
+      </c>
+      <c r="AC12" t="str">
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Air</v>
+        <v>Leaf</v>
       </c>
       <c r="B13" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="C13" t="str">
         <v>Water</v>
       </c>
-      <c r="C13" t="str">
-        <v>Fire</v>
-      </c>
       <c r="D13" t="str">
-        <v>10</v>
+        <v>Element</v>
       </c>
       <c r="E13" t="str">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F13" t="str">
         <v>1</v>
       </c>
       <c r="G13" t="str">
-        <v>A cool rush of wind drifts past your face</v>
+        <v>1</v>
       </c>
       <c r="H13" t="str">
-        <v>Air</v>
+        <v>Drops of dew glistle atop</v>
       </c>
       <c r="I13" t="str">
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <v/>
+        <v>Leaf</v>
       </c>
       <c r="K13" t="str">
-        <v/>
+        <v>energize</v>
       </c>
       <c r="L13" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="M13" t="str">
         <v/>
       </c>
       <c r="N13" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="O13" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="P13" t="str">
         <v/>
@@ -1499,51 +1532,54 @@
         <v/>
       </c>
       <c r="AB13" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="AC13" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Leaf</v>
+        <v>Ice</v>
       </c>
       <c r="B14" t="str">
-        <v>Earth</v>
+        <v>Water</v>
       </c>
       <c r="C14" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="D14" t="str">
-        <v>8</v>
+        <v>Element</v>
       </c>
       <c r="E14" t="str">
+        <v>10</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2</v>
+      </c>
+      <c r="G14" t="str">
         <v>1</v>
       </c>
-      <c r="F14" t="str">
-        <v>1</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Drops of dew glistle atop</v>
-      </c>
       <c r="H14" t="str">
-        <v>Earth</v>
+        <v>A biting chill that settles in your bones</v>
       </c>
       <c r="I14" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="J14" t="str">
-        <v>energize</v>
+        <v/>
       </c>
       <c r="K14" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="L14" t="str">
         <v/>
       </c>
       <c r="M14" t="str">
-        <v>1</v>
+        <v/>
       </c>
       <c r="N14" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O14" t="str">
         <v/>
@@ -1582,39 +1618,42 @@
         <v/>
       </c>
       <c r="AA14" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
       <c r="AB14" t="str">
+        <v/>
+      </c>
+      <c r="AC14" t="str">
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Ice</v>
+        <v>Glass</v>
       </c>
       <c r="B15" t="str">
-        <v>Water</v>
+        <v>Sand</v>
       </c>
       <c r="C15" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="D15" t="str">
-        <v>10</v>
+        <v>Element</v>
       </c>
       <c r="E15" t="str">
+        <v>12</v>
+      </c>
+      <c r="F15" t="str">
+        <v>3</v>
+      </c>
+      <c r="G15" t="str">
         <v>1</v>
       </c>
-      <c r="F15" t="str">
-        <v>1</v>
-      </c>
-      <c r="G15" t="str">
-        <v>A biting chill that settles in your bones</v>
-      </c>
       <c r="H15" t="str">
-        <v>Ice</v>
+        <v>Smooth and brittle, it catches the light</v>
       </c>
       <c r="I15" t="str">
-        <v/>
+        <v>Glass</v>
       </c>
       <c r="J15" t="str">
         <v/>
@@ -1671,6 +1710,9 @@
         <v/>
       </c>
       <c r="AB15" t="str">
+        <v/>
+      </c>
+      <c r="AC15" t="str">
         <v/>
       </c>
     </row>
@@ -1682,26 +1724,26 @@
         <v>Sand</v>
       </c>
       <c r="C16" t="str">
-        <v>Fire</v>
+        <v>Lightning</v>
       </c>
       <c r="D16" t="str">
+        <v>Element</v>
+      </c>
+      <c r="E16" t="str">
         <v>12</v>
       </c>
-      <c r="E16" t="str">
-        <v>2</v>
-      </c>
       <c r="F16" t="str">
+        <v>3</v>
+      </c>
+      <c r="G16" t="str">
         <v>1</v>
       </c>
-      <c r="G16" t="str">
+      <c r="H16" t="str">
         <v>Smooth and brittle, it catches the light</v>
       </c>
-      <c r="H16" t="str">
+      <c r="I16" t="str">
         <v>Glass</v>
       </c>
-      <c r="I16" t="str">
-        <v/>
-      </c>
       <c r="J16" t="str">
         <v/>
       </c>
@@ -1757,36 +1799,39 @@
         <v/>
       </c>
       <c r="AB16" t="str">
+        <v/>
+      </c>
+      <c r="AC16" t="str">
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Glass</v>
+        <v>Dark Matter</v>
       </c>
       <c r="B17" t="str">
-        <v>Sand</v>
+        <v>Unstable Element</v>
       </c>
       <c r="C17" t="str">
-        <v>Lightning</v>
+        <v>Unstable Element</v>
       </c>
       <c r="D17" t="str">
-        <v>12</v>
+        <v>Element</v>
       </c>
       <c r="E17" t="str">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F17" t="str">
         <v>1</v>
       </c>
       <c r="G17" t="str">
-        <v>Smooth and brittle, it catches the light</v>
+        <v>2</v>
       </c>
       <c r="H17" t="str">
-        <v>Glass</v>
+        <v>A quiet humming radiates from inside</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>Void</v>
       </c>
       <c r="J17" t="str">
         <v/>
@@ -1843,45 +1888,48 @@
         <v/>
       </c>
       <c r="AB17" t="str">
+        <v/>
+      </c>
+      <c r="AC17" t="str">
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Dark Matter</v>
+        <v>Worble</v>
       </c>
       <c r="B18" t="str">
-        <v>Unstable Element</v>
+        <v>Water</v>
       </c>
       <c r="C18" t="str">
-        <v>Unstable Element</v>
+        <v>Water</v>
       </c>
       <c r="D18" t="str">
-        <v>18</v>
+        <v>Spell</v>
       </c>
       <c r="E18" t="str">
-        <v>1</v>
+        <v>126</v>
       </c>
       <c r="F18" t="str">
         <v>2</v>
       </c>
       <c r="G18" t="str">
-        <v>A quiet humming radiates from inside</v>
+        <v>5</v>
       </c>
       <c r="H18" t="str">
-        <v>Void</v>
+        <v>The tide is high today my friend</v>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="J18" t="str">
-        <v/>
+        <v>Water</v>
       </c>
       <c r="K18" t="str">
-        <v/>
+        <v>soak</v>
       </c>
       <c r="L18" t="str">
-        <v/>
+        <v>4</v>
       </c>
       <c r="M18" t="str">
         <v/>
@@ -1890,7 +1938,7 @@
         <v/>
       </c>
       <c r="O18" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="P18" t="str">
         <v/>
@@ -1929,70 +1977,64 @@
         <v/>
       </c>
       <c r="AB18" t="str">
-        <v/>
+        <v>Water</v>
+      </c>
+      <c r="AC18" t="str">
+        <v>Water</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Worble</v>
+        <v>Blaze</v>
       </c>
       <c r="B19" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="C19" t="str">
-        <v>Water</v>
+        <v>Fire</v>
       </c>
       <c r="D19" t="str">
-        <v>126</v>
+        <v>Spell</v>
       </c>
       <c r="E19" t="str">
+        <v>109</v>
+      </c>
+      <c r="F19" t="str">
         <v>2</v>
       </c>
-      <c r="F19" t="str">
+      <c r="G19" t="str">
         <v>5</v>
       </c>
-      <c r="G19" t="str">
-        <v>The tide is high today my friend</v>
-      </c>
       <c r="H19" t="str">
-        <v>Water</v>
+        <v>Forest floor erupts in scorching flame</v>
       </c>
       <c r="I19" t="str">
-        <v>Water</v>
+        <v>Leaf</v>
       </c>
       <c r="J19" t="str">
-        <v>soak</v>
+        <v>Fire</v>
       </c>
       <c r="K19" t="str">
-        <v>4</v>
+        <v>burn</v>
       </c>
       <c r="L19" t="str">
-        <v/>
+        <v>6</v>
       </c>
       <c r="M19" t="str">
         <v/>
       </c>
       <c r="N19" t="str">
+        <v>2</v>
+      </c>
+      <c r="O19" t="str">
         <v>enemy</v>
       </c>
-      <c r="O19" t="str">
-        <v/>
-      </c>
-      <c r="P19" t="str">
-        <v/>
-      </c>
-      <c r="Q19" t="str">
-        <v/>
-      </c>
       <c r="R19" t="str">
         <v/>
       </c>
       <c r="S19" t="str">
         <v/>
       </c>
-      <c r="T19" t="str">
-        <v/>
-      </c>
       <c r="U19" t="str">
         <v/>
       </c>
@@ -2012,62 +2054,65 @@
         <v/>
       </c>
       <c r="AA19" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="AB19" t="str">
-        <v>Water</v>
+        <v>Fire</v>
+      </c>
+      <c r="AC19" t="str">
+        <v>Leaf</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Blaze</v>
+        <v>Regen</v>
       </c>
       <c r="B20" t="str">
         <v>Leaf</v>
       </c>
       <c r="C20" t="str">
-        <v>Fire</v>
+        <v>Water</v>
       </c>
       <c r="D20" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E20" t="str">
         <v>109</v>
       </c>
-      <c r="E20" t="str">
+      <c r="F20" t="str">
         <v>2</v>
       </c>
-      <c r="F20" t="str">
+      <c r="G20" t="str">
         <v>5</v>
       </c>
-      <c r="G20" t="str">
-        <v>Forest floor erupts in scorching flame</v>
-      </c>
       <c r="H20" t="str">
+        <v>Living vines wrap wounds in cool water</v>
+      </c>
+      <c r="I20" t="str">
         <v>Leaf</v>
       </c>
-      <c r="I20" t="str">
-        <v>Fire</v>
-      </c>
       <c r="J20" t="str">
-        <v>burn</v>
+        <v>Water</v>
       </c>
       <c r="K20" t="str">
-        <v>6</v>
+        <v>shield</v>
       </c>
       <c r="L20" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="M20" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="N20" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="Q20" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="O20" t="str">
+        <v>self</v>
       </c>
       <c r="R20" t="str">
         <v/>
       </c>
-      <c r="T20" t="str">
+      <c r="S20" t="str">
         <v/>
       </c>
       <c r="U20" t="str">
@@ -2089,62 +2134,65 @@
         <v/>
       </c>
       <c r="AA20" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
       <c r="AB20" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AC20" t="str">
         <v>Leaf</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Regen</v>
+        <v>Thorns</v>
       </c>
       <c r="B21" t="str">
         <v>Leaf</v>
       </c>
       <c r="C21" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E21" t="str">
+        <v>109</v>
+      </c>
+      <c r="F21" t="str">
+        <v>2</v>
+      </c>
+      <c r="G21" t="str">
+        <v>5</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Spiked vines wrap around you</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="J21" t="str">
         <v>Water</v>
       </c>
-      <c r="D21" t="str">
-        <v>109</v>
-      </c>
-      <c r="E21" t="str">
-        <v>2</v>
-      </c>
-      <c r="F21" t="str">
-        <v>5</v>
-      </c>
-      <c r="G21" t="str">
-        <v>Living vines wrap wounds in cool water</v>
-      </c>
-      <c r="H21" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="I21" t="str">
-        <v>Water</v>
-      </c>
-      <c r="J21" t="str">
+      <c r="K21" t="str">
         <v>shield</v>
       </c>
-      <c r="K21" t="str">
+      <c r="L21" t="str">
         <v>8</v>
       </c>
-      <c r="L21" t="str">
-        <v/>
-      </c>
       <c r="M21" t="str">
         <v/>
       </c>
       <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
         <v>self</v>
       </c>
-      <c r="Q21" t="str">
-        <v/>
-      </c>
       <c r="R21" t="str">
         <v/>
       </c>
-      <c r="T21" t="str">
+      <c r="S21" t="str">
         <v/>
       </c>
       <c r="U21" t="str">
@@ -2166,61 +2214,73 @@
         <v/>
       </c>
       <c r="AA21" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="AB21" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AC21" t="str">
         <v>Leaf</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Thorns</v>
+        <v>Levitate</v>
       </c>
       <c r="B22" t="str">
         <v>Leaf</v>
       </c>
       <c r="C22" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="D22" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E22" t="str">
         <v>109</v>
       </c>
-      <c r="E22" t="str">
-        <v>2</v>
-      </c>
       <c r="F22" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G22" t="str">
-        <v>Spiked vines protect you</v>
+        <v>3</v>
       </c>
       <c r="H22" t="str">
+        <v>Peacefully hover inches above the ground</v>
+      </c>
+      <c r="I22" t="str">
         <v>Leaf</v>
       </c>
-      <c r="I22" t="str">
-        <v>Water</v>
-      </c>
       <c r="J22" t="str">
+        <v>Air</v>
+      </c>
+      <c r="K22" t="str">
         <v>shield</v>
       </c>
-      <c r="K22" t="str">
+      <c r="L22" t="str">
         <v>8</v>
       </c>
-      <c r="L22" t="str">
-        <v/>
-      </c>
       <c r="M22" t="str">
         <v/>
       </c>
       <c r="N22" t="str">
+        <v/>
+      </c>
+      <c r="O22" t="str">
         <v>self</v>
       </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
       <c r="Q22" t="str">
         <v/>
       </c>
       <c r="R22" t="str">
         <v/>
       </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
       <c r="T22" t="str">
         <v/>
       </c>
@@ -2243,58 +2303,61 @@
         <v/>
       </c>
       <c r="AA22" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AB22" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AC22" t="str">
         <v>Leaf</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Tornado</v>
+        <v>Blizzard</v>
       </c>
       <c r="B23" t="str">
         <v>Leaf</v>
       </c>
       <c r="C23" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D23" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E23" t="str">
         <v>109</v>
       </c>
-      <c r="E23" t="str">
-        <v>2</v>
-      </c>
       <c r="F23" t="str">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G23" t="str">
-        <v>Wind whips and slashes about</v>
+        <v>5</v>
       </c>
       <c r="H23" t="str">
+        <v>Snow flurries block your vision</v>
+      </c>
+      <c r="I23" t="str">
         <v>Leaf</v>
       </c>
-      <c r="I23" t="str">
-        <v>Air</v>
-      </c>
       <c r="J23" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="K23" t="str">
         <v>shield</v>
       </c>
-      <c r="K23" t="str">
+      <c r="L23" t="str">
         <v>8</v>
       </c>
-      <c r="L23" t="str">
-        <v/>
-      </c>
       <c r="M23" t="str">
         <v/>
       </c>
       <c r="N23" t="str">
+        <v/>
+      </c>
+      <c r="O23" t="str">
         <v>self</v>
       </c>
-      <c r="O23" t="str">
-        <v/>
-      </c>
       <c r="P23" t="str">
         <v/>
       </c>
@@ -2329,73 +2392,67 @@
         <v/>
       </c>
       <c r="AA23" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AB23" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="AC23" t="str">
         <v>Leaf</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Blizzard</v>
+        <v>Leaf Blade</v>
       </c>
       <c r="B24" t="str">
         <v>Leaf</v>
       </c>
       <c r="C24" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="D24" t="str">
-        <v>109</v>
+        <v>Spell</v>
       </c>
       <c r="E24" t="str">
-        <v>2</v>
+        <v>159</v>
       </c>
       <c r="F24" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G24" t="str">
-        <v>Snow flurries block your vision</v>
+        <v>0</v>
       </c>
       <c r="H24" t="str">
+        <v>A razor edge honed from living wood</v>
+      </c>
+      <c r="I24" t="str">
         <v>Leaf</v>
       </c>
-      <c r="I24" t="str">
-        <v>Ice</v>
-      </c>
       <c r="J24" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="K24" t="str">
         <v>shield</v>
       </c>
-      <c r="K24" t="str">
+      <c r="L24" t="str">
         <v>8</v>
       </c>
-      <c r="L24" t="str">
-        <v/>
-      </c>
       <c r="M24" t="str">
         <v/>
       </c>
       <c r="N24" t="str">
+        <v/>
+      </c>
+      <c r="O24" t="str">
         <v>self</v>
       </c>
-      <c r="O24" t="str">
-        <v/>
-      </c>
-      <c r="P24" t="str">
-        <v/>
-      </c>
-      <c r="Q24" t="str">
-        <v/>
-      </c>
       <c r="R24" t="str">
         <v/>
       </c>
       <c r="S24" t="str">
         <v/>
       </c>
-      <c r="T24" t="str">
-        <v/>
-      </c>
       <c r="U24" t="str">
         <v/>
       </c>
@@ -2415,62 +2472,65 @@
         <v/>
       </c>
       <c r="AA24" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
       <c r="AB24" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AC24" t="str">
         <v>Leaf</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Leaf Blade</v>
+        <v>Needle Storm</v>
       </c>
       <c r="B25" t="str">
         <v>Leaf</v>
       </c>
       <c r="C25" t="str">
-        <v>Steel</v>
+        <v>Sand</v>
       </c>
       <c r="D25" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E25" t="str">
         <v>159</v>
       </c>
-      <c r="E25" t="str">
-        <v>2</v>
-      </c>
       <c r="F25" t="str">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G25" t="str">
-        <v>A razor edge honed from living wood</v>
+        <v>7</v>
       </c>
       <c r="H25" t="str">
+        <v>Tiny needles prick from every angle</v>
+      </c>
+      <c r="I25" t="str">
         <v>Leaf</v>
       </c>
-      <c r="I25" t="str">
-        <v>Steel</v>
-      </c>
       <c r="J25" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="K25" t="str">
         <v>shield</v>
       </c>
-      <c r="K25" t="str">
+      <c r="L25" t="str">
         <v>8</v>
       </c>
-      <c r="L25" t="str">
-        <v/>
-      </c>
       <c r="M25" t="str">
         <v/>
       </c>
       <c r="N25" t="str">
+        <v/>
+      </c>
+      <c r="O25" t="str">
         <v>self</v>
       </c>
-      <c r="Q25" t="str">
-        <v/>
-      </c>
       <c r="R25" t="str">
         <v/>
       </c>
-      <c r="T25" t="str">
+      <c r="S25" t="str">
         <v/>
       </c>
       <c r="U25" t="str">
@@ -2492,139 +2552,145 @@
         <v/>
       </c>
       <c r="AA25" t="str">
+        <v/>
+      </c>
+      <c r="AB25" t="str">
         <v>Earth</v>
       </c>
-      <c r="AB25" t="str">
+      <c r="AC25" t="str">
         <v>Leaf</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Needle Storm</v>
+        <v>Photosynthesis</v>
       </c>
       <c r="B26" t="str">
         <v>Leaf</v>
       </c>
       <c r="C26" t="str">
-        <v>Sand</v>
+        <v>Leaf</v>
       </c>
       <c r="D26" t="str">
-        <v>159</v>
+        <v>Spell</v>
       </c>
       <c r="E26" t="str">
+        <v>210</v>
+      </c>
+      <c r="F26" t="str">
+        <v>3</v>
+      </c>
+      <c r="G26" t="str">
+        <v>9</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Nature feeds itself to grow ever stronger</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Water</v>
+      </c>
+      <c r="K26" t="str">
+        <v>soak</v>
+      </c>
+      <c r="L26" t="str">
         <v>2</v>
       </c>
-      <c r="F26" t="str">
-        <v>7</v>
-      </c>
-      <c r="G26" t="str">
-        <v>Tiny needles prick from every angle</v>
-      </c>
-      <c r="H26" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="I26" t="str">
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
+      <c r="O26" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+      <c r="U26" t="str">
+        <v/>
+      </c>
+      <c r="V26" t="str">
+        <v/>
+      </c>
+      <c r="W26" t="str">
+        <v/>
+      </c>
+      <c r="X26" t="str">
+        <v/>
+      </c>
+      <c r="Y26" t="str">
+        <v/>
+      </c>
+      <c r="Z26" t="str">
+        <v/>
+      </c>
+      <c r="AA26" t="str">
+        <v/>
+      </c>
+      <c r="AB26" t="str">
         <v>Earth</v>
       </c>
-      <c r="J26" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K26" t="str">
-        <v>8</v>
-      </c>
-      <c r="L26" t="str">
-        <v/>
-      </c>
-      <c r="M26" t="str">
-        <v/>
-      </c>
-      <c r="N26" t="str">
-        <v>self</v>
-      </c>
-      <c r="Q26" t="str">
-        <v/>
-      </c>
-      <c r="R26" t="str">
-        <v/>
-      </c>
-      <c r="T26" t="str">
-        <v/>
-      </c>
-      <c r="U26" t="str">
-        <v/>
-      </c>
-      <c r="V26" t="str">
-        <v/>
-      </c>
-      <c r="W26" t="str">
-        <v/>
-      </c>
-      <c r="X26" t="str">
-        <v/>
-      </c>
-      <c r="Y26" t="str">
-        <v/>
-      </c>
-      <c r="Z26" t="str">
-        <v/>
-      </c>
-      <c r="AA26" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="AB26" t="str">
+      <c r="AC26" t="str">
         <v>Leaf</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Photosynthesis</v>
+        <v>Desert Blade</v>
       </c>
       <c r="B27" t="str">
-        <v>Leaf</v>
+        <v>Sand</v>
       </c>
       <c r="C27" t="str">
-        <v>Leaf</v>
+        <v>Steel</v>
       </c>
       <c r="D27" t="str">
-        <v>210</v>
+        <v>Spell</v>
       </c>
       <c r="E27" t="str">
-        <v>2</v>
+        <v>159</v>
       </c>
       <c r="F27" t="str">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G27" t="str">
-        <v>Nature feeds itself to grow ever stronger</v>
+        <v>0</v>
       </c>
       <c r="H27" t="str">
-        <v>Leaf</v>
+        <v>Sand-forged steel scorched by the desert sun</v>
       </c>
       <c r="I27" t="str">
-        <v>Water</v>
+        <v>Earth</v>
       </c>
       <c r="J27" t="str">
-        <v>soak</v>
+        <v>Steel</v>
       </c>
       <c r="K27" t="str">
-        <v>2</v>
+        <v>shield</v>
       </c>
       <c r="L27" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="M27" t="str">
         <v/>
       </c>
       <c r="N27" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="Q27" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v>self</v>
       </c>
       <c r="R27" t="str">
         <v/>
       </c>
-      <c r="T27" t="str">
+      <c r="S27" t="str">
         <v/>
       </c>
       <c r="U27" t="str">
@@ -2646,61 +2712,73 @@
         <v/>
       </c>
       <c r="AA27" t="str">
+        <v/>
+      </c>
+      <c r="AB27" t="str">
         <v>Earth</v>
       </c>
-      <c r="AB27" t="str">
-        <v>Leaf</v>
+      <c r="AC27" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Desert Blade</v>
+        <v>Sand Shield</v>
       </c>
       <c r="B28" t="str">
         <v>Sand</v>
       </c>
       <c r="C28" t="str">
-        <v>Steel</v>
+        <v>Earth</v>
       </c>
       <c r="D28" t="str">
-        <v>159</v>
+        <v>Spell</v>
       </c>
       <c r="E28" t="str">
-        <v>2</v>
+        <v>109</v>
       </c>
       <c r="F28" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G28" t="str">
-        <v>Sand-forged steel scorched by the desert sun</v>
+        <v>5</v>
       </c>
       <c r="H28" t="str">
+        <v>Grains pack tight into an earthen wall</v>
+      </c>
+      <c r="I28" t="str">
         <v>Earth</v>
       </c>
-      <c r="I28" t="str">
-        <v>Steel</v>
-      </c>
       <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
         <v>shield</v>
       </c>
-      <c r="K28" t="str">
+      <c r="L28" t="str">
         <v>8</v>
       </c>
-      <c r="L28" t="str">
-        <v/>
-      </c>
       <c r="M28" t="str">
         <v/>
       </c>
       <c r="N28" t="str">
+        <v/>
+      </c>
+      <c r="O28" t="str">
         <v>self</v>
       </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
       <c r="Q28" t="str">
         <v/>
       </c>
       <c r="R28" t="str">
         <v/>
       </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
       <c r="T28" t="str">
         <v/>
       </c>
@@ -2723,144 +2801,150 @@
         <v/>
       </c>
       <c r="AA28" t="str">
+        <v/>
+      </c>
+      <c r="AB28" t="str">
         <v>Earth</v>
       </c>
-      <c r="AB28" t="str">
-        <v>Fire</v>
+      <c r="AC28" t="str">
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Sand Shield</v>
+        <v>Sandstorm</v>
       </c>
       <c r="B29" t="str">
         <v>Sand</v>
       </c>
       <c r="C29" t="str">
+        <v>Air</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E29" t="str">
+        <v>109</v>
+      </c>
+      <c r="F29" t="str">
+        <v>4</v>
+      </c>
+      <c r="G29" t="str">
+        <v>3</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Blinding grit swirls on howling winds</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Air</v>
+      </c>
+      <c r="J29" t="str">
         <v>Earth</v>
       </c>
-      <c r="D29" t="str">
-        <v>109</v>
-      </c>
-      <c r="E29" t="str">
-        <v>2</v>
-      </c>
-      <c r="F29" t="str">
-        <v>5</v>
-      </c>
-      <c r="G29" t="str">
-        <v>Grains pack tight into an earthen wall</v>
-      </c>
-      <c r="H29" t="str">
+      <c r="K29" t="str">
+        <v>shield</v>
+      </c>
+      <c r="L29" t="str">
+        <v>8</v>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v/>
+      </c>
+      <c r="O29" t="str">
+        <v>self</v>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
+        <v/>
+      </c>
+      <c r="T29" t="str">
+        <v/>
+      </c>
+      <c r="U29" t="str">
+        <v/>
+      </c>
+      <c r="V29" t="str">
+        <v/>
+      </c>
+      <c r="W29" t="str">
+        <v/>
+      </c>
+      <c r="X29" t="str">
+        <v/>
+      </c>
+      <c r="Y29" t="str">
+        <v/>
+      </c>
+      <c r="Z29" t="str">
+        <v/>
+      </c>
+      <c r="AA29" t="str">
+        <v/>
+      </c>
+      <c r="AB29" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AC29" t="str">
         <v>Earth</v>
-      </c>
-      <c r="I29" t="str">
-        <v/>
-      </c>
-      <c r="J29" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K29" t="str">
-        <v>8</v>
-      </c>
-      <c r="L29" t="str">
-        <v/>
-      </c>
-      <c r="M29" t="str">
-        <v/>
-      </c>
-      <c r="N29" t="str">
-        <v>self</v>
-      </c>
-      <c r="O29" t="str">
-        <v/>
-      </c>
-      <c r="P29" t="str">
-        <v/>
-      </c>
-      <c r="Q29" t="str">
-        <v/>
-      </c>
-      <c r="R29" t="str">
-        <v/>
-      </c>
-      <c r="S29" t="str">
-        <v/>
-      </c>
-      <c r="T29" t="str">
-        <v/>
-      </c>
-      <c r="U29" t="str">
-        <v/>
-      </c>
-      <c r="V29" t="str">
-        <v/>
-      </c>
-      <c r="W29" t="str">
-        <v/>
-      </c>
-      <c r="X29" t="str">
-        <v/>
-      </c>
-      <c r="Y29" t="str">
-        <v/>
-      </c>
-      <c r="Z29" t="str">
-        <v/>
-      </c>
-      <c r="AA29" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="AB29" t="str">
-        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Sandstorm</v>
+        <v>Iceblast</v>
       </c>
       <c r="B30" t="str">
         <v>Sand</v>
       </c>
       <c r="C30" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D30" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E30" t="str">
         <v>109</v>
       </c>
-      <c r="E30" t="str">
-        <v>2</v>
-      </c>
       <c r="F30" t="str">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G30" t="str">
-        <v>Blinding grit swirls on howling winds</v>
+        <v>5</v>
       </c>
       <c r="H30" t="str">
-        <v>Air</v>
+        <v>Cold grit bites with a frosty sting</v>
       </c>
       <c r="I30" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="J30" t="str">
         <v>Earth</v>
       </c>
-      <c r="J30" t="str">
+      <c r="K30" t="str">
         <v>shield</v>
       </c>
-      <c r="K30" t="str">
+      <c r="L30" t="str">
         <v>8</v>
       </c>
-      <c r="L30" t="str">
-        <v/>
-      </c>
       <c r="M30" t="str">
         <v/>
       </c>
       <c r="N30" t="str">
+        <v/>
+      </c>
+      <c r="O30" t="str">
         <v>self</v>
       </c>
-      <c r="O30" t="str">
-        <v/>
-      </c>
       <c r="P30" t="str">
         <v/>
       </c>
@@ -2895,63 +2979,60 @@
         <v/>
       </c>
       <c r="AA30" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AB30" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="AC30" t="str">
         <v>Earth</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Iceblast</v>
+        <v>Blaze Blade</v>
       </c>
       <c r="B31" t="str">
-        <v>Sand</v>
+        <v>Steel</v>
       </c>
       <c r="C31" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="D31" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E31" t="str">
         <v>109</v>
       </c>
-      <c r="E31" t="str">
+      <c r="F31" t="str">
         <v>2</v>
       </c>
-      <c r="F31" t="str">
-        <v>5</v>
-      </c>
       <c r="G31" t="str">
-        <v>Cold grit bites with a frosty sting</v>
+        <v>0</v>
       </c>
       <c r="H31" t="str">
-        <v>Ice</v>
+        <v>A steel blade bathed in white-hot flame</v>
       </c>
       <c r="I31" t="str">
-        <v>Earth</v>
+        <v>Fire</v>
       </c>
       <c r="J31" t="str">
-        <v>shield</v>
+        <v>Steel</v>
       </c>
       <c r="K31" t="str">
-        <v>8</v>
+        <v>burn</v>
       </c>
       <c r="L31" t="str">
-        <v/>
+        <v>6</v>
       </c>
       <c r="M31" t="str">
         <v/>
       </c>
       <c r="N31" t="str">
-        <v>self</v>
+        <v>2</v>
       </c>
       <c r="O31" t="str">
-        <v/>
-      </c>
-      <c r="P31" t="str">
-        <v/>
-      </c>
-      <c r="Q31" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="R31" t="str">
         <v/>
@@ -2959,9 +3040,6 @@
       <c r="S31" t="str">
         <v/>
       </c>
-      <c r="T31" t="str">
-        <v/>
-      </c>
       <c r="U31" t="str">
         <v/>
       </c>
@@ -2981,133 +3059,136 @@
         <v/>
       </c>
       <c r="AA31" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
       <c r="AB31" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="AC31" t="str">
         <v>Earth</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Blaze Blade</v>
+        <v>Aqua Blade</v>
       </c>
       <c r="B32" t="str">
         <v>Steel</v>
       </c>
       <c r="C32" t="str">
+        <v>Water</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E32" t="str">
+        <v>109</v>
+      </c>
+      <c r="F32" t="str">
+        <v>2</v>
+      </c>
+      <c r="G32" t="str">
+        <v>0</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Steam rises where cold steel meets the wave</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Water</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="K32" t="str">
+        <v>soak</v>
+      </c>
+      <c r="L32" t="str">
+        <v>2</v>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+      <c r="N32" t="str">
+        <v/>
+      </c>
+      <c r="O32" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="U32" t="str">
+        <v/>
+      </c>
+      <c r="V32" t="str">
+        <v/>
+      </c>
+      <c r="W32" t="str">
+        <v/>
+      </c>
+      <c r="X32" t="str">
+        <v/>
+      </c>
+      <c r="Y32" t="str">
+        <v/>
+      </c>
+      <c r="Z32" t="str">
+        <v/>
+      </c>
+      <c r="AA32" t="str">
+        <v/>
+      </c>
+      <c r="AB32" t="str">
+        <v>Water</v>
+      </c>
+      <c r="AC32" t="str">
         <v>Fire</v>
-      </c>
-      <c r="D32" t="str">
-        <v>109</v>
-      </c>
-      <c r="E32" t="str">
-        <v>2</v>
-      </c>
-      <c r="F32" t="str">
-        <v>0</v>
-      </c>
-      <c r="G32" t="str">
-        <v>A steel blade bathed in white-hot flame</v>
-      </c>
-      <c r="H32" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="I32" t="str">
-        <v>Steel</v>
-      </c>
-      <c r="J32" t="str">
-        <v>burn</v>
-      </c>
-      <c r="K32" t="str">
-        <v>6</v>
-      </c>
-      <c r="L32" t="str">
-        <v/>
-      </c>
-      <c r="M32" t="str">
-        <v>2</v>
-      </c>
-      <c r="N32" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="Q32" t="str">
-        <v/>
-      </c>
-      <c r="R32" t="str">
-        <v/>
-      </c>
-      <c r="T32" t="str">
-        <v/>
-      </c>
-      <c r="U32" t="str">
-        <v/>
-      </c>
-      <c r="V32" t="str">
-        <v/>
-      </c>
-      <c r="W32" t="str">
-        <v/>
-      </c>
-      <c r="X32" t="str">
-        <v/>
-      </c>
-      <c r="Y32" t="str">
-        <v/>
-      </c>
-      <c r="Z32" t="str">
-        <v/>
-      </c>
-      <c r="AA32" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="AB32" t="str">
-        <v>Earth</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Aqua Blade</v>
+        <v>Thunder Blade</v>
       </c>
       <c r="B33" t="str">
         <v>Steel</v>
       </c>
       <c r="C33" t="str">
-        <v>Water</v>
+        <v>Lightning</v>
       </c>
       <c r="D33" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E33" t="str">
         <v>109</v>
       </c>
-      <c r="E33" t="str">
+      <c r="F33" t="str">
+        <v>4</v>
+      </c>
+      <c r="G33" t="str">
+        <v>0</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Sparks dance across the blades edge</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="K33" t="str">
+        <v>multi_hit</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
         <v>2</v>
       </c>
-      <c r="F33" t="str">
-        <v>0</v>
-      </c>
-      <c r="G33" t="str">
-        <v>Steam rises where cold steel meets the wave</v>
-      </c>
-      <c r="H33" t="str">
-        <v>Water</v>
-      </c>
-      <c r="I33" t="str">
-        <v>Steel</v>
-      </c>
-      <c r="J33" t="str">
-        <v>soak</v>
-      </c>
-      <c r="K33" t="str">
-        <v>2</v>
-      </c>
-      <c r="L33" t="str">
-        <v/>
-      </c>
-      <c r="M33" t="str">
-        <v/>
-      </c>
       <c r="N33" t="str">
+        <v/>
+      </c>
+      <c r="O33" t="str">
         <v>enemy</v>
       </c>
-      <c r="T33" t="str">
+      <c r="R33" t="str">
         <v/>
       </c>
       <c r="U33" t="str">
@@ -3129,60 +3210,60 @@
         <v/>
       </c>
       <c r="AA33" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="AB33" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="AC33" t="str">
         <v>Fire</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Thunder Blade</v>
+        <v>Earth Blade</v>
       </c>
       <c r="B34" t="str">
         <v>Steel</v>
       </c>
       <c r="C34" t="str">
-        <v>Lightning</v>
+        <v>Earth</v>
       </c>
       <c r="D34" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E34" t="str">
         <v>109</v>
       </c>
-      <c r="E34" t="str">
+      <c r="F34" t="str">
         <v>2</v>
       </c>
-      <c r="F34" t="str">
+      <c r="G34" t="str">
         <v>0</v>
       </c>
-      <c r="G34" t="str">
-        <v>Sparks dance across the blades edge</v>
-      </c>
       <c r="H34" t="str">
-        <v>Lightning</v>
+        <v>Heavy as bedrock</v>
       </c>
       <c r="I34" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="J34" t="str">
         <v>Steel</v>
       </c>
-      <c r="J34" t="str">
-        <v>multi_hit</v>
-      </c>
       <c r="K34" t="str">
-        <v/>
+        <v>shield</v>
       </c>
       <c r="L34" t="str">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M34" t="str">
         <v/>
       </c>
       <c r="N34" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="Q34" t="str">
-        <v/>
-      </c>
-      <c r="T34" t="str">
-        <v/>
+        <v/>
+      </c>
+      <c r="O34" t="str">
+        <v>self</v>
       </c>
       <c r="U34" t="str">
         <v/>
@@ -3203,54 +3284,60 @@
         <v/>
       </c>
       <c r="AA34" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
       <c r="AB34" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="AC34" t="str">
         <v>Fire</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Earth Blade</v>
+        <v>Air Blade</v>
       </c>
       <c r="B35" t="str">
         <v>Steel</v>
       </c>
       <c r="C35" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="D35" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E35" t="str">
         <v>109</v>
       </c>
-      <c r="E35" t="str">
-        <v>2</v>
-      </c>
       <c r="F35" t="str">
+        <v>3</v>
+      </c>
+      <c r="G35" t="str">
         <v>0</v>
       </c>
-      <c r="G35" t="str">
-        <v>Heavy as bedrock</v>
-      </c>
       <c r="H35" t="str">
-        <v>Earth</v>
+        <v>Cuts the air so fast it ignites</v>
       </c>
       <c r="I35" t="str">
+        <v>Air</v>
+      </c>
+      <c r="J35" t="str">
         <v>Steel</v>
       </c>
-      <c r="J35" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K35" t="str">
-        <v>8</v>
-      </c>
-      <c r="L35" t="str">
-        <v/>
-      </c>
       <c r="M35" t="str">
         <v/>
       </c>
-      <c r="N35" t="str">
-        <v>self</v>
+      <c r="P35" t="str">
+        <v/>
+      </c>
+      <c r="Q35" t="str">
+        <v/>
+      </c>
+      <c r="R35" t="str">
+        <v/>
+      </c>
+      <c r="S35" t="str">
+        <v/>
       </c>
       <c r="T35" t="str">
         <v/>
@@ -3274,44 +3361,47 @@
         <v/>
       </c>
       <c r="AA35" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AB35" t="str">
+        <v>Air</v>
+      </c>
+      <c r="AC35" t="str">
         <v>Fire</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Air Blade</v>
+        <v>Ice Blade</v>
       </c>
       <c r="B36" t="str">
         <v>Steel</v>
       </c>
       <c r="C36" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D36" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E36" t="str">
         <v>109</v>
       </c>
-      <c r="E36" t="str">
-        <v>2</v>
-      </c>
       <c r="F36" t="str">
+        <v>4</v>
+      </c>
+      <c r="G36" t="str">
         <v>0</v>
       </c>
-      <c r="G36" t="str">
-        <v>Cuts the air so fast it ignites</v>
-      </c>
       <c r="H36" t="str">
-        <v>Air</v>
+        <v>Cold steel that somehow scorches on contact</v>
       </c>
       <c r="I36" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="J36" t="str">
         <v>Steel</v>
       </c>
-      <c r="L36" t="str">
-        <v/>
-      </c>
-      <c r="O36" t="str">
+      <c r="M36" t="str">
         <v/>
       </c>
       <c r="P36" t="str">
@@ -3348,50 +3438,47 @@
         <v/>
       </c>
       <c r="AA36" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AB36" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="AC36" t="str">
         <v>Fire</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Ice Blade</v>
+        <v>Refined Steel</v>
       </c>
       <c r="B37" t="str">
         <v>Steel</v>
       </c>
       <c r="C37" t="str">
-        <v>Ice</v>
+        <v>Steel</v>
       </c>
       <c r="D37" t="str">
-        <v>109</v>
+        <v>Element</v>
       </c>
       <c r="E37" t="str">
-        <v>2</v>
+        <v>210</v>
       </c>
       <c r="F37" t="str">
+        <v>3</v>
+      </c>
+      <c r="G37" t="str">
         <v>0</v>
       </c>
-      <c r="G37" t="str">
-        <v>Cold steel that somehow scorches on contact</v>
-      </c>
       <c r="H37" t="str">
-        <v>Ice</v>
+        <v>Folded a thousand times until perfect</v>
       </c>
       <c r="I37" t="str">
         <v>Steel</v>
       </c>
-      <c r="L37" t="str">
-        <v/>
-      </c>
-      <c r="O37" t="str">
-        <v/>
-      </c>
-      <c r="P37" t="str">
-        <v/>
-      </c>
-      <c r="Q37" t="str">
+      <c r="J37" t="str">
+        <v>Steel</v>
+      </c>
+      <c r="M37" t="str">
         <v/>
       </c>
       <c r="R37" t="str">
@@ -3400,9 +3487,6 @@
       <c r="S37" t="str">
         <v/>
       </c>
-      <c r="T37" t="str">
-        <v/>
-      </c>
       <c r="U37" t="str">
         <v/>
       </c>
@@ -3422,51 +3506,75 @@
         <v/>
       </c>
       <c r="AA37" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
       <c r="AB37" t="str">
         <v>Fire</v>
       </c>
+      <c r="AC37" t="str">
+        <v>Earth</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Refined Steel</v>
+        <v>Water Bolt</v>
       </c>
       <c r="B38" t="str">
-        <v>Steel</v>
+        <v>Lightning</v>
       </c>
       <c r="C38" t="str">
-        <v>Steel</v>
+        <v>Water</v>
       </c>
       <c r="D38" t="str">
-        <v>210</v>
+        <v>Spell</v>
       </c>
       <c r="E38" t="str">
+        <v>58</v>
+      </c>
+      <c r="F38" t="str">
+        <v>3</v>
+      </c>
+      <c r="G38" t="str">
+        <v>3</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Crackling bolts that drench what they strike</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Water</v>
+      </c>
+      <c r="K38" t="str">
+        <v>multi_hit</v>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
         <v>2</v>
       </c>
-      <c r="F38" t="str">
-        <v>0</v>
-      </c>
-      <c r="G38" t="str">
-        <v>Folded a thousand times until perfect</v>
-      </c>
-      <c r="H38" t="str">
-        <v>Steel</v>
-      </c>
-      <c r="I38" t="str">
-        <v>Steel</v>
-      </c>
-      <c r="L38" t="str">
-        <v/>
+      <c r="N38" t="str">
+        <v/>
+      </c>
+      <c r="O38" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="P38" t="str">
+        <v>soak</v>
       </c>
       <c r="Q38" t="str">
-        <v/>
+        <v>2</v>
       </c>
       <c r="R38" t="str">
         <v/>
       </c>
+      <c r="S38" t="str">
+        <v/>
+      </c>
       <c r="T38" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="U38" t="str">
         <v/>
@@ -3487,245 +3595,254 @@
         <v/>
       </c>
       <c r="AA38" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
       <c r="AB38" t="str">
-        <v>Earth</v>
+        <v>Lightning</v>
+      </c>
+      <c r="AC38" t="str">
+        <v>Water</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Water Bolt</v>
+        <v>Ice Bolt</v>
       </c>
       <c r="B39" t="str">
         <v>Lightning</v>
       </c>
       <c r="C39" t="str">
-        <v>Water</v>
+        <v>Ice</v>
       </c>
       <c r="D39" t="str">
+        <v>Spell</v>
+      </c>
+      <c r="E39" t="str">
         <v>58</v>
       </c>
-      <c r="E39" t="str">
+      <c r="F39" t="str">
+        <v>5</v>
+      </c>
+      <c r="G39" t="str">
+        <v>3</v>
+      </c>
+      <c r="H39" t="str">
+        <v>A frozen shard launched like a thunderbolt</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="K39" t="str">
+        <v>multi_hit</v>
+      </c>
+      <c r="L39" t="str">
+        <v/>
+      </c>
+      <c r="M39" t="str">
         <v>2</v>
       </c>
-      <c r="F39" t="str">
-        <v>3</v>
-      </c>
-      <c r="G39" t="str">
-        <v>Crackling bolts that drench what they strike</v>
-      </c>
-      <c r="H39" t="str">
+      <c r="N39" t="str">
+        <v/>
+      </c>
+      <c r="O39" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="P39" t="str">
+        <v/>
+      </c>
+      <c r="Q39" t="str">
+        <v/>
+      </c>
+      <c r="R39" t="str">
+        <v/>
+      </c>
+      <c r="S39" t="str">
+        <v/>
+      </c>
+      <c r="T39" t="str">
+        <v/>
+      </c>
+      <c r="U39" t="str">
+        <v/>
+      </c>
+      <c r="V39" t="str">
+        <v/>
+      </c>
+      <c r="W39" t="str">
+        <v/>
+      </c>
+      <c r="X39" t="str">
+        <v/>
+      </c>
+      <c r="Y39" t="str">
+        <v/>
+      </c>
+      <c r="Z39" t="str">
+        <v/>
+      </c>
+      <c r="AA39" t="str">
+        <v/>
+      </c>
+      <c r="AB39" t="str">
         <v>Lightning</v>
       </c>
-      <c r="I39" t="str">
-        <v>Water</v>
-      </c>
-      <c r="J39" t="str">
-        <v>multi_hit</v>
-      </c>
-      <c r="K39" t="str">
-        <v/>
-      </c>
-      <c r="L39" t="str">
-        <v>2</v>
-      </c>
-      <c r="M39" t="str">
-        <v/>
-      </c>
-      <c r="N39" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="O39" t="str">
-        <v>soak</v>
-      </c>
-      <c r="P39" t="str">
-        <v>2</v>
-      </c>
-      <c r="Q39" t="str">
-        <v/>
-      </c>
-      <c r="R39" t="str">
-        <v/>
-      </c>
-      <c r="S39" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="T39" t="str">
-        <v/>
-      </c>
-      <c r="U39" t="str">
-        <v/>
-      </c>
-      <c r="V39" t="str">
-        <v/>
-      </c>
-      <c r="W39" t="str">
-        <v/>
-      </c>
-      <c r="X39" t="str">
-        <v/>
-      </c>
-      <c r="Y39" t="str">
-        <v/>
-      </c>
-      <c r="Z39" t="str">
-        <v/>
-      </c>
-      <c r="AA39" t="str">
-        <v>Lightning</v>
-      </c>
-      <c r="AB39" t="str">
-        <v>Water</v>
+      <c r="AC39" t="str">
+        <v>Ice</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Ice Bolt</v>
+        <v>Thunder</v>
       </c>
       <c r="B40" t="str">
         <v>Lightning</v>
       </c>
       <c r="C40" t="str">
-        <v>Ice</v>
+        <v>Lightning</v>
       </c>
       <c r="D40" t="str">
-        <v>58</v>
+        <v>Spell</v>
       </c>
       <c r="E40" t="str">
-        <v>2</v>
+        <v>126</v>
       </c>
       <c r="F40" t="str">
+        <v>5</v>
+      </c>
+      <c r="G40" t="str">
+        <v>5</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Strikes once, twice, three times in a flash</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="K40" t="str">
+        <v>multi_hit</v>
+      </c>
+      <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
         <v>3</v>
       </c>
-      <c r="G40" t="str">
-        <v>A frozen shard launched like a thunderbolt</v>
-      </c>
-      <c r="H40" t="str">
+      <c r="N40" t="str">
+        <v/>
+      </c>
+      <c r="O40" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
+      <c r="R40" t="str">
+        <v/>
+      </c>
+      <c r="S40" t="str">
+        <v/>
+      </c>
+      <c r="T40" t="str">
+        <v/>
+      </c>
+      <c r="U40" t="str">
+        <v/>
+      </c>
+      <c r="V40" t="str">
+        <v/>
+      </c>
+      <c r="W40" t="str">
+        <v/>
+      </c>
+      <c r="X40" t="str">
+        <v/>
+      </c>
+      <c r="Y40" t="str">
+        <v/>
+      </c>
+      <c r="Z40" t="str">
+        <v/>
+      </c>
+      <c r="AA40" t="str">
+        <v/>
+      </c>
+      <c r="AB40" t="str">
         <v>Lightning</v>
       </c>
-      <c r="I40" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="J40" t="str">
-        <v>multi_hit</v>
-      </c>
-      <c r="K40" t="str">
-        <v/>
-      </c>
-      <c r="L40" t="str">
-        <v>2</v>
-      </c>
-      <c r="M40" t="str">
-        <v/>
-      </c>
-      <c r="N40" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="O40" t="str">
-        <v/>
-      </c>
-      <c r="P40" t="str">
-        <v/>
-      </c>
-      <c r="Q40" t="str">
-        <v/>
-      </c>
-      <c r="R40" t="str">
-        <v/>
-      </c>
-      <c r="S40" t="str">
-        <v/>
-      </c>
-      <c r="T40" t="str">
-        <v/>
-      </c>
-      <c r="U40" t="str">
-        <v/>
-      </c>
-      <c r="V40" t="str">
-        <v/>
-      </c>
-      <c r="W40" t="str">
-        <v/>
-      </c>
-      <c r="X40" t="str">
-        <v/>
-      </c>
-      <c r="Y40" t="str">
-        <v/>
-      </c>
-      <c r="Z40" t="str">
-        <v/>
-      </c>
-      <c r="AA40" t="str">
+      <c r="AC40" t="str">
         <v>Lightning</v>
-      </c>
-      <c r="AB40" t="str">
-        <v>Ice</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Thunder</v>
+        <v>Mud Shot</v>
       </c>
       <c r="B41" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
       </c>
       <c r="C41" t="str">
-        <v>Lightning</v>
+        <v>Sand</v>
       </c>
       <c r="D41" t="str">
-        <v>126</v>
+        <v>Spell</v>
       </c>
       <c r="E41" t="str">
+        <v>60</v>
+      </c>
+      <c r="F41" t="str">
+        <v>3</v>
+      </c>
+      <c r="G41" t="str">
+        <v>5</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Thick sludge launched with surprising force</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Water</v>
+      </c>
+      <c r="J41" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="K41" t="str">
+        <v>shield</v>
+      </c>
+      <c r="L41" t="str">
+        <v>8</v>
+      </c>
+      <c r="M41" t="str">
+        <v/>
+      </c>
+      <c r="N41" t="str">
+        <v/>
+      </c>
+      <c r="O41" t="str">
+        <v>self</v>
+      </c>
+      <c r="P41" t="str">
+        <v>soak</v>
+      </c>
+      <c r="Q41" t="str">
         <v>2</v>
       </c>
-      <c r="F41" t="str">
-        <v>5</v>
-      </c>
-      <c r="G41" t="str">
-        <v>Strikes once, twice, three times in a flash</v>
-      </c>
-      <c r="H41" t="str">
-        <v>Lightning</v>
-      </c>
-      <c r="I41" t="str">
-        <v>Lightning</v>
-      </c>
-      <c r="J41" t="str">
-        <v>multi_hit</v>
-      </c>
-      <c r="K41" t="str">
-        <v/>
-      </c>
-      <c r="L41" t="str">
-        <v>3</v>
-      </c>
-      <c r="M41" t="str">
-        <v/>
-      </c>
-      <c r="N41" t="str">
+      <c r="R41" t="str">
+        <v/>
+      </c>
+      <c r="S41" t="str">
+        <v/>
+      </c>
+      <c r="T41" t="str">
         <v>enemy</v>
       </c>
-      <c r="O41" t="str">
-        <v/>
-      </c>
-      <c r="P41" t="str">
-        <v/>
-      </c>
-      <c r="Q41" t="str">
-        <v/>
-      </c>
-      <c r="R41" t="str">
-        <v/>
-      </c>
-      <c r="S41" t="str">
-        <v/>
-      </c>
-      <c r="T41" t="str">
-        <v/>
-      </c>
       <c r="U41" t="str">
         <v/>
       </c>
@@ -3745,45 +3862,48 @@
         <v/>
       </c>
       <c r="AA41" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
       <c r="AB41" t="str">
-        <v>Lightning</v>
+        <v>Water</v>
+      </c>
+      <c r="AC41" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Mud Shot</v>
+        <v>Tornado</v>
       </c>
       <c r="B42" t="str">
-        <v>Water</v>
+        <v>Air</v>
       </c>
       <c r="C42" t="str">
-        <v>Sand</v>
+        <v>Air</v>
       </c>
       <c r="D42" t="str">
-        <v>60</v>
+        <v>Spell</v>
       </c>
       <c r="E42" t="str">
+        <v>126</v>
+      </c>
+      <c r="F42" t="str">
+        <v>3</v>
+      </c>
+      <c r="G42" t="str">
         <v>2</v>
       </c>
-      <c r="F42" t="str">
-        <v>5</v>
-      </c>
-      <c r="G42" t="str">
-        <v>Thick sludge launched with surprising force</v>
-      </c>
       <c r="H42" t="str">
-        <v>Water</v>
+        <v>A perfect spiral of destruction and fury</v>
       </c>
       <c r="I42" t="str">
-        <v>Earth</v>
+        <v>Air</v>
       </c>
       <c r="J42" t="str">
-        <v>shield</v>
+        <v>Air</v>
       </c>
       <c r="K42" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="L42" t="str">
         <v/>
@@ -3792,13 +3912,13 @@
         <v/>
       </c>
       <c r="N42" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O42" t="str">
-        <v>soak</v>
+        <v/>
       </c>
       <c r="P42" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="Q42" t="str">
         <v/>
@@ -3807,7 +3927,7 @@
         <v/>
       </c>
       <c r="S42" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="T42" t="str">
         <v/>
@@ -3831,42 +3951,45 @@
         <v/>
       </c>
       <c r="AA42" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="AB42" t="str">
-        <v>Earth</v>
+        <v>Air</v>
+      </c>
+      <c r="AC42" t="str">
+        <v>Air</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Tornado</v>
+        <v>Hailstorm</v>
       </c>
       <c r="B43" t="str">
         <v>Air</v>
       </c>
       <c r="C43" t="str">
-        <v>Air</v>
+        <v>Ice</v>
       </c>
       <c r="D43" t="str">
-        <v>126</v>
+        <v>Spell</v>
       </c>
       <c r="E43" t="str">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="F43" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G43" t="str">
-        <v>A perfect spiral of destruction and fury</v>
+        <v>1</v>
       </c>
       <c r="H43" t="str">
-        <v>Air</v>
+        <v>Ice pellets rain down in a furious torrent</v>
       </c>
       <c r="I43" t="str">
         <v>Air</v>
       </c>
       <c r="J43" t="str">
-        <v/>
+        <v>Ice</v>
       </c>
       <c r="K43" t="str">
         <v/>
@@ -3917,57 +4040,60 @@
         <v/>
       </c>
       <c r="AA43" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AB43" t="str">
         <v>Air</v>
       </c>
+      <c r="AC43" t="str">
+        <v>Ice</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Hailstorm</v>
+        <v>Pyreball</v>
       </c>
       <c r="B44" t="str">
-        <v>Air</v>
+        <v>Fire</v>
       </c>
       <c r="C44" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="D44" t="str">
-        <v>58</v>
+        <v>Spell</v>
       </c>
       <c r="E44" t="str">
-        <v>2</v>
+        <v>126</v>
       </c>
       <c r="F44" t="str">
         <v>1</v>
       </c>
       <c r="G44" t="str">
-        <v>Ice pellets rain down in a furious torrent</v>
+        <v>5</v>
       </c>
       <c r="H44" t="str">
-        <v>Air</v>
+        <v>A massive fireball of pure concentrated flame</v>
       </c>
       <c r="I44" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
       </c>
       <c r="J44" t="str">
-        <v/>
+        <v>Fire</v>
       </c>
       <c r="K44" t="str">
-        <v/>
+        <v>burn</v>
       </c>
       <c r="L44" t="str">
-        <v/>
+        <v>10</v>
       </c>
       <c r="M44" t="str">
         <v/>
       </c>
       <c r="N44" t="str">
-        <v/>
+        <v>3</v>
       </c>
       <c r="O44" t="str">
-        <v/>
+        <v>enemy</v>
       </c>
       <c r="P44" t="str">
         <v/>
@@ -4003,57 +4129,60 @@
         <v/>
       </c>
       <c r="AA44" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AB44" t="str">
-        <v>Ice</v>
+        <v>Fire</v>
+      </c>
+      <c r="AC44" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Pyreball</v>
+        <v>Ice Shield</v>
       </c>
       <c r="B45" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="C45" t="str">
-        <v>Fire</v>
+        <v>Earth</v>
       </c>
       <c r="D45" t="str">
-        <v>126</v>
+        <v>Spell</v>
       </c>
       <c r="E45" t="str">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="F45" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G45" t="str">
-        <v>A massive fireball of pure concentrated flame</v>
+        <v>3</v>
       </c>
       <c r="H45" t="str">
-        <v>Fire</v>
+        <v>Frozen barrier as solid and cold as bedrock</v>
       </c>
       <c r="I45" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
       </c>
       <c r="J45" t="str">
-        <v>burn</v>
+        <v>Earth</v>
       </c>
       <c r="K45" t="str">
-        <v>10</v>
+        <v>shield</v>
       </c>
       <c r="L45" t="str">
-        <v/>
+        <v>8</v>
       </c>
       <c r="M45" t="str">
-        <v>3</v>
+        <v/>
       </c>
       <c r="N45" t="str">
-        <v>enemy</v>
+        <v/>
       </c>
       <c r="O45" t="str">
-        <v/>
+        <v>self</v>
       </c>
       <c r="P45" t="str">
         <v/>
@@ -4089,45 +4218,48 @@
         <v/>
       </c>
       <c r="AA45" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
       <c r="AB45" t="str">
-        <v>Fire</v>
+        <v>Ice</v>
+      </c>
+      <c r="AC45" t="str">
+        <v>Earth</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Ice Shield</v>
+        <v>Glacier</v>
       </c>
       <c r="B46" t="str">
         <v>Ice</v>
       </c>
       <c r="C46" t="str">
-        <v>Earth</v>
+        <v>Ice</v>
       </c>
       <c r="D46" t="str">
-        <v>58</v>
+        <v>Spell</v>
       </c>
       <c r="E46" t="str">
-        <v>2</v>
+        <v>126</v>
       </c>
       <c r="F46" t="str">
         <v>3</v>
       </c>
       <c r="G46" t="str">
-        <v>Frozen barrier as solid and cold as bedrock</v>
+        <v>5</v>
       </c>
       <c r="H46" t="str">
+        <v>Ancient ice creaks and grinds slowly forward</v>
+      </c>
+      <c r="I46" t="str">
         <v>Ice</v>
       </c>
-      <c r="I46" t="str">
-        <v>Earth</v>
-      </c>
       <c r="J46" t="str">
-        <v>shield</v>
+        <v>Ice</v>
       </c>
       <c r="K46" t="str">
-        <v>8</v>
+        <v/>
       </c>
       <c r="L46" t="str">
         <v/>
@@ -4136,7 +4268,7 @@
         <v/>
       </c>
       <c r="N46" t="str">
-        <v>self</v>
+        <v/>
       </c>
       <c r="O46" t="str">
         <v/>
@@ -4175,187 +4307,18 @@
         <v/>
       </c>
       <c r="AA46" t="str">
+        <v/>
+      </c>
+      <c r="AB46" t="str">
         <v>Ice</v>
       </c>
-      <c r="AB46" t="str">
-        <v>Earth</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>Glacier</v>
-      </c>
-      <c r="B47" t="str">
+      <c r="AC46" t="str">
         <v>Ice</v>
-      </c>
-      <c r="C47" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="D47" t="str">
-        <v>126</v>
-      </c>
-      <c r="E47" t="str">
-        <v>2</v>
-      </c>
-      <c r="F47" t="str">
-        <v>5</v>
-      </c>
-      <c r="G47" t="str">
-        <v>Ancient ice creaks and grinds slowly forward</v>
-      </c>
-      <c r="H47" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="I47" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="J47" t="str">
-        <v/>
-      </c>
-      <c r="K47" t="str">
-        <v/>
-      </c>
-      <c r="L47" t="str">
-        <v/>
-      </c>
-      <c r="M47" t="str">
-        <v/>
-      </c>
-      <c r="N47" t="str">
-        <v/>
-      </c>
-      <c r="O47" t="str">
-        <v/>
-      </c>
-      <c r="P47" t="str">
-        <v/>
-      </c>
-      <c r="Q47" t="str">
-        <v/>
-      </c>
-      <c r="R47" t="str">
-        <v/>
-      </c>
-      <c r="S47" t="str">
-        <v/>
-      </c>
-      <c r="T47" t="str">
-        <v/>
-      </c>
-      <c r="U47" t="str">
-        <v/>
-      </c>
-      <c r="V47" t="str">
-        <v/>
-      </c>
-      <c r="W47" t="str">
-        <v/>
-      </c>
-      <c r="X47" t="str">
-        <v/>
-      </c>
-      <c r="Y47" t="str">
-        <v/>
-      </c>
-      <c r="Z47" t="str">
-        <v/>
-      </c>
-      <c r="AA47" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="AB47" t="str">
-        <v>Ice</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>Earthquake</v>
-      </c>
-      <c r="B48" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="C48" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="D48" t="str">
-        <v>126</v>
-      </c>
-      <c r="E48" t="str">
-        <v>2</v>
-      </c>
-      <c r="F48" t="str">
-        <v>5</v>
-      </c>
-      <c r="G48" t="str">
-        <v>The ground splits open beneath your foe</v>
-      </c>
-      <c r="H48" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="I48" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="J48" t="str">
-        <v>shield</v>
-      </c>
-      <c r="K48" t="str">
-        <v>16</v>
-      </c>
-      <c r="L48" t="str">
-        <v/>
-      </c>
-      <c r="M48" t="str">
-        <v/>
-      </c>
-      <c r="N48" t="str">
-        <v>self</v>
-      </c>
-      <c r="O48" t="str">
-        <v/>
-      </c>
-      <c r="P48" t="str">
-        <v/>
-      </c>
-      <c r="Q48" t="str">
-        <v/>
-      </c>
-      <c r="R48" t="str">
-        <v/>
-      </c>
-      <c r="S48" t="str">
-        <v/>
-      </c>
-      <c r="T48" t="str">
-        <v/>
-      </c>
-      <c r="U48" t="str">
-        <v/>
-      </c>
-      <c r="V48" t="str">
-        <v/>
-      </c>
-      <c r="W48" t="str">
-        <v/>
-      </c>
-      <c r="X48" t="str">
-        <v/>
-      </c>
-      <c r="Y48" t="str">
-        <v/>
-      </c>
-      <c r="Z48" t="str">
-        <v/>
-      </c>
-      <c r="AA48" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="AB48" t="str">
-        <v>Earth</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AB48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC46"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Build: (80f0809) Balance Update
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -443,49 +443,49 @@
         <v>Effect 1 Duration</v>
       </c>
       <c r="O1" t="str">
+        <v>Effect 2 Target</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Effect 3 Kind</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Effect 3 Amount</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Effect 3 Hits</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Effect 3 Duration</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Effect 3 Target</v>
+      </c>
+      <c r="U1" t="str">
+        <v>__EMPTY</v>
+      </c>
+      <c r="V1" t="str">
+        <v>__EMPTY_1</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Type 1</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Type 2</v>
+      </c>
+      <c r="Y1" t="str">
         <v>Effect 1 Target</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Z1" t="str">
         <v>Effect 2 Kind</v>
       </c>
-      <c r="Q1" t="str">
+      <c r="AA1" t="str">
         <v>Effect 2 Amount</v>
       </c>
-      <c r="R1" t="str">
+      <c r="AB1" t="str">
         <v>Effect 2 Hits</v>
       </c>
-      <c r="S1" t="str">
+      <c r="AC1" t="str">
         <v>Effect 2 Duration</v>
-      </c>
-      <c r="T1" t="str">
-        <v>Effect 2 Target</v>
-      </c>
-      <c r="U1" t="str">
-        <v>Effect 3 Kind</v>
-      </c>
-      <c r="V1" t="str">
-        <v>Effect 3 Amount</v>
-      </c>
-      <c r="W1" t="str">
-        <v>Effect 3 Hits</v>
-      </c>
-      <c r="X1" t="str">
-        <v>Effect 3 Duration</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>Effect 3 Target</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>__EMPTY</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>__EMPTY_1</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>Type 1</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>Type 2</v>
       </c>
     </row>
     <row r="2">
@@ -531,6 +531,21 @@
       <c r="N2" t="str">
         <v>3</v>
       </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
       <c r="T2" t="str">
         <v/>
       </c>
@@ -544,21 +559,6 @@
         <v/>
       </c>
       <c r="X2" t="str">
-        <v/>
-      </c>
-      <c r="Y2" t="str">
-        <v/>
-      </c>
-      <c r="Z2" t="str">
-        <v/>
-      </c>
-      <c r="AA2" t="str">
-        <v/>
-      </c>
-      <c r="AB2" t="str">
-        <v/>
-      </c>
-      <c r="AC2" t="str">
         <v/>
       </c>
     </row>
@@ -633,7 +633,7 @@
         <v/>
       </c>
       <c r="X3" t="str">
-        <v/>
+        <v>Leaf</v>
       </c>
       <c r="Y3" t="str">
         <v/>
@@ -648,7 +648,7 @@
         <v/>
       </c>
       <c r="AC3" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -1131,7 +1131,7 @@
         <v>shield</v>
       </c>
       <c r="L9" t="str">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="M9" t="str">
         <v/>
@@ -1493,38 +1493,38 @@
         <v>1</v>
       </c>
       <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+      <c r="R13" t="str">
+        <v/>
+      </c>
+      <c r="S13" t="str">
+        <v/>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v/>
+      </c>
+      <c r="V13" t="str">
+        <v/>
+      </c>
+      <c r="W13" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="X13" t="str">
+        <v/>
+      </c>
+      <c r="Y13" t="str">
         <v>self</v>
       </c>
-      <c r="P13" t="str">
-        <v/>
-      </c>
-      <c r="Q13" t="str">
-        <v/>
-      </c>
-      <c r="R13" t="str">
-        <v/>
-      </c>
-      <c r="S13" t="str">
-        <v/>
-      </c>
-      <c r="T13" t="str">
-        <v/>
-      </c>
-      <c r="U13" t="str">
-        <v/>
-      </c>
-      <c r="V13" t="str">
-        <v/>
-      </c>
-      <c r="W13" t="str">
-        <v/>
-      </c>
-      <c r="X13" t="str">
-        <v/>
-      </c>
-      <c r="Y13" t="str">
-        <v/>
-      </c>
       <c r="Z13" t="str">
         <v/>
       </c>
@@ -1532,7 +1532,7 @@
         <v/>
       </c>
       <c r="AB13" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
       <c r="AC13" t="str">
         <v/>
@@ -1908,7 +1908,7 @@
         <v>Spell</v>
       </c>
       <c r="E18" t="str">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="F18" t="str">
         <v>2</v>
@@ -1938,38 +1938,38 @@
         <v/>
       </c>
       <c r="O18" t="str">
+        <v/>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
+        <v/>
+      </c>
+      <c r="R18" t="str">
+        <v/>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
+      <c r="U18" t="str">
+        <v/>
+      </c>
+      <c r="V18" t="str">
+        <v/>
+      </c>
+      <c r="W18" t="str">
+        <v>Water</v>
+      </c>
+      <c r="X18" t="str">
+        <v>Water</v>
+      </c>
+      <c r="Y18" t="str">
         <v>enemy</v>
       </c>
-      <c r="P18" t="str">
-        <v/>
-      </c>
-      <c r="Q18" t="str">
-        <v/>
-      </c>
-      <c r="R18" t="str">
-        <v/>
-      </c>
-      <c r="S18" t="str">
-        <v/>
-      </c>
-      <c r="T18" t="str">
-        <v/>
-      </c>
-      <c r="U18" t="str">
-        <v/>
-      </c>
-      <c r="V18" t="str">
-        <v/>
-      </c>
-      <c r="W18" t="str">
-        <v/>
-      </c>
-      <c r="X18" t="str">
-        <v/>
-      </c>
-      <c r="Y18" t="str">
-        <v/>
-      </c>
       <c r="Z18" t="str">
         <v/>
       </c>
@@ -1977,10 +1977,10 @@
         <v/>
       </c>
       <c r="AB18" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="AC18" t="str">
-        <v>Water</v>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -1997,7 +1997,7 @@
         <v>Spell</v>
       </c>
       <c r="E19" t="str">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="F19" t="str">
         <v>2</v>
@@ -2026,41 +2026,41 @@
       <c r="N19" t="str">
         <v>2</v>
       </c>
-      <c r="O19" t="str">
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
+      <c r="R19" t="str">
+        <v/>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
+      <c r="U19" t="str">
+        <v/>
+      </c>
+      <c r="V19" t="str">
+        <v/>
+      </c>
+      <c r="W19" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="X19" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="Y19" t="str">
         <v>enemy</v>
       </c>
-      <c r="R19" t="str">
-        <v/>
-      </c>
-      <c r="S19" t="str">
-        <v/>
-      </c>
-      <c r="U19" t="str">
-        <v/>
-      </c>
-      <c r="V19" t="str">
-        <v/>
-      </c>
-      <c r="W19" t="str">
-        <v/>
-      </c>
-      <c r="X19" t="str">
-        <v/>
-      </c>
-      <c r="Y19" t="str">
-        <v/>
-      </c>
-      <c r="Z19" t="str">
-        <v/>
-      </c>
-      <c r="AA19" t="str">
-        <v/>
-      </c>
       <c r="AB19" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
       <c r="AC19" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -2077,7 +2077,7 @@
         <v>Spell</v>
       </c>
       <c r="E20" t="str">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="F20" t="str">
         <v>2</v>
@@ -2098,7 +2098,7 @@
         <v>shield</v>
       </c>
       <c r="L20" t="str">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M20" t="str">
         <v/>
@@ -2106,41 +2106,41 @@
       <c r="N20" t="str">
         <v/>
       </c>
-      <c r="O20" t="str">
+      <c r="P20" t="str">
+        <v/>
+      </c>
+      <c r="Q20" t="str">
+        <v/>
+      </c>
+      <c r="R20" t="str">
+        <v/>
+      </c>
+      <c r="S20" t="str">
+        <v/>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
+        <v/>
+      </c>
+      <c r="V20" t="str">
+        <v/>
+      </c>
+      <c r="W20" t="str">
+        <v>Water</v>
+      </c>
+      <c r="X20" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="Y20" t="str">
         <v>self</v>
       </c>
-      <c r="R20" t="str">
-        <v/>
-      </c>
-      <c r="S20" t="str">
-        <v/>
-      </c>
-      <c r="U20" t="str">
-        <v/>
-      </c>
-      <c r="V20" t="str">
-        <v/>
-      </c>
-      <c r="W20" t="str">
-        <v/>
-      </c>
-      <c r="X20" t="str">
-        <v/>
-      </c>
-      <c r="Y20" t="str">
-        <v/>
-      </c>
-      <c r="Z20" t="str">
-        <v/>
-      </c>
-      <c r="AA20" t="str">
-        <v/>
-      </c>
       <c r="AB20" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="AC20" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="21">
@@ -2157,7 +2157,7 @@
         <v>Spell</v>
       </c>
       <c r="E21" t="str">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="F21" t="str">
         <v>2</v>
@@ -2178,7 +2178,7 @@
         <v>shield</v>
       </c>
       <c r="L21" t="str">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M21" t="str">
         <v/>
@@ -2186,41 +2186,41 @@
       <c r="N21" t="str">
         <v/>
       </c>
-      <c r="O21" t="str">
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
+      <c r="R21" t="str">
+        <v/>
+      </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
+      <c r="U21" t="str">
+        <v/>
+      </c>
+      <c r="V21" t="str">
+        <v/>
+      </c>
+      <c r="W21" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="X21" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="Y21" t="str">
         <v>self</v>
       </c>
-      <c r="R21" t="str">
-        <v/>
-      </c>
-      <c r="S21" t="str">
-        <v/>
-      </c>
-      <c r="U21" t="str">
-        <v/>
-      </c>
-      <c r="V21" t="str">
-        <v/>
-      </c>
-      <c r="W21" t="str">
-        <v/>
-      </c>
-      <c r="X21" t="str">
-        <v/>
-      </c>
-      <c r="Y21" t="str">
-        <v/>
-      </c>
-      <c r="Z21" t="str">
-        <v/>
-      </c>
-      <c r="AA21" t="str">
-        <v/>
-      </c>
       <c r="AB21" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AC21" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -2237,7 +2237,7 @@
         <v>Spell</v>
       </c>
       <c r="E22" t="str">
-        <v>109</v>
+        <v>130</v>
       </c>
       <c r="F22" t="str">
         <v>3</v>
@@ -2258,7 +2258,7 @@
         <v>shield</v>
       </c>
       <c r="L22" t="str">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M22" t="str">
         <v/>
@@ -2267,38 +2267,38 @@
         <v/>
       </c>
       <c r="O22" t="str">
+        <v/>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+      <c r="Q22" t="str">
+        <v/>
+      </c>
+      <c r="R22" t="str">
+        <v/>
+      </c>
+      <c r="S22" t="str">
+        <v/>
+      </c>
+      <c r="T22" t="str">
+        <v/>
+      </c>
+      <c r="U22" t="str">
+        <v/>
+      </c>
+      <c r="V22" t="str">
+        <v/>
+      </c>
+      <c r="W22" t="str">
+        <v>Air</v>
+      </c>
+      <c r="X22" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="Y22" t="str">
         <v>self</v>
       </c>
-      <c r="P22" t="str">
-        <v/>
-      </c>
-      <c r="Q22" t="str">
-        <v/>
-      </c>
-      <c r="R22" t="str">
-        <v/>
-      </c>
-      <c r="S22" t="str">
-        <v/>
-      </c>
-      <c r="T22" t="str">
-        <v/>
-      </c>
-      <c r="U22" t="str">
-        <v/>
-      </c>
-      <c r="V22" t="str">
-        <v/>
-      </c>
-      <c r="W22" t="str">
-        <v/>
-      </c>
-      <c r="X22" t="str">
-        <v/>
-      </c>
-      <c r="Y22" t="str">
-        <v/>
-      </c>
       <c r="Z22" t="str">
         <v/>
       </c>
@@ -2306,10 +2306,10 @@
         <v/>
       </c>
       <c r="AB22" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AC22" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -2326,7 +2326,7 @@
         <v>Spell</v>
       </c>
       <c r="E23" t="str">
-        <v>109</v>
+        <v>165</v>
       </c>
       <c r="F23" t="str">
         <v>4</v>
@@ -2347,7 +2347,7 @@
         <v>shield</v>
       </c>
       <c r="L23" t="str">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="M23" t="str">
         <v/>
@@ -2356,38 +2356,38 @@
         <v/>
       </c>
       <c r="O23" t="str">
+        <v/>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
+      <c r="R23" t="str">
+        <v/>
+      </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v/>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="X23" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="Y23" t="str">
         <v>self</v>
       </c>
-      <c r="P23" t="str">
-        <v/>
-      </c>
-      <c r="Q23" t="str">
-        <v/>
-      </c>
-      <c r="R23" t="str">
-        <v/>
-      </c>
-      <c r="S23" t="str">
-        <v/>
-      </c>
-      <c r="T23" t="str">
-        <v/>
-      </c>
-      <c r="U23" t="str">
-        <v/>
-      </c>
-      <c r="V23" t="str">
-        <v/>
-      </c>
-      <c r="W23" t="str">
-        <v/>
-      </c>
-      <c r="X23" t="str">
-        <v/>
-      </c>
-      <c r="Y23" t="str">
-        <v/>
-      </c>
       <c r="Z23" t="str">
         <v/>
       </c>
@@ -2395,10 +2395,10 @@
         <v/>
       </c>
       <c r="AB23" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
       <c r="AC23" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="24">
@@ -2415,7 +2415,7 @@
         <v>Spell</v>
       </c>
       <c r="E24" t="str">
-        <v>159</v>
+        <v>140</v>
       </c>
       <c r="F24" t="str">
         <v>3</v>
@@ -2436,7 +2436,7 @@
         <v>shield</v>
       </c>
       <c r="L24" t="str">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M24" t="str">
         <v/>
@@ -2444,41 +2444,41 @@
       <c r="N24" t="str">
         <v/>
       </c>
-      <c r="O24" t="str">
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
+      <c r="R24" t="str">
+        <v/>
+      </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v/>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="X24" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="Y24" t="str">
         <v>self</v>
       </c>
-      <c r="R24" t="str">
-        <v/>
-      </c>
-      <c r="S24" t="str">
-        <v/>
-      </c>
-      <c r="U24" t="str">
-        <v/>
-      </c>
-      <c r="V24" t="str">
-        <v/>
-      </c>
-      <c r="W24" t="str">
-        <v/>
-      </c>
-      <c r="X24" t="str">
-        <v/>
-      </c>
-      <c r="Y24" t="str">
-        <v/>
-      </c>
-      <c r="Z24" t="str">
-        <v/>
-      </c>
-      <c r="AA24" t="str">
-        <v/>
-      </c>
       <c r="AB24" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AC24" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -2495,7 +2495,7 @@
         <v>Spell</v>
       </c>
       <c r="E25" t="str">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="F25" t="str">
         <v>4</v>
@@ -2516,7 +2516,7 @@
         <v>shield</v>
       </c>
       <c r="L25" t="str">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M25" t="str">
         <v/>
@@ -2524,41 +2524,41 @@
       <c r="N25" t="str">
         <v/>
       </c>
-      <c r="O25" t="str">
+      <c r="P25" t="str">
+        <v/>
+      </c>
+      <c r="Q25" t="str">
+        <v/>
+      </c>
+      <c r="R25" t="str">
+        <v/>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+      <c r="T25" t="str">
+        <v/>
+      </c>
+      <c r="U25" t="str">
+        <v/>
+      </c>
+      <c r="V25" t="str">
+        <v/>
+      </c>
+      <c r="W25" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="X25" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="Y25" t="str">
         <v>self</v>
       </c>
-      <c r="R25" t="str">
-        <v/>
-      </c>
-      <c r="S25" t="str">
-        <v/>
-      </c>
-      <c r="U25" t="str">
-        <v/>
-      </c>
-      <c r="V25" t="str">
-        <v/>
-      </c>
-      <c r="W25" t="str">
-        <v/>
-      </c>
-      <c r="X25" t="str">
-        <v/>
-      </c>
-      <c r="Y25" t="str">
-        <v/>
-      </c>
-      <c r="Z25" t="str">
-        <v/>
-      </c>
-      <c r="AA25" t="str">
-        <v/>
-      </c>
       <c r="AB25" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AC25" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -2575,7 +2575,7 @@
         <v>Spell</v>
       </c>
       <c r="E26" t="str">
-        <v>210</v>
+        <v>145</v>
       </c>
       <c r="F26" t="str">
         <v>3</v>
@@ -2604,41 +2604,41 @@
       <c r="N26" t="str">
         <v/>
       </c>
-      <c r="O26" t="str">
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
+      <c r="R26" t="str">
+        <v/>
+      </c>
+      <c r="S26" t="str">
+        <v/>
+      </c>
+      <c r="T26" t="str">
+        <v/>
+      </c>
+      <c r="U26" t="str">
+        <v/>
+      </c>
+      <c r="V26" t="str">
+        <v/>
+      </c>
+      <c r="W26" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="X26" t="str">
+        <v>Leaf</v>
+      </c>
+      <c r="Y26" t="str">
         <v>enemy</v>
       </c>
-      <c r="R26" t="str">
-        <v/>
-      </c>
-      <c r="S26" t="str">
-        <v/>
-      </c>
-      <c r="U26" t="str">
-        <v/>
-      </c>
-      <c r="V26" t="str">
-        <v/>
-      </c>
-      <c r="W26" t="str">
-        <v/>
-      </c>
-      <c r="X26" t="str">
-        <v/>
-      </c>
-      <c r="Y26" t="str">
-        <v/>
-      </c>
-      <c r="Z26" t="str">
-        <v/>
-      </c>
-      <c r="AA26" t="str">
-        <v/>
-      </c>
       <c r="AB26" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AC26" t="str">
-        <v>Leaf</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -2655,7 +2655,7 @@
         <v>Spell</v>
       </c>
       <c r="E27" t="str">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="F27" t="str">
         <v>4</v>
@@ -2676,7 +2676,7 @@
         <v>shield</v>
       </c>
       <c r="L27" t="str">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M27" t="str">
         <v/>
@@ -2684,41 +2684,41 @@
       <c r="N27" t="str">
         <v/>
       </c>
-      <c r="O27" t="str">
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
+      <c r="R27" t="str">
+        <v/>
+      </c>
+      <c r="S27" t="str">
+        <v/>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+      <c r="U27" t="str">
+        <v/>
+      </c>
+      <c r="V27" t="str">
+        <v/>
+      </c>
+      <c r="W27" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="X27" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="Y27" t="str">
         <v>self</v>
       </c>
-      <c r="R27" t="str">
-        <v/>
-      </c>
-      <c r="S27" t="str">
-        <v/>
-      </c>
-      <c r="U27" t="str">
-        <v/>
-      </c>
-      <c r="V27" t="str">
-        <v/>
-      </c>
-      <c r="W27" t="str">
-        <v/>
-      </c>
-      <c r="X27" t="str">
-        <v/>
-      </c>
-      <c r="Y27" t="str">
-        <v/>
-      </c>
-      <c r="Z27" t="str">
-        <v/>
-      </c>
-      <c r="AA27" t="str">
-        <v/>
-      </c>
       <c r="AB27" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AC27" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -2735,7 +2735,7 @@
         <v>Spell</v>
       </c>
       <c r="E28" t="str">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="F28" t="str">
         <v>3</v>
@@ -2756,7 +2756,7 @@
         <v>shield</v>
       </c>
       <c r="L28" t="str">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="M28" t="str">
         <v/>
@@ -2765,38 +2765,38 @@
         <v/>
       </c>
       <c r="O28" t="str">
+        <v/>
+      </c>
+      <c r="P28" t="str">
+        <v/>
+      </c>
+      <c r="Q28" t="str">
+        <v/>
+      </c>
+      <c r="R28" t="str">
+        <v/>
+      </c>
+      <c r="S28" t="str">
+        <v/>
+      </c>
+      <c r="T28" t="str">
+        <v/>
+      </c>
+      <c r="U28" t="str">
+        <v/>
+      </c>
+      <c r="V28" t="str">
+        <v/>
+      </c>
+      <c r="W28" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="X28" t="str">
+        <v/>
+      </c>
+      <c r="Y28" t="str">
         <v>self</v>
       </c>
-      <c r="P28" t="str">
-        <v/>
-      </c>
-      <c r="Q28" t="str">
-        <v/>
-      </c>
-      <c r="R28" t="str">
-        <v/>
-      </c>
-      <c r="S28" t="str">
-        <v/>
-      </c>
-      <c r="T28" t="str">
-        <v/>
-      </c>
-      <c r="U28" t="str">
-        <v/>
-      </c>
-      <c r="V28" t="str">
-        <v/>
-      </c>
-      <c r="W28" t="str">
-        <v/>
-      </c>
-      <c r="X28" t="str">
-        <v/>
-      </c>
-      <c r="Y28" t="str">
-        <v/>
-      </c>
       <c r="Z28" t="str">
         <v/>
       </c>
@@ -2804,7 +2804,7 @@
         <v/>
       </c>
       <c r="AB28" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
       <c r="AC28" t="str">
         <v/>
@@ -2824,7 +2824,7 @@
         <v>Spell</v>
       </c>
       <c r="E29" t="str">
-        <v>109</v>
+        <v>165</v>
       </c>
       <c r="F29" t="str">
         <v>4</v>
@@ -2845,7 +2845,7 @@
         <v>shield</v>
       </c>
       <c r="L29" t="str">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="M29" t="str">
         <v/>
@@ -2854,38 +2854,38 @@
         <v/>
       </c>
       <c r="O29" t="str">
+        <v/>
+      </c>
+      <c r="P29" t="str">
+        <v/>
+      </c>
+      <c r="Q29" t="str">
+        <v/>
+      </c>
+      <c r="R29" t="str">
+        <v/>
+      </c>
+      <c r="S29" t="str">
+        <v/>
+      </c>
+      <c r="T29" t="str">
+        <v/>
+      </c>
+      <c r="U29" t="str">
+        <v/>
+      </c>
+      <c r="V29" t="str">
+        <v/>
+      </c>
+      <c r="W29" t="str">
+        <v>Air</v>
+      </c>
+      <c r="X29" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="Y29" t="str">
         <v>self</v>
       </c>
-      <c r="P29" t="str">
-        <v/>
-      </c>
-      <c r="Q29" t="str">
-        <v/>
-      </c>
-      <c r="R29" t="str">
-        <v/>
-      </c>
-      <c r="S29" t="str">
-        <v/>
-      </c>
-      <c r="T29" t="str">
-        <v/>
-      </c>
-      <c r="U29" t="str">
-        <v/>
-      </c>
-      <c r="V29" t="str">
-        <v/>
-      </c>
-      <c r="W29" t="str">
-        <v/>
-      </c>
-      <c r="X29" t="str">
-        <v/>
-      </c>
-      <c r="Y29" t="str">
-        <v/>
-      </c>
       <c r="Z29" t="str">
         <v/>
       </c>
@@ -2893,10 +2893,10 @@
         <v/>
       </c>
       <c r="AB29" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AC29" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -2913,7 +2913,7 @@
         <v>Spell</v>
       </c>
       <c r="E30" t="str">
-        <v>109</v>
+        <v>370</v>
       </c>
       <c r="F30" t="str">
         <v>5</v>
@@ -2934,7 +2934,7 @@
         <v>shield</v>
       </c>
       <c r="L30" t="str">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="M30" t="str">
         <v/>
@@ -2943,38 +2943,38 @@
         <v/>
       </c>
       <c r="O30" t="str">
+        <v/>
+      </c>
+      <c r="P30" t="str">
+        <v/>
+      </c>
+      <c r="Q30" t="str">
+        <v/>
+      </c>
+      <c r="R30" t="str">
+        <v/>
+      </c>
+      <c r="S30" t="str">
+        <v/>
+      </c>
+      <c r="T30" t="str">
+        <v/>
+      </c>
+      <c r="U30" t="str">
+        <v/>
+      </c>
+      <c r="V30" t="str">
+        <v/>
+      </c>
+      <c r="W30" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="X30" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="Y30" t="str">
         <v>self</v>
       </c>
-      <c r="P30" t="str">
-        <v/>
-      </c>
-      <c r="Q30" t="str">
-        <v/>
-      </c>
-      <c r="R30" t="str">
-        <v/>
-      </c>
-      <c r="S30" t="str">
-        <v/>
-      </c>
-      <c r="T30" t="str">
-        <v/>
-      </c>
-      <c r="U30" t="str">
-        <v/>
-      </c>
-      <c r="V30" t="str">
-        <v/>
-      </c>
-      <c r="W30" t="str">
-        <v/>
-      </c>
-      <c r="X30" t="str">
-        <v/>
-      </c>
-      <c r="Y30" t="str">
-        <v/>
-      </c>
       <c r="Z30" t="str">
         <v/>
       </c>
@@ -2982,10 +2982,10 @@
         <v/>
       </c>
       <c r="AB30" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
       <c r="AC30" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
     </row>
     <row r="31">
@@ -3002,7 +3002,7 @@
         <v>Spell</v>
       </c>
       <c r="E31" t="str">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="F31" t="str">
         <v>2</v>
@@ -3031,41 +3031,41 @@
       <c r="N31" t="str">
         <v>2</v>
       </c>
-      <c r="O31" t="str">
+      <c r="P31" t="str">
+        <v/>
+      </c>
+      <c r="Q31" t="str">
+        <v/>
+      </c>
+      <c r="R31" t="str">
+        <v/>
+      </c>
+      <c r="S31" t="str">
+        <v/>
+      </c>
+      <c r="T31" t="str">
+        <v/>
+      </c>
+      <c r="U31" t="str">
+        <v/>
+      </c>
+      <c r="V31" t="str">
+        <v/>
+      </c>
+      <c r="W31" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="X31" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="Y31" t="str">
         <v>enemy</v>
       </c>
-      <c r="R31" t="str">
-        <v/>
-      </c>
-      <c r="S31" t="str">
-        <v/>
-      </c>
-      <c r="U31" t="str">
-        <v/>
-      </c>
-      <c r="V31" t="str">
-        <v/>
-      </c>
-      <c r="W31" t="str">
-        <v/>
-      </c>
-      <c r="X31" t="str">
-        <v/>
-      </c>
-      <c r="Y31" t="str">
-        <v/>
-      </c>
-      <c r="Z31" t="str">
-        <v/>
-      </c>
-      <c r="AA31" t="str">
-        <v/>
-      </c>
       <c r="AB31" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
       <c r="AC31" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -3082,7 +3082,7 @@
         <v>Spell</v>
       </c>
       <c r="E32" t="str">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="F32" t="str">
         <v>2</v>
@@ -3111,35 +3111,35 @@
       <c r="N32" t="str">
         <v/>
       </c>
-      <c r="O32" t="str">
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
+      <c r="R32" t="str">
+        <v/>
+      </c>
+      <c r="S32" t="str">
+        <v/>
+      </c>
+      <c r="T32" t="str">
+        <v/>
+      </c>
+      <c r="U32" t="str">
+        <v/>
+      </c>
+      <c r="V32" t="str">
+        <v/>
+      </c>
+      <c r="W32" t="str">
+        <v>Water</v>
+      </c>
+      <c r="X32" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="Y32" t="str">
         <v>enemy</v>
-      </c>
-      <c r="U32" t="str">
-        <v/>
-      </c>
-      <c r="V32" t="str">
-        <v/>
-      </c>
-      <c r="W32" t="str">
-        <v/>
-      </c>
-      <c r="X32" t="str">
-        <v/>
-      </c>
-      <c r="Y32" t="str">
-        <v/>
-      </c>
-      <c r="Z32" t="str">
-        <v/>
-      </c>
-      <c r="AA32" t="str">
-        <v/>
-      </c>
-      <c r="AB32" t="str">
-        <v>Water</v>
-      </c>
-      <c r="AC32" t="str">
-        <v>Fire</v>
       </c>
     </row>
     <row r="33">
@@ -3156,7 +3156,7 @@
         <v>Spell</v>
       </c>
       <c r="E33" t="str">
-        <v>109</v>
+        <v>85</v>
       </c>
       <c r="F33" t="str">
         <v>4</v>
@@ -3185,38 +3185,38 @@
       <c r="N33" t="str">
         <v/>
       </c>
-      <c r="O33" t="str">
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
+      <c r="R33" t="str">
+        <v/>
+      </c>
+      <c r="S33" t="str">
+        <v/>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
+        <v/>
+      </c>
+      <c r="V33" t="str">
+        <v/>
+      </c>
+      <c r="W33" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="X33" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="Y33" t="str">
         <v>enemy</v>
       </c>
-      <c r="R33" t="str">
-        <v/>
-      </c>
-      <c r="U33" t="str">
-        <v/>
-      </c>
-      <c r="V33" t="str">
-        <v/>
-      </c>
-      <c r="W33" t="str">
-        <v/>
-      </c>
-      <c r="X33" t="str">
-        <v/>
-      </c>
-      <c r="Y33" t="str">
-        <v/>
-      </c>
-      <c r="Z33" t="str">
-        <v/>
-      </c>
-      <c r="AA33" t="str">
-        <v/>
-      </c>
       <c r="AB33" t="str">
-        <v>Lightning</v>
-      </c>
-      <c r="AC33" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -3233,7 +3233,7 @@
         <v>Spell</v>
       </c>
       <c r="E34" t="str">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="F34" t="str">
         <v>2</v>
@@ -3254,7 +3254,7 @@
         <v>shield</v>
       </c>
       <c r="L34" t="str">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M34" t="str">
         <v/>
@@ -3262,35 +3262,35 @@
       <c r="N34" t="str">
         <v/>
       </c>
-      <c r="O34" t="str">
+      <c r="P34" t="str">
+        <v/>
+      </c>
+      <c r="Q34" t="str">
+        <v/>
+      </c>
+      <c r="R34" t="str">
+        <v/>
+      </c>
+      <c r="S34" t="str">
+        <v/>
+      </c>
+      <c r="T34" t="str">
+        <v/>
+      </c>
+      <c r="U34" t="str">
+        <v/>
+      </c>
+      <c r="V34" t="str">
+        <v/>
+      </c>
+      <c r="W34" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="X34" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="Y34" t="str">
         <v>self</v>
-      </c>
-      <c r="U34" t="str">
-        <v/>
-      </c>
-      <c r="V34" t="str">
-        <v/>
-      </c>
-      <c r="W34" t="str">
-        <v/>
-      </c>
-      <c r="X34" t="str">
-        <v/>
-      </c>
-      <c r="Y34" t="str">
-        <v/>
-      </c>
-      <c r="Z34" t="str">
-        <v/>
-      </c>
-      <c r="AA34" t="str">
-        <v/>
-      </c>
-      <c r="AB34" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="AC34" t="str">
-        <v>Fire</v>
       </c>
     </row>
     <row r="35">
@@ -3307,7 +3307,7 @@
         <v>Spell</v>
       </c>
       <c r="E35" t="str">
-        <v>109</v>
+        <v>135</v>
       </c>
       <c r="F35" t="str">
         <v>3</v>
@@ -3327,6 +3327,9 @@
       <c r="M35" t="str">
         <v/>
       </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
       <c r="P35" t="str">
         <v/>
       </c>
@@ -3349,13 +3352,10 @@
         <v/>
       </c>
       <c r="W35" t="str">
-        <v/>
+        <v>Air</v>
       </c>
       <c r="X35" t="str">
-        <v/>
-      </c>
-      <c r="Y35" t="str">
-        <v/>
+        <v>Fire</v>
       </c>
       <c r="Z35" t="str">
         <v/>
@@ -3364,10 +3364,10 @@
         <v/>
       </c>
       <c r="AB35" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AC35" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -3384,7 +3384,7 @@
         <v>Spell</v>
       </c>
       <c r="E36" t="str">
-        <v>109</v>
+        <v>170</v>
       </c>
       <c r="F36" t="str">
         <v>4</v>
@@ -3404,6 +3404,9 @@
       <c r="M36" t="str">
         <v/>
       </c>
+      <c r="O36" t="str">
+        <v/>
+      </c>
       <c r="P36" t="str">
         <v/>
       </c>
@@ -3426,13 +3429,10 @@
         <v/>
       </c>
       <c r="W36" t="str">
-        <v/>
+        <v>Ice</v>
       </c>
       <c r="X36" t="str">
-        <v/>
-      </c>
-      <c r="Y36" t="str">
-        <v/>
+        <v>Fire</v>
       </c>
       <c r="Z36" t="str">
         <v/>
@@ -3441,10 +3441,10 @@
         <v/>
       </c>
       <c r="AB36" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
       <c r="AC36" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
     </row>
     <row r="37">
@@ -3481,12 +3481,21 @@
       <c r="M37" t="str">
         <v/>
       </c>
+      <c r="P37" t="str">
+        <v/>
+      </c>
+      <c r="Q37" t="str">
+        <v/>
+      </c>
       <c r="R37" t="str">
         <v/>
       </c>
       <c r="S37" t="str">
         <v/>
       </c>
+      <c r="T37" t="str">
+        <v/>
+      </c>
       <c r="U37" t="str">
         <v/>
       </c>
@@ -3494,25 +3503,16 @@
         <v/>
       </c>
       <c r="W37" t="str">
-        <v/>
+        <v>Fire</v>
       </c>
       <c r="X37" t="str">
-        <v/>
-      </c>
-      <c r="Y37" t="str">
-        <v/>
-      </c>
-      <c r="Z37" t="str">
-        <v/>
-      </c>
-      <c r="AA37" t="str">
-        <v/>
+        <v>Earth</v>
       </c>
       <c r="AB37" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
       <c r="AC37" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -3529,7 +3529,7 @@
         <v>Spell</v>
       </c>
       <c r="E38" t="str">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="F38" t="str">
         <v>3</v>
@@ -3562,46 +3562,46 @@
         <v>enemy</v>
       </c>
       <c r="P38" t="str">
+        <v/>
+      </c>
+      <c r="Q38" t="str">
+        <v/>
+      </c>
+      <c r="R38" t="str">
+        <v/>
+      </c>
+      <c r="S38" t="str">
+        <v/>
+      </c>
+      <c r="T38" t="str">
+        <v/>
+      </c>
+      <c r="U38" t="str">
+        <v/>
+      </c>
+      <c r="V38" t="str">
+        <v/>
+      </c>
+      <c r="W38" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="X38" t="str">
+        <v>Water</v>
+      </c>
+      <c r="Y38" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="Z38" t="str">
         <v>soak</v>
       </c>
-      <c r="Q38" t="str">
+      <c r="AA38" t="str">
         <v>2</v>
       </c>
-      <c r="R38" t="str">
-        <v/>
-      </c>
-      <c r="S38" t="str">
-        <v/>
-      </c>
-      <c r="T38" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="U38" t="str">
-        <v/>
-      </c>
-      <c r="V38" t="str">
-        <v/>
-      </c>
-      <c r="W38" t="str">
-        <v/>
-      </c>
-      <c r="X38" t="str">
-        <v/>
-      </c>
-      <c r="Y38" t="str">
-        <v/>
-      </c>
-      <c r="Z38" t="str">
-        <v/>
-      </c>
-      <c r="AA38" t="str">
-        <v/>
-      </c>
       <c r="AB38" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
       <c r="AC38" t="str">
-        <v>Water</v>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -3618,7 +3618,7 @@
         <v>Spell</v>
       </c>
       <c r="E39" t="str">
-        <v>58</v>
+        <v>190</v>
       </c>
       <c r="F39" t="str">
         <v>5</v>
@@ -3648,38 +3648,38 @@
         <v/>
       </c>
       <c r="O39" t="str">
+        <v/>
+      </c>
+      <c r="P39" t="str">
+        <v/>
+      </c>
+      <c r="Q39" t="str">
+        <v/>
+      </c>
+      <c r="R39" t="str">
+        <v/>
+      </c>
+      <c r="S39" t="str">
+        <v/>
+      </c>
+      <c r="T39" t="str">
+        <v/>
+      </c>
+      <c r="U39" t="str">
+        <v/>
+      </c>
+      <c r="V39" t="str">
+        <v/>
+      </c>
+      <c r="W39" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="X39" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="Y39" t="str">
         <v>enemy</v>
       </c>
-      <c r="P39" t="str">
-        <v/>
-      </c>
-      <c r="Q39" t="str">
-        <v/>
-      </c>
-      <c r="R39" t="str">
-        <v/>
-      </c>
-      <c r="S39" t="str">
-        <v/>
-      </c>
-      <c r="T39" t="str">
-        <v/>
-      </c>
-      <c r="U39" t="str">
-        <v/>
-      </c>
-      <c r="V39" t="str">
-        <v/>
-      </c>
-      <c r="W39" t="str">
-        <v/>
-      </c>
-      <c r="X39" t="str">
-        <v/>
-      </c>
-      <c r="Y39" t="str">
-        <v/>
-      </c>
       <c r="Z39" t="str">
         <v/>
       </c>
@@ -3687,10 +3687,10 @@
         <v/>
       </c>
       <c r="AB39" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
       <c r="AC39" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -3707,7 +3707,7 @@
         <v>Spell</v>
       </c>
       <c r="E40" t="str">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="F40" t="str">
         <v>5</v>
@@ -3737,38 +3737,38 @@
         <v/>
       </c>
       <c r="O40" t="str">
+        <v/>
+      </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
+      <c r="Q40" t="str">
+        <v/>
+      </c>
+      <c r="R40" t="str">
+        <v/>
+      </c>
+      <c r="S40" t="str">
+        <v/>
+      </c>
+      <c r="T40" t="str">
+        <v/>
+      </c>
+      <c r="U40" t="str">
+        <v/>
+      </c>
+      <c r="V40" t="str">
+        <v/>
+      </c>
+      <c r="W40" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="X40" t="str">
+        <v>Lightning</v>
+      </c>
+      <c r="Y40" t="str">
         <v>enemy</v>
       </c>
-      <c r="P40" t="str">
-        <v/>
-      </c>
-      <c r="Q40" t="str">
-        <v/>
-      </c>
-      <c r="R40" t="str">
-        <v/>
-      </c>
-      <c r="S40" t="str">
-        <v/>
-      </c>
-      <c r="T40" t="str">
-        <v/>
-      </c>
-      <c r="U40" t="str">
-        <v/>
-      </c>
-      <c r="V40" t="str">
-        <v/>
-      </c>
-      <c r="W40" t="str">
-        <v/>
-      </c>
-      <c r="X40" t="str">
-        <v/>
-      </c>
-      <c r="Y40" t="str">
-        <v/>
-      </c>
       <c r="Z40" t="str">
         <v/>
       </c>
@@ -3776,10 +3776,10 @@
         <v/>
       </c>
       <c r="AB40" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
       <c r="AC40" t="str">
-        <v>Lightning</v>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -3796,7 +3796,7 @@
         <v>Spell</v>
       </c>
       <c r="E41" t="str">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="F41" t="str">
         <v>3</v>
@@ -3817,7 +3817,7 @@
         <v>shield</v>
       </c>
       <c r="L41" t="str">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="M41" t="str">
         <v/>
@@ -3826,49 +3826,49 @@
         <v/>
       </c>
       <c r="O41" t="str">
+        <v>enemy</v>
+      </c>
+      <c r="P41" t="str">
+        <v/>
+      </c>
+      <c r="Q41" t="str">
+        <v/>
+      </c>
+      <c r="R41" t="str">
+        <v/>
+      </c>
+      <c r="S41" t="str">
+        <v/>
+      </c>
+      <c r="T41" t="str">
+        <v/>
+      </c>
+      <c r="U41" t="str">
+        <v/>
+      </c>
+      <c r="V41" t="str">
+        <v/>
+      </c>
+      <c r="W41" t="str">
+        <v>Water</v>
+      </c>
+      <c r="X41" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="Y41" t="str">
         <v>self</v>
       </c>
-      <c r="P41" t="str">
+      <c r="Z41" t="str">
         <v>soak</v>
       </c>
-      <c r="Q41" t="str">
+      <c r="AA41" t="str">
         <v>2</v>
       </c>
-      <c r="R41" t="str">
-        <v/>
-      </c>
-      <c r="S41" t="str">
-        <v/>
-      </c>
-      <c r="T41" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="U41" t="str">
-        <v/>
-      </c>
-      <c r="V41" t="str">
-        <v/>
-      </c>
-      <c r="W41" t="str">
-        <v/>
-      </c>
-      <c r="X41" t="str">
-        <v/>
-      </c>
-      <c r="Y41" t="str">
-        <v/>
-      </c>
-      <c r="Z41" t="str">
-        <v/>
-      </c>
-      <c r="AA41" t="str">
-        <v/>
-      </c>
       <c r="AB41" t="str">
-        <v>Water</v>
+        <v/>
       </c>
       <c r="AC41" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
     </row>
     <row r="42">
@@ -3885,7 +3885,7 @@
         <v>Spell</v>
       </c>
       <c r="E42" t="str">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="F42" t="str">
         <v>3</v>
@@ -3939,10 +3939,10 @@
         <v/>
       </c>
       <c r="W42" t="str">
-        <v/>
+        <v>Air</v>
       </c>
       <c r="X42" t="str">
-        <v/>
+        <v>Air</v>
       </c>
       <c r="Y42" t="str">
         <v/>
@@ -3954,10 +3954,10 @@
         <v/>
       </c>
       <c r="AB42" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AC42" t="str">
-        <v>Air</v>
+        <v/>
       </c>
     </row>
     <row r="43">
@@ -3974,7 +3974,7 @@
         <v>Spell</v>
       </c>
       <c r="E43" t="str">
-        <v>58</v>
+        <v>165</v>
       </c>
       <c r="F43" t="str">
         <v>4</v>
@@ -4028,10 +4028,10 @@
         <v/>
       </c>
       <c r="W43" t="str">
-        <v/>
+        <v>Air</v>
       </c>
       <c r="X43" t="str">
-        <v/>
+        <v>Ice</v>
       </c>
       <c r="Y43" t="str">
         <v/>
@@ -4043,10 +4043,10 @@
         <v/>
       </c>
       <c r="AB43" t="str">
-        <v>Air</v>
+        <v/>
       </c>
       <c r="AC43" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -4063,7 +4063,7 @@
         <v>Spell</v>
       </c>
       <c r="E44" t="str">
-        <v>126</v>
+        <v>75</v>
       </c>
       <c r="F44" t="str">
         <v>1</v>
@@ -4093,38 +4093,38 @@
         <v>3</v>
       </c>
       <c r="O44" t="str">
+        <v/>
+      </c>
+      <c r="P44" t="str">
+        <v/>
+      </c>
+      <c r="Q44" t="str">
+        <v/>
+      </c>
+      <c r="R44" t="str">
+        <v/>
+      </c>
+      <c r="S44" t="str">
+        <v/>
+      </c>
+      <c r="T44" t="str">
+        <v/>
+      </c>
+      <c r="U44" t="str">
+        <v/>
+      </c>
+      <c r="V44" t="str">
+        <v/>
+      </c>
+      <c r="W44" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="X44" t="str">
+        <v>Fire</v>
+      </c>
+      <c r="Y44" t="str">
         <v>enemy</v>
       </c>
-      <c r="P44" t="str">
-        <v/>
-      </c>
-      <c r="Q44" t="str">
-        <v/>
-      </c>
-      <c r="R44" t="str">
-        <v/>
-      </c>
-      <c r="S44" t="str">
-        <v/>
-      </c>
-      <c r="T44" t="str">
-        <v/>
-      </c>
-      <c r="U44" t="str">
-        <v/>
-      </c>
-      <c r="V44" t="str">
-        <v/>
-      </c>
-      <c r="W44" t="str">
-        <v/>
-      </c>
-      <c r="X44" t="str">
-        <v/>
-      </c>
-      <c r="Y44" t="str">
-        <v/>
-      </c>
       <c r="Z44" t="str">
         <v/>
       </c>
@@ -4132,10 +4132,10 @@
         <v/>
       </c>
       <c r="AB44" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
       <c r="AC44" t="str">
-        <v>Fire</v>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -4152,7 +4152,7 @@
         <v>Spell</v>
       </c>
       <c r="E45" t="str">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F45" t="str">
         <v>3</v>
@@ -4173,7 +4173,7 @@
         <v>shield</v>
       </c>
       <c r="L45" t="str">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="M45" t="str">
         <v/>
@@ -4182,38 +4182,38 @@
         <v/>
       </c>
       <c r="O45" t="str">
+        <v/>
+      </c>
+      <c r="P45" t="str">
+        <v/>
+      </c>
+      <c r="Q45" t="str">
+        <v/>
+      </c>
+      <c r="R45" t="str">
+        <v/>
+      </c>
+      <c r="S45" t="str">
+        <v/>
+      </c>
+      <c r="T45" t="str">
+        <v/>
+      </c>
+      <c r="U45" t="str">
+        <v/>
+      </c>
+      <c r="V45" t="str">
+        <v/>
+      </c>
+      <c r="W45" t="str">
+        <v>Ice</v>
+      </c>
+      <c r="X45" t="str">
+        <v>Earth</v>
+      </c>
+      <c r="Y45" t="str">
         <v>self</v>
       </c>
-      <c r="P45" t="str">
-        <v/>
-      </c>
-      <c r="Q45" t="str">
-        <v/>
-      </c>
-      <c r="R45" t="str">
-        <v/>
-      </c>
-      <c r="S45" t="str">
-        <v/>
-      </c>
-      <c r="T45" t="str">
-        <v/>
-      </c>
-      <c r="U45" t="str">
-        <v/>
-      </c>
-      <c r="V45" t="str">
-        <v/>
-      </c>
-      <c r="W45" t="str">
-        <v/>
-      </c>
-      <c r="X45" t="str">
-        <v/>
-      </c>
-      <c r="Y45" t="str">
-        <v/>
-      </c>
       <c r="Z45" t="str">
         <v/>
       </c>
@@ -4221,10 +4221,10 @@
         <v/>
       </c>
       <c r="AB45" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
       <c r="AC45" t="str">
-        <v>Earth</v>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -4241,7 +4241,7 @@
         <v>Spell</v>
       </c>
       <c r="E46" t="str">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="F46" t="str">
         <v>3</v>
@@ -4295,10 +4295,10 @@
         <v/>
       </c>
       <c r="W46" t="str">
-        <v/>
+        <v>Ice</v>
       </c>
       <c r="X46" t="str">
-        <v/>
+        <v>Ice</v>
       </c>
       <c r="Y46" t="str">
         <v/>
@@ -4310,10 +4310,10 @@
         <v/>
       </c>
       <c r="AB46" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
       <c r="AC46" t="str">
-        <v>Ice</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Build: (0f5a2f9) Update rewards to increase as you unlock new elements
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -460,33 +460,6 @@
       <c r="T1" t="str">
         <v>Effect 3 Target</v>
       </c>
-      <c r="U1" t="str">
-        <v>__EMPTY</v>
-      </c>
-      <c r="V1" t="str">
-        <v>__EMPTY_1</v>
-      </c>
-      <c r="W1" t="str">
-        <v>Type 1</v>
-      </c>
-      <c r="X1" t="str">
-        <v>Type 2</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>Effect 1 Target</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>Effect 2 Kind</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>Effect 2 Amount</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>Effect 2 Hits</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>Effect 2 Duration</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -632,9 +605,6 @@
       <c r="W3" t="str">
         <v/>
       </c>
-      <c r="X3" t="str">
-        <v>Leaf</v>
-      </c>
       <c r="Y3" t="str">
         <v/>
       </c>
@@ -1516,14 +1486,8 @@
       <c r="V13" t="str">
         <v/>
       </c>
-      <c r="W13" t="str">
-        <v>Leaf</v>
-      </c>
       <c r="X13" t="str">
         <v/>
-      </c>
-      <c r="Y13" t="str">
-        <v>self</v>
       </c>
       <c r="Z13" t="str">
         <v/>
@@ -1961,15 +1925,6 @@
       <c r="V18" t="str">
         <v/>
       </c>
-      <c r="W18" t="str">
-        <v>Water</v>
-      </c>
-      <c r="X18" t="str">
-        <v>Water</v>
-      </c>
-      <c r="Y18" t="str">
-        <v>enemy</v>
-      </c>
       <c r="Z18" t="str">
         <v/>
       </c>
@@ -2047,15 +2002,6 @@
       <c r="V19" t="str">
         <v/>
       </c>
-      <c r="W19" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="X19" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="Y19" t="str">
-        <v>enemy</v>
-      </c>
       <c r="AB19" t="str">
         <v/>
       </c>
@@ -2127,15 +2073,6 @@
       <c r="V20" t="str">
         <v/>
       </c>
-      <c r="W20" t="str">
-        <v>Water</v>
-      </c>
-      <c r="X20" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="Y20" t="str">
-        <v>self</v>
-      </c>
       <c r="AB20" t="str">
         <v/>
       </c>
@@ -2207,15 +2144,6 @@
       <c r="V21" t="str">
         <v/>
       </c>
-      <c r="W21" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="X21" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="Y21" t="str">
-        <v>self</v>
-      </c>
       <c r="AB21" t="str">
         <v/>
       </c>
@@ -2290,15 +2218,6 @@
       <c r="V22" t="str">
         <v/>
       </c>
-      <c r="W22" t="str">
-        <v>Air</v>
-      </c>
-      <c r="X22" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="Y22" t="str">
-        <v>self</v>
-      </c>
       <c r="Z22" t="str">
         <v/>
       </c>
@@ -2379,15 +2298,6 @@
       <c r="V23" t="str">
         <v/>
       </c>
-      <c r="W23" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="X23" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="Y23" t="str">
-        <v>self</v>
-      </c>
       <c r="Z23" t="str">
         <v/>
       </c>
@@ -2465,15 +2375,6 @@
       <c r="V24" t="str">
         <v/>
       </c>
-      <c r="W24" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="X24" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="Y24" t="str">
-        <v>self</v>
-      </c>
       <c r="AB24" t="str">
         <v/>
       </c>
@@ -2545,15 +2446,6 @@
       <c r="V25" t="str">
         <v/>
       </c>
-      <c r="W25" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="X25" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="Y25" t="str">
-        <v>self</v>
-      </c>
       <c r="AB25" t="str">
         <v/>
       </c>
@@ -2625,15 +2517,6 @@
       <c r="V26" t="str">
         <v/>
       </c>
-      <c r="W26" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="X26" t="str">
-        <v>Leaf</v>
-      </c>
-      <c r="Y26" t="str">
-        <v>enemy</v>
-      </c>
       <c r="AB26" t="str">
         <v/>
       </c>
@@ -2705,15 +2588,6 @@
       <c r="V27" t="str">
         <v/>
       </c>
-      <c r="W27" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="X27" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="Y27" t="str">
-        <v>self</v>
-      </c>
       <c r="AB27" t="str">
         <v/>
       </c>
@@ -2788,14 +2662,8 @@
       <c r="V28" t="str">
         <v/>
       </c>
-      <c r="W28" t="str">
-        <v>Earth</v>
-      </c>
       <c r="X28" t="str">
         <v/>
-      </c>
-      <c r="Y28" t="str">
-        <v>self</v>
       </c>
       <c r="Z28" t="str">
         <v/>
@@ -2877,15 +2745,6 @@
       <c r="V29" t="str">
         <v/>
       </c>
-      <c r="W29" t="str">
-        <v>Air</v>
-      </c>
-      <c r="X29" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="Y29" t="str">
-        <v>self</v>
-      </c>
       <c r="Z29" t="str">
         <v/>
       </c>
@@ -2966,15 +2825,6 @@
       <c r="V30" t="str">
         <v/>
       </c>
-      <c r="W30" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="X30" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="Y30" t="str">
-        <v>self</v>
-      </c>
       <c r="Z30" t="str">
         <v/>
       </c>
@@ -3052,15 +2902,6 @@
       <c r="V31" t="str">
         <v/>
       </c>
-      <c r="W31" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="X31" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="Y31" t="str">
-        <v>enemy</v>
-      </c>
       <c r="AB31" t="str">
         <v/>
       </c>
@@ -3132,15 +2973,6 @@
       <c r="V32" t="str">
         <v/>
       </c>
-      <c r="W32" t="str">
-        <v>Water</v>
-      </c>
-      <c r="X32" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="Y32" t="str">
-        <v>enemy</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -3206,15 +3038,6 @@
       <c r="V33" t="str">
         <v/>
       </c>
-      <c r="W33" t="str">
-        <v>Lightning</v>
-      </c>
-      <c r="X33" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="Y33" t="str">
-        <v>enemy</v>
-      </c>
       <c r="AB33" t="str">
         <v/>
       </c>
@@ -3283,15 +3106,6 @@
       <c r="V34" t="str">
         <v/>
       </c>
-      <c r="W34" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="X34" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="Y34" t="str">
-        <v>self</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -3351,12 +3165,6 @@
       <c r="V35" t="str">
         <v/>
       </c>
-      <c r="W35" t="str">
-        <v>Air</v>
-      </c>
-      <c r="X35" t="str">
-        <v>Fire</v>
-      </c>
       <c r="Z35" t="str">
         <v/>
       </c>
@@ -3428,12 +3236,6 @@
       <c r="V36" t="str">
         <v/>
       </c>
-      <c r="W36" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="X36" t="str">
-        <v>Fire</v>
-      </c>
       <c r="Z36" t="str">
         <v/>
       </c>
@@ -3502,12 +3304,6 @@
       <c r="V37" t="str">
         <v/>
       </c>
-      <c r="W37" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="X37" t="str">
-        <v>Earth</v>
-      </c>
       <c r="AB37" t="str">
         <v/>
       </c>
@@ -3582,21 +3378,6 @@
       <c r="V38" t="str">
         <v/>
       </c>
-      <c r="W38" t="str">
-        <v>Lightning</v>
-      </c>
-      <c r="X38" t="str">
-        <v>Water</v>
-      </c>
-      <c r="Y38" t="str">
-        <v>enemy</v>
-      </c>
-      <c r="Z38" t="str">
-        <v>soak</v>
-      </c>
-      <c r="AA38" t="str">
-        <v>2</v>
-      </c>
       <c r="AB38" t="str">
         <v/>
       </c>
@@ -3671,15 +3452,6 @@
       <c r="V39" t="str">
         <v/>
       </c>
-      <c r="W39" t="str">
-        <v>Lightning</v>
-      </c>
-      <c r="X39" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="Y39" t="str">
-        <v>enemy</v>
-      </c>
       <c r="Z39" t="str">
         <v/>
       </c>
@@ -3760,15 +3532,6 @@
       <c r="V40" t="str">
         <v/>
       </c>
-      <c r="W40" t="str">
-        <v>Lightning</v>
-      </c>
-      <c r="X40" t="str">
-        <v>Lightning</v>
-      </c>
-      <c r="Y40" t="str">
-        <v>enemy</v>
-      </c>
       <c r="Z40" t="str">
         <v/>
       </c>
@@ -3849,21 +3612,6 @@
       <c r="V41" t="str">
         <v/>
       </c>
-      <c r="W41" t="str">
-        <v>Water</v>
-      </c>
-      <c r="X41" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="Y41" t="str">
-        <v>self</v>
-      </c>
-      <c r="Z41" t="str">
-        <v>soak</v>
-      </c>
-      <c r="AA41" t="str">
-        <v>2</v>
-      </c>
       <c r="AB41" t="str">
         <v/>
       </c>
@@ -3938,12 +3686,6 @@
       <c r="V42" t="str">
         <v/>
       </c>
-      <c r="W42" t="str">
-        <v>Air</v>
-      </c>
-      <c r="X42" t="str">
-        <v>Air</v>
-      </c>
       <c r="Y42" t="str">
         <v/>
       </c>
@@ -4027,12 +3769,6 @@
       <c r="V43" t="str">
         <v/>
       </c>
-      <c r="W43" t="str">
-        <v>Air</v>
-      </c>
-      <c r="X43" t="str">
-        <v>Ice</v>
-      </c>
       <c r="Y43" t="str">
         <v/>
       </c>
@@ -4116,15 +3852,6 @@
       <c r="V44" t="str">
         <v/>
       </c>
-      <c r="W44" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="X44" t="str">
-        <v>Fire</v>
-      </c>
-      <c r="Y44" t="str">
-        <v>enemy</v>
-      </c>
       <c r="Z44" t="str">
         <v/>
       </c>
@@ -4205,15 +3932,6 @@
       <c r="V45" t="str">
         <v/>
       </c>
-      <c r="W45" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="X45" t="str">
-        <v>Earth</v>
-      </c>
-      <c r="Y45" t="str">
-        <v>self</v>
-      </c>
       <c r="Z45" t="str">
         <v/>
       </c>
@@ -4293,12 +4011,6 @@
       </c>
       <c r="V46" t="str">
         <v/>
-      </c>
-      <c r="W46" t="str">
-        <v>Ice</v>
-      </c>
-      <c r="X46" t="str">
-        <v>Ice</v>
       </c>
       <c r="Y46" t="str">
         <v/>

</xml_diff>

<commit_message>
Build: (cd095f4) Minor QoL Updates
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -633,7 +633,7 @@
         <v>10</v>
       </c>
       <c r="F6" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" t="str">
         <v>1</v>
@@ -643,6 +643,15 @@
       </c>
       <c r="I6" t="str">
         <v>Air</v>
+      </c>
+      <c r="K6" t="str">
+        <v>combo</v>
+      </c>
+      <c r="L6" t="str">
+        <v>1</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Fire</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Build: (7df739b) A bunch of little QoL changes
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -505,13 +505,13 @@
         <v>Water</v>
       </c>
       <c r="K2" t="str">
-        <v>soak</v>
+        <v>shield</v>
       </c>
       <c r="L2" t="str">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N2" t="str">
-        <v>1</v>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -549,7 +549,7 @@
         <v>1</v>
       </c>
       <c r="N3" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -557,10 +557,10 @@
         <v>Earth</v>
       </c>
       <c r="B4" t="str">
-        <v>Sand</v>
+        <v>Light</v>
       </c>
       <c r="C4" t="str">
-        <v>Sand</v>
+        <v>Water</v>
       </c>
       <c r="D4" t="str">
         <v>Element</v>
@@ -572,19 +572,22 @@
         <v>0</v>
       </c>
       <c r="G4" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" t="str">
-        <v>It's a rock</v>
+        <v>It's a leaf</v>
       </c>
       <c r="I4" t="str">
         <v>Earth</v>
       </c>
       <c r="K4" t="str">
-        <v>shield</v>
+        <v>energize</v>
       </c>
       <c r="L4" t="str">
-        <v>5</v>
+        <v>1</v>
+      </c>
+      <c r="N4" t="str">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -636,7 +639,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6" t="str">
         <v>A cool rush of wind drifts past your face</v>
@@ -1070,7 +1073,7 @@
         <v>10</v>
       </c>
       <c r="N19" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -1111,7 +1114,7 @@
         <v>4</v>
       </c>
       <c r="N20" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -1152,7 +1155,7 @@
         <v>6</v>
       </c>
       <c r="N21" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P21" t="str">
         <v>energize</v>
@@ -1308,7 +1311,7 @@
         <v>6</v>
       </c>
       <c r="N24" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -1349,7 +1352,7 @@
         <v>2</v>
       </c>
       <c r="N25" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -1519,7 +1522,7 @@
         <v>2</v>
       </c>
       <c r="N29" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P29" t="str">
         <v>energize</v>
@@ -1793,6 +1796,9 @@
       <c r="K36" t="str">
         <v>freeze</v>
       </c>
+      <c r="N36" t="str">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2030,6 +2036,9 @@
       <c r="K42" t="str">
         <v>freeze</v>
       </c>
+      <c r="N42" t="str">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2064,6 +2073,9 @@
       </c>
       <c r="K43" t="str">
         <v>freeze</v>
+      </c>
+      <c r="N43" t="str">
+        <v>1</v>
       </c>
     </row>
     <row r="44">

</xml_diff>

<commit_message>
Build: (cab4446) Pipeline fix
</commit_message>
<xml_diff>
--- a/elements.xlsx
+++ b/elements.xlsx
@@ -490,7 +490,7 @@
         <v>Element</v>
       </c>
       <c r="E2" t="str">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F2" t="str">
         <v>0</v>
@@ -503,12 +503,6 @@
       </c>
       <c r="I2" t="str">
         <v>Water</v>
-      </c>
-      <c r="K2" t="str">
-        <v>shield</v>
-      </c>
-      <c r="L2" t="str">
-        <v>5</v>
       </c>
       <c r="N2" t="str">
         <v/>
@@ -534,22 +528,13 @@
         <v>0</v>
       </c>
       <c r="G3" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="str">
         <v>A bright flame burning hot</v>
       </c>
       <c r="I3" t="str">
         <v>Fire</v>
-      </c>
-      <c r="K3" t="str">
-        <v>burn</v>
-      </c>
-      <c r="L3" t="str">
-        <v>1</v>
-      </c>
-      <c r="N3" t="str">
-        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -566,28 +551,19 @@
         <v>Element</v>
       </c>
       <c r="E4" t="str">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F4" t="str">
         <v>0</v>
       </c>
       <c r="G4" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H4" t="str">
         <v>It's a leaf</v>
       </c>
       <c r="I4" t="str">
         <v>Earth</v>
-      </c>
-      <c r="K4" t="str">
-        <v>energize</v>
-      </c>
-      <c r="L4" t="str">
-        <v>1</v>
-      </c>
-      <c r="N4" t="str">
-        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -639,22 +615,13 @@
         <v>0</v>
       </c>
       <c r="G6" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" t="str">
         <v>A cool rush of wind drifts past your face</v>
       </c>
       <c r="I6" t="str">
         <v>Air</v>
-      </c>
-      <c r="K6" t="str">
-        <v>combo</v>
-      </c>
-      <c r="L6" t="str">
-        <v>1</v>
-      </c>
-      <c r="O6" t="str">
-        <v>Fire</v>
       </c>
     </row>
     <row r="7">

</xml_diff>